<commit_message>
Removed grids, added fragile walls
</commit_message>
<xml_diff>
--- a/Translations/Translations.xlsx
+++ b/Translations/Translations.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programacion\MelonLoader\FS_LevelEditor\Translations\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Codes\c#\FrSLE\Translations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51C7A83E-5509-4020-9352-7F868F992264}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C40685B5-79CC-44E2-9567-3C747D734598}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{F5C22481-FF1A-482C-BF7E-EB5A7718AF49}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15900" xr2:uid="{F5C22481-FF1A-482C-BF7E-EB5A7718AF49}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="557" uniqueCount="512">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="563" uniqueCount="518">
   <si>
     <t>ID</t>
   </si>
@@ -1570,6 +1570,24 @@
   </si>
   <si>
     <t>DESBLOQUEADA</t>
+  </si>
+  <si>
+    <t>object.DESTRUCTIBLE_WALL</t>
+  </si>
+  <si>
+    <t>Fragile Wall</t>
+  </si>
+  <si>
+    <t>Крихка стіна</t>
+  </si>
+  <si>
+    <t>events.OnBreak</t>
+  </si>
+  <si>
+    <t>On Break</t>
+  </si>
+  <si>
+    <t>При розваленні</t>
   </si>
 </sst>
 </file>
@@ -1656,7 +1674,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Звичайний" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1672,9 +1690,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Тема &quot;Office 2013 – 2022&quot;">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013–2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1712,7 +1730,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013–2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1818,7 +1836,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013–2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1960,7 +1978,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1969,8 +1987,8 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6961A5F-F8EA-4989-8112-A0ACE51D011E}">
   <sheetPr codeName="Hoja1"/>
-  <dimension ref="A1:D145"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:D147"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="37" style="2" customWidth="1"/>
     <col min="2" max="4" width="45.7109375" style="2" customWidth="1"/>
@@ -2667,1274 +2685,1296 @@
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
-        <v>69</v>
+        <v>512</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="C51" s="2" t="s">
-        <v>101</v>
+        <v>513</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>365</v>
+        <v>514</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
-        <v>105</v>
+        <v>69</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>2</v>
+        <v>69</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A55" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>111</v>
+        <v>4</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57" s="2" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" s="2" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
-        <v>446</v>
+        <v>118</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>447</v>
+        <v>122</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>460</v>
+        <v>121</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>448</v>
+        <v>371</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61" s="2" t="s">
-        <v>154</v>
+        <v>446</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>155</v>
+        <v>447</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>156</v>
+        <v>460</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>372</v>
+        <v>448</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" s="2" t="s">
-        <v>164</v>
+        <v>515</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>165</v>
-      </c>
-      <c r="C62" s="2" t="s">
-        <v>166</v>
+        <v>516</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>373</v>
+        <v>517</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63" s="2" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" s="2" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A65" s="2" t="s">
-        <v>141</v>
+        <v>157</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>142</v>
+        <v>158</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>143</v>
+        <v>159</v>
       </c>
       <c r="D65" s="2" t="s">
-        <v>376</v>
-      </c>
-    </row>
-    <row r="66" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66" s="2" t="s">
-        <v>144</v>
+        <v>167</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>145</v>
+        <v>169</v>
       </c>
       <c r="D66" s="2" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A67" s="2" t="s">
-        <v>153</v>
+        <v>141</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="D67" s="2" t="s">
-        <v>329</v>
-      </c>
-    </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A68" s="2" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>148</v>
+        <v>163</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="D68" s="2" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A69" s="2" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="D69" s="2" t="s">
-        <v>379</v>
+        <v>329</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A70" s="2" t="s">
-        <v>172</v>
+        <v>147</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>170</v>
+        <v>148</v>
       </c>
       <c r="C70" s="2" t="s">
-        <v>171</v>
+        <v>149</v>
       </c>
       <c r="D70" s="2" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A71" s="2" t="s">
-        <v>173</v>
+        <v>150</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>174</v>
+        <v>151</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>175</v>
+        <v>152</v>
       </c>
       <c r="D71" s="2" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A72" s="2" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="D72" s="2" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A73" s="2" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="C73" s="2" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="D73" s="2" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A74" s="2" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="C74" s="2" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="D74" s="2" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A75" s="2" t="s">
-        <v>244</v>
+        <v>178</v>
       </c>
       <c r="B75" s="2" t="s">
-        <v>244</v>
+        <v>178</v>
       </c>
       <c r="C75" s="2" t="s">
-        <v>95</v>
+        <v>179</v>
       </c>
       <c r="D75" s="2" t="s">
-        <v>385</v>
-      </c>
-    </row>
-    <row r="76" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A76" s="2" t="s">
-        <v>138</v>
-      </c>
-      <c r="B76" s="1" t="s">
-        <v>140</v>
+        <v>180</v>
+      </c>
+      <c r="B76" s="2" t="s">
+        <v>180</v>
       </c>
       <c r="C76" s="2" t="s">
-        <v>139</v>
+        <v>181</v>
       </c>
       <c r="D76" s="2" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A77" s="2" t="s">
-        <v>182</v>
+        <v>244</v>
       </c>
       <c r="B77" s="2" t="s">
-        <v>183</v>
+        <v>244</v>
       </c>
       <c r="C77" s="2" t="s">
-        <v>183</v>
+        <v>95</v>
       </c>
       <c r="D77" s="2" t="s">
-        <v>387</v>
-      </c>
-    </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A78" s="2" t="s">
-        <v>184</v>
-      </c>
-      <c r="B78" s="2" t="s">
-        <v>184</v>
+        <v>138</v>
+      </c>
+      <c r="B78" s="1" t="s">
+        <v>140</v>
       </c>
       <c r="C78" s="2" t="s">
-        <v>185</v>
+        <v>139</v>
       </c>
       <c r="D78" s="2" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A79" s="2" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="B79" s="2" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="C79" s="2" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="D79" s="2" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="B80" s="2" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
       <c r="C80" s="2" t="s">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="D80" s="2" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A81" s="2" t="s">
-        <v>191</v>
+        <v>186</v>
       </c>
       <c r="B81" s="2" t="s">
-        <v>191</v>
+        <v>186</v>
       </c>
       <c r="C81" s="2" t="s">
-        <v>192</v>
+        <v>187</v>
       </c>
       <c r="D81" s="2" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A82" s="2" t="s">
-        <v>193</v>
+        <v>188</v>
       </c>
       <c r="B82" s="2" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="C82" s="2" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
       <c r="D82" s="2" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A83" s="2" t="s">
-        <v>435</v>
-      </c>
-      <c r="B83" s="4" t="s">
-        <v>436</v>
-      </c>
-      <c r="C83" s="4" t="s">
-        <v>437</v>
+        <v>191</v>
+      </c>
+      <c r="B83" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="C83" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="D83" s="2" t="s">
+        <v>391</v>
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A84" s="2" t="s">
-        <v>438</v>
-      </c>
-      <c r="B84" s="4" t="s">
-        <v>439</v>
-      </c>
-      <c r="C84" s="4" t="s">
-        <v>440</v>
+        <v>193</v>
+      </c>
+      <c r="B84" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="C84" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="D84" s="2" t="s">
+        <v>392</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A85" s="2" t="s">
-        <v>474</v>
+        <v>435</v>
       </c>
       <c r="B85" s="4" t="s">
-        <v>475</v>
+        <v>436</v>
       </c>
       <c r="C85" s="4" t="s">
-        <v>476</v>
+        <v>437</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A86" s="2" t="s">
-        <v>196</v>
-      </c>
-      <c r="B86" s="2" t="s">
-        <v>197</v>
-      </c>
-      <c r="C86" s="2" t="s">
-        <v>198</v>
-      </c>
-      <c r="D86" s="2" t="s">
-        <v>393</v>
+        <v>438</v>
+      </c>
+      <c r="B86" s="4" t="s">
+        <v>439</v>
+      </c>
+      <c r="C86" s="4" t="s">
+        <v>440</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A87" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="B87" s="2" t="s">
-        <v>200</v>
-      </c>
-      <c r="C87" s="2" t="s">
-        <v>201</v>
-      </c>
-      <c r="D87" s="2" t="s">
-        <v>394</v>
+        <v>474</v>
+      </c>
+      <c r="B87" s="4" t="s">
+        <v>475</v>
+      </c>
+      <c r="C87" s="4" t="s">
+        <v>476</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A88" s="2" t="s">
-        <v>202</v>
+        <v>196</v>
       </c>
       <c r="B88" s="2" t="s">
-        <v>202</v>
+        <v>197</v>
       </c>
       <c r="C88" s="2" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
       <c r="D88" s="2" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A89" s="2" t="s">
-        <v>204</v>
+        <v>199</v>
       </c>
       <c r="B89" s="2" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="C89" s="2" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="D89" s="2" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A90" s="2" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="B90" s="2" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="C90" s="2" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="D90" s="2" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A91" s="2" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="B91" s="2" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
       <c r="C91" s="2" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="D91" s="2" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A92" s="2" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="B92" s="2" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="C92" s="2" t="s">
-        <v>212</v>
+        <v>206</v>
       </c>
       <c r="D92" s="2" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A93" s="2" t="s">
-        <v>213</v>
+        <v>207</v>
       </c>
       <c r="B93" s="2" t="s">
-        <v>214</v>
+        <v>208</v>
       </c>
       <c r="C93" s="2" t="s">
-        <v>215</v>
+        <v>209</v>
       </c>
       <c r="D93" s="2" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A94" s="2" t="s">
-        <v>216</v>
+        <v>210</v>
       </c>
       <c r="B94" s="2" t="s">
-        <v>217</v>
+        <v>211</v>
       </c>
       <c r="C94" s="2" t="s">
-        <v>218</v>
+        <v>212</v>
       </c>
       <c r="D94" s="2" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A95" s="2" t="s">
-        <v>221</v>
+        <v>213</v>
       </c>
       <c r="B95" s="2" t="s">
-        <v>220</v>
+        <v>214</v>
       </c>
       <c r="C95" s="2" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
       <c r="D95" s="2" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A96" s="2" t="s">
-        <v>293</v>
+        <v>216</v>
       </c>
       <c r="B96" s="2" t="s">
-        <v>293</v>
+        <v>217</v>
       </c>
       <c r="C96" s="2" t="s">
-        <v>294</v>
+        <v>218</v>
       </c>
       <c r="D96" s="2" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A97" s="2" t="s">
-        <v>295</v>
+        <v>221</v>
       </c>
       <c r="B97" s="2" t="s">
-        <v>296</v>
+        <v>220</v>
       </c>
       <c r="C97" s="2" t="s">
-        <v>297</v>
+        <v>219</v>
       </c>
       <c r="D97" s="2" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A98" s="2" t="s">
-        <v>298</v>
+        <v>293</v>
       </c>
       <c r="B98" s="2" t="s">
-        <v>299</v>
+        <v>293</v>
       </c>
       <c r="C98" s="2" t="s">
-        <v>300</v>
+        <v>294</v>
       </c>
       <c r="D98" s="2" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A99" s="2" t="s">
-        <v>222</v>
+        <v>295</v>
       </c>
       <c r="B99" s="2" t="s">
-        <v>222</v>
+        <v>296</v>
       </c>
       <c r="C99" s="2" t="s">
-        <v>223</v>
+        <v>297</v>
       </c>
       <c r="D99" s="2" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A100" s="2" t="s">
-        <v>224</v>
+        <v>298</v>
       </c>
       <c r="B100" s="2" t="s">
-        <v>225</v>
+        <v>299</v>
       </c>
       <c r="C100" s="2" t="s">
-        <v>226</v>
+        <v>300</v>
       </c>
       <c r="D100" s="2" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A101" s="2" t="s">
-        <v>227</v>
+        <v>222</v>
       </c>
       <c r="B101" s="2" t="s">
-        <v>228</v>
+        <v>222</v>
       </c>
       <c r="C101" s="2" t="s">
-        <v>229</v>
+        <v>223</v>
       </c>
       <c r="D101" s="2" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A102" s="2" t="s">
-        <v>230</v>
+        <v>224</v>
       </c>
       <c r="B102" s="2" t="s">
-        <v>230</v>
+        <v>225</v>
       </c>
       <c r="C102" s="2" t="s">
-        <v>230</v>
+        <v>226</v>
       </c>
       <c r="D102" s="2" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A103" s="2" t="s">
-        <v>231</v>
+        <v>227</v>
       </c>
       <c r="B103" s="2" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="C103" s="2" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="D103" s="2" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A104" s="2" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="B104" s="2" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="C104" s="2" t="s">
-        <v>234</v>
+        <v>230</v>
       </c>
       <c r="D104" s="2" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A105" s="2" t="s">
-        <v>235</v>
+        <v>231</v>
       </c>
       <c r="B105" s="2" t="s">
-        <v>236</v>
+        <v>231</v>
       </c>
       <c r="C105" s="2" t="s">
-        <v>237</v>
+        <v>232</v>
       </c>
       <c r="D105" s="2" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A106" s="2" t="s">
-        <v>238</v>
+        <v>233</v>
       </c>
       <c r="B106" s="2" t="s">
-        <v>239</v>
+        <v>233</v>
       </c>
       <c r="C106" s="2" t="s">
-        <v>240</v>
+        <v>234</v>
       </c>
       <c r="D106" s="2" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A107" s="2" t="s">
-        <v>301</v>
+        <v>235</v>
       </c>
       <c r="B107" s="2" t="s">
-        <v>302</v>
+        <v>236</v>
       </c>
       <c r="C107" s="2" t="s">
-        <v>303</v>
+        <v>237</v>
       </c>
       <c r="D107" s="2" t="s">
-        <v>414</v>
+        <v>412</v>
       </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A108" s="2" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="B108" s="2" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="C108" s="2" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="D108" s="2" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A109" s="2" t="s">
-        <v>245</v>
+        <v>301</v>
       </c>
       <c r="B109" s="2" t="s">
-        <v>253</v>
+        <v>302</v>
       </c>
       <c r="C109" s="2" t="s">
-        <v>252</v>
+        <v>303</v>
       </c>
       <c r="D109" s="2" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A110" s="2" t="s">
-        <v>246</v>
+        <v>241</v>
       </c>
       <c r="B110" s="2" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="C110" s="2" t="s">
-        <v>247</v>
+        <v>243</v>
       </c>
       <c r="D110" s="2" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A111" s="2" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="B111" s="2" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
       <c r="C111" s="2" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="D111" s="2" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A112" s="2" t="s">
-        <v>250</v>
+        <v>246</v>
       </c>
       <c r="B112" s="2" t="s">
-        <v>250</v>
+        <v>246</v>
       </c>
       <c r="C112" s="2" t="s">
-        <v>251</v>
+        <v>247</v>
       </c>
       <c r="D112" s="2" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A113" s="2" t="s">
-        <v>254</v>
+        <v>248</v>
       </c>
       <c r="B113" s="2" t="s">
-        <v>255</v>
+        <v>248</v>
       </c>
       <c r="C113" s="2" t="s">
-        <v>256</v>
+        <v>249</v>
       </c>
       <c r="D113" s="2" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A114" s="2" t="s">
-        <v>257</v>
+        <v>250</v>
       </c>
       <c r="B114" s="2" t="s">
-        <v>258</v>
+        <v>250</v>
       </c>
       <c r="C114" s="2" t="s">
-        <v>259</v>
+        <v>251</v>
       </c>
       <c r="D114" s="2" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A115" s="2" t="s">
-        <v>260</v>
+        <v>254</v>
       </c>
       <c r="B115" s="2" t="s">
-        <v>261</v>
+        <v>255</v>
       </c>
       <c r="C115" s="2" t="s">
-        <v>262</v>
+        <v>256</v>
       </c>
       <c r="D115" s="2" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A116" s="2" t="s">
-        <v>263</v>
+        <v>257</v>
       </c>
       <c r="B116" s="2" t="s">
-        <v>264</v>
+        <v>258</v>
       </c>
       <c r="C116" s="2" t="s">
-        <v>265</v>
+        <v>259</v>
       </c>
       <c r="D116" s="2" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A117" s="2" t="s">
-        <v>266</v>
+        <v>260</v>
       </c>
       <c r="B117" s="2" t="s">
-        <v>266</v>
+        <v>261</v>
       </c>
       <c r="C117" s="2" t="s">
-        <v>266</v>
+        <v>262</v>
       </c>
       <c r="D117" s="2" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A118" s="2" t="s">
-        <v>267</v>
+        <v>263</v>
       </c>
       <c r="B118" s="2" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="C118" s="2" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="D118" s="2" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
     </row>
     <row r="119" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A119" s="2" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="B119" s="2" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="C119" s="2" t="s">
-        <v>270</v>
+        <v>266</v>
       </c>
       <c r="D119" s="2" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A120" s="2" t="s">
-        <v>271</v>
+        <v>267</v>
       </c>
       <c r="B120" s="2" t="s">
-        <v>271</v>
+        <v>267</v>
       </c>
       <c r="C120" s="2" t="s">
-        <v>274</v>
+        <v>268</v>
       </c>
       <c r="D120" s="2" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A121" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="B121" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="C121" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="D121" s="2" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="122" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A122" s="2" t="s">
+        <v>271</v>
+      </c>
+      <c r="B122" s="2" t="s">
+        <v>271</v>
+      </c>
+      <c r="C122" s="2" t="s">
+        <v>274</v>
+      </c>
+      <c r="D122" s="2" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="123" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A123" s="2" t="s">
         <v>272</v>
       </c>
-      <c r="B121" s="2" t="s">
+      <c r="B123" s="2" t="s">
         <v>272</v>
       </c>
-      <c r="C121" s="2" t="s">
+      <c r="C123" s="2" t="s">
         <v>273</v>
       </c>
-      <c r="D121" s="2" t="s">
+      <c r="D123" s="2" t="s">
         <v>428</v>
       </c>
     </row>
-    <row r="122" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A122" s="2" t="s">
+    <row r="124" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A124" s="2" t="s">
         <v>275</v>
       </c>
-      <c r="B122" s="2" t="s">
+      <c r="B124" s="2" t="s">
         <v>277</v>
       </c>
-      <c r="C122" s="2" t="s">
+      <c r="C124" s="2" t="s">
         <v>280</v>
       </c>
     </row>
-    <row r="123" spans="1:4" ht="45" x14ac:dyDescent="0.25">
-      <c r="A123" s="2" t="s">
+    <row r="125" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="A125" s="2" t="s">
         <v>276</v>
       </c>
-      <c r="B123" s="2" t="s">
+      <c r="B125" s="2" t="s">
         <v>278</v>
       </c>
-      <c r="C123" s="2" t="s">
+      <c r="C125" s="2" t="s">
         <v>279</v>
       </c>
     </row>
-    <row r="124" spans="1:4" ht="75" x14ac:dyDescent="0.25">
-      <c r="A124" s="2" t="s">
+    <row r="126" spans="1:4" ht="75" x14ac:dyDescent="0.25">
+      <c r="A126" s="2" t="s">
         <v>290</v>
       </c>
-      <c r="B124" s="2" t="s">
+      <c r="B126" s="2" t="s">
         <v>291</v>
       </c>
-      <c r="C124" s="2" t="s">
+      <c r="C126" s="2" t="s">
         <v>292</v>
-      </c>
-    </row>
-    <row r="125" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A125" s="2" t="s">
-        <v>307</v>
-      </c>
-      <c r="B125" s="2" t="s">
-        <v>308</v>
-      </c>
-      <c r="C125" s="2" t="s">
-        <v>309</v>
-      </c>
-      <c r="D125" s="2" t="s">
-        <v>429</v>
-      </c>
-    </row>
-    <row r="126" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A126" s="2" t="s">
-        <v>310</v>
-      </c>
-      <c r="B126" s="2" t="s">
-        <v>312</v>
-      </c>
-      <c r="C126" s="2" t="s">
-        <v>313</v>
-      </c>
-      <c r="D126" s="2" t="s">
-        <v>430</v>
       </c>
     </row>
     <row r="127" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A127" s="2" t="s">
-        <v>311</v>
+        <v>307</v>
       </c>
       <c r="B127" s="2" t="s">
-        <v>315</v>
+        <v>308</v>
       </c>
       <c r="C127" s="2" t="s">
-        <v>314</v>
+        <v>309</v>
       </c>
       <c r="D127" s="2" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
     </row>
     <row r="128" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A128" s="2" t="s">
-        <v>316</v>
+        <v>310</v>
       </c>
       <c r="B128" s="2" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="C128" s="2" t="s">
-        <v>317</v>
+        <v>313</v>
       </c>
       <c r="D128" s="2" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
     </row>
     <row r="129" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A129" s="2" t="s">
-        <v>318</v>
+        <v>311</v>
       </c>
       <c r="B129" s="2" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="C129" s="2" t="s">
-        <v>461</v>
+        <v>314</v>
       </c>
       <c r="D129" s="2" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
     </row>
     <row r="130" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A130" s="2" t="s">
-        <v>320</v>
+        <v>316</v>
       </c>
       <c r="B130" s="2" t="s">
-        <v>321</v>
+        <v>316</v>
       </c>
       <c r="C130" s="2" t="s">
-        <v>462</v>
+        <v>317</v>
       </c>
       <c r="D130" s="2" t="s">
-        <v>434</v>
+        <v>432</v>
       </c>
     </row>
     <row r="131" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A131" s="2" t="s">
-        <v>449</v>
+        <v>318</v>
       </c>
       <c r="B131" s="2" t="s">
-        <v>449</v>
+        <v>319</v>
       </c>
       <c r="C131" s="2" t="s">
-        <v>463</v>
+        <v>461</v>
       </c>
       <c r="D131" s="2" t="s">
-        <v>346</v>
+        <v>433</v>
       </c>
     </row>
     <row r="132" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A132" s="2" t="s">
-        <v>450</v>
+        <v>320</v>
       </c>
       <c r="B132" s="2" t="s">
-        <v>451</v>
+        <v>321</v>
       </c>
       <c r="C132" s="2" t="s">
-        <v>464</v>
+        <v>462</v>
       </c>
       <c r="D132" s="2" t="s">
-        <v>452</v>
+        <v>434</v>
       </c>
     </row>
     <row r="133" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A133" s="2" t="s">
-        <v>477</v>
+        <v>449</v>
       </c>
       <c r="B133" s="2" t="s">
-        <v>478</v>
+        <v>449</v>
       </c>
       <c r="C133" s="2" t="s">
-        <v>479</v>
+        <v>463</v>
+      </c>
+      <c r="D133" s="2" t="s">
+        <v>346</v>
       </c>
     </row>
     <row r="134" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A134" s="2" t="s">
-        <v>480</v>
+        <v>450</v>
       </c>
       <c r="B134" s="2" t="s">
-        <v>481</v>
+        <v>451</v>
       </c>
       <c r="C134" s="2" t="s">
-        <v>482</v>
+        <v>464</v>
+      </c>
+      <c r="D134" s="2" t="s">
+        <v>452</v>
       </c>
     </row>
     <row r="135" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A135" s="2" t="s">
-        <v>483</v>
+        <v>477</v>
       </c>
       <c r="B135" s="2" t="s">
-        <v>484</v>
+        <v>478</v>
       </c>
       <c r="C135" s="2" t="s">
-        <v>485</v>
+        <v>479</v>
       </c>
     </row>
     <row r="136" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A136" s="2" t="s">
-        <v>486</v>
+        <v>480</v>
       </c>
       <c r="B136" s="2" t="s">
-        <v>487</v>
+        <v>481</v>
       </c>
       <c r="C136" s="2" t="s">
-        <v>488</v>
+        <v>482</v>
       </c>
     </row>
     <row r="137" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A137" s="2" t="s">
-        <v>489</v>
+        <v>483</v>
       </c>
       <c r="B137" s="2" t="s">
-        <v>490</v>
+        <v>484</v>
       </c>
       <c r="C137" s="2" t="s">
-        <v>491</v>
+        <v>485</v>
       </c>
     </row>
     <row r="138" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A138" s="2" t="s">
-        <v>492</v>
+        <v>486</v>
       </c>
       <c r="B138" s="2" t="s">
-        <v>493</v>
+        <v>487</v>
       </c>
       <c r="C138" s="2" t="s">
-        <v>494</v>
+        <v>488</v>
       </c>
     </row>
     <row r="139" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A139" s="2" t="s">
-        <v>495</v>
+        <v>489</v>
       </c>
       <c r="B139" s="2" t="s">
-        <v>496</v>
+        <v>490</v>
       </c>
       <c r="C139" s="2" t="s">
-        <v>497</v>
+        <v>491</v>
       </c>
     </row>
     <row r="140" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A140" s="2" t="s">
-        <v>498</v>
+        <v>492</v>
       </c>
       <c r="B140" s="2" t="s">
-        <v>499</v>
+        <v>493</v>
       </c>
       <c r="C140" s="2" t="s">
-        <v>500</v>
+        <v>494</v>
       </c>
     </row>
     <row r="141" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A141" s="2" t="s">
-        <v>501</v>
+        <v>495</v>
       </c>
       <c r="B141" s="2" t="s">
-        <v>502</v>
+        <v>496</v>
       </c>
       <c r="C141" s="2" t="s">
-        <v>503</v>
+        <v>497</v>
       </c>
     </row>
     <row r="142" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A142" s="2" t="s">
-        <v>504</v>
+        <v>498</v>
       </c>
       <c r="B142" s="2" t="s">
-        <v>504</v>
+        <v>499</v>
       </c>
       <c r="C142" s="2" t="s">
-        <v>505</v>
+        <v>500</v>
       </c>
     </row>
     <row r="143" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A143" s="2" t="s">
-        <v>506</v>
+        <v>501</v>
       </c>
       <c r="B143" s="2" t="s">
-        <v>506</v>
+        <v>502</v>
       </c>
       <c r="C143" s="2" t="s">
-        <v>507</v>
+        <v>503</v>
       </c>
     </row>
     <row r="144" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A144" s="2" t="s">
-        <v>508</v>
+        <v>504</v>
       </c>
       <c r="B144" s="2" t="s">
-        <v>508</v>
+        <v>504</v>
       </c>
       <c r="C144" s="2" t="s">
-        <v>509</v>
+        <v>505</v>
       </c>
     </row>
     <row r="145" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A145" s="2" t="s">
+        <v>506</v>
+      </c>
+      <c r="B145" s="2" t="s">
+        <v>506</v>
+      </c>
+      <c r="C145" s="2" t="s">
+        <v>507</v>
+      </c>
+    </row>
+    <row r="146" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A146" s="2" t="s">
+        <v>508</v>
+      </c>
+      <c r="B146" s="2" t="s">
+        <v>508</v>
+      </c>
+      <c r="C146" s="2" t="s">
+        <v>509</v>
+      </c>
+    </row>
+    <row r="147" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A147" s="2" t="s">
         <v>510</v>
       </c>
-      <c r="B145" s="2" t="s">
+      <c r="B147" s="2" t="s">
         <v>510</v>
       </c>
-      <c r="C145" s="2" t="s">
+      <c r="C147" s="2" t="s">
         <v>511</v>
       </c>
     </row>

</xml_diff>

<commit_message>
correct normals and bridge improvements
</commit_message>
<xml_diff>
--- a/Translations/Translations.xlsx
+++ b/Translations/Translations.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Codes\c#\FrSLE\Translations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C40685B5-79CC-44E2-9567-3C747D734598}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1967C7D-4CC3-4849-9540-7F7172268945}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15900" xr2:uid="{F5C22481-FF1A-482C-BF7E-EB5A7718AF49}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="563" uniqueCount="518">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="572" uniqueCount="527">
   <si>
     <t>ID</t>
   </si>
@@ -1588,6 +1588,33 @@
   </si>
   <si>
     <t>При розваленні</t>
+  </si>
+  <si>
+    <t>object.BRIDGE</t>
+  </si>
+  <si>
+    <t>Bridge</t>
+  </si>
+  <si>
+    <t>Міст</t>
+  </si>
+  <si>
+    <t>events.OnDeploy</t>
+  </si>
+  <si>
+    <t>On Deploy</t>
+  </si>
+  <si>
+    <t>При розкритті</t>
+  </si>
+  <si>
+    <t>events.OnRetract</t>
+  </si>
+  <si>
+    <t>On Retract</t>
+  </si>
+  <si>
+    <t>При скритті</t>
   </si>
 </sst>
 </file>
@@ -1987,7 +2014,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6961A5F-F8EA-4989-8112-A0ACE51D011E}">
   <sheetPr codeName="Hoja1"/>
-  <dimension ref="A1:D147"/>
+  <dimension ref="A1:D150"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="37" style="2" customWidth="1"/>
@@ -2696,1285 +2723,1318 @@
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
-        <v>69</v>
+        <v>518</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="C52" s="2" t="s">
-        <v>101</v>
+        <v>519</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>365</v>
+        <v>520</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" s="2" t="s">
-        <v>105</v>
+        <v>69</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>2</v>
+        <v>69</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A55" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>111</v>
+        <v>4</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57" s="2" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" s="2" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" s="2" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61" s="2" t="s">
-        <v>446</v>
+        <v>118</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>447</v>
+        <v>122</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>460</v>
+        <v>121</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>448</v>
+        <v>371</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" s="2" t="s">
-        <v>515</v>
+        <v>446</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>516</v>
+        <v>447</v>
+      </c>
+      <c r="C62" s="2" t="s">
+        <v>460</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>517</v>
+        <v>448</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63" s="2" t="s">
-        <v>154</v>
+        <v>515</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="C63" s="2" t="s">
-        <v>156</v>
+        <v>516</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>372</v>
+        <v>517</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" s="2" t="s">
-        <v>164</v>
+        <v>521</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>165</v>
-      </c>
-      <c r="C64" s="2" t="s">
-        <v>166</v>
+        <v>522</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>373</v>
+        <v>523</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A65" s="2" t="s">
-        <v>157</v>
+        <v>524</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>158</v>
-      </c>
-      <c r="C65" s="2" t="s">
-        <v>159</v>
+        <v>525</v>
       </c>
       <c r="D65" s="2" t="s">
-        <v>374</v>
+        <v>526</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66" s="2" t="s">
-        <v>167</v>
+        <v>154</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>168</v>
+        <v>155</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>169</v>
+        <v>156</v>
       </c>
       <c r="D66" s="2" t="s">
-        <v>375</v>
+        <v>372</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A67" s="2" t="s">
-        <v>141</v>
+        <v>164</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>142</v>
+        <v>165</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>143</v>
+        <v>166</v>
       </c>
       <c r="D67" s="2" t="s">
-        <v>376</v>
-      </c>
-    </row>
-    <row r="68" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A68" s="2" t="s">
-        <v>144</v>
+        <v>157</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>145</v>
+        <v>159</v>
       </c>
       <c r="D68" s="2" t="s">
-        <v>377</v>
+        <v>374</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A69" s="2" t="s">
-        <v>153</v>
+        <v>167</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>146</v>
+        <v>168</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>146</v>
+        <v>169</v>
       </c>
       <c r="D69" s="2" t="s">
-        <v>329</v>
+        <v>375</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A70" s="2" t="s">
-        <v>147</v>
+        <v>141</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="C70" s="2" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
       <c r="D70" s="2" t="s">
-        <v>378</v>
-      </c>
-    </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A71" s="2" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>151</v>
+        <v>163</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>152</v>
+        <v>145</v>
       </c>
       <c r="D71" s="2" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A72" s="2" t="s">
-        <v>172</v>
+        <v>153</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>170</v>
+        <v>146</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>171</v>
+        <v>146</v>
       </c>
       <c r="D72" s="2" t="s">
-        <v>380</v>
+        <v>329</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A73" s="2" t="s">
-        <v>173</v>
+        <v>147</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>174</v>
+        <v>148</v>
       </c>
       <c r="C73" s="2" t="s">
-        <v>175</v>
+        <v>149</v>
       </c>
       <c r="D73" s="2" t="s">
-        <v>381</v>
+        <v>378</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A74" s="2" t="s">
-        <v>176</v>
+        <v>150</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>176</v>
+        <v>151</v>
       </c>
       <c r="C74" s="2" t="s">
-        <v>177</v>
+        <v>152</v>
       </c>
       <c r="D74" s="2" t="s">
-        <v>382</v>
+        <v>379</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A75" s="2" t="s">
-        <v>178</v>
+        <v>172</v>
       </c>
       <c r="B75" s="2" t="s">
-        <v>178</v>
+        <v>170</v>
       </c>
       <c r="C75" s="2" t="s">
-        <v>179</v>
+        <v>171</v>
       </c>
       <c r="D75" s="2" t="s">
-        <v>383</v>
+        <v>380</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A76" s="2" t="s">
-        <v>180</v>
+        <v>173</v>
       </c>
       <c r="B76" s="2" t="s">
-        <v>180</v>
+        <v>174</v>
       </c>
       <c r="C76" s="2" t="s">
-        <v>181</v>
+        <v>175</v>
       </c>
       <c r="D76" s="2" t="s">
-        <v>384</v>
+        <v>381</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A77" s="2" t="s">
-        <v>244</v>
+        <v>176</v>
       </c>
       <c r="B77" s="2" t="s">
-        <v>244</v>
+        <v>176</v>
       </c>
       <c r="C77" s="2" t="s">
-        <v>95</v>
+        <v>177</v>
       </c>
       <c r="D77" s="2" t="s">
-        <v>385</v>
-      </c>
-    </row>
-    <row r="78" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A78" s="2" t="s">
-        <v>138</v>
-      </c>
-      <c r="B78" s="1" t="s">
-        <v>140</v>
+        <v>178</v>
+      </c>
+      <c r="B78" s="2" t="s">
+        <v>178</v>
       </c>
       <c r="C78" s="2" t="s">
-        <v>139</v>
+        <v>179</v>
       </c>
       <c r="D78" s="2" t="s">
-        <v>386</v>
+        <v>383</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A79" s="2" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="B79" s="2" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="C79" s="2" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="D79" s="2" t="s">
-        <v>387</v>
+        <v>384</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
-        <v>184</v>
+        <v>244</v>
       </c>
       <c r="B80" s="2" t="s">
-        <v>184</v>
+        <v>244</v>
       </c>
       <c r="C80" s="2" t="s">
-        <v>185</v>
+        <v>95</v>
       </c>
       <c r="D80" s="2" t="s">
-        <v>388</v>
-      </c>
-    </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A81" s="2" t="s">
-        <v>186</v>
-      </c>
-      <c r="B81" s="2" t="s">
-        <v>186</v>
+        <v>138</v>
+      </c>
+      <c r="B81" s="1" t="s">
+        <v>140</v>
       </c>
       <c r="C81" s="2" t="s">
-        <v>187</v>
+        <v>139</v>
       </c>
       <c r="D81" s="2" t="s">
-        <v>389</v>
+        <v>386</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A82" s="2" t="s">
-        <v>188</v>
+        <v>182</v>
       </c>
       <c r="B82" s="2" t="s">
-        <v>189</v>
+        <v>183</v>
       </c>
       <c r="C82" s="2" t="s">
-        <v>190</v>
+        <v>183</v>
       </c>
       <c r="D82" s="2" t="s">
-        <v>390</v>
+        <v>387</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A83" s="2" t="s">
-        <v>191</v>
+        <v>184</v>
       </c>
       <c r="B83" s="2" t="s">
-        <v>191</v>
+        <v>184</v>
       </c>
       <c r="C83" s="2" t="s">
-        <v>192</v>
+        <v>185</v>
       </c>
       <c r="D83" s="2" t="s">
-        <v>391</v>
+        <v>388</v>
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A84" s="2" t="s">
-        <v>193</v>
+        <v>186</v>
       </c>
       <c r="B84" s="2" t="s">
-        <v>194</v>
+        <v>186</v>
       </c>
       <c r="C84" s="2" t="s">
-        <v>195</v>
+        <v>187</v>
       </c>
       <c r="D84" s="2" t="s">
-        <v>392</v>
+        <v>389</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A85" s="2" t="s">
-        <v>435</v>
-      </c>
-      <c r="B85" s="4" t="s">
-        <v>436</v>
-      </c>
-      <c r="C85" s="4" t="s">
-        <v>437</v>
+        <v>188</v>
+      </c>
+      <c r="B85" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="C85" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="D85" s="2" t="s">
+        <v>390</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A86" s="2" t="s">
-        <v>438</v>
-      </c>
-      <c r="B86" s="4" t="s">
-        <v>439</v>
-      </c>
-      <c r="C86" s="4" t="s">
-        <v>440</v>
+        <v>191</v>
+      </c>
+      <c r="B86" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="C86" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="D86" s="2" t="s">
+        <v>391</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A87" s="2" t="s">
-        <v>474</v>
-      </c>
-      <c r="B87" s="4" t="s">
-        <v>475</v>
-      </c>
-      <c r="C87" s="4" t="s">
-        <v>476</v>
+        <v>193</v>
+      </c>
+      <c r="B87" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="C87" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="D87" s="2" t="s">
+        <v>392</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A88" s="2" t="s">
-        <v>196</v>
-      </c>
-      <c r="B88" s="2" t="s">
-        <v>197</v>
-      </c>
-      <c r="C88" s="2" t="s">
-        <v>198</v>
-      </c>
-      <c r="D88" s="2" t="s">
-        <v>393</v>
+        <v>435</v>
+      </c>
+      <c r="B88" s="4" t="s">
+        <v>436</v>
+      </c>
+      <c r="C88" s="4" t="s">
+        <v>437</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A89" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="B89" s="2" t="s">
-        <v>200</v>
-      </c>
-      <c r="C89" s="2" t="s">
-        <v>201</v>
-      </c>
-      <c r="D89" s="2" t="s">
-        <v>394</v>
+        <v>438</v>
+      </c>
+      <c r="B89" s="4" t="s">
+        <v>439</v>
+      </c>
+      <c r="C89" s="4" t="s">
+        <v>440</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A90" s="2" t="s">
-        <v>202</v>
-      </c>
-      <c r="B90" s="2" t="s">
-        <v>202</v>
-      </c>
-      <c r="C90" s="2" t="s">
-        <v>203</v>
-      </c>
-      <c r="D90" s="2" t="s">
-        <v>395</v>
+        <v>474</v>
+      </c>
+      <c r="B90" s="4" t="s">
+        <v>475</v>
+      </c>
+      <c r="C90" s="4" t="s">
+        <v>476</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A91" s="2" t="s">
-        <v>204</v>
+        <v>196</v>
       </c>
       <c r="B91" s="2" t="s">
-        <v>204</v>
+        <v>197</v>
       </c>
       <c r="C91" s="2" t="s">
-        <v>205</v>
+        <v>198</v>
       </c>
       <c r="D91" s="2" t="s">
-        <v>396</v>
+        <v>393</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A92" s="2" t="s">
-        <v>206</v>
+        <v>199</v>
       </c>
       <c r="B92" s="2" t="s">
-        <v>206</v>
+        <v>200</v>
       </c>
       <c r="C92" s="2" t="s">
-        <v>206</v>
+        <v>201</v>
       </c>
       <c r="D92" s="2" t="s">
-        <v>397</v>
+        <v>394</v>
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A93" s="2" t="s">
-        <v>207</v>
+        <v>202</v>
       </c>
       <c r="B93" s="2" t="s">
-        <v>208</v>
+        <v>202</v>
       </c>
       <c r="C93" s="2" t="s">
-        <v>209</v>
+        <v>203</v>
       </c>
       <c r="D93" s="2" t="s">
-        <v>398</v>
+        <v>395</v>
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A94" s="2" t="s">
-        <v>210</v>
+        <v>204</v>
       </c>
       <c r="B94" s="2" t="s">
-        <v>211</v>
+        <v>204</v>
       </c>
       <c r="C94" s="2" t="s">
-        <v>212</v>
+        <v>205</v>
       </c>
       <c r="D94" s="2" t="s">
-        <v>399</v>
+        <v>396</v>
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A95" s="2" t="s">
-        <v>213</v>
+        <v>206</v>
       </c>
       <c r="B95" s="2" t="s">
-        <v>214</v>
+        <v>206</v>
       </c>
       <c r="C95" s="2" t="s">
-        <v>215</v>
+        <v>206</v>
       </c>
       <c r="D95" s="2" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A96" s="2" t="s">
-        <v>216</v>
+        <v>207</v>
       </c>
       <c r="B96" s="2" t="s">
-        <v>217</v>
+        <v>208</v>
       </c>
       <c r="C96" s="2" t="s">
-        <v>218</v>
+        <v>209</v>
       </c>
       <c r="D96" s="2" t="s">
-        <v>401</v>
+        <v>398</v>
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A97" s="2" t="s">
-        <v>221</v>
+        <v>210</v>
       </c>
       <c r="B97" s="2" t="s">
-        <v>220</v>
+        <v>211</v>
       </c>
       <c r="C97" s="2" t="s">
-        <v>219</v>
+        <v>212</v>
       </c>
       <c r="D97" s="2" t="s">
-        <v>402</v>
+        <v>399</v>
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A98" s="2" t="s">
-        <v>293</v>
+        <v>213</v>
       </c>
       <c r="B98" s="2" t="s">
-        <v>293</v>
+        <v>214</v>
       </c>
       <c r="C98" s="2" t="s">
-        <v>294</v>
+        <v>215</v>
       </c>
       <c r="D98" s="2" t="s">
-        <v>403</v>
+        <v>400</v>
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A99" s="2" t="s">
-        <v>295</v>
+        <v>216</v>
       </c>
       <c r="B99" s="2" t="s">
-        <v>296</v>
+        <v>217</v>
       </c>
       <c r="C99" s="2" t="s">
-        <v>297</v>
+        <v>218</v>
       </c>
       <c r="D99" s="2" t="s">
-        <v>404</v>
+        <v>401</v>
       </c>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A100" s="2" t="s">
-        <v>298</v>
+        <v>221</v>
       </c>
       <c r="B100" s="2" t="s">
-        <v>299</v>
+        <v>220</v>
       </c>
       <c r="C100" s="2" t="s">
-        <v>300</v>
+        <v>219</v>
       </c>
       <c r="D100" s="2" t="s">
-        <v>405</v>
+        <v>402</v>
       </c>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A101" s="2" t="s">
-        <v>222</v>
+        <v>293</v>
       </c>
       <c r="B101" s="2" t="s">
-        <v>222</v>
+        <v>293</v>
       </c>
       <c r="C101" s="2" t="s">
-        <v>223</v>
+        <v>294</v>
       </c>
       <c r="D101" s="2" t="s">
-        <v>406</v>
+        <v>403</v>
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A102" s="2" t="s">
-        <v>224</v>
+        <v>295</v>
       </c>
       <c r="B102" s="2" t="s">
-        <v>225</v>
+        <v>296</v>
       </c>
       <c r="C102" s="2" t="s">
-        <v>226</v>
+        <v>297</v>
       </c>
       <c r="D102" s="2" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A103" s="2" t="s">
-        <v>227</v>
+        <v>298</v>
       </c>
       <c r="B103" s="2" t="s">
-        <v>228</v>
+        <v>299</v>
       </c>
       <c r="C103" s="2" t="s">
-        <v>229</v>
+        <v>300</v>
       </c>
       <c r="D103" s="2" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A104" s="2" t="s">
-        <v>230</v>
+        <v>222</v>
       </c>
       <c r="B104" s="2" t="s">
-        <v>230</v>
+        <v>222</v>
       </c>
       <c r="C104" s="2" t="s">
-        <v>230</v>
+        <v>223</v>
       </c>
       <c r="D104" s="2" t="s">
-        <v>409</v>
+        <v>406</v>
       </c>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A105" s="2" t="s">
-        <v>231</v>
+        <v>224</v>
       </c>
       <c r="B105" s="2" t="s">
-        <v>231</v>
+        <v>225</v>
       </c>
       <c r="C105" s="2" t="s">
-        <v>232</v>
+        <v>226</v>
       </c>
       <c r="D105" s="2" t="s">
-        <v>410</v>
+        <v>407</v>
       </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A106" s="2" t="s">
-        <v>233</v>
+        <v>227</v>
       </c>
       <c r="B106" s="2" t="s">
-        <v>233</v>
+        <v>228</v>
       </c>
       <c r="C106" s="2" t="s">
-        <v>234</v>
+        <v>229</v>
       </c>
       <c r="D106" s="2" t="s">
-        <v>411</v>
+        <v>408</v>
       </c>
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A107" s="2" t="s">
-        <v>235</v>
+        <v>230</v>
       </c>
       <c r="B107" s="2" t="s">
-        <v>236</v>
+        <v>230</v>
       </c>
       <c r="C107" s="2" t="s">
-        <v>237</v>
+        <v>230</v>
       </c>
       <c r="D107" s="2" t="s">
-        <v>412</v>
+        <v>409</v>
       </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A108" s="2" t="s">
-        <v>238</v>
+        <v>231</v>
       </c>
       <c r="B108" s="2" t="s">
-        <v>239</v>
+        <v>231</v>
       </c>
       <c r="C108" s="2" t="s">
-        <v>240</v>
+        <v>232</v>
       </c>
       <c r="D108" s="2" t="s">
-        <v>413</v>
+        <v>410</v>
       </c>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A109" s="2" t="s">
-        <v>301</v>
+        <v>233</v>
       </c>
       <c r="B109" s="2" t="s">
-        <v>302</v>
+        <v>233</v>
       </c>
       <c r="C109" s="2" t="s">
-        <v>303</v>
+        <v>234</v>
       </c>
       <c r="D109" s="2" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A110" s="2" t="s">
-        <v>241</v>
+        <v>235</v>
       </c>
       <c r="B110" s="2" t="s">
-        <v>242</v>
+        <v>236</v>
       </c>
       <c r="C110" s="2" t="s">
-        <v>243</v>
+        <v>237</v>
       </c>
       <c r="D110" s="2" t="s">
-        <v>415</v>
+        <v>412</v>
       </c>
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A111" s="2" t="s">
-        <v>245</v>
+        <v>238</v>
       </c>
       <c r="B111" s="2" t="s">
-        <v>253</v>
+        <v>239</v>
       </c>
       <c r="C111" s="2" t="s">
-        <v>252</v>
+        <v>240</v>
       </c>
       <c r="D111" s="2" t="s">
-        <v>416</v>
+        <v>413</v>
       </c>
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A112" s="2" t="s">
-        <v>246</v>
+        <v>301</v>
       </c>
       <c r="B112" s="2" t="s">
-        <v>246</v>
+        <v>302</v>
       </c>
       <c r="C112" s="2" t="s">
-        <v>247</v>
+        <v>303</v>
       </c>
       <c r="D112" s="2" t="s">
-        <v>417</v>
+        <v>414</v>
       </c>
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A113" s="2" t="s">
-        <v>248</v>
+        <v>241</v>
       </c>
       <c r="B113" s="2" t="s">
-        <v>248</v>
+        <v>242</v>
       </c>
       <c r="C113" s="2" t="s">
-        <v>249</v>
+        <v>243</v>
       </c>
       <c r="D113" s="2" t="s">
-        <v>418</v>
+        <v>415</v>
       </c>
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A114" s="2" t="s">
-        <v>250</v>
+        <v>245</v>
       </c>
       <c r="B114" s="2" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="C114" s="2" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="D114" s="2" t="s">
-        <v>419</v>
+        <v>416</v>
       </c>
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A115" s="2" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
       <c r="B115" s="2" t="s">
-        <v>255</v>
+        <v>246</v>
       </c>
       <c r="C115" s="2" t="s">
-        <v>256</v>
+        <v>247</v>
       </c>
       <c r="D115" s="2" t="s">
-        <v>420</v>
+        <v>417</v>
       </c>
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A116" s="2" t="s">
-        <v>257</v>
+        <v>248</v>
       </c>
       <c r="B116" s="2" t="s">
-        <v>258</v>
+        <v>248</v>
       </c>
       <c r="C116" s="2" t="s">
-        <v>259</v>
+        <v>249</v>
       </c>
       <c r="D116" s="2" t="s">
-        <v>421</v>
+        <v>418</v>
       </c>
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A117" s="2" t="s">
-        <v>260</v>
+        <v>250</v>
       </c>
       <c r="B117" s="2" t="s">
-        <v>261</v>
+        <v>250</v>
       </c>
       <c r="C117" s="2" t="s">
-        <v>262</v>
+        <v>251</v>
       </c>
       <c r="D117" s="2" t="s">
-        <v>422</v>
+        <v>419</v>
       </c>
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A118" s="2" t="s">
-        <v>263</v>
+        <v>254</v>
       </c>
       <c r="B118" s="2" t="s">
-        <v>264</v>
+        <v>255</v>
       </c>
       <c r="C118" s="2" t="s">
-        <v>265</v>
+        <v>256</v>
       </c>
       <c r="D118" s="2" t="s">
-        <v>423</v>
+        <v>420</v>
       </c>
     </row>
     <row r="119" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A119" s="2" t="s">
-        <v>266</v>
+        <v>257</v>
       </c>
       <c r="B119" s="2" t="s">
-        <v>266</v>
+        <v>258</v>
       </c>
       <c r="C119" s="2" t="s">
-        <v>266</v>
+        <v>259</v>
       </c>
       <c r="D119" s="2" t="s">
-        <v>424</v>
+        <v>421</v>
       </c>
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A120" s="2" t="s">
-        <v>267</v>
+        <v>260</v>
       </c>
       <c r="B120" s="2" t="s">
-        <v>267</v>
+        <v>261</v>
       </c>
       <c r="C120" s="2" t="s">
-        <v>268</v>
+        <v>262</v>
       </c>
       <c r="D120" s="2" t="s">
-        <v>425</v>
+        <v>422</v>
       </c>
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A121" s="2" t="s">
-        <v>269</v>
+        <v>263</v>
       </c>
       <c r="B121" s="2" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="C121" s="2" t="s">
-        <v>270</v>
+        <v>265</v>
       </c>
       <c r="D121" s="2" t="s">
-        <v>426</v>
+        <v>423</v>
       </c>
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A122" s="2" t="s">
-        <v>271</v>
+        <v>266</v>
       </c>
       <c r="B122" s="2" t="s">
-        <v>271</v>
+        <v>266</v>
       </c>
       <c r="C122" s="2" t="s">
-        <v>274</v>
+        <v>266</v>
       </c>
       <c r="D122" s="2" t="s">
-        <v>427</v>
+        <v>424</v>
       </c>
     </row>
     <row r="123" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A123" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="B123" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="C123" s="2" t="s">
+        <v>268</v>
+      </c>
+      <c r="D123" s="2" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="124" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A124" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="B124" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="C124" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="D124" s="2" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="125" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A125" s="2" t="s">
+        <v>271</v>
+      </c>
+      <c r="B125" s="2" t="s">
+        <v>271</v>
+      </c>
+      <c r="C125" s="2" t="s">
+        <v>274</v>
+      </c>
+      <c r="D125" s="2" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="126" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A126" s="2" t="s">
         <v>272</v>
       </c>
-      <c r="B123" s="2" t="s">
+      <c r="B126" s="2" t="s">
         <v>272</v>
       </c>
-      <c r="C123" s="2" t="s">
+      <c r="C126" s="2" t="s">
         <v>273</v>
       </c>
-      <c r="D123" s="2" t="s">
+      <c r="D126" s="2" t="s">
         <v>428</v>
       </c>
     </row>
-    <row r="124" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A124" s="2" t="s">
+    <row r="127" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A127" s="2" t="s">
         <v>275</v>
       </c>
-      <c r="B124" s="2" t="s">
+      <c r="B127" s="2" t="s">
         <v>277</v>
       </c>
-      <c r="C124" s="2" t="s">
+      <c r="C127" s="2" t="s">
         <v>280</v>
       </c>
     </row>
-    <row r="125" spans="1:4" ht="45" x14ac:dyDescent="0.25">
-      <c r="A125" s="2" t="s">
+    <row r="128" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="A128" s="2" t="s">
         <v>276</v>
       </c>
-      <c r="B125" s="2" t="s">
+      <c r="B128" s="2" t="s">
         <v>278</v>
       </c>
-      <c r="C125" s="2" t="s">
+      <c r="C128" s="2" t="s">
         <v>279</v>
       </c>
     </row>
-    <row r="126" spans="1:4" ht="75" x14ac:dyDescent="0.25">
-      <c r="A126" s="2" t="s">
+    <row r="129" spans="1:4" ht="75" x14ac:dyDescent="0.25">
+      <c r="A129" s="2" t="s">
         <v>290</v>
       </c>
-      <c r="B126" s="2" t="s">
+      <c r="B129" s="2" t="s">
         <v>291</v>
       </c>
-      <c r="C126" s="2" t="s">
+      <c r="C129" s="2" t="s">
         <v>292</v>
-      </c>
-    </row>
-    <row r="127" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A127" s="2" t="s">
-        <v>307</v>
-      </c>
-      <c r="B127" s="2" t="s">
-        <v>308</v>
-      </c>
-      <c r="C127" s="2" t="s">
-        <v>309</v>
-      </c>
-      <c r="D127" s="2" t="s">
-        <v>429</v>
-      </c>
-    </row>
-    <row r="128" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A128" s="2" t="s">
-        <v>310</v>
-      </c>
-      <c r="B128" s="2" t="s">
-        <v>312</v>
-      </c>
-      <c r="C128" s="2" t="s">
-        <v>313</v>
-      </c>
-      <c r="D128" s="2" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="129" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A129" s="2" t="s">
-        <v>311</v>
-      </c>
-      <c r="B129" s="2" t="s">
-        <v>315</v>
-      </c>
-      <c r="C129" s="2" t="s">
-        <v>314</v>
-      </c>
-      <c r="D129" s="2" t="s">
-        <v>431</v>
       </c>
     </row>
     <row r="130" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A130" s="2" t="s">
-        <v>316</v>
+        <v>307</v>
       </c>
       <c r="B130" s="2" t="s">
-        <v>316</v>
+        <v>308</v>
       </c>
       <c r="C130" s="2" t="s">
-        <v>317</v>
+        <v>309</v>
       </c>
       <c r="D130" s="2" t="s">
-        <v>432</v>
+        <v>429</v>
       </c>
     </row>
     <row r="131" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A131" s="2" t="s">
-        <v>318</v>
+        <v>310</v>
       </c>
       <c r="B131" s="2" t="s">
-        <v>319</v>
+        <v>312</v>
       </c>
       <c r="C131" s="2" t="s">
-        <v>461</v>
+        <v>313</v>
       </c>
       <c r="D131" s="2" t="s">
-        <v>433</v>
+        <v>430</v>
       </c>
     </row>
     <row r="132" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A132" s="2" t="s">
-        <v>320</v>
+        <v>311</v>
       </c>
       <c r="B132" s="2" t="s">
-        <v>321</v>
+        <v>315</v>
       </c>
       <c r="C132" s="2" t="s">
-        <v>462</v>
+        <v>314</v>
       </c>
       <c r="D132" s="2" t="s">
-        <v>434</v>
+        <v>431</v>
       </c>
     </row>
     <row r="133" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A133" s="2" t="s">
-        <v>449</v>
+        <v>316</v>
       </c>
       <c r="B133" s="2" t="s">
-        <v>449</v>
+        <v>316</v>
       </c>
       <c r="C133" s="2" t="s">
-        <v>463</v>
+        <v>317</v>
       </c>
       <c r="D133" s="2" t="s">
-        <v>346</v>
+        <v>432</v>
       </c>
     </row>
     <row r="134" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A134" s="2" t="s">
-        <v>450</v>
+        <v>318</v>
       </c>
       <c r="B134" s="2" t="s">
-        <v>451</v>
+        <v>319</v>
       </c>
       <c r="C134" s="2" t="s">
-        <v>464</v>
+        <v>461</v>
       </c>
       <c r="D134" s="2" t="s">
-        <v>452</v>
+        <v>433</v>
       </c>
     </row>
     <row r="135" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A135" s="2" t="s">
-        <v>477</v>
+        <v>320</v>
       </c>
       <c r="B135" s="2" t="s">
-        <v>478</v>
+        <v>321</v>
       </c>
       <c r="C135" s="2" t="s">
-        <v>479</v>
+        <v>462</v>
+      </c>
+      <c r="D135" s="2" t="s">
+        <v>434</v>
       </c>
     </row>
     <row r="136" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A136" s="2" t="s">
-        <v>480</v>
+        <v>449</v>
       </c>
       <c r="B136" s="2" t="s">
-        <v>481</v>
+        <v>449</v>
       </c>
       <c r="C136" s="2" t="s">
-        <v>482</v>
+        <v>463</v>
+      </c>
+      <c r="D136" s="2" t="s">
+        <v>346</v>
       </c>
     </row>
     <row r="137" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A137" s="2" t="s">
-        <v>483</v>
+        <v>450</v>
       </c>
       <c r="B137" s="2" t="s">
-        <v>484</v>
+        <v>451</v>
       </c>
       <c r="C137" s="2" t="s">
-        <v>485</v>
+        <v>464</v>
+      </c>
+      <c r="D137" s="2" t="s">
+        <v>452</v>
       </c>
     </row>
     <row r="138" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A138" s="2" t="s">
-        <v>486</v>
+        <v>477</v>
       </c>
       <c r="B138" s="2" t="s">
-        <v>487</v>
+        <v>478</v>
       </c>
       <c r="C138" s="2" t="s">
-        <v>488</v>
+        <v>479</v>
       </c>
     </row>
     <row r="139" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A139" s="2" t="s">
-        <v>489</v>
+        <v>480</v>
       </c>
       <c r="B139" s="2" t="s">
-        <v>490</v>
+        <v>481</v>
       </c>
       <c r="C139" s="2" t="s">
-        <v>491</v>
+        <v>482</v>
       </c>
     </row>
     <row r="140" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A140" s="2" t="s">
-        <v>492</v>
+        <v>483</v>
       </c>
       <c r="B140" s="2" t="s">
-        <v>493</v>
+        <v>484</v>
       </c>
       <c r="C140" s="2" t="s">
-        <v>494</v>
+        <v>485</v>
       </c>
     </row>
     <row r="141" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A141" s="2" t="s">
-        <v>495</v>
+        <v>486</v>
       </c>
       <c r="B141" s="2" t="s">
-        <v>496</v>
+        <v>487</v>
       </c>
       <c r="C141" s="2" t="s">
-        <v>497</v>
+        <v>488</v>
       </c>
     </row>
     <row r="142" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A142" s="2" t="s">
-        <v>498</v>
+        <v>489</v>
       </c>
       <c r="B142" s="2" t="s">
-        <v>499</v>
+        <v>490</v>
       </c>
       <c r="C142" s="2" t="s">
-        <v>500</v>
+        <v>491</v>
       </c>
     </row>
     <row r="143" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A143" s="2" t="s">
-        <v>501</v>
+        <v>492</v>
       </c>
       <c r="B143" s="2" t="s">
-        <v>502</v>
+        <v>493</v>
       </c>
       <c r="C143" s="2" t="s">
-        <v>503</v>
+        <v>494</v>
       </c>
     </row>
     <row r="144" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A144" s="2" t="s">
-        <v>504</v>
+        <v>495</v>
       </c>
       <c r="B144" s="2" t="s">
-        <v>504</v>
+        <v>496</v>
       </c>
       <c r="C144" s="2" t="s">
-        <v>505</v>
+        <v>497</v>
       </c>
     </row>
     <row r="145" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A145" s="2" t="s">
-        <v>506</v>
+        <v>498</v>
       </c>
       <c r="B145" s="2" t="s">
-        <v>506</v>
+        <v>499</v>
       </c>
       <c r="C145" s="2" t="s">
-        <v>507</v>
+        <v>500</v>
       </c>
     </row>
     <row r="146" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A146" s="2" t="s">
-        <v>508</v>
+        <v>501</v>
       </c>
       <c r="B146" s="2" t="s">
-        <v>508</v>
+        <v>502</v>
       </c>
       <c r="C146" s="2" t="s">
-        <v>509</v>
+        <v>503</v>
       </c>
     </row>
     <row r="147" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A147" s="2" t="s">
+        <v>504</v>
+      </c>
+      <c r="B147" s="2" t="s">
+        <v>504</v>
+      </c>
+      <c r="C147" s="2" t="s">
+        <v>505</v>
+      </c>
+    </row>
+    <row r="148" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A148" s="2" t="s">
+        <v>506</v>
+      </c>
+      <c r="B148" s="2" t="s">
+        <v>506</v>
+      </c>
+      <c r="C148" s="2" t="s">
+        <v>507</v>
+      </c>
+    </row>
+    <row r="149" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A149" s="2" t="s">
+        <v>508</v>
+      </c>
+      <c r="B149" s="2" t="s">
+        <v>508</v>
+      </c>
+      <c r="C149" s="2" t="s">
+        <v>509</v>
+      </c>
+    </row>
+    <row r="150" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A150" s="2" t="s">
         <v>510</v>
       </c>
-      <c r="B147" s="2" t="s">
+      <c r="B150" s="2" t="s">
         <v>510</v>
       </c>
-      <c r="C147" s="2" t="s">
+      <c r="C150" s="2" t="s">
         <v>511</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Changed two entries because Chrs wanted it.
</commit_message>
<xml_diff>
--- a/Translations/Translations.xlsx
+++ b/Translations/Translations.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Codes\c#\FrSLE\Translations\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programacion\MelonLoader\FS_LevelEditor\Translations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1967C7D-4CC3-4849-9540-7F7172268945}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8436EDEC-EAFE-4595-BBB7-A6783CBD918B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15900" xr2:uid="{F5C22481-FF1A-482C-BF7E-EB5A7718AF49}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{F5C22481-FF1A-482C-BF7E-EB5A7718AF49}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -603,9 +603,6 @@
     <t>ActivateOnStart</t>
   </si>
   <si>
-    <t>Activate On Start</t>
-  </si>
-  <si>
     <t>Activar Al Inicio</t>
   </si>
   <si>
@@ -1479,9 +1476,6 @@
     <t>StartMovingAtStart</t>
   </si>
   <si>
-    <t>Start Moving At Start</t>
-  </si>
-  <si>
     <t>Mover Al Inicio</t>
   </si>
   <si>
@@ -1615,6 +1609,12 @@
   </si>
   <si>
     <t>При скритті</t>
+  </si>
+  <si>
+    <t>Move At Start</t>
+  </si>
+  <si>
+    <t>Start Enabled</t>
   </si>
 </sst>
 </file>
@@ -1701,7 +1701,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Звичайний" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1717,9 +1717,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Тема &quot;Office 2013 – 2022&quot;">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
   <a:themeElements>
-    <a:clrScheme name="Office 2013–2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1757,7 +1757,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013–2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1863,7 +1863,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013–2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -2005,7 +2005,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -2015,7 +2015,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6961A5F-F8EA-4989-8112-A0ACE51D011E}">
   <sheetPr codeName="Hoja1"/>
   <dimension ref="A1:D150"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="37" style="2" customWidth="1"/>
     <col min="2" max="4" width="45.7109375" style="2" customWidth="1"/>
@@ -2033,7 +2033,7 @@
         <v>70</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
@@ -2047,7 +2047,7 @@
         <v>162</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -2061,7 +2061,7 @@
         <v>125</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -2075,7 +2075,7 @@
         <v>128</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -2089,7 +2089,7 @@
         <v>131</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -2103,7 +2103,7 @@
         <v>134</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -2117,7 +2117,7 @@
         <v>137</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -2131,7 +2131,7 @@
         <v>71</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -2145,7 +2145,7 @@
         <v>72</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
@@ -2159,7 +2159,7 @@
         <v>73</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
@@ -2173,7 +2173,7 @@
         <v>74</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
@@ -2187,7 +2187,7 @@
         <v>75</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
@@ -2201,7 +2201,7 @@
         <v>76</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
@@ -2215,7 +2215,7 @@
         <v>77</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
@@ -2229,7 +2229,7 @@
         <v>78</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
@@ -2243,7 +2243,7 @@
         <v>79</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
@@ -2257,7 +2257,7 @@
         <v>80</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
@@ -2271,7 +2271,7 @@
         <v>81</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
@@ -2285,7 +2285,7 @@
         <v>82</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
@@ -2299,7 +2299,7 @@
         <v>83</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
@@ -2313,7 +2313,7 @@
         <v>84</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
@@ -2327,7 +2327,7 @@
         <v>85</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
@@ -2341,7 +2341,7 @@
         <v>86</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
@@ -2355,7 +2355,7 @@
         <v>87</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
@@ -2369,7 +2369,7 @@
         <v>88</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
@@ -2383,7 +2383,7 @@
         <v>89</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
@@ -2397,7 +2397,7 @@
         <v>90</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
@@ -2411,7 +2411,7 @@
         <v>91</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
@@ -2425,7 +2425,7 @@
         <v>92</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
@@ -2439,7 +2439,7 @@
         <v>93</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
@@ -2453,7 +2453,7 @@
         <v>50</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
@@ -2467,7 +2467,7 @@
         <v>94</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
@@ -2481,7 +2481,7 @@
         <v>95</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
@@ -2495,7 +2495,7 @@
         <v>96</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
@@ -2509,7 +2509,7 @@
         <v>97</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
@@ -2523,7 +2523,7 @@
         <v>98</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
@@ -2537,7 +2537,7 @@
         <v>99</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
@@ -2551,7 +2551,7 @@
         <v>100</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
     </row>
     <row r="39" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2565,171 +2565,171 @@
         <v>66</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="B40" s="2" t="s">
         <v>281</v>
       </c>
-      <c r="B40" s="2" t="s">
+      <c r="C40" s="2" t="s">
         <v>282</v>
       </c>
-      <c r="C40" s="2" t="s">
-        <v>283</v>
-      </c>
       <c r="D40" s="2" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="B41" s="2" t="s">
         <v>284</v>
       </c>
-      <c r="B41" s="2" t="s">
+      <c r="C41" s="2" t="s">
         <v>285</v>
       </c>
-      <c r="C41" s="2" t="s">
-        <v>286</v>
-      </c>
       <c r="D41" s="2" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
+        <v>286</v>
+      </c>
+      <c r="B42" s="2" t="s">
         <v>287</v>
       </c>
-      <c r="B42" s="2" t="s">
+      <c r="C42" s="2" t="s">
         <v>288</v>
       </c>
-      <c r="C42" s="2" t="s">
-        <v>289</v>
-      </c>
       <c r="D42" s="2" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
+        <v>303</v>
+      </c>
+      <c r="B43" s="2" t="s">
         <v>304</v>
       </c>
-      <c r="B43" s="2" t="s">
+      <c r="C43" s="2" t="s">
         <v>305</v>
       </c>
-      <c r="C43" s="2" t="s">
-        <v>306</v>
-      </c>
       <c r="D43" s="2" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
+        <v>440</v>
+      </c>
+      <c r="B44" s="2" t="s">
         <v>441</v>
       </c>
-      <c r="B44" s="2" t="s">
-        <v>442</v>
-      </c>
       <c r="C44" s="2" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
+        <v>442</v>
+      </c>
+      <c r="B45" s="2" t="s">
         <v>443</v>
       </c>
-      <c r="B45" s="2" t="s">
+      <c r="C45" s="2" t="s">
+        <v>443</v>
+      </c>
+      <c r="D45" s="2" t="s">
         <v>444</v>
-      </c>
-      <c r="C45" s="2" t="s">
-        <v>444</v>
-      </c>
-      <c r="D45" s="2" t="s">
-        <v>445</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
+        <v>452</v>
+      </c>
+      <c r="B46" s="2" t="s">
         <v>453</v>
       </c>
-      <c r="B46" s="2" t="s">
+      <c r="C46" s="2" t="s">
+        <v>458</v>
+      </c>
+      <c r="D46" s="2" t="s">
         <v>454</v>
-      </c>
-      <c r="C46" s="2" t="s">
-        <v>459</v>
-      </c>
-      <c r="D46" s="2" t="s">
-        <v>455</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
+        <v>455</v>
+      </c>
+      <c r="B47" s="2" t="s">
         <v>456</v>
       </c>
-      <c r="B47" s="2" t="s">
+      <c r="C47" s="2" t="s">
+        <v>456</v>
+      </c>
+      <c r="D47" s="2" t="s">
         <v>457</v>
-      </c>
-      <c r="C47" s="2" t="s">
-        <v>457</v>
-      </c>
-      <c r="D47" s="2" t="s">
-        <v>458</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
+        <v>464</v>
+      </c>
+      <c r="B48" s="2" t="s">
         <v>465</v>
       </c>
-      <c r="B48" s="2" t="s">
+      <c r="C48" s="2" t="s">
         <v>466</v>
-      </c>
-      <c r="C48" s="2" t="s">
-        <v>467</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
+        <v>467</v>
+      </c>
+      <c r="B49" s="2" t="s">
         <v>468</v>
       </c>
-      <c r="B49" s="2" t="s">
+      <c r="C49" s="2" t="s">
         <v>469</v>
-      </c>
-      <c r="C49" s="2" t="s">
-        <v>470</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
+        <v>470</v>
+      </c>
+      <c r="B50" s="2" t="s">
         <v>471</v>
       </c>
-      <c r="B50" s="2" t="s">
+      <c r="C50" s="2" t="s">
         <v>472</v>
-      </c>
-      <c r="C50" s="2" t="s">
-        <v>473</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
+        <v>510</v>
+      </c>
+      <c r="B51" s="2" t="s">
+        <v>511</v>
+      </c>
+      <c r="D51" s="2" t="s">
         <v>512</v>
-      </c>
-      <c r="B51" s="2" t="s">
-        <v>513</v>
-      </c>
-      <c r="D51" s="2" t="s">
-        <v>514</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
+        <v>516</v>
+      </c>
+      <c r="B52" s="2" t="s">
+        <v>517</v>
+      </c>
+      <c r="D52" s="2" t="s">
         <v>518</v>
-      </c>
-      <c r="B52" s="2" t="s">
-        <v>519</v>
-      </c>
-      <c r="D52" s="2" t="s">
-        <v>520</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
@@ -2743,7 +2743,7 @@
         <v>101</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
@@ -2757,7 +2757,7 @@
         <v>102</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
@@ -2771,7 +2771,7 @@
         <v>103</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
@@ -2785,7 +2785,7 @@
         <v>104</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
@@ -2799,7 +2799,7 @@
         <v>109</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
@@ -2813,7 +2813,7 @@
         <v>113</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
@@ -2827,7 +2827,7 @@
         <v>116</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
@@ -2841,7 +2841,7 @@
         <v>120</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
@@ -2855,54 +2855,54 @@
         <v>121</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" s="2" t="s">
+        <v>445</v>
+      </c>
+      <c r="B62" s="2" t="s">
         <v>446</v>
       </c>
-      <c r="B62" s="2" t="s">
+      <c r="C62" s="2" t="s">
+        <v>459</v>
+      </c>
+      <c r="D62" s="2" t="s">
         <v>447</v>
-      </c>
-      <c r="C62" s="2" t="s">
-        <v>460</v>
-      </c>
-      <c r="D62" s="2" t="s">
-        <v>448</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63" s="2" t="s">
+        <v>513</v>
+      </c>
+      <c r="B63" s="2" t="s">
+        <v>514</v>
+      </c>
+      <c r="D63" s="2" t="s">
         <v>515</v>
-      </c>
-      <c r="B63" s="2" t="s">
-        <v>516</v>
-      </c>
-      <c r="D63" s="2" t="s">
-        <v>517</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" s="2" t="s">
+        <v>519</v>
+      </c>
+      <c r="B64" s="2" t="s">
+        <v>520</v>
+      </c>
+      <c r="D64" s="2" t="s">
         <v>521</v>
-      </c>
-      <c r="B64" s="2" t="s">
-        <v>522</v>
-      </c>
-      <c r="D64" s="2" t="s">
-        <v>523</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A65" s="2" t="s">
+        <v>522</v>
+      </c>
+      <c r="B65" s="2" t="s">
+        <v>523</v>
+      </c>
+      <c r="D65" s="2" t="s">
         <v>524</v>
-      </c>
-      <c r="B65" s="2" t="s">
-        <v>525</v>
-      </c>
-      <c r="D65" s="2" t="s">
-        <v>526</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
@@ -2916,7 +2916,7 @@
         <v>156</v>
       </c>
       <c r="D66" s="2" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
@@ -2930,7 +2930,7 @@
         <v>166</v>
       </c>
       <c r="D67" s="2" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
@@ -2944,7 +2944,7 @@
         <v>159</v>
       </c>
       <c r="D68" s="2" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
@@ -2958,7 +2958,7 @@
         <v>169</v>
       </c>
       <c r="D69" s="2" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.25">
@@ -2972,7 +2972,7 @@
         <v>143</v>
       </c>
       <c r="D70" s="2" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
     </row>
     <row r="71" spans="1:4" ht="45" x14ac:dyDescent="0.25">
@@ -2986,7 +2986,7 @@
         <v>145</v>
       </c>
       <c r="D71" s="2" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
@@ -3000,7 +3000,7 @@
         <v>146</v>
       </c>
       <c r="D72" s="2" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
@@ -3014,7 +3014,7 @@
         <v>149</v>
       </c>
       <c r="D73" s="2" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">
@@ -3028,7 +3028,7 @@
         <v>152</v>
       </c>
       <c r="D74" s="2" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
@@ -3042,7 +3042,7 @@
         <v>171</v>
       </c>
       <c r="D75" s="2" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
@@ -3056,7 +3056,7 @@
         <v>175</v>
       </c>
       <c r="D76" s="2" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
@@ -3070,7 +3070,7 @@
         <v>177</v>
       </c>
       <c r="D77" s="2" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.25">
@@ -3084,7 +3084,7 @@
         <v>179</v>
       </c>
       <c r="D78" s="2" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
@@ -3098,21 +3098,21 @@
         <v>181</v>
       </c>
       <c r="D79" s="2" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B80" s="2" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C80" s="2" t="s">
         <v>95</v>
       </c>
       <c r="D80" s="2" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
     </row>
     <row r="81" spans="1:4" ht="30" x14ac:dyDescent="0.25">
@@ -3126,7 +3126,7 @@
         <v>139</v>
       </c>
       <c r="D81" s="2" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">
@@ -3140,7 +3140,7 @@
         <v>183</v>
       </c>
       <c r="D82" s="2" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.25">
@@ -3154,7 +3154,7 @@
         <v>185</v>
       </c>
       <c r="D83" s="2" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.25">
@@ -3168,7 +3168,7 @@
         <v>187</v>
       </c>
       <c r="D84" s="2" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.25">
@@ -3176,866 +3176,866 @@
         <v>188</v>
       </c>
       <c r="B85" s="2" t="s">
+        <v>526</v>
+      </c>
+      <c r="C85" s="2" t="s">
         <v>189</v>
       </c>
-      <c r="C85" s="2" t="s">
-        <v>190</v>
-      </c>
       <c r="D85" s="2" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A86" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="B86" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="C86" s="2" t="s">
         <v>191</v>
       </c>
-      <c r="B86" s="2" t="s">
-        <v>191</v>
-      </c>
-      <c r="C86" s="2" t="s">
-        <v>192</v>
-      </c>
       <c r="D86" s="2" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A87" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="B87" s="2" t="s">
         <v>193</v>
       </c>
-      <c r="B87" s="2" t="s">
+      <c r="C87" s="2" t="s">
         <v>194</v>
       </c>
-      <c r="C87" s="2" t="s">
-        <v>195</v>
-      </c>
       <c r="D87" s="2" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A88" s="2" t="s">
+        <v>434</v>
+      </c>
+      <c r="B88" s="4" t="s">
         <v>435</v>
       </c>
-      <c r="B88" s="4" t="s">
+      <c r="C88" s="4" t="s">
         <v>436</v>
-      </c>
-      <c r="C88" s="4" t="s">
-        <v>437</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A89" s="2" t="s">
+        <v>437</v>
+      </c>
+      <c r="B89" s="4" t="s">
         <v>438</v>
       </c>
-      <c r="B89" s="4" t="s">
+      <c r="C89" s="4" t="s">
         <v>439</v>
-      </c>
-      <c r="C89" s="4" t="s">
-        <v>440</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A90" s="2" t="s">
+        <v>473</v>
+      </c>
+      <c r="B90" s="4" t="s">
         <v>474</v>
       </c>
-      <c r="B90" s="4" t="s">
+      <c r="C90" s="4" t="s">
         <v>475</v>
-      </c>
-      <c r="C90" s="4" t="s">
-        <v>476</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A91" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="B91" s="2" t="s">
         <v>196</v>
       </c>
-      <c r="B91" s="2" t="s">
+      <c r="C91" s="2" t="s">
         <v>197</v>
       </c>
-      <c r="C91" s="2" t="s">
-        <v>198</v>
-      </c>
       <c r="D91" s="2" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A92" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="B92" s="2" t="s">
         <v>199</v>
       </c>
-      <c r="B92" s="2" t="s">
+      <c r="C92" s="2" t="s">
         <v>200</v>
       </c>
-      <c r="C92" s="2" t="s">
-        <v>201</v>
-      </c>
       <c r="D92" s="2" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A93" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="B93" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="C93" s="2" t="s">
         <v>202</v>
       </c>
-      <c r="B93" s="2" t="s">
-        <v>202</v>
-      </c>
-      <c r="C93" s="2" t="s">
-        <v>203</v>
-      </c>
       <c r="D93" s="2" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A94" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="B94" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="C94" s="2" t="s">
         <v>204</v>
       </c>
-      <c r="B94" s="2" t="s">
-        <v>204</v>
-      </c>
-      <c r="C94" s="2" t="s">
-        <v>205</v>
-      </c>
       <c r="D94" s="2" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A95" s="2" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B95" s="2" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C95" s="2" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="D95" s="2" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A96" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="B96" s="2" t="s">
         <v>207</v>
       </c>
-      <c r="B96" s="2" t="s">
+      <c r="C96" s="2" t="s">
         <v>208</v>
       </c>
-      <c r="C96" s="2" t="s">
-        <v>209</v>
-      </c>
       <c r="D96" s="2" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A97" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="B97" s="2" t="s">
         <v>210</v>
       </c>
-      <c r="B97" s="2" t="s">
+      <c r="C97" s="2" t="s">
         <v>211</v>
       </c>
-      <c r="C97" s="2" t="s">
-        <v>212</v>
-      </c>
       <c r="D97" s="2" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A98" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="B98" s="2" t="s">
         <v>213</v>
       </c>
-      <c r="B98" s="2" t="s">
+      <c r="C98" s="2" t="s">
         <v>214</v>
       </c>
-      <c r="C98" s="2" t="s">
-        <v>215</v>
-      </c>
       <c r="D98" s="2" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A99" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="B99" s="2" t="s">
         <v>216</v>
       </c>
-      <c r="B99" s="2" t="s">
+      <c r="C99" s="2" t="s">
         <v>217</v>
       </c>
-      <c r="C99" s="2" t="s">
-        <v>218</v>
-      </c>
       <c r="D99" s="2" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A100" s="2" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="B100" s="2" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="C100" s="2" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="D100" s="2" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A101" s="2" t="s">
+        <v>292</v>
+      </c>
+      <c r="B101" s="2" t="s">
+        <v>292</v>
+      </c>
+      <c r="C101" s="2" t="s">
         <v>293</v>
       </c>
-      <c r="B101" s="2" t="s">
-        <v>293</v>
-      </c>
-      <c r="C101" s="2" t="s">
-        <v>294</v>
-      </c>
       <c r="D101" s="2" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A102" s="2" t="s">
+        <v>294</v>
+      </c>
+      <c r="B102" s="2" t="s">
         <v>295</v>
       </c>
-      <c r="B102" s="2" t="s">
+      <c r="C102" s="2" t="s">
         <v>296</v>
       </c>
-      <c r="C102" s="2" t="s">
-        <v>297</v>
-      </c>
       <c r="D102" s="2" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A103" s="2" t="s">
+        <v>297</v>
+      </c>
+      <c r="B103" s="2" t="s">
         <v>298</v>
       </c>
-      <c r="B103" s="2" t="s">
+      <c r="C103" s="2" t="s">
         <v>299</v>
       </c>
-      <c r="C103" s="2" t="s">
-        <v>300</v>
-      </c>
       <c r="D103" s="2" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A104" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="B104" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="C104" s="2" t="s">
         <v>222</v>
       </c>
-      <c r="B104" s="2" t="s">
-        <v>222</v>
-      </c>
-      <c r="C104" s="2" t="s">
-        <v>223</v>
-      </c>
       <c r="D104" s="2" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A105" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="B105" s="2" t="s">
         <v>224</v>
       </c>
-      <c r="B105" s="2" t="s">
+      <c r="C105" s="2" t="s">
         <v>225</v>
       </c>
-      <c r="C105" s="2" t="s">
-        <v>226</v>
-      </c>
       <c r="D105" s="2" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A106" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="B106" s="2" t="s">
         <v>227</v>
       </c>
-      <c r="B106" s="2" t="s">
+      <c r="C106" s="2" t="s">
         <v>228</v>
       </c>
-      <c r="C106" s="2" t="s">
-        <v>229</v>
-      </c>
       <c r="D106" s="2" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A107" s="2" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B107" s="2" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="C107" s="2" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="D107" s="2" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A108" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="B108" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="C108" s="2" t="s">
         <v>231</v>
       </c>
-      <c r="B108" s="2" t="s">
-        <v>231</v>
-      </c>
-      <c r="C108" s="2" t="s">
-        <v>232</v>
-      </c>
       <c r="D108" s="2" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A109" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="B109" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="C109" s="2" t="s">
         <v>233</v>
       </c>
-      <c r="B109" s="2" t="s">
-        <v>233</v>
-      </c>
-      <c r="C109" s="2" t="s">
-        <v>234</v>
-      </c>
       <c r="D109" s="2" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A110" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="B110" s="2" t="s">
         <v>235</v>
       </c>
-      <c r="B110" s="2" t="s">
+      <c r="C110" s="2" t="s">
         <v>236</v>
       </c>
-      <c r="C110" s="2" t="s">
-        <v>237</v>
-      </c>
       <c r="D110" s="2" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A111" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="B111" s="2" t="s">
         <v>238</v>
       </c>
-      <c r="B111" s="2" t="s">
+      <c r="C111" s="2" t="s">
         <v>239</v>
       </c>
-      <c r="C111" s="2" t="s">
-        <v>240</v>
-      </c>
       <c r="D111" s="2" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A112" s="2" t="s">
+        <v>300</v>
+      </c>
+      <c r="B112" s="2" t="s">
         <v>301</v>
       </c>
-      <c r="B112" s="2" t="s">
+      <c r="C112" s="2" t="s">
         <v>302</v>
       </c>
-      <c r="C112" s="2" t="s">
-        <v>303</v>
-      </c>
       <c r="D112" s="2" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A113" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="B113" s="2" t="s">
         <v>241</v>
       </c>
-      <c r="B113" s="2" t="s">
+      <c r="C113" s="2" t="s">
         <v>242</v>
       </c>
-      <c r="C113" s="2" t="s">
-        <v>243</v>
-      </c>
       <c r="D113" s="2" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A114" s="2" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B114" s="2" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="C114" s="2" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="D114" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A115" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="B115" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="C115" s="2" t="s">
         <v>246</v>
       </c>
-      <c r="B115" s="2" t="s">
-        <v>246</v>
-      </c>
-      <c r="C115" s="2" t="s">
-        <v>247</v>
-      </c>
       <c r="D115" s="2" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A116" s="2" t="s">
+        <v>247</v>
+      </c>
+      <c r="B116" s="2" t="s">
+        <v>247</v>
+      </c>
+      <c r="C116" s="2" t="s">
         <v>248</v>
       </c>
-      <c r="B116" s="2" t="s">
-        <v>248</v>
-      </c>
-      <c r="C116" s="2" t="s">
-        <v>249</v>
-      </c>
       <c r="D116" s="2" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A117" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="B117" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="C117" s="2" t="s">
         <v>250</v>
       </c>
-      <c r="B117" s="2" t="s">
-        <v>250</v>
-      </c>
-      <c r="C117" s="2" t="s">
-        <v>251</v>
-      </c>
       <c r="D117" s="2" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A118" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="B118" s="2" t="s">
         <v>254</v>
       </c>
-      <c r="B118" s="2" t="s">
+      <c r="C118" s="2" t="s">
         <v>255</v>
       </c>
-      <c r="C118" s="2" t="s">
-        <v>256</v>
-      </c>
       <c r="D118" s="2" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
     </row>
     <row r="119" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A119" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="B119" s="2" t="s">
         <v>257</v>
       </c>
-      <c r="B119" s="2" t="s">
+      <c r="C119" s="2" t="s">
         <v>258</v>
       </c>
-      <c r="C119" s="2" t="s">
-        <v>259</v>
-      </c>
       <c r="D119" s="2" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A120" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="B120" s="2" t="s">
         <v>260</v>
       </c>
-      <c r="B120" s="2" t="s">
+      <c r="C120" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="C120" s="2" t="s">
-        <v>262</v>
-      </c>
       <c r="D120" s="2" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A121" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="B121" s="2" t="s">
         <v>263</v>
       </c>
-      <c r="B121" s="2" t="s">
+      <c r="C121" s="2" t="s">
         <v>264</v>
       </c>
-      <c r="C121" s="2" t="s">
-        <v>265</v>
-      </c>
       <c r="D121" s="2" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A122" s="2" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="B122" s="2" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="C122" s="2" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="D122" s="2" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
     </row>
     <row r="123" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A123" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="B123" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="C123" s="2" t="s">
         <v>267</v>
       </c>
-      <c r="B123" s="2" t="s">
-        <v>267</v>
-      </c>
-      <c r="C123" s="2" t="s">
-        <v>268</v>
-      </c>
       <c r="D123" s="2" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
     </row>
     <row r="124" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A124" s="2" t="s">
+        <v>268</v>
+      </c>
+      <c r="B124" s="2" t="s">
+        <v>268</v>
+      </c>
+      <c r="C124" s="2" t="s">
         <v>269</v>
       </c>
-      <c r="B124" s="2" t="s">
-        <v>269</v>
-      </c>
-      <c r="C124" s="2" t="s">
-        <v>270</v>
-      </c>
       <c r="D124" s="2" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
     </row>
     <row r="125" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A125" s="2" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="B125" s="2" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="C125" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="D125" s="2" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
     </row>
     <row r="126" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A126" s="2" t="s">
+        <v>271</v>
+      </c>
+      <c r="B126" s="2" t="s">
+        <v>271</v>
+      </c>
+      <c r="C126" s="2" t="s">
         <v>272</v>
       </c>
-      <c r="B126" s="2" t="s">
-        <v>272</v>
-      </c>
-      <c r="C126" s="2" t="s">
-        <v>273</v>
-      </c>
       <c r="D126" s="2" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
     </row>
     <row r="127" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A127" s="2" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="B127" s="2" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="C127" s="2" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="128" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A128" s="2" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="B128" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="C128" s="2" t="s">
         <v>278</v>
-      </c>
-      <c r="C128" s="2" t="s">
-        <v>279</v>
       </c>
     </row>
     <row r="129" spans="1:4" ht="75" x14ac:dyDescent="0.25">
       <c r="A129" s="2" t="s">
+        <v>289</v>
+      </c>
+      <c r="B129" s="2" t="s">
         <v>290</v>
       </c>
-      <c r="B129" s="2" t="s">
+      <c r="C129" s="2" t="s">
         <v>291</v>
-      </c>
-      <c r="C129" s="2" t="s">
-        <v>292</v>
       </c>
     </row>
     <row r="130" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A130" s="2" t="s">
+        <v>306</v>
+      </c>
+      <c r="B130" s="2" t="s">
         <v>307</v>
       </c>
-      <c r="B130" s="2" t="s">
+      <c r="C130" s="2" t="s">
         <v>308</v>
       </c>
-      <c r="C130" s="2" t="s">
-        <v>309</v>
-      </c>
       <c r="D130" s="2" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
     </row>
     <row r="131" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A131" s="2" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="B131" s="2" t="s">
+        <v>311</v>
+      </c>
+      <c r="C131" s="2" t="s">
         <v>312</v>
       </c>
-      <c r="C131" s="2" t="s">
-        <v>313</v>
-      </c>
       <c r="D131" s="2" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
     </row>
     <row r="132" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A132" s="2" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="B132" s="2" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="C132" s="2" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="D132" s="2" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
     </row>
     <row r="133" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A133" s="2" t="s">
+        <v>315</v>
+      </c>
+      <c r="B133" s="2" t="s">
+        <v>315</v>
+      </c>
+      <c r="C133" s="2" t="s">
         <v>316</v>
       </c>
-      <c r="B133" s="2" t="s">
-        <v>316</v>
-      </c>
-      <c r="C133" s="2" t="s">
-        <v>317</v>
-      </c>
       <c r="D133" s="2" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
     </row>
     <row r="134" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A134" s="2" t="s">
+        <v>317</v>
+      </c>
+      <c r="B134" s="2" t="s">
         <v>318</v>
       </c>
-      <c r="B134" s="2" t="s">
-        <v>319</v>
-      </c>
       <c r="C134" s="2" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="D134" s="2" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
     </row>
     <row r="135" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A135" s="2" t="s">
+        <v>319</v>
+      </c>
+      <c r="B135" s="2" t="s">
         <v>320</v>
       </c>
-      <c r="B135" s="2" t="s">
-        <v>321</v>
-      </c>
       <c r="C135" s="2" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="D135" s="2" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="136" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A136" s="2" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="B136" s="2" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="C136" s="2" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="D136" s="2" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="137" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A137" s="2" t="s">
+        <v>449</v>
+      </c>
+      <c r="B137" s="2" t="s">
         <v>450</v>
       </c>
-      <c r="B137" s="2" t="s">
+      <c r="C137" s="2" t="s">
+        <v>463</v>
+      </c>
+      <c r="D137" s="2" t="s">
         <v>451</v>
-      </c>
-      <c r="C137" s="2" t="s">
-        <v>464</v>
-      </c>
-      <c r="D137" s="2" t="s">
-        <v>452</v>
       </c>
     </row>
     <row r="138" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A138" s="2" t="s">
+        <v>476</v>
+      </c>
+      <c r="B138" s="2" t="s">
         <v>477</v>
       </c>
-      <c r="B138" s="2" t="s">
+      <c r="C138" s="2" t="s">
         <v>478</v>
-      </c>
-      <c r="C138" s="2" t="s">
-        <v>479</v>
       </c>
     </row>
     <row r="139" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A139" s="2" t="s">
+        <v>479</v>
+      </c>
+      <c r="B139" s="2" t="s">
+        <v>525</v>
+      </c>
+      <c r="C139" s="2" t="s">
         <v>480</v>
-      </c>
-      <c r="B139" s="2" t="s">
-        <v>481</v>
-      </c>
-      <c r="C139" s="2" t="s">
-        <v>482</v>
       </c>
     </row>
     <row r="140" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A140" s="2" t="s">
+        <v>481</v>
+      </c>
+      <c r="B140" s="2" t="s">
+        <v>482</v>
+      </c>
+      <c r="C140" s="2" t="s">
         <v>483</v>
-      </c>
-      <c r="B140" s="2" t="s">
-        <v>484</v>
-      </c>
-      <c r="C140" s="2" t="s">
-        <v>485</v>
       </c>
     </row>
     <row r="141" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A141" s="2" t="s">
+        <v>484</v>
+      </c>
+      <c r="B141" s="2" t="s">
+        <v>485</v>
+      </c>
+      <c r="C141" s="2" t="s">
         <v>486</v>
-      </c>
-      <c r="B141" s="2" t="s">
-        <v>487</v>
-      </c>
-      <c r="C141" s="2" t="s">
-        <v>488</v>
       </c>
     </row>
     <row r="142" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A142" s="2" t="s">
+        <v>487</v>
+      </c>
+      <c r="B142" s="2" t="s">
+        <v>488</v>
+      </c>
+      <c r="C142" s="2" t="s">
         <v>489</v>
-      </c>
-      <c r="B142" s="2" t="s">
-        <v>490</v>
-      </c>
-      <c r="C142" s="2" t="s">
-        <v>491</v>
       </c>
     </row>
     <row r="143" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A143" s="2" t="s">
+        <v>490</v>
+      </c>
+      <c r="B143" s="2" t="s">
+        <v>491</v>
+      </c>
+      <c r="C143" s="2" t="s">
         <v>492</v>
-      </c>
-      <c r="B143" s="2" t="s">
-        <v>493</v>
-      </c>
-      <c r="C143" s="2" t="s">
-        <v>494</v>
       </c>
     </row>
     <row r="144" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A144" s="2" t="s">
+        <v>493</v>
+      </c>
+      <c r="B144" s="2" t="s">
+        <v>494</v>
+      </c>
+      <c r="C144" s="2" t="s">
         <v>495</v>
-      </c>
-      <c r="B144" s="2" t="s">
-        <v>496</v>
-      </c>
-      <c r="C144" s="2" t="s">
-        <v>497</v>
       </c>
     </row>
     <row r="145" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A145" s="2" t="s">
+        <v>496</v>
+      </c>
+      <c r="B145" s="2" t="s">
+        <v>497</v>
+      </c>
+      <c r="C145" s="2" t="s">
         <v>498</v>
-      </c>
-      <c r="B145" s="2" t="s">
-        <v>499</v>
-      </c>
-      <c r="C145" s="2" t="s">
-        <v>500</v>
       </c>
     </row>
     <row r="146" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A146" s="2" t="s">
+        <v>499</v>
+      </c>
+      <c r="B146" s="2" t="s">
+        <v>500</v>
+      </c>
+      <c r="C146" s="2" t="s">
         <v>501</v>
-      </c>
-      <c r="B146" s="2" t="s">
-        <v>502</v>
-      </c>
-      <c r="C146" s="2" t="s">
-        <v>503</v>
       </c>
     </row>
     <row r="147" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A147" s="2" t="s">
-        <v>504</v>
+        <v>502</v>
       </c>
       <c r="B147" s="2" t="s">
-        <v>504</v>
+        <v>502</v>
       </c>
       <c r="C147" s="2" t="s">
-        <v>505</v>
+        <v>503</v>
       </c>
     </row>
     <row r="148" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A148" s="2" t="s">
-        <v>506</v>
+        <v>504</v>
       </c>
       <c r="B148" s="2" t="s">
-        <v>506</v>
+        <v>504</v>
       </c>
       <c r="C148" s="2" t="s">
-        <v>507</v>
+        <v>505</v>
       </c>
     </row>
     <row r="149" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A149" s="2" t="s">
-        <v>508</v>
+        <v>506</v>
       </c>
       <c r="B149" s="2" t="s">
-        <v>508</v>
+        <v>506</v>
       </c>
       <c r="C149" s="2" t="s">
-        <v>509</v>
+        <v>507</v>
       </c>
     </row>
     <row r="150" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A150" s="2" t="s">
-        <v>510</v>
+        <v>508</v>
       </c>
       <c r="B150" s="2" t="s">
-        <v>510</v>
+        <v>508</v>
       </c>
       <c r="C150" s="2" t="s">
-        <v>511</v>
+        <v>509</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Reverted EVERYTHING and fixed EVERYTHING merging EVERYTHING and makingEVERYTHING work
</commit_message>
<xml_diff>
--- a/Translations/Translations.xlsx
+++ b/Translations/Translations.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programacion\MelonLoader\FS_LevelEditor\Translations\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Codes\c#\FrSLE\Translations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8436EDEC-EAFE-4595-BBB7-A6783CBD918B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B620771-43AB-47DC-B1FF-39E53DA3078C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{F5C22481-FF1A-482C-BF7E-EB5A7718AF49}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15900" xr2:uid="{F5C22481-FF1A-482C-BF7E-EB5A7718AF49}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="572" uniqueCount="527">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="592" uniqueCount="546">
   <si>
     <t>ID</t>
   </si>
@@ -1615,6 +1615,63 @@
   </si>
   <si>
     <t>Start Enabled</t>
+  </si>
+  <si>
+    <t>object.CUBE_KILLPLANE</t>
+  </si>
+  <si>
+    <t>Unauthorized Object</t>
+  </si>
+  <si>
+    <t>Неавторизований об'єкт</t>
+  </si>
+  <si>
+    <t>object.KEYPAD</t>
+  </si>
+  <si>
+    <t>Keypad</t>
+  </si>
+  <si>
+    <t>Циферблат</t>
+  </si>
+  <si>
+    <t>events.onWinEvents</t>
+  </si>
+  <si>
+    <t>On Win</t>
+  </si>
+  <si>
+    <t>При правильній комбінації</t>
+  </si>
+  <si>
+    <t>On Lose</t>
+  </si>
+  <si>
+    <t>При неправильній комбінації</t>
+  </si>
+  <si>
+    <t>leaveOnIncorrect</t>
+  </si>
+  <si>
+    <t>Leave on Incorrect</t>
+  </si>
+  <si>
+    <t>events.onFailEvents</t>
+  </si>
+  <si>
+    <t>Keycode</t>
+  </si>
+  <si>
+    <t>Код</t>
+  </si>
+  <si>
+    <t>IgnoreIfInHands</t>
+  </si>
+  <si>
+    <t>Ignore if currently picked up</t>
+  </si>
+  <si>
+    <t>Ігнорувати, якщо піднято</t>
   </si>
 </sst>
 </file>
@@ -1701,7 +1758,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Звичайний" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1717,9 +1774,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Тема &quot;Office 2013 – 2022&quot;">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013–2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1757,7 +1814,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013–2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1863,7 +1920,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013–2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -2005,7 +2062,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -2014,8 +2071,8 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6961A5F-F8EA-4989-8112-A0ACE51D011E}">
   <sheetPr codeName="Hoja1"/>
-  <dimension ref="A1:D150"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:D157"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="37" style="2" customWidth="1"/>
     <col min="2" max="4" width="45.7109375" style="2" customWidth="1"/>
@@ -2734,1307 +2791,1381 @@
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" s="2" t="s">
-        <v>69</v>
+        <v>527</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="C53" s="2" t="s">
-        <v>101</v>
+        <v>528</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>364</v>
+        <v>529</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" s="2" t="s">
-        <v>105</v>
+        <v>530</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="C54" s="2" t="s">
-        <v>102</v>
+        <v>531</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>365</v>
+        <v>532</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A55" s="2" t="s">
-        <v>106</v>
+        <v>69</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>3</v>
+        <v>69</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57" s="2" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>111</v>
+        <v>3</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" s="2" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>112</v>
+        <v>4</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>113</v>
+        <v>104</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" s="2" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>116</v>
+        <v>109</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>368</v>
+        <v>365</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
-        <v>117</v>
+        <v>110</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>119</v>
+        <v>112</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>120</v>
+        <v>113</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61" s="2" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" s="2" t="s">
-        <v>445</v>
+        <v>117</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>446</v>
+        <v>119</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>459</v>
+        <v>120</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>447</v>
+        <v>369</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63" s="2" t="s">
-        <v>513</v>
+        <v>118</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>514</v>
+        <v>122</v>
+      </c>
+      <c r="C63" s="2" t="s">
+        <v>121</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>515</v>
+        <v>370</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" s="2" t="s">
-        <v>519</v>
+        <v>445</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>520</v>
+        <v>446</v>
+      </c>
+      <c r="C64" s="2" t="s">
+        <v>459</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>521</v>
+        <v>447</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A65" s="2" t="s">
-        <v>522</v>
+        <v>513</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>523</v>
+        <v>514</v>
       </c>
       <c r="D65" s="2" t="s">
-        <v>524</v>
+        <v>515</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66" s="2" t="s">
-        <v>154</v>
+        <v>519</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="C66" s="2" t="s">
-        <v>156</v>
+        <v>520</v>
       </c>
       <c r="D66" s="2" t="s">
-        <v>371</v>
+        <v>521</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A67" s="2" t="s">
-        <v>164</v>
+        <v>522</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>165</v>
-      </c>
-      <c r="C67" s="2" t="s">
-        <v>166</v>
+        <v>523</v>
       </c>
       <c r="D67" s="2" t="s">
-        <v>372</v>
+        <v>524</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A68" s="2" t="s">
-        <v>157</v>
+        <v>533</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>158</v>
-      </c>
-      <c r="C68" s="2" t="s">
-        <v>159</v>
+        <v>534</v>
       </c>
       <c r="D68" s="2" t="s">
-        <v>373</v>
+        <v>535</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A69" s="2" t="s">
-        <v>167</v>
+        <v>540</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>168</v>
-      </c>
-      <c r="C69" s="2" t="s">
-        <v>169</v>
+        <v>536</v>
       </c>
       <c r="D69" s="2" t="s">
-        <v>374</v>
+        <v>537</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A70" s="2" t="s">
-        <v>141</v>
+        <v>154</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>142</v>
+        <v>155</v>
       </c>
       <c r="C70" s="2" t="s">
-        <v>143</v>
+        <v>156</v>
       </c>
       <c r="D70" s="2" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="71" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A71" s="2" t="s">
-        <v>144</v>
+        <v>164</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>145</v>
+        <v>166</v>
       </c>
       <c r="D71" s="2" t="s">
-        <v>376</v>
+        <v>372</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A72" s="2" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>146</v>
+        <v>158</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>146</v>
+        <v>159</v>
       </c>
       <c r="D72" s="2" t="s">
-        <v>328</v>
+        <v>373</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A73" s="2" t="s">
-        <v>147</v>
+        <v>167</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>148</v>
+        <v>168</v>
       </c>
       <c r="C73" s="2" t="s">
-        <v>149</v>
+        <v>169</v>
       </c>
       <c r="D73" s="2" t="s">
-        <v>377</v>
+        <v>374</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A74" s="2" t="s">
-        <v>150</v>
+        <v>141</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>151</v>
+        <v>142</v>
       </c>
       <c r="C74" s="2" t="s">
-        <v>152</v>
+        <v>143</v>
       </c>
       <c r="D74" s="2" t="s">
-        <v>378</v>
-      </c>
-    </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A75" s="2" t="s">
-        <v>172</v>
+        <v>144</v>
       </c>
       <c r="B75" s="2" t="s">
-        <v>170</v>
+        <v>163</v>
       </c>
       <c r="C75" s="2" t="s">
-        <v>171</v>
+        <v>145</v>
       </c>
       <c r="D75" s="2" t="s">
-        <v>379</v>
+        <v>376</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A76" s="2" t="s">
-        <v>173</v>
+        <v>153</v>
       </c>
       <c r="B76" s="2" t="s">
-        <v>174</v>
+        <v>146</v>
       </c>
       <c r="C76" s="2" t="s">
-        <v>175</v>
+        <v>146</v>
       </c>
       <c r="D76" s="2" t="s">
-        <v>380</v>
+        <v>328</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A77" s="2" t="s">
-        <v>176</v>
+        <v>147</v>
       </c>
       <c r="B77" s="2" t="s">
-        <v>176</v>
+        <v>148</v>
       </c>
       <c r="C77" s="2" t="s">
-        <v>177</v>
+        <v>149</v>
       </c>
       <c r="D77" s="2" t="s">
-        <v>381</v>
+        <v>377</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A78" s="2" t="s">
-        <v>178</v>
+        <v>150</v>
       </c>
       <c r="B78" s="2" t="s">
-        <v>178</v>
+        <v>151</v>
       </c>
       <c r="C78" s="2" t="s">
-        <v>179</v>
+        <v>152</v>
       </c>
       <c r="D78" s="2" t="s">
-        <v>382</v>
+        <v>378</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A79" s="2" t="s">
-        <v>180</v>
+        <v>172</v>
       </c>
       <c r="B79" s="2" t="s">
-        <v>180</v>
+        <v>170</v>
       </c>
       <c r="C79" s="2" t="s">
-        <v>181</v>
+        <v>171</v>
       </c>
       <c r="D79" s="2" t="s">
-        <v>383</v>
+        <v>379</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
-        <v>243</v>
+        <v>173</v>
       </c>
       <c r="B80" s="2" t="s">
-        <v>243</v>
+        <v>174</v>
       </c>
       <c r="C80" s="2" t="s">
-        <v>95</v>
+        <v>175</v>
       </c>
       <c r="D80" s="2" t="s">
-        <v>384</v>
-      </c>
-    </row>
-    <row r="81" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A81" s="2" t="s">
-        <v>138</v>
-      </c>
-      <c r="B81" s="1" t="s">
-        <v>140</v>
+        <v>176</v>
+      </c>
+      <c r="B81" s="2" t="s">
+        <v>176</v>
       </c>
       <c r="C81" s="2" t="s">
-        <v>139</v>
+        <v>177</v>
       </c>
       <c r="D81" s="2" t="s">
-        <v>385</v>
+        <v>381</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A82" s="2" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="B82" s="2" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
       <c r="C82" s="2" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="D82" s="2" t="s">
-        <v>386</v>
+        <v>382</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A83" s="2" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="B83" s="2" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="C83" s="2" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="D83" s="2" t="s">
-        <v>387</v>
+        <v>383</v>
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A84" s="2" t="s">
-        <v>186</v>
+        <v>243</v>
       </c>
       <c r="B84" s="2" t="s">
-        <v>186</v>
+        <v>243</v>
       </c>
       <c r="C84" s="2" t="s">
-        <v>187</v>
+        <v>95</v>
       </c>
       <c r="D84" s="2" t="s">
-        <v>388</v>
-      </c>
-    </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="85" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A85" s="2" t="s">
-        <v>188</v>
-      </c>
-      <c r="B85" s="2" t="s">
-        <v>526</v>
+        <v>138</v>
+      </c>
+      <c r="B85" s="1" t="s">
+        <v>140</v>
       </c>
       <c r="C85" s="2" t="s">
-        <v>189</v>
+        <v>139</v>
       </c>
       <c r="D85" s="2" t="s">
-        <v>389</v>
+        <v>385</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A86" s="2" t="s">
-        <v>190</v>
+        <v>182</v>
       </c>
       <c r="B86" s="2" t="s">
-        <v>190</v>
+        <v>183</v>
       </c>
       <c r="C86" s="2" t="s">
-        <v>191</v>
+        <v>183</v>
       </c>
       <c r="D86" s="2" t="s">
-        <v>390</v>
+        <v>386</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A87" s="2" t="s">
-        <v>192</v>
+        <v>184</v>
       </c>
       <c r="B87" s="2" t="s">
-        <v>193</v>
+        <v>184</v>
       </c>
       <c r="C87" s="2" t="s">
-        <v>194</v>
+        <v>185</v>
       </c>
       <c r="D87" s="2" t="s">
-        <v>391</v>
+        <v>387</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A88" s="2" t="s">
-        <v>434</v>
-      </c>
-      <c r="B88" s="4" t="s">
-        <v>435</v>
-      </c>
-      <c r="C88" s="4" t="s">
-        <v>436</v>
+        <v>186</v>
+      </c>
+      <c r="B88" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="C88" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="D88" s="2" t="s">
+        <v>388</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A89" s="2" t="s">
-        <v>437</v>
-      </c>
-      <c r="B89" s="4" t="s">
-        <v>438</v>
-      </c>
-      <c r="C89" s="4" t="s">
-        <v>439</v>
+        <v>188</v>
+      </c>
+      <c r="B89" s="2" t="s">
+        <v>526</v>
+      </c>
+      <c r="C89" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="D89" s="2" t="s">
+        <v>389</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A90" s="2" t="s">
-        <v>473</v>
-      </c>
-      <c r="B90" s="4" t="s">
-        <v>474</v>
-      </c>
-      <c r="C90" s="4" t="s">
-        <v>475</v>
+        <v>190</v>
+      </c>
+      <c r="B90" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="C90" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="D90" s="2" t="s">
+        <v>390</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A91" s="2" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="B91" s="2" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="C91" s="2" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="D91" s="2" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A92" s="2" t="s">
-        <v>198</v>
-      </c>
-      <c r="B92" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="C92" s="2" t="s">
-        <v>200</v>
-      </c>
-      <c r="D92" s="2" t="s">
-        <v>393</v>
+        <v>434</v>
+      </c>
+      <c r="B92" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="C92" s="4" t="s">
+        <v>436</v>
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A93" s="2" t="s">
-        <v>201</v>
-      </c>
-      <c r="B93" s="2" t="s">
-        <v>201</v>
-      </c>
-      <c r="C93" s="2" t="s">
-        <v>202</v>
-      </c>
-      <c r="D93" s="2" t="s">
-        <v>394</v>
+        <v>437</v>
+      </c>
+      <c r="B93" s="4" t="s">
+        <v>438</v>
+      </c>
+      <c r="C93" s="4" t="s">
+        <v>439</v>
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A94" s="2" t="s">
-        <v>203</v>
-      </c>
-      <c r="B94" s="2" t="s">
-        <v>203</v>
-      </c>
-      <c r="C94" s="2" t="s">
-        <v>204</v>
-      </c>
-      <c r="D94" s="2" t="s">
-        <v>395</v>
+        <v>473</v>
+      </c>
+      <c r="B94" s="4" t="s">
+        <v>474</v>
+      </c>
+      <c r="C94" s="4" t="s">
+        <v>475</v>
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A95" s="2" t="s">
-        <v>205</v>
+        <v>195</v>
       </c>
       <c r="B95" s="2" t="s">
-        <v>205</v>
+        <v>196</v>
       </c>
       <c r="C95" s="2" t="s">
-        <v>205</v>
+        <v>197</v>
       </c>
       <c r="D95" s="2" t="s">
-        <v>396</v>
+        <v>392</v>
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A96" s="2" t="s">
-        <v>206</v>
+        <v>198</v>
       </c>
       <c r="B96" s="2" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="C96" s="2" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="D96" s="2" t="s">
-        <v>397</v>
+        <v>393</v>
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A97" s="2" t="s">
-        <v>209</v>
+        <v>201</v>
       </c>
       <c r="B97" s="2" t="s">
-        <v>210</v>
+        <v>201</v>
       </c>
       <c r="C97" s="2" t="s">
-        <v>211</v>
+        <v>202</v>
       </c>
       <c r="D97" s="2" t="s">
-        <v>398</v>
+        <v>394</v>
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A98" s="2" t="s">
-        <v>212</v>
+        <v>203</v>
       </c>
       <c r="B98" s="2" t="s">
-        <v>213</v>
+        <v>203</v>
       </c>
       <c r="C98" s="2" t="s">
-        <v>214</v>
+        <v>204</v>
       </c>
       <c r="D98" s="2" t="s">
-        <v>399</v>
+        <v>395</v>
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A99" s="2" t="s">
-        <v>215</v>
+        <v>205</v>
       </c>
       <c r="B99" s="2" t="s">
-        <v>216</v>
+        <v>205</v>
       </c>
       <c r="C99" s="2" t="s">
-        <v>217</v>
+        <v>205</v>
       </c>
       <c r="D99" s="2" t="s">
-        <v>400</v>
+        <v>396</v>
       </c>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A100" s="2" t="s">
-        <v>220</v>
+        <v>206</v>
       </c>
       <c r="B100" s="2" t="s">
-        <v>219</v>
+        <v>207</v>
       </c>
       <c r="C100" s="2" t="s">
-        <v>218</v>
+        <v>208</v>
       </c>
       <c r="D100" s="2" t="s">
-        <v>401</v>
+        <v>397</v>
       </c>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A101" s="2" t="s">
-        <v>292</v>
+        <v>209</v>
       </c>
       <c r="B101" s="2" t="s">
-        <v>292</v>
+        <v>210</v>
       </c>
       <c r="C101" s="2" t="s">
-        <v>293</v>
+        <v>211</v>
       </c>
       <c r="D101" s="2" t="s">
-        <v>402</v>
+        <v>398</v>
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A102" s="2" t="s">
-        <v>294</v>
+        <v>212</v>
       </c>
       <c r="B102" s="2" t="s">
-        <v>295</v>
+        <v>213</v>
       </c>
       <c r="C102" s="2" t="s">
-        <v>296</v>
+        <v>214</v>
       </c>
       <c r="D102" s="2" t="s">
-        <v>403</v>
+        <v>399</v>
       </c>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A103" s="2" t="s">
-        <v>297</v>
+        <v>215</v>
       </c>
       <c r="B103" s="2" t="s">
-        <v>298</v>
+        <v>216</v>
       </c>
       <c r="C103" s="2" t="s">
-        <v>299</v>
+        <v>217</v>
       </c>
       <c r="D103" s="2" t="s">
-        <v>404</v>
+        <v>400</v>
       </c>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A104" s="2" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="B104" s="2" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="C104" s="2" t="s">
-        <v>222</v>
+        <v>218</v>
       </c>
       <c r="D104" s="2" t="s">
-        <v>405</v>
+        <v>401</v>
       </c>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A105" s="2" t="s">
-        <v>223</v>
+        <v>292</v>
       </c>
       <c r="B105" s="2" t="s">
-        <v>224</v>
+        <v>292</v>
       </c>
       <c r="C105" s="2" t="s">
-        <v>225</v>
+        <v>293</v>
       </c>
       <c r="D105" s="2" t="s">
-        <v>406</v>
+        <v>402</v>
       </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A106" s="2" t="s">
-        <v>226</v>
+        <v>294</v>
       </c>
       <c r="B106" s="2" t="s">
-        <v>227</v>
+        <v>295</v>
       </c>
       <c r="C106" s="2" t="s">
-        <v>228</v>
+        <v>296</v>
       </c>
       <c r="D106" s="2" t="s">
-        <v>407</v>
+        <v>403</v>
       </c>
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A107" s="2" t="s">
-        <v>229</v>
+        <v>297</v>
       </c>
       <c r="B107" s="2" t="s">
-        <v>229</v>
+        <v>298</v>
       </c>
       <c r="C107" s="2" t="s">
-        <v>229</v>
+        <v>299</v>
       </c>
       <c r="D107" s="2" t="s">
-        <v>408</v>
+        <v>404</v>
       </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A108" s="2" t="s">
-        <v>230</v>
+        <v>221</v>
       </c>
       <c r="B108" s="2" t="s">
-        <v>230</v>
+        <v>221</v>
       </c>
       <c r="C108" s="2" t="s">
-        <v>231</v>
+        <v>222</v>
       </c>
       <c r="D108" s="2" t="s">
-        <v>409</v>
+        <v>405</v>
       </c>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A109" s="2" t="s">
-        <v>232</v>
+        <v>223</v>
       </c>
       <c r="B109" s="2" t="s">
-        <v>232</v>
+        <v>224</v>
       </c>
       <c r="C109" s="2" t="s">
-        <v>233</v>
+        <v>225</v>
       </c>
       <c r="D109" s="2" t="s">
-        <v>410</v>
+        <v>406</v>
       </c>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A110" s="2" t="s">
-        <v>234</v>
+        <v>226</v>
       </c>
       <c r="B110" s="2" t="s">
-        <v>235</v>
+        <v>227</v>
       </c>
       <c r="C110" s="2" t="s">
-        <v>236</v>
+        <v>228</v>
       </c>
       <c r="D110" s="2" t="s">
-        <v>411</v>
+        <v>407</v>
       </c>
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A111" s="2" t="s">
-        <v>237</v>
+        <v>229</v>
       </c>
       <c r="B111" s="2" t="s">
-        <v>238</v>
+        <v>229</v>
       </c>
       <c r="C111" s="2" t="s">
-        <v>239</v>
+        <v>229</v>
       </c>
       <c r="D111" s="2" t="s">
-        <v>412</v>
+        <v>408</v>
       </c>
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A112" s="2" t="s">
-        <v>300</v>
+        <v>230</v>
       </c>
       <c r="B112" s="2" t="s">
-        <v>301</v>
+        <v>230</v>
       </c>
       <c r="C112" s="2" t="s">
-        <v>302</v>
+        <v>231</v>
       </c>
       <c r="D112" s="2" t="s">
-        <v>413</v>
+        <v>409</v>
       </c>
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A113" s="2" t="s">
-        <v>240</v>
+        <v>232</v>
       </c>
       <c r="B113" s="2" t="s">
-        <v>241</v>
+        <v>232</v>
       </c>
       <c r="C113" s="2" t="s">
-        <v>242</v>
+        <v>233</v>
       </c>
       <c r="D113" s="2" t="s">
-        <v>414</v>
+        <v>410</v>
       </c>
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A114" s="2" t="s">
-        <v>244</v>
+        <v>234</v>
       </c>
       <c r="B114" s="2" t="s">
-        <v>252</v>
+        <v>235</v>
       </c>
       <c r="C114" s="2" t="s">
-        <v>251</v>
+        <v>236</v>
       </c>
       <c r="D114" s="2" t="s">
-        <v>415</v>
+        <v>411</v>
       </c>
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A115" s="2" t="s">
-        <v>245</v>
+        <v>237</v>
       </c>
       <c r="B115" s="2" t="s">
-        <v>245</v>
+        <v>238</v>
       </c>
       <c r="C115" s="2" t="s">
-        <v>246</v>
+        <v>239</v>
       </c>
       <c r="D115" s="2" t="s">
-        <v>416</v>
+        <v>412</v>
       </c>
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A116" s="2" t="s">
-        <v>247</v>
+        <v>300</v>
       </c>
       <c r="B116" s="2" t="s">
-        <v>247</v>
+        <v>301</v>
       </c>
       <c r="C116" s="2" t="s">
-        <v>248</v>
+        <v>302</v>
       </c>
       <c r="D116" s="2" t="s">
-        <v>417</v>
+        <v>413</v>
       </c>
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A117" s="2" t="s">
-        <v>249</v>
+        <v>240</v>
       </c>
       <c r="B117" s="2" t="s">
-        <v>249</v>
+        <v>241</v>
       </c>
       <c r="C117" s="2" t="s">
-        <v>250</v>
+        <v>242</v>
       </c>
       <c r="D117" s="2" t="s">
-        <v>418</v>
+        <v>414</v>
       </c>
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A118" s="2" t="s">
-        <v>253</v>
+        <v>244</v>
       </c>
       <c r="B118" s="2" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="C118" s="2" t="s">
-        <v>255</v>
+        <v>251</v>
       </c>
       <c r="D118" s="2" t="s">
-        <v>419</v>
+        <v>415</v>
       </c>
     </row>
     <row r="119" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A119" s="2" t="s">
-        <v>256</v>
+        <v>245</v>
       </c>
       <c r="B119" s="2" t="s">
-        <v>257</v>
+        <v>245</v>
       </c>
       <c r="C119" s="2" t="s">
-        <v>258</v>
+        <v>246</v>
       </c>
       <c r="D119" s="2" t="s">
-        <v>420</v>
+        <v>416</v>
       </c>
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A120" s="2" t="s">
-        <v>259</v>
+        <v>247</v>
       </c>
       <c r="B120" s="2" t="s">
-        <v>260</v>
+        <v>247</v>
       </c>
       <c r="C120" s="2" t="s">
-        <v>261</v>
+        <v>248</v>
       </c>
       <c r="D120" s="2" t="s">
-        <v>421</v>
+        <v>417</v>
       </c>
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A121" s="2" t="s">
-        <v>262</v>
+        <v>249</v>
       </c>
       <c r="B121" s="2" t="s">
-        <v>263</v>
+        <v>249</v>
       </c>
       <c r="C121" s="2" t="s">
-        <v>264</v>
+        <v>250</v>
       </c>
       <c r="D121" s="2" t="s">
-        <v>422</v>
+        <v>418</v>
       </c>
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A122" s="2" t="s">
-        <v>265</v>
+        <v>253</v>
       </c>
       <c r="B122" s="2" t="s">
-        <v>265</v>
+        <v>254</v>
       </c>
       <c r="C122" s="2" t="s">
-        <v>265</v>
+        <v>255</v>
       </c>
       <c r="D122" s="2" t="s">
-        <v>423</v>
+        <v>419</v>
       </c>
     </row>
     <row r="123" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A123" s="2" t="s">
-        <v>266</v>
+        <v>256</v>
       </c>
       <c r="B123" s="2" t="s">
-        <v>266</v>
+        <v>257</v>
       </c>
       <c r="C123" s="2" t="s">
-        <v>267</v>
+        <v>258</v>
       </c>
       <c r="D123" s="2" t="s">
-        <v>424</v>
+        <v>420</v>
       </c>
     </row>
     <row r="124" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A124" s="2" t="s">
-        <v>268</v>
+        <v>259</v>
       </c>
       <c r="B124" s="2" t="s">
-        <v>268</v>
+        <v>260</v>
       </c>
       <c r="C124" s="2" t="s">
-        <v>269</v>
+        <v>261</v>
       </c>
       <c r="D124" s="2" t="s">
-        <v>425</v>
+        <v>421</v>
       </c>
     </row>
     <row r="125" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A125" s="2" t="s">
-        <v>270</v>
+        <v>262</v>
       </c>
       <c r="B125" s="2" t="s">
-        <v>270</v>
+        <v>263</v>
       </c>
       <c r="C125" s="2" t="s">
-        <v>273</v>
+        <v>264</v>
       </c>
       <c r="D125" s="2" t="s">
-        <v>426</v>
+        <v>422</v>
       </c>
     </row>
     <row r="126" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A126" s="2" t="s">
-        <v>271</v>
+        <v>265</v>
       </c>
       <c r="B126" s="2" t="s">
-        <v>271</v>
+        <v>265</v>
       </c>
       <c r="C126" s="2" t="s">
-        <v>272</v>
+        <v>265</v>
       </c>
       <c r="D126" s="2" t="s">
-        <v>427</v>
-      </c>
-    </row>
-    <row r="127" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="127" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A127" s="2" t="s">
-        <v>274</v>
+        <v>266</v>
       </c>
       <c r="B127" s="2" t="s">
-        <v>276</v>
+        <v>266</v>
       </c>
       <c r="C127" s="2" t="s">
-        <v>279</v>
-      </c>
-    </row>
-    <row r="128" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+        <v>267</v>
+      </c>
+      <c r="D127" s="2" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="128" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A128" s="2" t="s">
-        <v>275</v>
+        <v>268</v>
       </c>
       <c r="B128" s="2" t="s">
-        <v>277</v>
+        <v>268</v>
       </c>
       <c r="C128" s="2" t="s">
-        <v>278</v>
-      </c>
-    </row>
-    <row r="129" spans="1:4" ht="75" x14ac:dyDescent="0.25">
+        <v>269</v>
+      </c>
+      <c r="D128" s="2" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="129" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A129" s="2" t="s">
-        <v>289</v>
+        <v>270</v>
       </c>
       <c r="B129" s="2" t="s">
-        <v>290</v>
+        <v>270</v>
       </c>
       <c r="C129" s="2" t="s">
-        <v>291</v>
+        <v>273</v>
+      </c>
+      <c r="D129" s="2" t="s">
+        <v>426</v>
       </c>
     </row>
     <row r="130" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A130" s="2" t="s">
-        <v>306</v>
+        <v>271</v>
       </c>
       <c r="B130" s="2" t="s">
-        <v>307</v>
+        <v>271</v>
       </c>
       <c r="C130" s="2" t="s">
-        <v>308</v>
+        <v>272</v>
       </c>
       <c r="D130" s="2" t="s">
-        <v>428</v>
-      </c>
-    </row>
-    <row r="131" spans="1:4" x14ac:dyDescent="0.25">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="131" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A131" s="2" t="s">
-        <v>309</v>
+        <v>274</v>
       </c>
       <c r="B131" s="2" t="s">
-        <v>311</v>
+        <v>276</v>
       </c>
       <c r="C131" s="2" t="s">
-        <v>312</v>
-      </c>
-      <c r="D131" s="2" t="s">
-        <v>429</v>
-      </c>
-    </row>
-    <row r="132" spans="1:4" x14ac:dyDescent="0.25">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="132" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A132" s="2" t="s">
-        <v>310</v>
+        <v>275</v>
       </c>
       <c r="B132" s="2" t="s">
-        <v>314</v>
+        <v>277</v>
       </c>
       <c r="C132" s="2" t="s">
-        <v>313</v>
-      </c>
-      <c r="D132" s="2" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="133" spans="1:4" x14ac:dyDescent="0.25">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="133" spans="1:4" ht="75" x14ac:dyDescent="0.25">
       <c r="A133" s="2" t="s">
-        <v>315</v>
+        <v>289</v>
       </c>
       <c r="B133" s="2" t="s">
-        <v>315</v>
+        <v>290</v>
       </c>
       <c r="C133" s="2" t="s">
-        <v>316</v>
-      </c>
-      <c r="D133" s="2" t="s">
-        <v>431</v>
+        <v>291</v>
       </c>
     </row>
     <row r="134" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A134" s="2" t="s">
-        <v>317</v>
+        <v>306</v>
       </c>
       <c r="B134" s="2" t="s">
-        <v>318</v>
+        <v>307</v>
       </c>
       <c r="C134" s="2" t="s">
-        <v>460</v>
+        <v>308</v>
       </c>
       <c r="D134" s="2" t="s">
-        <v>432</v>
+        <v>428</v>
       </c>
     </row>
     <row r="135" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A135" s="2" t="s">
-        <v>319</v>
+        <v>309</v>
       </c>
       <c r="B135" s="2" t="s">
-        <v>320</v>
+        <v>311</v>
       </c>
       <c r="C135" s="2" t="s">
-        <v>461</v>
+        <v>312</v>
       </c>
       <c r="D135" s="2" t="s">
-        <v>433</v>
+        <v>429</v>
       </c>
     </row>
     <row r="136" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A136" s="2" t="s">
-        <v>448</v>
+        <v>310</v>
       </c>
       <c r="B136" s="2" t="s">
-        <v>448</v>
+        <v>314</v>
       </c>
       <c r="C136" s="2" t="s">
-        <v>462</v>
+        <v>313</v>
       </c>
       <c r="D136" s="2" t="s">
-        <v>345</v>
+        <v>430</v>
       </c>
     </row>
     <row r="137" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A137" s="2" t="s">
-        <v>449</v>
+        <v>315</v>
       </c>
       <c r="B137" s="2" t="s">
-        <v>450</v>
+        <v>315</v>
       </c>
       <c r="C137" s="2" t="s">
-        <v>463</v>
+        <v>316</v>
       </c>
       <c r="D137" s="2" t="s">
-        <v>451</v>
+        <v>431</v>
       </c>
     </row>
     <row r="138" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A138" s="2" t="s">
-        <v>476</v>
+        <v>317</v>
       </c>
       <c r="B138" s="2" t="s">
-        <v>477</v>
+        <v>318</v>
       </c>
       <c r="C138" s="2" t="s">
-        <v>478</v>
+        <v>460</v>
+      </c>
+      <c r="D138" s="2" t="s">
+        <v>432</v>
       </c>
     </row>
     <row r="139" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A139" s="2" t="s">
-        <v>479</v>
+        <v>319</v>
       </c>
       <c r="B139" s="2" t="s">
-        <v>525</v>
+        <v>320</v>
       </c>
       <c r="C139" s="2" t="s">
-        <v>480</v>
+        <v>461</v>
+      </c>
+      <c r="D139" s="2" t="s">
+        <v>433</v>
       </c>
     </row>
     <row r="140" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A140" s="2" t="s">
-        <v>481</v>
+        <v>448</v>
       </c>
       <c r="B140" s="2" t="s">
-        <v>482</v>
+        <v>448</v>
       </c>
       <c r="C140" s="2" t="s">
-        <v>483</v>
+        <v>462</v>
+      </c>
+      <c r="D140" s="2" t="s">
+        <v>345</v>
       </c>
     </row>
     <row r="141" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A141" s="2" t="s">
-        <v>484</v>
+        <v>449</v>
       </c>
       <c r="B141" s="2" t="s">
-        <v>485</v>
+        <v>450</v>
       </c>
       <c r="C141" s="2" t="s">
-        <v>486</v>
+        <v>463</v>
+      </c>
+      <c r="D141" s="2" t="s">
+        <v>451</v>
       </c>
     </row>
     <row r="142" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A142" s="2" t="s">
-        <v>487</v>
+        <v>476</v>
       </c>
       <c r="B142" s="2" t="s">
-        <v>488</v>
+        <v>477</v>
       </c>
       <c r="C142" s="2" t="s">
-        <v>489</v>
+        <v>478</v>
       </c>
     </row>
     <row r="143" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A143" s="2" t="s">
-        <v>490</v>
+        <v>479</v>
       </c>
       <c r="B143" s="2" t="s">
-        <v>491</v>
+        <v>525</v>
       </c>
       <c r="C143" s="2" t="s">
-        <v>492</v>
+        <v>480</v>
       </c>
     </row>
     <row r="144" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A144" s="2" t="s">
+        <v>481</v>
+      </c>
+      <c r="B144" s="2" t="s">
+        <v>482</v>
+      </c>
+      <c r="C144" s="2" t="s">
+        <v>483</v>
+      </c>
+    </row>
+    <row r="145" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A145" s="2" t="s">
+        <v>484</v>
+      </c>
+      <c r="B145" s="2" t="s">
+        <v>485</v>
+      </c>
+      <c r="C145" s="2" t="s">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="146" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A146" s="2" t="s">
+        <v>487</v>
+      </c>
+      <c r="B146" s="2" t="s">
+        <v>488</v>
+      </c>
+      <c r="C146" s="2" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="147" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A147" s="2" t="s">
+        <v>490</v>
+      </c>
+      <c r="B147" s="2" t="s">
+        <v>491</v>
+      </c>
+      <c r="C147" s="2" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="148" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A148" s="2" t="s">
+        <v>538</v>
+      </c>
+      <c r="B148" s="2" t="s">
+        <v>539</v>
+      </c>
+    </row>
+    <row r="149" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A149" s="2" t="s">
+        <v>541</v>
+      </c>
+      <c r="B149" s="2" t="s">
+        <v>541</v>
+      </c>
+      <c r="D149" s="2" t="s">
+        <v>542</v>
+      </c>
+    </row>
+    <row r="150" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A150" s="2" t="s">
+        <v>543</v>
+      </c>
+      <c r="B150" s="2" t="s">
+        <v>544</v>
+      </c>
+      <c r="D150" s="2" t="s">
+        <v>545</v>
+      </c>
+    </row>
+    <row r="151" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A151" s="2" t="s">
         <v>493</v>
       </c>
-      <c r="B144" s="2" t="s">
+      <c r="B151" s="2" t="s">
         <v>494</v>
       </c>
-      <c r="C144" s="2" t="s">
+      <c r="C151" s="2" t="s">
         <v>495</v>
       </c>
     </row>
-    <row r="145" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A145" s="2" t="s">
+    <row r="152" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A152" s="2" t="s">
         <v>496</v>
       </c>
-      <c r="B145" s="2" t="s">
+      <c r="B152" s="2" t="s">
         <v>497</v>
       </c>
-      <c r="C145" s="2" t="s">
+      <c r="C152" s="2" t="s">
         <v>498</v>
       </c>
     </row>
-    <row r="146" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A146" s="2" t="s">
+    <row r="153" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A153" s="2" t="s">
         <v>499</v>
       </c>
-      <c r="B146" s="2" t="s">
+      <c r="B153" s="2" t="s">
         <v>500</v>
       </c>
-      <c r="C146" s="2" t="s">
+      <c r="C153" s="2" t="s">
         <v>501</v>
       </c>
     </row>
-    <row r="147" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A147" s="2" t="s">
+    <row r="154" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A154" s="2" t="s">
         <v>502</v>
       </c>
-      <c r="B147" s="2" t="s">
+      <c r="B154" s="2" t="s">
         <v>502</v>
       </c>
-      <c r="C147" s="2" t="s">
+      <c r="C154" s="2" t="s">
         <v>503</v>
       </c>
     </row>
-    <row r="148" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A148" s="2" t="s">
+    <row r="155" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A155" s="2" t="s">
         <v>504</v>
       </c>
-      <c r="B148" s="2" t="s">
+      <c r="B155" s="2" t="s">
         <v>504</v>
       </c>
-      <c r="C148" s="2" t="s">
+      <c r="C155" s="2" t="s">
         <v>505</v>
       </c>
     </row>
-    <row r="149" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A149" s="2" t="s">
+    <row r="156" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A156" s="2" t="s">
         <v>506</v>
       </c>
-      <c r="B149" s="2" t="s">
+      <c r="B156" s="2" t="s">
         <v>506</v>
       </c>
-      <c r="C149" s="2" t="s">
+      <c r="C156" s="2" t="s">
         <v>507</v>
       </c>
     </row>
-    <row r="150" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A150" s="2" t="s">
+    <row r="157" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A157" s="2" t="s">
         <v>508</v>
       </c>
-      <c r="B150" s="2" t="s">
+      <c r="B157" s="2" t="s">
         <v>508</v>
       </c>
-      <c r="C150" s="2" t="s">
+      <c r="C157" s="2" t="s">
         <v>509</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Mine(crap) and upgrades fixes.
</commit_message>
<xml_diff>
--- a/Translations/Translations.xlsx
+++ b/Translations/Translations.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Codes\c#\FrSLE\Translations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B620771-43AB-47DC-B1FF-39E53DA3078C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F2C483A-E7FA-49AD-8E45-BFDA3107184B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15900" xr2:uid="{F5C22481-FF1A-482C-BF7E-EB5A7718AF49}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15900" xr2:uid="{F5C22481-FF1A-482C-BF7E-EB5A7718AF49}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="592" uniqueCount="546">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="595" uniqueCount="549">
   <si>
     <t>ID</t>
   </si>
@@ -1672,6 +1672,15 @@
   </si>
   <si>
     <t>Ігнорувати, якщо піднято</t>
+  </si>
+  <si>
+    <t>object.MINE</t>
+  </si>
+  <si>
+    <t>Mine</t>
+  </si>
+  <si>
+    <t>Міна</t>
   </si>
 </sst>
 </file>
@@ -2071,7 +2080,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6961A5F-F8EA-4989-8112-A0ACE51D011E}">
   <sheetPr codeName="Hoja1"/>
-  <dimension ref="A1:D157"/>
+  <dimension ref="A1:D158"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="37" style="2" customWidth="1"/>
@@ -2813,1359 +2822,1370 @@
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A55" s="2" t="s">
-        <v>69</v>
+        <v>546</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="C55" s="2" t="s">
-        <v>101</v>
+        <v>547</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>364</v>
+        <v>548</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
-        <v>105</v>
+        <v>69</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>2</v>
+        <v>69</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>111</v>
+        <v>4</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61" s="2" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" s="2" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" s="2" t="s">
-        <v>445</v>
+        <v>118</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>446</v>
+        <v>122</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>459</v>
+        <v>121</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>447</v>
+        <v>370</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A65" s="2" t="s">
-        <v>513</v>
+        <v>445</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>514</v>
+        <v>446</v>
+      </c>
+      <c r="C65" s="2" t="s">
+        <v>459</v>
       </c>
       <c r="D65" s="2" t="s">
-        <v>515</v>
+        <v>447</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66" s="2" t="s">
-        <v>519</v>
+        <v>513</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>520</v>
+        <v>514</v>
       </c>
       <c r="D66" s="2" t="s">
-        <v>521</v>
+        <v>515</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A67" s="2" t="s">
-        <v>522</v>
+        <v>519</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>523</v>
+        <v>520</v>
       </c>
       <c r="D67" s="2" t="s">
-        <v>524</v>
+        <v>521</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A68" s="2" t="s">
-        <v>533</v>
+        <v>522</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>534</v>
+        <v>523</v>
       </c>
       <c r="D68" s="2" t="s">
-        <v>535</v>
+        <v>524</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A69" s="2" t="s">
-        <v>540</v>
+        <v>533</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>536</v>
+        <v>534</v>
       </c>
       <c r="D69" s="2" t="s">
-        <v>537</v>
+        <v>535</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A70" s="2" t="s">
-        <v>154</v>
+        <v>540</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="C70" s="2" t="s">
-        <v>156</v>
+        <v>536</v>
       </c>
       <c r="D70" s="2" t="s">
-        <v>371</v>
+        <v>537</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A71" s="2" t="s">
-        <v>164</v>
+        <v>154</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>165</v>
+        <v>155</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>166</v>
+        <v>156</v>
       </c>
       <c r="D71" s="2" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A72" s="2" t="s">
-        <v>157</v>
+        <v>164</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>158</v>
+        <v>165</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>159</v>
+        <v>166</v>
       </c>
       <c r="D72" s="2" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A73" s="2" t="s">
-        <v>167</v>
+        <v>157</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>168</v>
+        <v>158</v>
       </c>
       <c r="C73" s="2" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="D73" s="2" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A74" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="B74" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="C74" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="D74" s="2" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A75" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="B74" s="2" t="s">
+      <c r="B75" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="C74" s="2" t="s">
+      <c r="C75" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="D74" s="2" t="s">
+      <c r="D75" s="2" t="s">
         <v>375</v>
       </c>
     </row>
-    <row r="75" spans="1:4" ht="45" x14ac:dyDescent="0.25">
-      <c r="A75" s="2" t="s">
+    <row r="76" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="A76" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="B75" s="2" t="s">
+      <c r="B76" s="2" t="s">
         <v>163</v>
       </c>
-      <c r="C75" s="2" t="s">
+      <c r="C76" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="D75" s="2" t="s">
+      <c r="D76" s="2" t="s">
         <v>376</v>
-      </c>
-    </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A76" s="2" t="s">
-        <v>153</v>
-      </c>
-      <c r="B76" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="C76" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="D76" s="2" t="s">
-        <v>328</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A77" s="2" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="B77" s="2" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="C77" s="2" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="D77" s="2" t="s">
-        <v>377</v>
+        <v>328</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A78" s="2" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="B78" s="2" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="C78" s="2" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="D78" s="2" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A79" s="2" t="s">
-        <v>172</v>
+        <v>150</v>
       </c>
       <c r="B79" s="2" t="s">
-        <v>170</v>
+        <v>151</v>
       </c>
       <c r="C79" s="2" t="s">
-        <v>171</v>
+        <v>152</v>
       </c>
       <c r="D79" s="2" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B80" s="2" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="C80" s="2" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="D80" s="2" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A81" s="2" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="B81" s="2" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="C81" s="2" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="D81" s="2" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A82" s="2" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="B82" s="2" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="C82" s="2" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="D82" s="2" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A83" s="2" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="B83" s="2" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="C83" s="2" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="D83" s="2" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A84" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="B84" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="C84" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="D84" s="2" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A85" s="2" t="s">
         <v>243</v>
       </c>
-      <c r="B84" s="2" t="s">
+      <c r="B85" s="2" t="s">
         <v>243</v>
       </c>
-      <c r="C84" s="2" t="s">
+      <c r="C85" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="D84" s="2" t="s">
+      <c r="D85" s="2" t="s">
         <v>384</v>
       </c>
     </row>
-    <row r="85" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A85" s="2" t="s">
+    <row r="86" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A86" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="B85" s="1" t="s">
+      <c r="B86" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="C85" s="2" t="s">
+      <c r="C86" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="D85" s="2" t="s">
+      <c r="D86" s="2" t="s">
         <v>385</v>
-      </c>
-    </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A86" s="2" t="s">
-        <v>182</v>
-      </c>
-      <c r="B86" s="2" t="s">
-        <v>183</v>
-      </c>
-      <c r="C86" s="2" t="s">
-        <v>183</v>
-      </c>
-      <c r="D86" s="2" t="s">
-        <v>386</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A87" s="2" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="B87" s="2" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C87" s="2" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="D87" s="2" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A88" s="2" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="B88" s="2" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="C88" s="2" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="D88" s="2" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A89" s="2" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="B89" s="2" t="s">
-        <v>526</v>
+        <v>186</v>
       </c>
       <c r="C89" s="2" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="D89" s="2" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A90" s="2" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="B90" s="2" t="s">
-        <v>190</v>
+        <v>526</v>
       </c>
       <c r="C90" s="2" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="D90" s="2" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A91" s="2" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="B91" s="2" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="C91" s="2" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="D91" s="2" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A92" s="2" t="s">
-        <v>434</v>
-      </c>
-      <c r="B92" s="4" t="s">
-        <v>435</v>
-      </c>
-      <c r="C92" s="4" t="s">
-        <v>436</v>
+        <v>192</v>
+      </c>
+      <c r="B92" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="C92" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="D92" s="2" t="s">
+        <v>391</v>
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A93" s="2" t="s">
-        <v>437</v>
+        <v>434</v>
       </c>
       <c r="B93" s="4" t="s">
-        <v>438</v>
+        <v>435</v>
       </c>
       <c r="C93" s="4" t="s">
-        <v>439</v>
+        <v>436</v>
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A94" s="2" t="s">
-        <v>473</v>
+        <v>437</v>
       </c>
       <c r="B94" s="4" t="s">
-        <v>474</v>
+        <v>438</v>
       </c>
       <c r="C94" s="4" t="s">
-        <v>475</v>
+        <v>439</v>
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A95" s="2" t="s">
-        <v>195</v>
-      </c>
-      <c r="B95" s="2" t="s">
-        <v>196</v>
-      </c>
-      <c r="C95" s="2" t="s">
-        <v>197</v>
-      </c>
-      <c r="D95" s="2" t="s">
-        <v>392</v>
+        <v>473</v>
+      </c>
+      <c r="B95" s="4" t="s">
+        <v>474</v>
+      </c>
+      <c r="C95" s="4" t="s">
+        <v>475</v>
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A96" s="2" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="B96" s="2" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="C96" s="2" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="D96" s="2" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A97" s="2" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="B97" s="2" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="C97" s="2" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="D97" s="2" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A98" s="2" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="B98" s="2" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="C98" s="2" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="D98" s="2" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A99" s="2" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="B99" s="2" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="C99" s="2" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="D99" s="2" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A100" s="2" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B100" s="2" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="C100" s="2" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="D100" s="2" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A101" s="2" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="B101" s="2" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="C101" s="2" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="D101" s="2" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A102" s="2" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="B102" s="2" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="C102" s="2" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="D102" s="2" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A103" s="2" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="B103" s="2" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="C103" s="2" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="D103" s="2" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A104" s="2" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="B104" s="2" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="C104" s="2" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="D104" s="2" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A105" s="2" t="s">
-        <v>292</v>
+        <v>220</v>
       </c>
       <c r="B105" s="2" t="s">
-        <v>292</v>
+        <v>219</v>
       </c>
       <c r="C105" s="2" t="s">
-        <v>293</v>
+        <v>218</v>
       </c>
       <c r="D105" s="2" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A106" s="2" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="B106" s="2" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="C106" s="2" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
       <c r="D106" s="2" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A107" s="2" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
       <c r="B107" s="2" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="C107" s="2" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="D107" s="2" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A108" s="2" t="s">
-        <v>221</v>
+        <v>297</v>
       </c>
       <c r="B108" s="2" t="s">
-        <v>221</v>
+        <v>298</v>
       </c>
       <c r="C108" s="2" t="s">
-        <v>222</v>
+        <v>299</v>
       </c>
       <c r="D108" s="2" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A109" s="2" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="B109" s="2" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="C109" s="2" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="D109" s="2" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A110" s="2" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="B110" s="2" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="C110" s="2" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="D110" s="2" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A111" s="2" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="B111" s="2" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="C111" s="2" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="D111" s="2" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A112" s="2" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B112" s="2" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="C112" s="2" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="D112" s="2" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A113" s="2" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="B113" s="2" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="C113" s="2" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="D113" s="2" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A114" s="2" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="B114" s="2" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="C114" s="2" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="D114" s="2" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A115" s="2" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="B115" s="2" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="C115" s="2" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="D115" s="2" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A116" s="2" t="s">
-        <v>300</v>
+        <v>237</v>
       </c>
       <c r="B116" s="2" t="s">
-        <v>301</v>
+        <v>238</v>
       </c>
       <c r="C116" s="2" t="s">
-        <v>302</v>
+        <v>239</v>
       </c>
       <c r="D116" s="2" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A117" s="2" t="s">
-        <v>240</v>
+        <v>300</v>
       </c>
       <c r="B117" s="2" t="s">
-        <v>241</v>
+        <v>301</v>
       </c>
       <c r="C117" s="2" t="s">
-        <v>242</v>
+        <v>302</v>
       </c>
       <c r="D117" s="2" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A118" s="2" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="B118" s="2" t="s">
-        <v>252</v>
+        <v>241</v>
       </c>
       <c r="C118" s="2" t="s">
-        <v>251</v>
+        <v>242</v>
       </c>
       <c r="D118" s="2" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="119" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A119" s="2" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B119" s="2" t="s">
-        <v>245</v>
+        <v>252</v>
       </c>
       <c r="C119" s="2" t="s">
-        <v>246</v>
+        <v>251</v>
       </c>
       <c r="D119" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A120" s="2" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="B120" s="2" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="C120" s="2" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="D120" s="2" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A121" s="2" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="B121" s="2" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="C121" s="2" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="D121" s="2" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A122" s="2" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="B122" s="2" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="C122" s="2" t="s">
-        <v>255</v>
+        <v>250</v>
       </c>
       <c r="D122" s="2" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
     </row>
     <row r="123" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A123" s="2" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="B123" s="2" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="C123" s="2" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="D123" s="2" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
     </row>
     <row r="124" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A124" s="2" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="B124" s="2" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="C124" s="2" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="D124" s="2" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
     </row>
     <row r="125" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A125" s="2" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="B125" s="2" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="C125" s="2" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="D125" s="2" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="126" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A126" s="2" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="B126" s="2" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="C126" s="2" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="D126" s="2" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
     </row>
     <row r="127" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A127" s="2" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="B127" s="2" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="C127" s="2" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="D127" s="2" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
     </row>
     <row r="128" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A128" s="2" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="B128" s="2" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="C128" s="2" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="D128" s="2" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
     </row>
     <row r="129" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A129" s="2" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="B129" s="2" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="C129" s="2" t="s">
-        <v>273</v>
+        <v>269</v>
       </c>
       <c r="D129" s="2" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
     </row>
     <row r="130" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A130" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="B130" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="C130" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="D130" s="2" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="131" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A131" s="2" t="s">
         <v>271</v>
       </c>
-      <c r="B130" s="2" t="s">
+      <c r="B131" s="2" t="s">
         <v>271</v>
       </c>
-      <c r="C130" s="2" t="s">
+      <c r="C131" s="2" t="s">
         <v>272</v>
       </c>
-      <c r="D130" s="2" t="s">
+      <c r="D131" s="2" t="s">
         <v>427</v>
       </c>
     </row>
-    <row r="131" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A131" s="2" t="s">
+    <row r="132" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A132" s="2" t="s">
         <v>274</v>
       </c>
-      <c r="B131" s="2" t="s">
+      <c r="B132" s="2" t="s">
         <v>276</v>
       </c>
-      <c r="C131" s="2" t="s">
+      <c r="C132" s="2" t="s">
         <v>279</v>
       </c>
     </row>
-    <row r="132" spans="1:4" ht="45" x14ac:dyDescent="0.25">
-      <c r="A132" s="2" t="s">
+    <row r="133" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="A133" s="2" t="s">
         <v>275</v>
       </c>
-      <c r="B132" s="2" t="s">
+      <c r="B133" s="2" t="s">
         <v>277</v>
       </c>
-      <c r="C132" s="2" t="s">
+      <c r="C133" s="2" t="s">
         <v>278</v>
       </c>
     </row>
-    <row r="133" spans="1:4" ht="75" x14ac:dyDescent="0.25">
-      <c r="A133" s="2" t="s">
+    <row r="134" spans="1:4" ht="75" x14ac:dyDescent="0.25">
+      <c r="A134" s="2" t="s">
         <v>289</v>
       </c>
-      <c r="B133" s="2" t="s">
+      <c r="B134" s="2" t="s">
         <v>290</v>
       </c>
-      <c r="C133" s="2" t="s">
+      <c r="C134" s="2" t="s">
         <v>291</v>
-      </c>
-    </row>
-    <row r="134" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A134" s="2" t="s">
-        <v>306</v>
-      </c>
-      <c r="B134" s="2" t="s">
-        <v>307</v>
-      </c>
-      <c r="C134" s="2" t="s">
-        <v>308</v>
-      </c>
-      <c r="D134" s="2" t="s">
-        <v>428</v>
       </c>
     </row>
     <row r="135" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A135" s="2" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
       <c r="B135" s="2" t="s">
-        <v>311</v>
+        <v>307</v>
       </c>
       <c r="C135" s="2" t="s">
-        <v>312</v>
+        <v>308</v>
       </c>
       <c r="D135" s="2" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
     </row>
     <row r="136" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A136" s="2" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="B136" s="2" t="s">
-        <v>314</v>
+        <v>311</v>
       </c>
       <c r="C136" s="2" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="D136" s="2" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
     </row>
     <row r="137" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A137" s="2" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="B137" s="2" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="C137" s="2" t="s">
-        <v>316</v>
+        <v>313</v>
       </c>
       <c r="D137" s="2" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
     </row>
     <row r="138" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A138" s="2" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="B138" s="2" t="s">
-        <v>318</v>
+        <v>315</v>
       </c>
       <c r="C138" s="2" t="s">
-        <v>460</v>
+        <v>316</v>
       </c>
       <c r="D138" s="2" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
     </row>
     <row r="139" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A139" s="2" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="B139" s="2" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="C139" s="2" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="D139" s="2" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
     </row>
     <row r="140" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A140" s="2" t="s">
-        <v>448</v>
+        <v>319</v>
       </c>
       <c r="B140" s="2" t="s">
-        <v>448</v>
+        <v>320</v>
       </c>
       <c r="C140" s="2" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="D140" s="2" t="s">
-        <v>345</v>
+        <v>433</v>
       </c>
     </row>
     <row r="141" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A141" s="2" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="B141" s="2" t="s">
-        <v>450</v>
+        <v>448</v>
       </c>
       <c r="C141" s="2" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="D141" s="2" t="s">
-        <v>451</v>
+        <v>345</v>
       </c>
     </row>
     <row r="142" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A142" s="2" t="s">
-        <v>476</v>
+        <v>449</v>
       </c>
       <c r="B142" s="2" t="s">
-        <v>477</v>
+        <v>450</v>
       </c>
       <c r="C142" s="2" t="s">
-        <v>478</v>
+        <v>463</v>
+      </c>
+      <c r="D142" s="2" t="s">
+        <v>451</v>
       </c>
     </row>
     <row r="143" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A143" s="2" t="s">
-        <v>479</v>
+        <v>476</v>
       </c>
       <c r="B143" s="2" t="s">
-        <v>525</v>
+        <v>477</v>
       </c>
       <c r="C143" s="2" t="s">
-        <v>480</v>
+        <v>478</v>
       </c>
     </row>
     <row r="144" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A144" s="2" t="s">
-        <v>481</v>
+        <v>479</v>
       </c>
       <c r="B144" s="2" t="s">
-        <v>482</v>
+        <v>525</v>
       </c>
       <c r="C144" s="2" t="s">
-        <v>483</v>
+        <v>480</v>
       </c>
     </row>
     <row r="145" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A145" s="2" t="s">
-        <v>484</v>
+        <v>481</v>
       </c>
       <c r="B145" s="2" t="s">
-        <v>485</v>
+        <v>482</v>
       </c>
       <c r="C145" s="2" t="s">
-        <v>486</v>
+        <v>483</v>
       </c>
     </row>
     <row r="146" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A146" s="2" t="s">
-        <v>487</v>
+        <v>484</v>
       </c>
       <c r="B146" s="2" t="s">
-        <v>488</v>
+        <v>485</v>
       </c>
       <c r="C146" s="2" t="s">
-        <v>489</v>
+        <v>486</v>
       </c>
     </row>
     <row r="147" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A147" s="2" t="s">
-        <v>490</v>
+        <v>487</v>
       </c>
       <c r="B147" s="2" t="s">
-        <v>491</v>
+        <v>488</v>
       </c>
       <c r="C147" s="2" t="s">
-        <v>492</v>
+        <v>489</v>
       </c>
     </row>
     <row r="148" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A148" s="2" t="s">
-        <v>538</v>
+        <v>490</v>
       </c>
       <c r="B148" s="2" t="s">
-        <v>539</v>
+        <v>491</v>
+      </c>
+      <c r="C148" s="2" t="s">
+        <v>492</v>
       </c>
     </row>
     <row r="149" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A149" s="2" t="s">
-        <v>541</v>
+        <v>538</v>
       </c>
       <c r="B149" s="2" t="s">
-        <v>541</v>
-      </c>
-      <c r="D149" s="2" t="s">
-        <v>542</v>
+        <v>539</v>
       </c>
     </row>
     <row r="150" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A150" s="2" t="s">
-        <v>543</v>
+        <v>541</v>
       </c>
       <c r="B150" s="2" t="s">
-        <v>544</v>
+        <v>541</v>
       </c>
       <c r="D150" s="2" t="s">
-        <v>545</v>
+        <v>542</v>
       </c>
     </row>
     <row r="151" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A151" s="2" t="s">
-        <v>493</v>
+        <v>543</v>
       </c>
       <c r="B151" s="2" t="s">
-        <v>494</v>
-      </c>
-      <c r="C151" s="2" t="s">
-        <v>495</v>
+        <v>544</v>
+      </c>
+      <c r="D151" s="2" t="s">
+        <v>545</v>
       </c>
     </row>
     <row r="152" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A152" s="2" t="s">
-        <v>496</v>
+        <v>493</v>
       </c>
       <c r="B152" s="2" t="s">
-        <v>497</v>
+        <v>494</v>
       </c>
       <c r="C152" s="2" t="s">
-        <v>498</v>
+        <v>495</v>
       </c>
     </row>
     <row r="153" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A153" s="2" t="s">
-        <v>499</v>
+        <v>496</v>
       </c>
       <c r="B153" s="2" t="s">
-        <v>500</v>
+        <v>497</v>
       </c>
       <c r="C153" s="2" t="s">
-        <v>501</v>
+        <v>498</v>
       </c>
     </row>
     <row r="154" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A154" s="2" t="s">
-        <v>502</v>
+        <v>499</v>
       </c>
       <c r="B154" s="2" t="s">
-        <v>502</v>
+        <v>500</v>
       </c>
       <c r="C154" s="2" t="s">
-        <v>503</v>
+        <v>501</v>
       </c>
     </row>
     <row r="155" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A155" s="2" t="s">
-        <v>504</v>
+        <v>502</v>
       </c>
       <c r="B155" s="2" t="s">
-        <v>504</v>
+        <v>502</v>
       </c>
       <c r="C155" s="2" t="s">
-        <v>505</v>
+        <v>503</v>
       </c>
     </row>
     <row r="156" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A156" s="2" t="s">
-        <v>506</v>
+        <v>504</v>
       </c>
       <c r="B156" s="2" t="s">
-        <v>506</v>
+        <v>504</v>
       </c>
       <c r="C156" s="2" t="s">
-        <v>507</v>
+        <v>505</v>
       </c>
     </row>
     <row r="157" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A157" s="2" t="s">
+        <v>506</v>
+      </c>
+      <c r="B157" s="2" t="s">
+        <v>506</v>
+      </c>
+      <c r="C157" s="2" t="s">
+        <v>507</v>
+      </c>
+    </row>
+    <row r="158" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A158" s="2" t="s">
         <v>508</v>
       </c>
-      <c r="B157" s="2" t="s">
+      <c r="B158" s="2" t="s">
         <v>508</v>
       </c>
-      <c r="C157" s="2" t="s">
+      <c r="C158" s="2" t="s">
         <v>509</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Notification system, jetpack events, RGB wall, fixes to slowdown bug
</commit_message>
<xml_diff>
--- a/Translations/Translations.xlsx
+++ b/Translations/Translations.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Codes\c#\FrSLE\Translations\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Codes\c#\gLE\Translations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F2C483A-E7FA-49AD-8E45-BFDA3107184B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5DEFF9D4-91D6-4E8E-A03F-126553FB2C07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15900" xr2:uid="{F5C22481-FF1A-482C-BF7E-EB5A7718AF49}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{F5C22481-FF1A-482C-BF7E-EB5A7718AF49}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="595" uniqueCount="549">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="598" uniqueCount="549">
   <si>
     <t>ID</t>
   </si>
@@ -1767,7 +1767,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Звичайний" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1783,9 +1783,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Тема &quot;Office 2013 – 2022&quot;">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013–2022">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1823,7 +1823,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013–2022">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1929,7 +1929,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013–2022">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -2080,7 +2080,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6961A5F-F8EA-4989-8112-A0ACE51D011E}">
   <sheetPr codeName="Hoja1"/>
-  <dimension ref="A1:D158"/>
+  <dimension ref="A1:D159"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="37" style="2" customWidth="1"/>
@@ -2847,1345 +2847,1356 @@
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57" s="2" t="s">
-        <v>105</v>
+        <v>456</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="C57" s="2" t="s">
-        <v>102</v>
+        <v>456</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>365</v>
+        <v>457</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>111</v>
+        <v>4</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61" s="2" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" s="2" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63" s="2" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A65" s="2" t="s">
-        <v>445</v>
+        <v>118</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>446</v>
+        <v>122</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>459</v>
+        <v>121</v>
       </c>
       <c r="D65" s="2" t="s">
-        <v>447</v>
+        <v>370</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66" s="2" t="s">
-        <v>513</v>
+        <v>445</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>514</v>
+        <v>446</v>
+      </c>
+      <c r="C66" s="2" t="s">
+        <v>459</v>
       </c>
       <c r="D66" s="2" t="s">
-        <v>515</v>
+        <v>447</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A67" s="2" t="s">
-        <v>519</v>
+        <v>513</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>520</v>
+        <v>514</v>
       </c>
       <c r="D67" s="2" t="s">
-        <v>521</v>
+        <v>515</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A68" s="2" t="s">
-        <v>522</v>
+        <v>519</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>523</v>
+        <v>520</v>
       </c>
       <c r="D68" s="2" t="s">
-        <v>524</v>
+        <v>521</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A69" s="2" t="s">
-        <v>533</v>
+        <v>522</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>534</v>
+        <v>523</v>
       </c>
       <c r="D69" s="2" t="s">
-        <v>535</v>
+        <v>524</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A70" s="2" t="s">
-        <v>540</v>
+        <v>533</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>536</v>
+        <v>534</v>
       </c>
       <c r="D70" s="2" t="s">
-        <v>537</v>
+        <v>535</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A71" s="2" t="s">
-        <v>154</v>
+        <v>540</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="C71" s="2" t="s">
-        <v>156</v>
+        <v>536</v>
       </c>
       <c r="D71" s="2" t="s">
-        <v>371</v>
+        <v>537</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A72" s="2" t="s">
-        <v>164</v>
+        <v>154</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>165</v>
+        <v>155</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>166</v>
+        <v>156</v>
       </c>
       <c r="D72" s="2" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A73" s="2" t="s">
-        <v>157</v>
+        <v>164</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>158</v>
+        <v>165</v>
       </c>
       <c r="C73" s="2" t="s">
-        <v>159</v>
+        <v>166</v>
       </c>
       <c r="D73" s="2" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A74" s="2" t="s">
-        <v>167</v>
+        <v>157</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>168</v>
+        <v>158</v>
       </c>
       <c r="C74" s="2" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="D74" s="2" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A75" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="B75" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="C75" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="D75" s="2" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A76" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="B75" s="2" t="s">
+      <c r="B76" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="C75" s="2" t="s">
+      <c r="C76" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="D75" s="2" t="s">
+      <c r="D76" s="2" t="s">
         <v>375</v>
       </c>
     </row>
-    <row r="76" spans="1:4" ht="45" x14ac:dyDescent="0.25">
-      <c r="A76" s="2" t="s">
+    <row r="77" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="A77" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="B76" s="2" t="s">
+      <c r="B77" s="2" t="s">
         <v>163</v>
       </c>
-      <c r="C76" s="2" t="s">
+      <c r="C77" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="D76" s="2" t="s">
+      <c r="D77" s="2" t="s">
         <v>376</v>
-      </c>
-    </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A77" s="2" t="s">
-        <v>153</v>
-      </c>
-      <c r="B77" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="C77" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="D77" s="2" t="s">
-        <v>328</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A78" s="2" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="B78" s="2" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="C78" s="2" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="D78" s="2" t="s">
-        <v>377</v>
+        <v>328</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A79" s="2" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="B79" s="2" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="C79" s="2" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="D79" s="2" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
-        <v>172</v>
+        <v>150</v>
       </c>
       <c r="B80" s="2" t="s">
-        <v>170</v>
+        <v>151</v>
       </c>
       <c r="C80" s="2" t="s">
-        <v>171</v>
+        <v>152</v>
       </c>
       <c r="D80" s="2" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A81" s="2" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B81" s="2" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="C81" s="2" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="D81" s="2" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A82" s="2" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="B82" s="2" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="C82" s="2" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="D82" s="2" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A83" s="2" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="B83" s="2" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="C83" s="2" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="D83" s="2" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A84" s="2" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="B84" s="2" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="C84" s="2" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="D84" s="2" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A85" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="B85" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="C85" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="D85" s="2" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A86" s="2" t="s">
         <v>243</v>
       </c>
-      <c r="B85" s="2" t="s">
+      <c r="B86" s="2" t="s">
         <v>243</v>
       </c>
-      <c r="C85" s="2" t="s">
+      <c r="C86" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="D85" s="2" t="s">
+      <c r="D86" s="2" t="s">
         <v>384</v>
       </c>
     </row>
-    <row r="86" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A86" s="2" t="s">
+    <row r="87" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A87" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="B86" s="1" t="s">
+      <c r="B87" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="C86" s="2" t="s">
+      <c r="C87" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="D86" s="2" t="s">
+      <c r="D87" s="2" t="s">
         <v>385</v>
-      </c>
-    </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A87" s="2" t="s">
-        <v>182</v>
-      </c>
-      <c r="B87" s="2" t="s">
-        <v>183</v>
-      </c>
-      <c r="C87" s="2" t="s">
-        <v>183</v>
-      </c>
-      <c r="D87" s="2" t="s">
-        <v>386</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A88" s="2" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="B88" s="2" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C88" s="2" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="D88" s="2" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A89" s="2" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="B89" s="2" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="C89" s="2" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="D89" s="2" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A90" s="2" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="B90" s="2" t="s">
-        <v>526</v>
+        <v>186</v>
       </c>
       <c r="C90" s="2" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="D90" s="2" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A91" s="2" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="B91" s="2" t="s">
-        <v>190</v>
+        <v>526</v>
       </c>
       <c r="C91" s="2" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="D91" s="2" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A92" s="2" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="B92" s="2" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="C92" s="2" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="D92" s="2" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A93" s="2" t="s">
-        <v>434</v>
-      </c>
-      <c r="B93" s="4" t="s">
-        <v>435</v>
-      </c>
-      <c r="C93" s="4" t="s">
-        <v>436</v>
+        <v>192</v>
+      </c>
+      <c r="B93" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="C93" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="D93" s="2" t="s">
+        <v>391</v>
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A94" s="2" t="s">
-        <v>437</v>
+        <v>434</v>
       </c>
       <c r="B94" s="4" t="s">
-        <v>438</v>
+        <v>435</v>
       </c>
       <c r="C94" s="4" t="s">
-        <v>439</v>
+        <v>436</v>
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A95" s="2" t="s">
-        <v>473</v>
+        <v>437</v>
       </c>
       <c r="B95" s="4" t="s">
-        <v>474</v>
+        <v>438</v>
       </c>
       <c r="C95" s="4" t="s">
-        <v>475</v>
+        <v>439</v>
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A96" s="2" t="s">
-        <v>195</v>
-      </c>
-      <c r="B96" s="2" t="s">
-        <v>196</v>
-      </c>
-      <c r="C96" s="2" t="s">
-        <v>197</v>
-      </c>
-      <c r="D96" s="2" t="s">
-        <v>392</v>
+        <v>473</v>
+      </c>
+      <c r="B96" s="4" t="s">
+        <v>474</v>
+      </c>
+      <c r="C96" s="4" t="s">
+        <v>475</v>
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A97" s="2" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="B97" s="2" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="C97" s="2" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="D97" s="2" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A98" s="2" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="B98" s="2" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="C98" s="2" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="D98" s="2" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A99" s="2" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="B99" s="2" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="C99" s="2" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="D99" s="2" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A100" s="2" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="B100" s="2" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="C100" s="2" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="D100" s="2" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A101" s="2" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B101" s="2" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="C101" s="2" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="D101" s="2" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A102" s="2" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="B102" s="2" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="C102" s="2" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="D102" s="2" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A103" s="2" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="B103" s="2" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="C103" s="2" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="D103" s="2" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A104" s="2" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="B104" s="2" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="C104" s="2" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="D104" s="2" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A105" s="2" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="B105" s="2" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="C105" s="2" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="D105" s="2" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A106" s="2" t="s">
-        <v>292</v>
+        <v>220</v>
       </c>
       <c r="B106" s="2" t="s">
-        <v>292</v>
+        <v>219</v>
       </c>
       <c r="C106" s="2" t="s">
-        <v>293</v>
+        <v>218</v>
       </c>
       <c r="D106" s="2" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A107" s="2" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="B107" s="2" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="C107" s="2" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
       <c r="D107" s="2" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A108" s="2" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
       <c r="B108" s="2" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="C108" s="2" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="D108" s="2" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A109" s="2" t="s">
-        <v>221</v>
+        <v>297</v>
       </c>
       <c r="B109" s="2" t="s">
-        <v>221</v>
+        <v>298</v>
       </c>
       <c r="C109" s="2" t="s">
-        <v>222</v>
+        <v>299</v>
       </c>
       <c r="D109" s="2" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A110" s="2" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="B110" s="2" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="C110" s="2" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="D110" s="2" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A111" s="2" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="B111" s="2" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="C111" s="2" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="D111" s="2" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A112" s="2" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="B112" s="2" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="C112" s="2" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="D112" s="2" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A113" s="2" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B113" s="2" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="C113" s="2" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="D113" s="2" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A114" s="2" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="B114" s="2" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="C114" s="2" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="D114" s="2" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A115" s="2" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="B115" s="2" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="C115" s="2" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="D115" s="2" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A116" s="2" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="B116" s="2" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="C116" s="2" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="D116" s="2" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A117" s="2" t="s">
-        <v>300</v>
+        <v>237</v>
       </c>
       <c r="B117" s="2" t="s">
-        <v>301</v>
+        <v>238</v>
       </c>
       <c r="C117" s="2" t="s">
-        <v>302</v>
+        <v>239</v>
       </c>
       <c r="D117" s="2" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A118" s="2" t="s">
-        <v>240</v>
+        <v>300</v>
       </c>
       <c r="B118" s="2" t="s">
-        <v>241</v>
+        <v>301</v>
       </c>
       <c r="C118" s="2" t="s">
-        <v>242</v>
+        <v>302</v>
       </c>
       <c r="D118" s="2" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
     </row>
     <row r="119" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A119" s="2" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="B119" s="2" t="s">
-        <v>252</v>
+        <v>241</v>
       </c>
       <c r="C119" s="2" t="s">
-        <v>251</v>
+        <v>242</v>
       </c>
       <c r="D119" s="2" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A120" s="2" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B120" s="2" t="s">
-        <v>245</v>
+        <v>252</v>
       </c>
       <c r="C120" s="2" t="s">
-        <v>246</v>
+        <v>251</v>
       </c>
       <c r="D120" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A121" s="2" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="B121" s="2" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="C121" s="2" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="D121" s="2" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A122" s="2" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="B122" s="2" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="C122" s="2" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="D122" s="2" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
     </row>
     <row r="123" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A123" s="2" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="B123" s="2" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="C123" s="2" t="s">
-        <v>255</v>
+        <v>250</v>
       </c>
       <c r="D123" s="2" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
     </row>
     <row r="124" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A124" s="2" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="B124" s="2" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="C124" s="2" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="D124" s="2" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
     </row>
     <row r="125" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A125" s="2" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="B125" s="2" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="C125" s="2" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="D125" s="2" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
     </row>
     <row r="126" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A126" s="2" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="B126" s="2" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="C126" s="2" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="D126" s="2" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="127" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A127" s="2" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="B127" s="2" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="C127" s="2" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="D127" s="2" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
     </row>
     <row r="128" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A128" s="2" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="B128" s="2" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="C128" s="2" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="D128" s="2" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
     </row>
     <row r="129" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A129" s="2" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="B129" s="2" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="C129" s="2" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="D129" s="2" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
     </row>
     <row r="130" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A130" s="2" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="B130" s="2" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="C130" s="2" t="s">
-        <v>273</v>
+        <v>269</v>
       </c>
       <c r="D130" s="2" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
     </row>
     <row r="131" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A131" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="B131" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="C131" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="D131" s="2" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="132" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A132" s="2" t="s">
         <v>271</v>
       </c>
-      <c r="B131" s="2" t="s">
+      <c r="B132" s="2" t="s">
         <v>271</v>
       </c>
-      <c r="C131" s="2" t="s">
+      <c r="C132" s="2" t="s">
         <v>272</v>
       </c>
-      <c r="D131" s="2" t="s">
+      <c r="D132" s="2" t="s">
         <v>427</v>
       </c>
     </row>
-    <row r="132" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A132" s="2" t="s">
+    <row r="133" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A133" s="2" t="s">
         <v>274</v>
       </c>
-      <c r="B132" s="2" t="s">
+      <c r="B133" s="2" t="s">
         <v>276</v>
       </c>
-      <c r="C132" s="2" t="s">
+      <c r="C133" s="2" t="s">
         <v>279</v>
       </c>
     </row>
-    <row r="133" spans="1:4" ht="45" x14ac:dyDescent="0.25">
-      <c r="A133" s="2" t="s">
+    <row r="134" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="A134" s="2" t="s">
         <v>275</v>
       </c>
-      <c r="B133" s="2" t="s">
+      <c r="B134" s="2" t="s">
         <v>277</v>
       </c>
-      <c r="C133" s="2" t="s">
+      <c r="C134" s="2" t="s">
         <v>278</v>
       </c>
     </row>
-    <row r="134" spans="1:4" ht="75" x14ac:dyDescent="0.25">
-      <c r="A134" s="2" t="s">
+    <row r="135" spans="1:4" ht="75" x14ac:dyDescent="0.25">
+      <c r="A135" s="2" t="s">
         <v>289</v>
       </c>
-      <c r="B134" s="2" t="s">
+      <c r="B135" s="2" t="s">
         <v>290</v>
       </c>
-      <c r="C134" s="2" t="s">
+      <c r="C135" s="2" t="s">
         <v>291</v>
-      </c>
-    </row>
-    <row r="135" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A135" s="2" t="s">
-        <v>306</v>
-      </c>
-      <c r="B135" s="2" t="s">
-        <v>307</v>
-      </c>
-      <c r="C135" s="2" t="s">
-        <v>308</v>
-      </c>
-      <c r="D135" s="2" t="s">
-        <v>428</v>
       </c>
     </row>
     <row r="136" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A136" s="2" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
       <c r="B136" s="2" t="s">
-        <v>311</v>
+        <v>307</v>
       </c>
       <c r="C136" s="2" t="s">
-        <v>312</v>
+        <v>308</v>
       </c>
       <c r="D136" s="2" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
     </row>
     <row r="137" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A137" s="2" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="B137" s="2" t="s">
-        <v>314</v>
+        <v>311</v>
       </c>
       <c r="C137" s="2" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="D137" s="2" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
     </row>
     <row r="138" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A138" s="2" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="B138" s="2" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="C138" s="2" t="s">
-        <v>316</v>
+        <v>313</v>
       </c>
       <c r="D138" s="2" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
     </row>
     <row r="139" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A139" s="2" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="B139" s="2" t="s">
-        <v>318</v>
+        <v>315</v>
       </c>
       <c r="C139" s="2" t="s">
-        <v>460</v>
+        <v>316</v>
       </c>
       <c r="D139" s="2" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
     </row>
     <row r="140" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A140" s="2" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="B140" s="2" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="C140" s="2" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="D140" s="2" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
     </row>
     <row r="141" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A141" s="2" t="s">
-        <v>448</v>
+        <v>319</v>
       </c>
       <c r="B141" s="2" t="s">
-        <v>448</v>
+        <v>320</v>
       </c>
       <c r="C141" s="2" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="D141" s="2" t="s">
-        <v>345</v>
+        <v>433</v>
       </c>
     </row>
     <row r="142" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A142" s="2" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="B142" s="2" t="s">
-        <v>450</v>
+        <v>448</v>
       </c>
       <c r="C142" s="2" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="D142" s="2" t="s">
-        <v>451</v>
+        <v>345</v>
       </c>
     </row>
     <row r="143" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A143" s="2" t="s">
-        <v>476</v>
+        <v>449</v>
       </c>
       <c r="B143" s="2" t="s">
-        <v>477</v>
+        <v>450</v>
       </c>
       <c r="C143" s="2" t="s">
-        <v>478</v>
+        <v>463</v>
+      </c>
+      <c r="D143" s="2" t="s">
+        <v>451</v>
       </c>
     </row>
     <row r="144" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A144" s="2" t="s">
-        <v>479</v>
+        <v>476</v>
       </c>
       <c r="B144" s="2" t="s">
-        <v>525</v>
+        <v>477</v>
       </c>
       <c r="C144" s="2" t="s">
-        <v>480</v>
+        <v>478</v>
       </c>
     </row>
     <row r="145" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A145" s="2" t="s">
-        <v>481</v>
+        <v>479</v>
       </c>
       <c r="B145" s="2" t="s">
-        <v>482</v>
+        <v>525</v>
       </c>
       <c r="C145" s="2" t="s">
-        <v>483</v>
+        <v>480</v>
       </c>
     </row>
     <row r="146" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A146" s="2" t="s">
-        <v>484</v>
+        <v>481</v>
       </c>
       <c r="B146" s="2" t="s">
-        <v>485</v>
+        <v>482</v>
       </c>
       <c r="C146" s="2" t="s">
-        <v>486</v>
+        <v>483</v>
       </c>
     </row>
     <row r="147" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A147" s="2" t="s">
-        <v>487</v>
+        <v>484</v>
       </c>
       <c r="B147" s="2" t="s">
-        <v>488</v>
+        <v>485</v>
       </c>
       <c r="C147" s="2" t="s">
-        <v>489</v>
+        <v>486</v>
       </c>
     </row>
     <row r="148" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A148" s="2" t="s">
-        <v>490</v>
+        <v>487</v>
       </c>
       <c r="B148" s="2" t="s">
-        <v>491</v>
+        <v>488</v>
       </c>
       <c r="C148" s="2" t="s">
-        <v>492</v>
+        <v>489</v>
       </c>
     </row>
     <row r="149" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A149" s="2" t="s">
-        <v>538</v>
+        <v>490</v>
       </c>
       <c r="B149" s="2" t="s">
-        <v>539</v>
+        <v>491</v>
+      </c>
+      <c r="C149" s="2" t="s">
+        <v>492</v>
       </c>
     </row>
     <row r="150" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A150" s="2" t="s">
-        <v>541</v>
+        <v>538</v>
       </c>
       <c r="B150" s="2" t="s">
-        <v>541</v>
-      </c>
-      <c r="D150" s="2" t="s">
-        <v>542</v>
+        <v>539</v>
       </c>
     </row>
     <row r="151" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A151" s="2" t="s">
-        <v>543</v>
+        <v>541</v>
       </c>
       <c r="B151" s="2" t="s">
-        <v>544</v>
+        <v>541</v>
       </c>
       <c r="D151" s="2" t="s">
-        <v>545</v>
+        <v>542</v>
       </c>
     </row>
     <row r="152" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A152" s="2" t="s">
-        <v>493</v>
+        <v>543</v>
       </c>
       <c r="B152" s="2" t="s">
-        <v>494</v>
-      </c>
-      <c r="C152" s="2" t="s">
-        <v>495</v>
+        <v>544</v>
+      </c>
+      <c r="D152" s="2" t="s">
+        <v>545</v>
       </c>
     </row>
     <row r="153" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A153" s="2" t="s">
-        <v>496</v>
+        <v>493</v>
       </c>
       <c r="B153" s="2" t="s">
-        <v>497</v>
+        <v>494</v>
       </c>
       <c r="C153" s="2" t="s">
-        <v>498</v>
+        <v>495</v>
       </c>
     </row>
     <row r="154" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A154" s="2" t="s">
-        <v>499</v>
+        <v>496</v>
       </c>
       <c r="B154" s="2" t="s">
-        <v>500</v>
+        <v>497</v>
       </c>
       <c r="C154" s="2" t="s">
-        <v>501</v>
+        <v>498</v>
       </c>
     </row>
     <row r="155" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A155" s="2" t="s">
-        <v>502</v>
+        <v>499</v>
       </c>
       <c r="B155" s="2" t="s">
-        <v>502</v>
+        <v>500</v>
       </c>
       <c r="C155" s="2" t="s">
-        <v>503</v>
+        <v>501</v>
       </c>
     </row>
     <row r="156" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A156" s="2" t="s">
-        <v>504</v>
+        <v>502</v>
       </c>
       <c r="B156" s="2" t="s">
-        <v>504</v>
+        <v>502</v>
       </c>
       <c r="C156" s="2" t="s">
-        <v>505</v>
+        <v>503</v>
       </c>
     </row>
     <row r="157" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A157" s="2" t="s">
-        <v>506</v>
+        <v>504</v>
       </c>
       <c r="B157" s="2" t="s">
-        <v>506</v>
+        <v>504</v>
       </c>
       <c r="C157" s="2" t="s">
-        <v>507</v>
+        <v>505</v>
       </c>
     </row>
     <row r="158" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A158" s="2" t="s">
+        <v>506</v>
+      </c>
+      <c r="B158" s="2" t="s">
+        <v>506</v>
+      </c>
+      <c r="C158" s="2" t="s">
+        <v>507</v>
+      </c>
+    </row>
+    <row r="159" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A159" s="2" t="s">
         <v>508</v>
       </c>
-      <c r="B158" s="2" t="s">
+      <c r="B159" s="2" t="s">
         <v>508</v>
       </c>
-      <c r="C158" s="2" t="s">
+      <c r="C159" s="2" t="s">
         <v>509</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Tons of fixes and new stuff
</commit_message>
<xml_diff>
--- a/Translations/Translations.xlsx
+++ b/Translations/Translations.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Codes\c#\gLE\Translations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5DEFF9D4-91D6-4E8E-A03F-126553FB2C07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7E3333C-AF25-4DF7-9286-0CEC035B97DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{F5C22481-FF1A-482C-BF7E-EB5A7718AF49}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="598" uniqueCount="549">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="625" uniqueCount="574">
   <si>
     <t>ID</t>
   </si>
@@ -1650,12 +1650,6 @@
     <t>При неправильній комбінації</t>
   </si>
   <si>
-    <t>leaveOnIncorrect</t>
-  </si>
-  <si>
-    <t>Leave on Incorrect</t>
-  </si>
-  <si>
     <t>events.onFailEvents</t>
   </si>
   <si>
@@ -1681,6 +1675,87 @@
   </si>
   <si>
     <t>Міна</t>
+  </si>
+  <si>
+    <t>object.HEAL_AREA</t>
+  </si>
+  <si>
+    <t>Heal Area</t>
+  </si>
+  <si>
+    <t>Лікувальна зона</t>
+  </si>
+  <si>
+    <t>object.RGB_WALL</t>
+  </si>
+  <si>
+    <t>Color Wall</t>
+  </si>
+  <si>
+    <t>Кольорова стіна</t>
+  </si>
+  <si>
+    <t>Джетпак</t>
+  </si>
+  <si>
+    <t>Точка переміщення</t>
+  </si>
+  <si>
+    <t>Рухома платформа</t>
+  </si>
+  <si>
+    <t>Точка переміщення рухомої платформа</t>
+  </si>
+  <si>
+    <t>Ворона</t>
+  </si>
+  <si>
+    <t>+ Додати глобальну точку руху</t>
+  </si>
+  <si>
+    <t>+ Додати точку руху пили</t>
+  </si>
+  <si>
+    <t>+ Додати точку руху платформи</t>
+  </si>
+  <si>
+    <t>РОЗБЛОКОВАНІ</t>
+  </si>
+  <si>
+    <t>ЗАБЛОКОВАНІ</t>
+  </si>
+  <si>
+    <t>ВІДКРИТІ</t>
+  </si>
+  <si>
+    <t>ЗАКРИТІ</t>
+  </si>
+  <si>
+    <t>Автоматичні?</t>
+  </si>
+  <si>
+    <t>ЗАЦИКЛЕНО</t>
+  </si>
+  <si>
+    <t>ПОВЕРНУТИСЯ</t>
+  </si>
+  <si>
+    <t>НІЧОГО</t>
+  </si>
+  <si>
+    <t>Тип руху</t>
+  </si>
+  <si>
+    <t>Затримка початку</t>
+  </si>
+  <si>
+    <t>Швидкість руху</t>
+  </si>
+  <si>
+    <t>Почати рух при старті</t>
+  </si>
+  <si>
+    <t>Невидимі бортики</t>
   </si>
 </sst>
 </file>
@@ -2080,7 +2155,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6961A5F-F8EA-4989-8112-A0ACE51D011E}">
   <sheetPr codeName="Hoja1"/>
-  <dimension ref="A1:D159"/>
+  <dimension ref="A1:D161"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="37" style="2" customWidth="1"/>
@@ -2700,6 +2775,9 @@
       <c r="C44" s="2" t="s">
         <v>441</v>
       </c>
+      <c r="D44" s="2" t="s">
+        <v>554</v>
+      </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
@@ -2753,6 +2831,9 @@
       <c r="C48" s="2" t="s">
         <v>466</v>
       </c>
+      <c r="D48" s="2" t="s">
+        <v>555</v>
+      </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
@@ -2764,6 +2845,9 @@
       <c r="C49" s="2" t="s">
         <v>469</v>
       </c>
+      <c r="D49" s="2" t="s">
+        <v>556</v>
+      </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
@@ -2775,6 +2859,9 @@
       <c r="C50" s="2" t="s">
         <v>472</v>
       </c>
+      <c r="D50" s="2" t="s">
+        <v>557</v>
+      </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
@@ -2822,91 +2909,82 @@
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A55" s="2" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
-        <v>69</v>
+        <v>550</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="C56" s="2" t="s">
-        <v>101</v>
+        <v>551</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>364</v>
+        <v>552</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57" s="2" t="s">
-        <v>456</v>
+        <v>544</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>456</v>
+        <v>545</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>457</v>
+        <v>546</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" s="2" t="s">
-        <v>105</v>
+        <v>69</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>2</v>
+        <v>69</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" s="2" t="s">
-        <v>106</v>
+        <v>443</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C59" s="2" t="s">
-        <v>103</v>
+        <v>443</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>366</v>
+        <v>553</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
-        <v>107</v>
+        <v>456</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C60" s="2" t="s">
-        <v>104</v>
+        <v>456</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>367</v>
+        <v>457</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61" s="2" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>111</v>
+        <v>2</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>109</v>
+        <v>102</v>
       </c>
       <c r="D61" s="2" t="s">
         <v>365</v>
@@ -2914,13 +2992,13 @@
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" s="2" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>112</v>
+        <v>3</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>113</v>
+        <v>103</v>
       </c>
       <c r="D62" s="2" t="s">
         <v>366</v>
@@ -2928,1276 +3006,1358 @@
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63" s="2" t="s">
-        <v>114</v>
+        <v>107</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>115</v>
+        <v>4</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>116</v>
+        <v>104</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" s="2" t="s">
-        <v>117</v>
+        <v>108</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>369</v>
+        <v>365</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A65" s="2" t="s">
-        <v>118</v>
+        <v>110</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>122</v>
+        <v>112</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>121</v>
+        <v>113</v>
       </c>
       <c r="D65" s="2" t="s">
-        <v>370</v>
+        <v>366</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66" s="2" t="s">
-        <v>445</v>
+        <v>114</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>446</v>
+        <v>115</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>459</v>
+        <v>116</v>
       </c>
       <c r="D66" s="2" t="s">
-        <v>447</v>
+        <v>368</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A67" s="2" t="s">
-        <v>513</v>
+        <v>117</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>514</v>
+        <v>119</v>
+      </c>
+      <c r="C67" s="2" t="s">
+        <v>120</v>
       </c>
       <c r="D67" s="2" t="s">
-        <v>515</v>
+        <v>369</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A68" s="2" t="s">
-        <v>519</v>
+        <v>118</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>520</v>
+        <v>122</v>
+      </c>
+      <c r="C68" s="2" t="s">
+        <v>121</v>
       </c>
       <c r="D68" s="2" t="s">
-        <v>521</v>
+        <v>370</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A69" s="2" t="s">
-        <v>522</v>
+        <v>445</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>523</v>
+        <v>446</v>
+      </c>
+      <c r="C69" s="2" t="s">
+        <v>459</v>
       </c>
       <c r="D69" s="2" t="s">
-        <v>524</v>
+        <v>447</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A70" s="2" t="s">
-        <v>533</v>
+        <v>513</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>534</v>
+        <v>514</v>
       </c>
       <c r="D70" s="2" t="s">
-        <v>535</v>
+        <v>515</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A71" s="2" t="s">
-        <v>540</v>
+        <v>519</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>536</v>
+        <v>520</v>
       </c>
       <c r="D71" s="2" t="s">
-        <v>537</v>
+        <v>521</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A72" s="2" t="s">
-        <v>154</v>
+        <v>522</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="C72" s="2" t="s">
-        <v>156</v>
+        <v>523</v>
       </c>
       <c r="D72" s="2" t="s">
-        <v>371</v>
+        <v>524</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A73" s="2" t="s">
-        <v>164</v>
+        <v>533</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>165</v>
-      </c>
-      <c r="C73" s="2" t="s">
-        <v>166</v>
+        <v>534</v>
       </c>
       <c r="D73" s="2" t="s">
-        <v>372</v>
+        <v>535</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A74" s="2" t="s">
-        <v>157</v>
+        <v>538</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>158</v>
-      </c>
-      <c r="C74" s="2" t="s">
-        <v>159</v>
+        <v>536</v>
       </c>
       <c r="D74" s="2" t="s">
-        <v>373</v>
+        <v>537</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A75" s="2" t="s">
-        <v>167</v>
+        <v>154</v>
       </c>
       <c r="B75" s="2" t="s">
-        <v>168</v>
+        <v>155</v>
       </c>
       <c r="C75" s="2" t="s">
-        <v>169</v>
+        <v>156</v>
       </c>
       <c r="D75" s="2" t="s">
-        <v>374</v>
+        <v>371</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A76" s="2" t="s">
-        <v>141</v>
+        <v>164</v>
       </c>
       <c r="B76" s="2" t="s">
-        <v>142</v>
+        <v>165</v>
       </c>
       <c r="C76" s="2" t="s">
-        <v>143</v>
+        <v>166</v>
       </c>
       <c r="D76" s="2" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="77" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A77" s="2" t="s">
-        <v>144</v>
+        <v>157</v>
       </c>
       <c r="B77" s="2" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="C77" s="2" t="s">
-        <v>145</v>
+        <v>159</v>
       </c>
       <c r="D77" s="2" t="s">
-        <v>376</v>
+        <v>373</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A78" s="2" t="s">
-        <v>153</v>
+        <v>167</v>
       </c>
       <c r="B78" s="2" t="s">
-        <v>146</v>
+        <v>168</v>
       </c>
       <c r="C78" s="2" t="s">
-        <v>146</v>
+        <v>169</v>
       </c>
       <c r="D78" s="2" t="s">
-        <v>328</v>
+        <v>374</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A79" s="2" t="s">
-        <v>147</v>
+        <v>141</v>
       </c>
       <c r="B79" s="2" t="s">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="C79" s="2" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
       <c r="D79" s="2" t="s">
-        <v>377</v>
-      </c>
-    </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="B80" s="2" t="s">
-        <v>151</v>
+        <v>163</v>
       </c>
       <c r="C80" s="2" t="s">
-        <v>152</v>
+        <v>145</v>
       </c>
       <c r="D80" s="2" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A81" s="2" t="s">
-        <v>172</v>
+        <v>153</v>
       </c>
       <c r="B81" s="2" t="s">
-        <v>170</v>
+        <v>146</v>
       </c>
       <c r="C81" s="2" t="s">
-        <v>171</v>
+        <v>146</v>
       </c>
       <c r="D81" s="2" t="s">
-        <v>379</v>
+        <v>328</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A82" s="2" t="s">
-        <v>173</v>
+        <v>147</v>
       </c>
       <c r="B82" s="2" t="s">
-        <v>174</v>
+        <v>148</v>
       </c>
       <c r="C82" s="2" t="s">
-        <v>175</v>
+        <v>149</v>
       </c>
       <c r="D82" s="2" t="s">
-        <v>380</v>
+        <v>377</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A83" s="2" t="s">
-        <v>176</v>
+        <v>150</v>
       </c>
       <c r="B83" s="2" t="s">
-        <v>176</v>
+        <v>151</v>
       </c>
       <c r="C83" s="2" t="s">
-        <v>177</v>
+        <v>152</v>
       </c>
       <c r="D83" s="2" t="s">
-        <v>381</v>
+        <v>378</v>
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A84" s="2" t="s">
-        <v>178</v>
+        <v>172</v>
       </c>
       <c r="B84" s="2" t="s">
-        <v>178</v>
+        <v>170</v>
       </c>
       <c r="C84" s="2" t="s">
-        <v>179</v>
+        <v>171</v>
       </c>
       <c r="D84" s="2" t="s">
-        <v>382</v>
+        <v>379</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A85" s="2" t="s">
-        <v>180</v>
+        <v>173</v>
       </c>
       <c r="B85" s="2" t="s">
-        <v>180</v>
+        <v>174</v>
       </c>
       <c r="C85" s="2" t="s">
-        <v>181</v>
+        <v>175</v>
       </c>
       <c r="D85" s="2" t="s">
-        <v>383</v>
+        <v>380</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A86" s="2" t="s">
-        <v>243</v>
+        <v>176</v>
       </c>
       <c r="B86" s="2" t="s">
-        <v>243</v>
+        <v>176</v>
       </c>
       <c r="C86" s="2" t="s">
-        <v>95</v>
+        <v>177</v>
       </c>
       <c r="D86" s="2" t="s">
-        <v>384</v>
-      </c>
-    </row>
-    <row r="87" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A87" s="2" t="s">
-        <v>138</v>
-      </c>
-      <c r="B87" s="1" t="s">
-        <v>140</v>
+        <v>178</v>
+      </c>
+      <c r="B87" s="2" t="s">
+        <v>178</v>
       </c>
       <c r="C87" s="2" t="s">
-        <v>139</v>
+        <v>179</v>
       </c>
       <c r="D87" s="2" t="s">
-        <v>385</v>
+        <v>382</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A88" s="2" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="B88" s="2" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="C88" s="2" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="D88" s="2" t="s">
-        <v>386</v>
+        <v>383</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A89" s="2" t="s">
-        <v>184</v>
+        <v>243</v>
       </c>
       <c r="B89" s="2" t="s">
-        <v>184</v>
+        <v>243</v>
       </c>
       <c r="C89" s="2" t="s">
-        <v>185</v>
+        <v>95</v>
       </c>
       <c r="D89" s="2" t="s">
-        <v>387</v>
-      </c>
-    </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="90" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A90" s="2" t="s">
-        <v>186</v>
-      </c>
-      <c r="B90" s="2" t="s">
-        <v>186</v>
+        <v>138</v>
+      </c>
+      <c r="B90" s="1" t="s">
+        <v>140</v>
       </c>
       <c r="C90" s="2" t="s">
-        <v>187</v>
+        <v>139</v>
       </c>
       <c r="D90" s="2" t="s">
-        <v>388</v>
+        <v>385</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A91" s="2" t="s">
-        <v>188</v>
+        <v>182</v>
       </c>
       <c r="B91" s="2" t="s">
-        <v>526</v>
+        <v>183</v>
       </c>
       <c r="C91" s="2" t="s">
-        <v>189</v>
+        <v>183</v>
       </c>
       <c r="D91" s="2" t="s">
-        <v>389</v>
+        <v>386</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A92" s="2" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="B92" s="2" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="C92" s="2" t="s">
-        <v>191</v>
+        <v>185</v>
       </c>
       <c r="D92" s="2" t="s">
-        <v>390</v>
+        <v>387</v>
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A93" s="2" t="s">
-        <v>192</v>
+        <v>186</v>
       </c>
       <c r="B93" s="2" t="s">
-        <v>193</v>
+        <v>186</v>
       </c>
       <c r="C93" s="2" t="s">
-        <v>194</v>
+        <v>187</v>
       </c>
       <c r="D93" s="2" t="s">
-        <v>391</v>
+        <v>388</v>
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A94" s="2" t="s">
-        <v>434</v>
-      </c>
-      <c r="B94" s="4" t="s">
-        <v>435</v>
-      </c>
-      <c r="C94" s="4" t="s">
-        <v>436</v>
+        <v>188</v>
+      </c>
+      <c r="B94" s="2" t="s">
+        <v>526</v>
+      </c>
+      <c r="C94" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="D94" s="2" t="s">
+        <v>389</v>
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A95" s="2" t="s">
-        <v>437</v>
-      </c>
-      <c r="B95" s="4" t="s">
-        <v>438</v>
-      </c>
-      <c r="C95" s="4" t="s">
-        <v>439</v>
+        <v>190</v>
+      </c>
+      <c r="B95" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="C95" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="D95" s="2" t="s">
+        <v>390</v>
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A96" s="2" t="s">
-        <v>473</v>
-      </c>
-      <c r="B96" s="4" t="s">
-        <v>474</v>
-      </c>
-      <c r="C96" s="4" t="s">
-        <v>475</v>
+        <v>192</v>
+      </c>
+      <c r="B96" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="C96" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="D96" s="2" t="s">
+        <v>391</v>
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A97" s="2" t="s">
-        <v>195</v>
-      </c>
-      <c r="B97" s="2" t="s">
-        <v>196</v>
-      </c>
-      <c r="C97" s="2" t="s">
-        <v>197</v>
-      </c>
-      <c r="D97" s="2" t="s">
-        <v>392</v>
+        <v>434</v>
+      </c>
+      <c r="B97" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="C97" s="4" t="s">
+        <v>436</v>
+      </c>
+      <c r="D97" s="4" t="s">
+        <v>558</v>
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A98" s="2" t="s">
-        <v>198</v>
-      </c>
-      <c r="B98" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="C98" s="2" t="s">
-        <v>200</v>
-      </c>
-      <c r="D98" s="2" t="s">
-        <v>393</v>
+        <v>437</v>
+      </c>
+      <c r="B98" s="4" t="s">
+        <v>438</v>
+      </c>
+      <c r="C98" s="4" t="s">
+        <v>439</v>
+      </c>
+      <c r="D98" s="4" t="s">
+        <v>559</v>
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A99" s="2" t="s">
-        <v>201</v>
-      </c>
-      <c r="B99" s="2" t="s">
-        <v>201</v>
-      </c>
-      <c r="C99" s="2" t="s">
-        <v>202</v>
-      </c>
-      <c r="D99" s="2" t="s">
-        <v>394</v>
+        <v>473</v>
+      </c>
+      <c r="B99" s="4" t="s">
+        <v>474</v>
+      </c>
+      <c r="C99" s="4" t="s">
+        <v>475</v>
+      </c>
+      <c r="D99" s="4" t="s">
+        <v>560</v>
       </c>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A100" s="2" t="s">
-        <v>203</v>
+        <v>195</v>
       </c>
       <c r="B100" s="2" t="s">
-        <v>203</v>
+        <v>196</v>
       </c>
       <c r="C100" s="2" t="s">
-        <v>204</v>
+        <v>197</v>
       </c>
       <c r="D100" s="2" t="s">
-        <v>395</v>
+        <v>392</v>
       </c>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A101" s="2" t="s">
-        <v>205</v>
+        <v>198</v>
       </c>
       <c r="B101" s="2" t="s">
-        <v>205</v>
+        <v>199</v>
       </c>
       <c r="C101" s="2" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
       <c r="D101" s="2" t="s">
-        <v>396</v>
+        <v>393</v>
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A102" s="2" t="s">
-        <v>206</v>
+        <v>201</v>
       </c>
       <c r="B102" s="2" t="s">
-        <v>207</v>
+        <v>201</v>
       </c>
       <c r="C102" s="2" t="s">
-        <v>208</v>
+        <v>202</v>
       </c>
       <c r="D102" s="2" t="s">
-        <v>397</v>
+        <v>394</v>
       </c>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A103" s="2" t="s">
-        <v>209</v>
+        <v>203</v>
       </c>
       <c r="B103" s="2" t="s">
-        <v>210</v>
+        <v>203</v>
       </c>
       <c r="C103" s="2" t="s">
-        <v>211</v>
+        <v>204</v>
       </c>
       <c r="D103" s="2" t="s">
-        <v>398</v>
+        <v>395</v>
       </c>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A104" s="2" t="s">
-        <v>212</v>
+        <v>205</v>
       </c>
       <c r="B104" s="2" t="s">
-        <v>213</v>
+        <v>205</v>
       </c>
       <c r="C104" s="2" t="s">
-        <v>214</v>
+        <v>205</v>
       </c>
       <c r="D104" s="2" t="s">
-        <v>399</v>
+        <v>396</v>
       </c>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A105" s="2" t="s">
-        <v>215</v>
+        <v>206</v>
       </c>
       <c r="B105" s="2" t="s">
-        <v>216</v>
+        <v>207</v>
       </c>
       <c r="C105" s="2" t="s">
-        <v>217</v>
+        <v>208</v>
       </c>
       <c r="D105" s="2" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A106" s="2" t="s">
-        <v>220</v>
+        <v>209</v>
       </c>
       <c r="B106" s="2" t="s">
-        <v>219</v>
+        <v>210</v>
       </c>
       <c r="C106" s="2" t="s">
-        <v>218</v>
+        <v>211</v>
       </c>
       <c r="D106" s="2" t="s">
-        <v>401</v>
+        <v>398</v>
       </c>
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A107" s="2" t="s">
-        <v>292</v>
+        <v>212</v>
       </c>
       <c r="B107" s="2" t="s">
-        <v>292</v>
+        <v>213</v>
       </c>
       <c r="C107" s="2" t="s">
-        <v>293</v>
+        <v>214</v>
       </c>
       <c r="D107" s="2" t="s">
-        <v>402</v>
+        <v>399</v>
       </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A108" s="2" t="s">
-        <v>294</v>
+        <v>215</v>
       </c>
       <c r="B108" s="2" t="s">
-        <v>295</v>
+        <v>216</v>
       </c>
       <c r="C108" s="2" t="s">
-        <v>296</v>
+        <v>217</v>
       </c>
       <c r="D108" s="2" t="s">
-        <v>403</v>
+        <v>400</v>
       </c>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A109" s="2" t="s">
-        <v>297</v>
+        <v>220</v>
       </c>
       <c r="B109" s="2" t="s">
-        <v>298</v>
+        <v>219</v>
       </c>
       <c r="C109" s="2" t="s">
-        <v>299</v>
+        <v>218</v>
       </c>
       <c r="D109" s="2" t="s">
-        <v>404</v>
+        <v>401</v>
       </c>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A110" s="2" t="s">
-        <v>221</v>
+        <v>292</v>
       </c>
       <c r="B110" s="2" t="s">
-        <v>221</v>
+        <v>292</v>
       </c>
       <c r="C110" s="2" t="s">
-        <v>222</v>
+        <v>293</v>
       </c>
       <c r="D110" s="2" t="s">
-        <v>405</v>
+        <v>402</v>
       </c>
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A111" s="2" t="s">
-        <v>223</v>
+        <v>294</v>
       </c>
       <c r="B111" s="2" t="s">
-        <v>224</v>
+        <v>295</v>
       </c>
       <c r="C111" s="2" t="s">
-        <v>225</v>
+        <v>296</v>
       </c>
       <c r="D111" s="2" t="s">
-        <v>406</v>
+        <v>403</v>
       </c>
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A112" s="2" t="s">
-        <v>226</v>
+        <v>297</v>
       </c>
       <c r="B112" s="2" t="s">
-        <v>227</v>
+        <v>298</v>
       </c>
       <c r="C112" s="2" t="s">
-        <v>228</v>
+        <v>299</v>
       </c>
       <c r="D112" s="2" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A113" s="2" t="s">
-        <v>229</v>
+        <v>221</v>
       </c>
       <c r="B113" s="2" t="s">
-        <v>229</v>
+        <v>221</v>
       </c>
       <c r="C113" s="2" t="s">
-        <v>229</v>
+        <v>222</v>
       </c>
       <c r="D113" s="2" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A114" s="2" t="s">
-        <v>230</v>
+        <v>223</v>
       </c>
       <c r="B114" s="2" t="s">
-        <v>230</v>
+        <v>224</v>
       </c>
       <c r="C114" s="2" t="s">
-        <v>231</v>
+        <v>225</v>
       </c>
       <c r="D114" s="2" t="s">
-        <v>409</v>
+        <v>406</v>
       </c>
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A115" s="2" t="s">
-        <v>232</v>
+        <v>226</v>
       </c>
       <c r="B115" s="2" t="s">
-        <v>232</v>
+        <v>227</v>
       </c>
       <c r="C115" s="2" t="s">
-        <v>233</v>
+        <v>228</v>
       </c>
       <c r="D115" s="2" t="s">
-        <v>410</v>
+        <v>407</v>
       </c>
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A116" s="2" t="s">
-        <v>234</v>
+        <v>229</v>
       </c>
       <c r="B116" s="2" t="s">
-        <v>235</v>
+        <v>229</v>
       </c>
       <c r="C116" s="2" t="s">
-        <v>236</v>
+        <v>229</v>
       </c>
       <c r="D116" s="2" t="s">
-        <v>411</v>
+        <v>408</v>
       </c>
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A117" s="2" t="s">
-        <v>237</v>
+        <v>230</v>
       </c>
       <c r="B117" s="2" t="s">
-        <v>238</v>
+        <v>230</v>
       </c>
       <c r="C117" s="2" t="s">
-        <v>239</v>
+        <v>231</v>
       </c>
       <c r="D117" s="2" t="s">
-        <v>412</v>
+        <v>409</v>
       </c>
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A118" s="2" t="s">
-        <v>300</v>
+        <v>232</v>
       </c>
       <c r="B118" s="2" t="s">
-        <v>301</v>
+        <v>232</v>
       </c>
       <c r="C118" s="2" t="s">
-        <v>302</v>
+        <v>233</v>
       </c>
       <c r="D118" s="2" t="s">
-        <v>413</v>
+        <v>410</v>
       </c>
     </row>
     <row r="119" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A119" s="2" t="s">
-        <v>240</v>
+        <v>234</v>
       </c>
       <c r="B119" s="2" t="s">
-        <v>241</v>
+        <v>235</v>
       </c>
       <c r="C119" s="2" t="s">
-        <v>242</v>
+        <v>236</v>
       </c>
       <c r="D119" s="2" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A120" s="2" t="s">
-        <v>244</v>
+        <v>237</v>
       </c>
       <c r="B120" s="2" t="s">
-        <v>252</v>
+        <v>238</v>
       </c>
       <c r="C120" s="2" t="s">
-        <v>251</v>
+        <v>239</v>
       </c>
       <c r="D120" s="2" t="s">
-        <v>415</v>
+        <v>412</v>
       </c>
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A121" s="2" t="s">
-        <v>245</v>
+        <v>300</v>
       </c>
       <c r="B121" s="2" t="s">
-        <v>245</v>
+        <v>301</v>
       </c>
       <c r="C121" s="2" t="s">
-        <v>246</v>
+        <v>302</v>
       </c>
       <c r="D121" s="2" t="s">
-        <v>416</v>
+        <v>413</v>
       </c>
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A122" s="2" t="s">
-        <v>247</v>
+        <v>240</v>
       </c>
       <c r="B122" s="2" t="s">
-        <v>247</v>
+        <v>241</v>
       </c>
       <c r="C122" s="2" t="s">
-        <v>248</v>
+        <v>242</v>
       </c>
       <c r="D122" s="2" t="s">
-        <v>417</v>
+        <v>414</v>
       </c>
     </row>
     <row r="123" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A123" s="2" t="s">
-        <v>249</v>
+        <v>244</v>
       </c>
       <c r="B123" s="2" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="C123" s="2" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="D123" s="2" t="s">
-        <v>418</v>
+        <v>415</v>
       </c>
     </row>
     <row r="124" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A124" s="2" t="s">
-        <v>253</v>
+        <v>245</v>
       </c>
       <c r="B124" s="2" t="s">
-        <v>254</v>
+        <v>245</v>
       </c>
       <c r="C124" s="2" t="s">
-        <v>255</v>
+        <v>246</v>
       </c>
       <c r="D124" s="2" t="s">
-        <v>419</v>
+        <v>416</v>
       </c>
     </row>
     <row r="125" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A125" s="2" t="s">
-        <v>256</v>
+        <v>247</v>
       </c>
       <c r="B125" s="2" t="s">
-        <v>257</v>
+        <v>247</v>
       </c>
       <c r="C125" s="2" t="s">
-        <v>258</v>
+        <v>248</v>
       </c>
       <c r="D125" s="2" t="s">
-        <v>420</v>
+        <v>417</v>
       </c>
     </row>
     <row r="126" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A126" s="2" t="s">
-        <v>259</v>
+        <v>249</v>
       </c>
       <c r="B126" s="2" t="s">
-        <v>260</v>
+        <v>249</v>
       </c>
       <c r="C126" s="2" t="s">
-        <v>261</v>
+        <v>250</v>
       </c>
       <c r="D126" s="2" t="s">
-        <v>421</v>
+        <v>418</v>
       </c>
     </row>
     <row r="127" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A127" s="2" t="s">
-        <v>262</v>
+        <v>253</v>
       </c>
       <c r="B127" s="2" t="s">
-        <v>263</v>
+        <v>254</v>
       </c>
       <c r="C127" s="2" t="s">
-        <v>264</v>
+        <v>255</v>
       </c>
       <c r="D127" s="2" t="s">
-        <v>422</v>
+        <v>419</v>
       </c>
     </row>
     <row r="128" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A128" s="2" t="s">
-        <v>265</v>
+        <v>256</v>
       </c>
       <c r="B128" s="2" t="s">
-        <v>265</v>
+        <v>257</v>
       </c>
       <c r="C128" s="2" t="s">
-        <v>265</v>
+        <v>258</v>
       </c>
       <c r="D128" s="2" t="s">
-        <v>423</v>
+        <v>420</v>
       </c>
     </row>
     <row r="129" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A129" s="2" t="s">
-        <v>266</v>
+        <v>259</v>
       </c>
       <c r="B129" s="2" t="s">
-        <v>266</v>
+        <v>260</v>
       </c>
       <c r="C129" s="2" t="s">
-        <v>267</v>
+        <v>261</v>
       </c>
       <c r="D129" s="2" t="s">
-        <v>424</v>
+        <v>421</v>
       </c>
     </row>
     <row r="130" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A130" s="2" t="s">
-        <v>268</v>
+        <v>262</v>
       </c>
       <c r="B130" s="2" t="s">
-        <v>268</v>
+        <v>263</v>
       </c>
       <c r="C130" s="2" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="D130" s="2" t="s">
-        <v>425</v>
+        <v>422</v>
       </c>
     </row>
     <row r="131" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A131" s="2" t="s">
-        <v>270</v>
+        <v>265</v>
       </c>
       <c r="B131" s="2" t="s">
-        <v>270</v>
+        <v>265</v>
       </c>
       <c r="C131" s="2" t="s">
-        <v>273</v>
+        <v>265</v>
       </c>
       <c r="D131" s="2" t="s">
-        <v>426</v>
+        <v>423</v>
       </c>
     </row>
     <row r="132" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A132" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="B132" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="C132" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="D132" s="2" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="133" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A133" s="2" t="s">
+        <v>268</v>
+      </c>
+      <c r="B133" s="2" t="s">
+        <v>268</v>
+      </c>
+      <c r="C133" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="D133" s="2" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="134" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A134" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="B134" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="C134" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="D134" s="2" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="135" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A135" s="2" t="s">
         <v>271</v>
       </c>
-      <c r="B132" s="2" t="s">
+      <c r="B135" s="2" t="s">
         <v>271</v>
       </c>
-      <c r="C132" s="2" t="s">
+      <c r="C135" s="2" t="s">
         <v>272</v>
       </c>
-      <c r="D132" s="2" t="s">
+      <c r="D135" s="2" t="s">
         <v>427</v>
       </c>
     </row>
-    <row r="133" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A133" s="2" t="s">
+    <row r="136" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A136" s="2" t="s">
         <v>274</v>
       </c>
-      <c r="B133" s="2" t="s">
+      <c r="B136" s="2" t="s">
         <v>276</v>
       </c>
-      <c r="C133" s="2" t="s">
+      <c r="C136" s="2" t="s">
         <v>279</v>
       </c>
     </row>
-    <row r="134" spans="1:4" ht="45" x14ac:dyDescent="0.25">
-      <c r="A134" s="2" t="s">
+    <row r="137" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="A137" s="2" t="s">
         <v>275</v>
       </c>
-      <c r="B134" s="2" t="s">
+      <c r="B137" s="2" t="s">
         <v>277</v>
       </c>
-      <c r="C134" s="2" t="s">
+      <c r="C137" s="2" t="s">
         <v>278</v>
       </c>
     </row>
-    <row r="135" spans="1:4" ht="75" x14ac:dyDescent="0.25">
-      <c r="A135" s="2" t="s">
+    <row r="138" spans="1:4" ht="75" x14ac:dyDescent="0.25">
+      <c r="A138" s="2" t="s">
         <v>289</v>
       </c>
-      <c r="B135" s="2" t="s">
+      <c r="B138" s="2" t="s">
         <v>290</v>
       </c>
-      <c r="C135" s="2" t="s">
+      <c r="C138" s="2" t="s">
         <v>291</v>
-      </c>
-    </row>
-    <row r="136" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A136" s="2" t="s">
-        <v>306</v>
-      </c>
-      <c r="B136" s="2" t="s">
-        <v>307</v>
-      </c>
-      <c r="C136" s="2" t="s">
-        <v>308</v>
-      </c>
-      <c r="D136" s="2" t="s">
-        <v>428</v>
-      </c>
-    </row>
-    <row r="137" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A137" s="2" t="s">
-        <v>309</v>
-      </c>
-      <c r="B137" s="2" t="s">
-        <v>311</v>
-      </c>
-      <c r="C137" s="2" t="s">
-        <v>312</v>
-      </c>
-      <c r="D137" s="2" t="s">
-        <v>429</v>
-      </c>
-    </row>
-    <row r="138" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A138" s="2" t="s">
-        <v>310</v>
-      </c>
-      <c r="B138" s="2" t="s">
-        <v>314</v>
-      </c>
-      <c r="C138" s="2" t="s">
-        <v>313</v>
-      </c>
-      <c r="D138" s="2" t="s">
-        <v>430</v>
       </c>
     </row>
     <row r="139" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A139" s="2" t="s">
-        <v>315</v>
+        <v>306</v>
       </c>
       <c r="B139" s="2" t="s">
-        <v>315</v>
+        <v>307</v>
       </c>
       <c r="C139" s="2" t="s">
-        <v>316</v>
+        <v>308</v>
       </c>
       <c r="D139" s="2" t="s">
-        <v>431</v>
+        <v>428</v>
       </c>
     </row>
     <row r="140" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A140" s="2" t="s">
-        <v>317</v>
+        <v>309</v>
       </c>
       <c r="B140" s="2" t="s">
-        <v>318</v>
+        <v>311</v>
       </c>
       <c r="C140" s="2" t="s">
-        <v>460</v>
+        <v>312</v>
       </c>
       <c r="D140" s="2" t="s">
-        <v>432</v>
+        <v>429</v>
       </c>
     </row>
     <row r="141" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A141" s="2" t="s">
-        <v>319</v>
+        <v>310</v>
       </c>
       <c r="B141" s="2" t="s">
-        <v>320</v>
+        <v>314</v>
       </c>
       <c r="C141" s="2" t="s">
-        <v>461</v>
+        <v>313</v>
       </c>
       <c r="D141" s="2" t="s">
-        <v>433</v>
+        <v>430</v>
       </c>
     </row>
     <row r="142" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A142" s="2" t="s">
-        <v>448</v>
+        <v>315</v>
       </c>
       <c r="B142" s="2" t="s">
-        <v>448</v>
+        <v>315</v>
       </c>
       <c r="C142" s="2" t="s">
-        <v>462</v>
+        <v>316</v>
       </c>
       <c r="D142" s="2" t="s">
-        <v>345</v>
+        <v>431</v>
       </c>
     </row>
     <row r="143" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A143" s="2" t="s">
-        <v>449</v>
+        <v>317</v>
       </c>
       <c r="B143" s="2" t="s">
-        <v>450</v>
+        <v>318</v>
       </c>
       <c r="C143" s="2" t="s">
-        <v>463</v>
+        <v>460</v>
       </c>
       <c r="D143" s="2" t="s">
-        <v>451</v>
+        <v>432</v>
       </c>
     </row>
     <row r="144" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A144" s="2" t="s">
-        <v>476</v>
+        <v>319</v>
       </c>
       <c r="B144" s="2" t="s">
-        <v>477</v>
+        <v>320</v>
       </c>
       <c r="C144" s="2" t="s">
-        <v>478</v>
+        <v>461</v>
+      </c>
+      <c r="D144" s="2" t="s">
+        <v>433</v>
       </c>
     </row>
     <row r="145" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A145" s="2" t="s">
-        <v>479</v>
+        <v>448</v>
       </c>
       <c r="B145" s="2" t="s">
-        <v>525</v>
+        <v>448</v>
       </c>
       <c r="C145" s="2" t="s">
-        <v>480</v>
+        <v>462</v>
+      </c>
+      <c r="D145" s="2" t="s">
+        <v>345</v>
       </c>
     </row>
     <row r="146" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A146" s="2" t="s">
-        <v>481</v>
+        <v>449</v>
       </c>
       <c r="B146" s="2" t="s">
-        <v>482</v>
+        <v>450</v>
       </c>
       <c r="C146" s="2" t="s">
-        <v>483</v>
+        <v>463</v>
+      </c>
+      <c r="D146" s="2" t="s">
+        <v>451</v>
       </c>
     </row>
     <row r="147" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A147" s="2" t="s">
-        <v>484</v>
+        <v>476</v>
       </c>
       <c r="B147" s="2" t="s">
-        <v>485</v>
+        <v>477</v>
       </c>
       <c r="C147" s="2" t="s">
-        <v>486</v>
+        <v>478</v>
+      </c>
+      <c r="D147" s="2" t="s">
+        <v>573</v>
       </c>
     </row>
     <row r="148" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A148" s="2" t="s">
-        <v>487</v>
+        <v>479</v>
       </c>
       <c r="B148" s="2" t="s">
-        <v>488</v>
+        <v>525</v>
       </c>
       <c r="C148" s="2" t="s">
-        <v>489</v>
+        <v>480</v>
+      </c>
+      <c r="D148" s="2" t="s">
+        <v>572</v>
       </c>
     </row>
     <row r="149" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A149" s="2" t="s">
-        <v>490</v>
+        <v>481</v>
       </c>
       <c r="B149" s="2" t="s">
-        <v>491</v>
+        <v>482</v>
       </c>
       <c r="C149" s="2" t="s">
-        <v>492</v>
+        <v>483</v>
+      </c>
+      <c r="D149" s="2" t="s">
+        <v>571</v>
       </c>
     </row>
     <row r="150" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A150" s="2" t="s">
-        <v>538</v>
+        <v>484</v>
       </c>
       <c r="B150" s="2" t="s">
-        <v>539</v>
+        <v>485</v>
+      </c>
+      <c r="C150" s="2" t="s">
+        <v>486</v>
+      </c>
+      <c r="D150" s="2" t="s">
+        <v>570</v>
       </c>
     </row>
     <row r="151" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A151" s="2" t="s">
-        <v>541</v>
+        <v>487</v>
       </c>
       <c r="B151" s="2" t="s">
-        <v>541</v>
+        <v>488</v>
+      </c>
+      <c r="C151" s="2" t="s">
+        <v>489</v>
       </c>
       <c r="D151" s="2" t="s">
-        <v>542</v>
+        <v>569</v>
       </c>
     </row>
     <row r="152" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A152" s="2" t="s">
-        <v>543</v>
+        <v>490</v>
       </c>
       <c r="B152" s="2" t="s">
-        <v>544</v>
+        <v>491</v>
+      </c>
+      <c r="C152" s="2" t="s">
+        <v>492</v>
       </c>
       <c r="D152" s="2" t="s">
-        <v>545</v>
+        <v>568</v>
       </c>
     </row>
     <row r="153" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A153" s="2" t="s">
-        <v>493</v>
+        <v>539</v>
       </c>
       <c r="B153" s="2" t="s">
-        <v>494</v>
-      </c>
-      <c r="C153" s="2" t="s">
-        <v>495</v>
+        <v>539</v>
+      </c>
+      <c r="D153" s="2" t="s">
+        <v>540</v>
       </c>
     </row>
     <row r="154" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A154" s="2" t="s">
-        <v>496</v>
+        <v>541</v>
       </c>
       <c r="B154" s="2" t="s">
-        <v>497</v>
-      </c>
-      <c r="C154" s="2" t="s">
-        <v>498</v>
+        <v>542</v>
+      </c>
+      <c r="D154" s="2" t="s">
+        <v>543</v>
       </c>
     </row>
     <row r="155" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A155" s="2" t="s">
-        <v>499</v>
+        <v>493</v>
       </c>
       <c r="B155" s="2" t="s">
-        <v>500</v>
+        <v>494</v>
       </c>
       <c r="C155" s="2" t="s">
-        <v>501</v>
+        <v>495</v>
+      </c>
+      <c r="D155" s="2" t="s">
+        <v>567</v>
       </c>
     </row>
     <row r="156" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A156" s="2" t="s">
-        <v>502</v>
+        <v>496</v>
       </c>
       <c r="B156" s="2" t="s">
-        <v>502</v>
+        <v>497</v>
       </c>
       <c r="C156" s="2" t="s">
-        <v>503</v>
+        <v>498</v>
+      </c>
+      <c r="D156" s="2" t="s">
+        <v>566</v>
       </c>
     </row>
     <row r="157" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A157" s="2" t="s">
-        <v>504</v>
+        <v>499</v>
       </c>
       <c r="B157" s="2" t="s">
-        <v>504</v>
+        <v>500</v>
       </c>
       <c r="C157" s="2" t="s">
-        <v>505</v>
+        <v>501</v>
+      </c>
+      <c r="D157" s="2" t="s">
+        <v>565</v>
       </c>
     </row>
     <row r="158" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A158" s="2" t="s">
-        <v>506</v>
+        <v>502</v>
       </c>
       <c r="B158" s="2" t="s">
-        <v>506</v>
+        <v>502</v>
       </c>
       <c r="C158" s="2" t="s">
-        <v>507</v>
+        <v>503</v>
+      </c>
+      <c r="D158" s="2" t="s">
+        <v>564</v>
       </c>
     </row>
     <row r="159" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A159" s="2" t="s">
+        <v>504</v>
+      </c>
+      <c r="B159" s="2" t="s">
+        <v>504</v>
+      </c>
+      <c r="C159" s="2" t="s">
+        <v>505</v>
+      </c>
+      <c r="D159" s="2" t="s">
+        <v>563</v>
+      </c>
+    </row>
+    <row r="160" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A160" s="2" t="s">
+        <v>506</v>
+      </c>
+      <c r="B160" s="2" t="s">
+        <v>506</v>
+      </c>
+      <c r="C160" s="2" t="s">
+        <v>507</v>
+      </c>
+      <c r="D160" s="2" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="161" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A161" s="2" t="s">
         <v>508</v>
       </c>
-      <c r="B159" s="2" t="s">
+      <c r="B161" s="2" t="s">
         <v>508</v>
       </c>
-      <c r="C159" s="2" t="s">
+      <c r="C161" s="2" t="s">
         <v>509</v>
+      </c>
+      <c r="D161" s="2" t="s">
+        <v>561</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fixed some broken translations with the new system added in the past commit.
</commit_message>
<xml_diff>
--- a/Translations/Translations.xlsx
+++ b/Translations/Translations.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programacion\MelonLoader\FS_LevelEditor\Translations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6A5CE93-E473-44A7-ACAD-0C2FB45F8A21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F44A1C6D-A77C-4BF0-B5CF-21C4165213D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{F5C22481-FF1A-482C-BF7E-EB5A7718AF49}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1319" uniqueCount="629">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1322" uniqueCount="632">
   <si>
     <t>ID</t>
   </si>
@@ -1925,6 +1925,15 @@
   </si>
   <si>
     <t>DESPLEGADO</t>
+  </si>
+  <si>
+    <t>allCorrect</t>
+  </si>
+  <si>
+    <t>All Correct</t>
+  </si>
+  <si>
+    <t>Todo Correcto</t>
   </si>
 </sst>
 </file>
@@ -2324,7 +2333,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6961A5F-F8EA-4989-8112-A0ACE51D011E}">
   <sheetPr codeName="Hoja1"/>
-  <dimension ref="A1:D175"/>
+  <dimension ref="A1:D176"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="37" style="2" customWidth="1"/>
@@ -4729,6 +4738,17 @@
       </c>
       <c r="C175" s="2" t="s">
         <v>628</v>
+      </c>
+    </row>
+    <row r="176" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A176" s="2" t="s">
+        <v>629</v>
+      </c>
+      <c r="B176" s="2" t="s">
+        <v>630</v>
+      </c>
+      <c r="C176" s="2" t="s">
+        <v>631</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Now the respawn point for death triggers can be specified with a small waypoint!
</commit_message>
<xml_diff>
--- a/Translations/Translations.xlsx
+++ b/Translations/Translations.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programacion\MelonLoader\FS_LevelEditor\Translations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F44A1C6D-A77C-4BF0-B5CF-21C4165213D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7F04CC1-D9F1-4691-A5CD-28B7CCCF7EDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{F5C22481-FF1A-482C-BF7E-EB5A7718AF49}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1322" uniqueCount="632">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1331" uniqueCount="641">
   <si>
     <t>ID</t>
   </si>
@@ -1934,6 +1934,33 @@
   </si>
   <si>
     <t>Todo Correcto</t>
+  </si>
+  <si>
+    <t>AddDeathTriggerWaypoint</t>
+  </si>
+  <si>
+    <t>+ Add Respawn Point</t>
+  </si>
+  <si>
+    <t>+ Añadir Punto de Reaparición</t>
+  </si>
+  <si>
+    <t>object.DEATH_TRIGGER_WAYPOINT</t>
+  </si>
+  <si>
+    <t>Respawn Point</t>
+  </si>
+  <si>
+    <t>Punto de Reaparición</t>
+  </si>
+  <si>
+    <t>RotatePlayer</t>
+  </si>
+  <si>
+    <t>Rotate Player</t>
+  </si>
+  <si>
+    <t>Rotar al Jugador</t>
   </si>
 </sst>
 </file>
@@ -2333,7 +2360,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6961A5F-F8EA-4989-8112-A0ACE51D011E}">
   <sheetPr codeName="Hoja1"/>
-  <dimension ref="A1:D176"/>
+  <dimension ref="A1:D179"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="37" style="2" customWidth="1"/>
@@ -3141,1614 +3168,1647 @@
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" s="2" t="s">
-        <v>69</v>
+        <v>635</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>69</v>
+        <v>636</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="D58" s="2" t="s">
-        <v>364</v>
+        <v>637</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" s="2" t="s">
-        <v>443</v>
+        <v>69</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>443</v>
+        <v>69</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>601</v>
+        <v>101</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>552</v>
+        <v>364</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
-        <v>456</v>
+        <v>443</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>456</v>
+        <v>443</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>456</v>
+        <v>601</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>457</v>
+        <v>552</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61" s="2" t="s">
-        <v>105</v>
+        <v>456</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>2</v>
+        <v>456</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>102</v>
+        <v>456</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>365</v>
+        <v>457</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>111</v>
+        <v>4</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A65" s="2" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="D65" s="2" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66" s="2" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="D66" s="2" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A67" s="2" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="D67" s="2" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A68" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D68" s="2" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A69" s="2" t="s">
-        <v>445</v>
+        <v>118</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>446</v>
+        <v>122</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>459</v>
+        <v>121</v>
       </c>
       <c r="D69" s="2" t="s">
-        <v>447</v>
+        <v>370</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A70" s="2" t="s">
-        <v>512</v>
+        <v>445</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>513</v>
+        <v>446</v>
       </c>
       <c r="C70" s="2" t="s">
-        <v>602</v>
+        <v>459</v>
       </c>
       <c r="D70" s="2" t="s">
-        <v>514</v>
+        <v>447</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A71" s="2" t="s">
-        <v>518</v>
+        <v>512</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>519</v>
+        <v>513</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="D71" s="2" t="s">
-        <v>520</v>
+        <v>514</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A72" s="2" t="s">
-        <v>521</v>
+        <v>518</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>522</v>
+        <v>519</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="D72" s="2" t="s">
-        <v>523</v>
+        <v>520</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A73" s="2" t="s">
-        <v>532</v>
+        <v>521</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>533</v>
+        <v>522</v>
       </c>
       <c r="C73" s="2" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="D73" s="2" t="s">
-        <v>534</v>
+        <v>523</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A74" s="2" t="s">
-        <v>537</v>
+        <v>532</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>535</v>
+        <v>533</v>
       </c>
       <c r="C74" s="2" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="D74" s="2" t="s">
-        <v>536</v>
+        <v>534</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A75" s="2" t="s">
-        <v>154</v>
+        <v>537</v>
       </c>
       <c r="B75" s="2" t="s">
-        <v>155</v>
+        <v>535</v>
       </c>
       <c r="C75" s="2" t="s">
-        <v>156</v>
+        <v>606</v>
       </c>
       <c r="D75" s="2" t="s">
-        <v>371</v>
+        <v>536</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A76" s="2" t="s">
-        <v>164</v>
+        <v>154</v>
       </c>
       <c r="B76" s="2" t="s">
-        <v>165</v>
+        <v>155</v>
       </c>
       <c r="C76" s="2" t="s">
-        <v>166</v>
+        <v>156</v>
       </c>
       <c r="D76" s="2" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A77" s="2" t="s">
-        <v>157</v>
+        <v>164</v>
       </c>
       <c r="B77" s="2" t="s">
-        <v>158</v>
+        <v>165</v>
       </c>
       <c r="C77" s="2" t="s">
-        <v>159</v>
+        <v>166</v>
       </c>
       <c r="D77" s="2" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A78" s="2" t="s">
-        <v>167</v>
+        <v>157</v>
       </c>
       <c r="B78" s="2" t="s">
-        <v>168</v>
+        <v>158</v>
       </c>
       <c r="C78" s="2" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="D78" s="2" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A79" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="B79" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="C79" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="D79" s="2" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A80" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="B79" s="2" t="s">
+      <c r="B80" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="C79" s="2" t="s">
+      <c r="C80" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="D79" s="2" t="s">
+      <c r="D80" s="2" t="s">
         <v>375</v>
       </c>
     </row>
-    <row r="80" spans="1:4" ht="45" x14ac:dyDescent="0.25">
-      <c r="A80" s="2" t="s">
+    <row r="81" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="A81" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="B80" s="2" t="s">
+      <c r="B81" s="2" t="s">
         <v>163</v>
       </c>
-      <c r="C80" s="2" t="s">
+      <c r="C81" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="D80" s="2" t="s">
+      <c r="D81" s="2" t="s">
         <v>376</v>
-      </c>
-    </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A81" s="2" t="s">
-        <v>153</v>
-      </c>
-      <c r="B81" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="C81" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="D81" s="2" t="s">
-        <v>328</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A82" s="2" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="B82" s="2" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="C82" s="2" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="D82" s="2" t="s">
-        <v>377</v>
+        <v>328</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A83" s="2" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="B83" s="2" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="C83" s="2" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="D83" s="2" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A84" s="2" t="s">
-        <v>172</v>
+        <v>150</v>
       </c>
       <c r="B84" s="2" t="s">
-        <v>170</v>
+        <v>151</v>
       </c>
       <c r="C84" s="2" t="s">
-        <v>171</v>
+        <v>152</v>
       </c>
       <c r="D84" s="2" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A85" s="2" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B85" s="2" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="C85" s="2" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="D85" s="2" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A86" s="2" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="B86" s="2" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="C86" s="2" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="D86" s="2" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A87" s="2" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="B87" s="2" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="C87" s="2" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="D87" s="2" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A88" s="2" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="B88" s="2" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="C88" s="2" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="D88" s="2" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A89" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="B89" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="C89" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="D89" s="2" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A90" s="2" t="s">
         <v>243</v>
       </c>
-      <c r="B89" s="2" t="s">
+      <c r="B90" s="2" t="s">
         <v>243</v>
       </c>
-      <c r="C89" s="2" t="s">
+      <c r="C90" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="D89" s="2" t="s">
+      <c r="D90" s="2" t="s">
         <v>384</v>
       </c>
     </row>
-    <row r="90" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A90" s="2" t="s">
+    <row r="91" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A91" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="B90" s="1" t="s">
+      <c r="B91" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="C90" s="2" t="s">
+      <c r="C91" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="D90" s="2" t="s">
+      <c r="D91" s="2" t="s">
         <v>385</v>
-      </c>
-    </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A91" s="2" t="s">
-        <v>182</v>
-      </c>
-      <c r="B91" s="2" t="s">
-        <v>183</v>
-      </c>
-      <c r="C91" s="2" t="s">
-        <v>183</v>
-      </c>
-      <c r="D91" s="2" t="s">
-        <v>386</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A92" s="2" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="B92" s="2" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C92" s="2" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="D92" s="2" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A93" s="2" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="B93" s="2" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="C93" s="2" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="D93" s="2" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A94" s="2" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="B94" s="2" t="s">
-        <v>525</v>
+        <v>186</v>
       </c>
       <c r="C94" s="2" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="D94" s="2" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A95" s="2" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="B95" s="2" t="s">
-        <v>190</v>
+        <v>525</v>
       </c>
       <c r="C95" s="2" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="D95" s="2" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A96" s="2" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="B96" s="2" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="C96" s="2" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="D96" s="2" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A97" s="2" t="s">
-        <v>434</v>
-      </c>
-      <c r="B97" s="4" t="s">
-        <v>435</v>
-      </c>
-      <c r="C97" s="4" t="s">
-        <v>436</v>
-      </c>
-      <c r="D97" s="4" t="s">
-        <v>591</v>
+        <v>192</v>
+      </c>
+      <c r="B97" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="C97" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="D97" s="2" t="s">
+        <v>391</v>
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A98" s="2" t="s">
-        <v>437</v>
+        <v>434</v>
       </c>
       <c r="B98" s="4" t="s">
-        <v>438</v>
+        <v>435</v>
       </c>
       <c r="C98" s="4" t="s">
-        <v>439</v>
+        <v>436</v>
       </c>
       <c r="D98" s="4" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A99" s="2" t="s">
-        <v>473</v>
+        <v>437</v>
       </c>
       <c r="B99" s="4" t="s">
-        <v>590</v>
+        <v>438</v>
       </c>
       <c r="C99" s="4" t="s">
-        <v>474</v>
+        <v>439</v>
       </c>
       <c r="D99" s="4" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A100" s="2" t="s">
-        <v>195</v>
-      </c>
-      <c r="B100" s="2" t="s">
-        <v>196</v>
-      </c>
-      <c r="C100" s="2" t="s">
-        <v>197</v>
-      </c>
-      <c r="D100" s="2" t="s">
-        <v>392</v>
+        <v>473</v>
+      </c>
+      <c r="B100" s="4" t="s">
+        <v>590</v>
+      </c>
+      <c r="C100" s="4" t="s">
+        <v>474</v>
+      </c>
+      <c r="D100" s="4" t="s">
+        <v>593</v>
       </c>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A101" s="2" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="B101" s="2" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="C101" s="2" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="D101" s="2" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A102" s="2" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="B102" s="2" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="C102" s="2" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="D102" s="2" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A103" s="2" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="B103" s="2" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="C103" s="2" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="D103" s="2" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A104" s="2" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="B104" s="2" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="C104" s="2" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="D104" s="2" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A105" s="2" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B105" s="2" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="C105" s="2" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="D105" s="2" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A106" s="2" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="B106" s="2" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="C106" s="2" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="D106" s="2" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A107" s="2" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="B107" s="2" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="C107" s="2" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="D107" s="2" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A108" s="2" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="B108" s="2" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="C108" s="2" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="D108" s="2" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A109" s="2" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="B109" s="2" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="C109" s="2" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="D109" s="2" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A110" s="2" t="s">
-        <v>292</v>
+        <v>220</v>
       </c>
       <c r="B110" s="2" t="s">
-        <v>292</v>
+        <v>219</v>
       </c>
       <c r="C110" s="2" t="s">
-        <v>293</v>
+        <v>218</v>
       </c>
       <c r="D110" s="2" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A111" s="2" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="B111" s="2" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="C111" s="2" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
       <c r="D111" s="2" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A112" s="2" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
       <c r="B112" s="2" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="C112" s="2" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="D112" s="2" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A113" s="2" t="s">
-        <v>221</v>
+        <v>297</v>
       </c>
       <c r="B113" s="2" t="s">
-        <v>221</v>
+        <v>298</v>
       </c>
       <c r="C113" s="2" t="s">
-        <v>222</v>
+        <v>299</v>
       </c>
       <c r="D113" s="2" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A114" s="2" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="B114" s="2" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="C114" s="2" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="D114" s="2" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A115" s="2" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="B115" s="2" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="C115" s="2" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="D115" s="2" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A116" s="2" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="B116" s="2" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="C116" s="2" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="D116" s="2" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A117" s="2" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B117" s="2" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="C117" s="2" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="D117" s="2" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A118" s="2" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="B118" s="2" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="C118" s="2" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="D118" s="2" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
     </row>
     <row r="119" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A119" s="2" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="B119" s="2" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="C119" s="2" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="D119" s="2" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A120" s="2" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="B120" s="2" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="C120" s="2" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="D120" s="2" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A121" s="2" t="s">
-        <v>300</v>
+        <v>237</v>
       </c>
       <c r="B121" s="2" t="s">
-        <v>301</v>
+        <v>238</v>
       </c>
       <c r="C121" s="2" t="s">
-        <v>302</v>
+        <v>239</v>
       </c>
       <c r="D121" s="2" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A122" s="2" t="s">
-        <v>240</v>
+        <v>300</v>
       </c>
       <c r="B122" s="2" t="s">
-        <v>241</v>
+        <v>301</v>
       </c>
       <c r="C122" s="2" t="s">
-        <v>242</v>
+        <v>302</v>
       </c>
       <c r="D122" s="2" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
     </row>
     <row r="123" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A123" s="2" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="B123" s="2" t="s">
-        <v>252</v>
+        <v>241</v>
       </c>
       <c r="C123" s="2" t="s">
-        <v>251</v>
+        <v>242</v>
       </c>
       <c r="D123" s="2" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="124" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A124" s="2" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B124" s="2" t="s">
-        <v>245</v>
+        <v>252</v>
       </c>
       <c r="C124" s="2" t="s">
-        <v>246</v>
+        <v>251</v>
       </c>
       <c r="D124" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
     </row>
     <row r="125" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A125" s="2" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="B125" s="2" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="C125" s="2" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="D125" s="2" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
     </row>
     <row r="126" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A126" s="2" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="B126" s="2" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="C126" s="2" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="D126" s="2" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
     </row>
     <row r="127" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A127" s="2" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="B127" s="2" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="C127" s="2" t="s">
-        <v>255</v>
+        <v>250</v>
       </c>
       <c r="D127" s="2" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
     </row>
     <row r="128" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A128" s="2" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="B128" s="2" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="C128" s="2" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="D128" s="2" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
     </row>
     <row r="129" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A129" s="2" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="B129" s="2" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="C129" s="2" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="D129" s="2" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
     </row>
     <row r="130" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A130" s="2" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="B130" s="2" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="C130" s="2" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="D130" s="2" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="131" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A131" s="2" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="B131" s="2" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="C131" s="2" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="D131" s="2" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
     </row>
     <row r="132" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A132" s="2" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="B132" s="2" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="C132" s="2" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="D132" s="2" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
     </row>
     <row r="133" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A133" s="2" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="B133" s="2" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="C133" s="2" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="D133" s="2" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
     </row>
     <row r="134" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A134" s="2" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="B134" s="2" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="C134" s="2" t="s">
-        <v>273</v>
+        <v>269</v>
       </c>
       <c r="D134" s="2" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
     </row>
     <row r="135" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A135" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="B135" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="C135" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="D135" s="2" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="136" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A136" s="2" t="s">
         <v>271</v>
       </c>
-      <c r="B135" s="2" t="s">
+      <c r="B136" s="2" t="s">
         <v>271</v>
       </c>
-      <c r="C135" s="2" t="s">
+      <c r="C136" s="2" t="s">
         <v>272</v>
       </c>
-      <c r="D135" s="2" t="s">
+      <c r="D136" s="2" t="s">
         <v>427</v>
       </c>
     </row>
-    <row r="136" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A136" s="2" t="s">
+    <row r="137" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A137" s="2" t="s">
         <v>274</v>
       </c>
-      <c r="B136" s="2" t="s">
+      <c r="B137" s="2" t="s">
         <v>276</v>
       </c>
-      <c r="C136" s="2" t="s">
+      <c r="C137" s="2" t="s">
         <v>279</v>
       </c>
     </row>
-    <row r="137" spans="1:4" ht="45" x14ac:dyDescent="0.25">
-      <c r="A137" s="2" t="s">
+    <row r="138" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="A138" s="2" t="s">
         <v>275</v>
       </c>
-      <c r="B137" s="2" t="s">
+      <c r="B138" s="2" t="s">
         <v>277</v>
       </c>
-      <c r="C137" s="2" t="s">
+      <c r="C138" s="2" t="s">
         <v>278</v>
       </c>
     </row>
-    <row r="138" spans="1:4" ht="75" x14ac:dyDescent="0.25">
-      <c r="A138" s="2" t="s">
+    <row r="139" spans="1:4" ht="75" x14ac:dyDescent="0.25">
+      <c r="A139" s="2" t="s">
         <v>289</v>
       </c>
-      <c r="B138" s="2" t="s">
+      <c r="B139" s="2" t="s">
         <v>290</v>
       </c>
-      <c r="C138" s="2" t="s">
+      <c r="C139" s="2" t="s">
         <v>291</v>
-      </c>
-    </row>
-    <row r="139" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A139" s="2" t="s">
-        <v>306</v>
-      </c>
-      <c r="B139" s="2" t="s">
-        <v>307</v>
-      </c>
-      <c r="C139" s="2" t="s">
-        <v>308</v>
-      </c>
-      <c r="D139" s="2" t="s">
-        <v>428</v>
       </c>
     </row>
     <row r="140" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A140" s="2" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
       <c r="B140" s="2" t="s">
-        <v>311</v>
+        <v>307</v>
       </c>
       <c r="C140" s="2" t="s">
-        <v>312</v>
+        <v>308</v>
       </c>
       <c r="D140" s="2" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
     </row>
     <row r="141" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A141" s="2" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="B141" s="2" t="s">
-        <v>314</v>
+        <v>311</v>
       </c>
       <c r="C141" s="2" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="D141" s="2" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
     </row>
     <row r="142" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A142" s="2" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="B142" s="2" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="C142" s="2" t="s">
-        <v>316</v>
+        <v>313</v>
       </c>
       <c r="D142" s="2" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
     </row>
     <row r="143" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A143" s="2" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="B143" s="2" t="s">
-        <v>318</v>
+        <v>315</v>
       </c>
       <c r="C143" s="2" t="s">
-        <v>460</v>
+        <v>316</v>
       </c>
       <c r="D143" s="2" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
     </row>
     <row r="144" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A144" s="2" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="B144" s="2" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="C144" s="2" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="D144" s="2" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
     </row>
     <row r="145" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A145" s="2" t="s">
-        <v>448</v>
+        <v>319</v>
       </c>
       <c r="B145" s="2" t="s">
-        <v>448</v>
+        <v>320</v>
       </c>
       <c r="C145" s="2" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="D145" s="2" t="s">
-        <v>345</v>
+        <v>433</v>
       </c>
     </row>
     <row r="146" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A146" s="2" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="B146" s="2" t="s">
-        <v>450</v>
+        <v>448</v>
       </c>
       <c r="C146" s="2" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="D146" s="2" t="s">
-        <v>451</v>
+        <v>345</v>
       </c>
     </row>
     <row r="147" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A147" s="2" t="s">
-        <v>475</v>
+        <v>449</v>
       </c>
       <c r="B147" s="2" t="s">
-        <v>476</v>
+        <v>450</v>
       </c>
       <c r="C147" s="2" t="s">
-        <v>619</v>
+        <v>463</v>
       </c>
       <c r="D147" s="2" t="s">
-        <v>569</v>
+        <v>451</v>
       </c>
     </row>
     <row r="148" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A148" s="2" t="s">
-        <v>478</v>
+        <v>475</v>
       </c>
       <c r="B148" s="2" t="s">
-        <v>524</v>
+        <v>476</v>
       </c>
       <c r="C148" s="2" t="s">
-        <v>479</v>
+        <v>619</v>
       </c>
       <c r="D148" s="2" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
     </row>
     <row r="149" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A149" s="2" t="s">
-        <v>480</v>
+        <v>478</v>
       </c>
       <c r="B149" s="2" t="s">
-        <v>481</v>
+        <v>524</v>
       </c>
       <c r="C149" s="2" t="s">
-        <v>482</v>
+        <v>479</v>
       </c>
       <c r="D149" s="2" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
     </row>
     <row r="150" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A150" s="2" t="s">
-        <v>483</v>
+        <v>480</v>
       </c>
       <c r="B150" s="2" t="s">
-        <v>484</v>
+        <v>481</v>
       </c>
       <c r="C150" s="2" t="s">
-        <v>485</v>
+        <v>482</v>
       </c>
       <c r="D150" s="2" t="s">
-        <v>566</v>
+        <v>567</v>
       </c>
     </row>
     <row r="151" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A151" s="2" t="s">
-        <v>486</v>
+        <v>483</v>
       </c>
       <c r="B151" s="2" t="s">
-        <v>487</v>
+        <v>484</v>
       </c>
       <c r="C151" s="2" t="s">
-        <v>488</v>
+        <v>485</v>
       </c>
       <c r="D151" s="2" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
     </row>
     <row r="152" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A152" s="2" t="s">
-        <v>489</v>
+        <v>486</v>
       </c>
       <c r="B152" s="2" t="s">
-        <v>490</v>
+        <v>487</v>
       </c>
       <c r="C152" s="2" t="s">
-        <v>491</v>
+        <v>488</v>
       </c>
       <c r="D152" s="2" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
     </row>
     <row r="153" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A153" s="2" t="s">
-        <v>538</v>
+        <v>489</v>
       </c>
       <c r="B153" s="2" t="s">
-        <v>538</v>
+        <v>490</v>
       </c>
       <c r="C153" s="2" t="s">
-        <v>607</v>
+        <v>491</v>
       </c>
       <c r="D153" s="2" t="s">
-        <v>539</v>
+        <v>564</v>
       </c>
     </row>
     <row r="154" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A154" s="2" t="s">
-        <v>540</v>
+        <v>538</v>
       </c>
       <c r="B154" s="2" t="s">
-        <v>541</v>
+        <v>538</v>
       </c>
       <c r="C154" s="2" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="D154" s="2" t="s">
-        <v>542</v>
+        <v>539</v>
       </c>
     </row>
     <row r="155" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A155" s="2" t="s">
-        <v>492</v>
+        <v>540</v>
       </c>
       <c r="B155" s="2" t="s">
-        <v>493</v>
+        <v>541</v>
       </c>
       <c r="C155" s="2" t="s">
-        <v>494</v>
+        <v>608</v>
       </c>
       <c r="D155" s="2" t="s">
-        <v>563</v>
+        <v>542</v>
       </c>
     </row>
     <row r="156" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A156" s="2" t="s">
-        <v>495</v>
+        <v>492</v>
       </c>
       <c r="B156" s="2" t="s">
-        <v>496</v>
+        <v>493</v>
       </c>
       <c r="C156" s="2" t="s">
-        <v>497</v>
+        <v>494</v>
       </c>
       <c r="D156" s="2" t="s">
-        <v>562</v>
+        <v>563</v>
       </c>
     </row>
     <row r="157" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A157" s="2" t="s">
-        <v>498</v>
+        <v>495</v>
       </c>
       <c r="B157" s="2" t="s">
-        <v>499</v>
+        <v>496</v>
       </c>
       <c r="C157" s="2" t="s">
-        <v>500</v>
+        <v>497</v>
       </c>
       <c r="D157" s="2" t="s">
-        <v>561</v>
+        <v>562</v>
       </c>
     </row>
     <row r="158" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A158" s="2" t="s">
-        <v>501</v>
+        <v>498</v>
       </c>
       <c r="B158" s="2" t="s">
-        <v>501</v>
+        <v>499</v>
       </c>
       <c r="C158" s="2" t="s">
-        <v>502</v>
+        <v>500</v>
       </c>
       <c r="D158" s="2" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
     </row>
     <row r="159" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A159" s="2" t="s">
-        <v>503</v>
+        <v>501</v>
       </c>
       <c r="B159" s="2" t="s">
-        <v>503</v>
+        <v>501</v>
       </c>
       <c r="C159" s="2" t="s">
-        <v>504</v>
+        <v>502</v>
       </c>
       <c r="D159" s="2" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
     </row>
     <row r="160" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A160" s="2" t="s">
-        <v>505</v>
+        <v>503</v>
       </c>
       <c r="B160" s="2" t="s">
-        <v>505</v>
+        <v>503</v>
       </c>
       <c r="C160" s="2" t="s">
-        <v>506</v>
+        <v>504</v>
       </c>
       <c r="D160" s="2" t="s">
-        <v>558</v>
+        <v>559</v>
       </c>
     </row>
     <row r="161" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A161" s="2" t="s">
-        <v>507</v>
+        <v>505</v>
       </c>
       <c r="B161" s="2" t="s">
-        <v>507</v>
+        <v>505</v>
       </c>
       <c r="C161" s="2" t="s">
-        <v>508</v>
+        <v>506</v>
       </c>
       <c r="D161" s="2" t="s">
-        <v>557</v>
+        <v>558</v>
       </c>
     </row>
     <row r="162" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A162" s="2" t="s">
-        <v>570</v>
+        <v>507</v>
       </c>
       <c r="B162" s="2" t="s">
-        <v>571</v>
+        <v>507</v>
       </c>
       <c r="C162" s="2" t="s">
-        <v>609</v>
+        <v>508</v>
+      </c>
+      <c r="D162" s="2" t="s">
+        <v>557</v>
       </c>
     </row>
     <row r="163" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A163" s="2" t="s">
-        <v>572</v>
+        <v>570</v>
       </c>
       <c r="B163" s="2" t="s">
-        <v>573</v>
+        <v>571</v>
       </c>
       <c r="C163" s="2" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
     </row>
     <row r="164" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A164" s="2" t="s">
-        <v>574</v>
+        <v>572</v>
       </c>
       <c r="B164" s="2" t="s">
-        <v>575</v>
+        <v>573</v>
       </c>
       <c r="C164" s="2" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
     </row>
     <row r="165" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A165" s="2" t="s">
-        <v>576</v>
+        <v>574</v>
       </c>
       <c r="B165" s="2" t="s">
-        <v>577</v>
+        <v>575</v>
       </c>
       <c r="C165" s="2" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
     </row>
     <row r="166" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A166" s="2" t="s">
-        <v>578</v>
+        <v>576</v>
       </c>
       <c r="B166" s="2" t="s">
-        <v>579</v>
+        <v>577</v>
       </c>
       <c r="C166" s="2" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
     </row>
     <row r="167" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A167" s="2" t="s">
-        <v>580</v>
+        <v>578</v>
       </c>
       <c r="B167" s="2" t="s">
-        <v>581</v>
+        <v>579</v>
       </c>
       <c r="C167" s="2" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
     </row>
     <row r="168" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A168" s="2" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
       <c r="B168" s="2" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="C168" s="2" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
     </row>
     <row r="169" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A169" s="2" t="s">
-        <v>584</v>
+        <v>582</v>
       </c>
       <c r="B169" s="2" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="C169" s="2" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
     </row>
     <row r="170" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A170" s="2" t="s">
-        <v>586</v>
+        <v>584</v>
       </c>
       <c r="B170" s="2" t="s">
-        <v>587</v>
+        <v>585</v>
       </c>
       <c r="C170" s="2" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
     </row>
     <row r="171" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A171" s="2" t="s">
-        <v>588</v>
+        <v>586</v>
       </c>
       <c r="B171" s="2" t="s">
-        <v>589</v>
+        <v>587</v>
       </c>
       <c r="C171" s="2" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
     </row>
     <row r="172" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A172" s="2" t="s">
-        <v>620</v>
+        <v>588</v>
       </c>
       <c r="B172" s="2" t="s">
-        <v>621</v>
+        <v>589</v>
       </c>
       <c r="C172" s="2" t="s">
-        <v>622</v>
+        <v>618</v>
       </c>
     </row>
     <row r="173" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A173" s="2" t="s">
-        <v>623</v>
+        <v>620</v>
       </c>
       <c r="B173" s="2" t="s">
-        <v>623</v>
+        <v>621</v>
       </c>
       <c r="C173" s="2" t="s">
-        <v>624</v>
+        <v>622</v>
       </c>
     </row>
     <row r="174" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A174" s="2" t="s">
-        <v>625</v>
+        <v>623</v>
       </c>
       <c r="B174" s="2" t="s">
-        <v>625</v>
+        <v>623</v>
       </c>
       <c r="C174" s="2" t="s">
-        <v>627</v>
+        <v>624</v>
       </c>
     </row>
     <row r="175" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A175" s="2" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="B175" s="2" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="C175" s="2" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
     </row>
     <row r="176" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A176" s="2" t="s">
+        <v>626</v>
+      </c>
+      <c r="B176" s="2" t="s">
+        <v>626</v>
+      </c>
+      <c r="C176" s="2" t="s">
+        <v>628</v>
+      </c>
+    </row>
+    <row r="177" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A177" s="2" t="s">
         <v>629</v>
       </c>
-      <c r="B176" s="2" t="s">
+      <c r="B177" s="2" t="s">
         <v>630</v>
       </c>
-      <c r="C176" s="2" t="s">
+      <c r="C177" s="2" t="s">
         <v>631</v>
+      </c>
+    </row>
+    <row r="178" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A178" s="2" t="s">
+        <v>632</v>
+      </c>
+      <c r="B178" s="4" t="s">
+        <v>633</v>
+      </c>
+      <c r="C178" s="4" t="s">
+        <v>634</v>
+      </c>
+    </row>
+    <row r="179" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A179" s="2" t="s">
+        <v>638</v>
+      </c>
+      <c r="B179" s="2" t="s">
+        <v>639</v>
+      </c>
+      <c r="C179" s="2" t="s">
+        <v>640</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Changed "Set Door State" options. "Close" and "Close Fast" Translations are useless for now btw
</commit_message>
<xml_diff>
--- a/Translations/Translations.xlsx
+++ b/Translations/Translations.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programacion\MelonLoader\FS_LevelEditor\Translations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7F04CC1-D9F1-4691-A5CD-28B7CCCF7EDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92AF2B07-4B17-4CC1-940B-45245397C336}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{F5C22481-FF1A-482C-BF7E-EB5A7718AF49}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1331" uniqueCount="641">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1340" uniqueCount="649">
   <si>
     <t>ID</t>
   </si>
@@ -1961,6 +1961,30 @@
   </si>
   <si>
     <t>Rotar al Jugador</t>
+  </si>
+  <si>
+    <t>Close</t>
+  </si>
+  <si>
+    <t>Cerrar</t>
+  </si>
+  <si>
+    <t>CloseFast</t>
+  </si>
+  <si>
+    <t>Close Fast</t>
+  </si>
+  <si>
+    <t>Cerrar Rápido</t>
+  </si>
+  <si>
+    <t>DoNothing</t>
+  </si>
+  <si>
+    <t>Do Nothing</t>
+  </si>
+  <si>
+    <t>No hacer nada</t>
   </si>
 </sst>
 </file>
@@ -2360,7 +2384,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6961A5F-F8EA-4989-8112-A0ACE51D011E}">
   <sheetPr codeName="Hoja1"/>
-  <dimension ref="A1:D179"/>
+  <dimension ref="A1:D182"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="37" style="2" customWidth="1"/>
@@ -4809,6 +4833,39 @@
       </c>
       <c r="C179" s="2" t="s">
         <v>640</v>
+      </c>
+    </row>
+    <row r="180" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A180" s="2" t="s">
+        <v>641</v>
+      </c>
+      <c r="B180" s="2" t="s">
+        <v>641</v>
+      </c>
+      <c r="C180" s="2" t="s">
+        <v>642</v>
+      </c>
+    </row>
+    <row r="181" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A181" s="2" t="s">
+        <v>643</v>
+      </c>
+      <c r="B181" s="2" t="s">
+        <v>644</v>
+      </c>
+      <c r="C181" s="2" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="182" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A182" s="2" t="s">
+        <v>646</v>
+      </c>
+      <c r="B182" s="2" t="s">
+        <v>647</v>
+      </c>
+      <c r="C182" s="2" t="s">
+        <v>648</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added a property for breakable windows to decide if it should break with dodge or not.
</commit_message>
<xml_diff>
--- a/Translations/Translations.xlsx
+++ b/Translations/Translations.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programacion\MelonLoader\FS_LevelEditor\Translations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92AF2B07-4B17-4CC1-940B-45245397C336}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB786E76-A019-42D4-8F79-498282CA4782}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{F5C22481-FF1A-482C-BF7E-EB5A7718AF49}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1340" uniqueCount="649">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1343" uniqueCount="652">
   <si>
     <t>ID</t>
   </si>
@@ -1985,6 +1985,15 @@
   </si>
   <si>
     <t>No hacer nada</t>
+  </si>
+  <si>
+    <t>BreakWithDodge</t>
+  </si>
+  <si>
+    <t>Break With Dodge</t>
+  </si>
+  <si>
+    <t>Romper Al Evadir</t>
   </si>
 </sst>
 </file>
@@ -2384,7 +2393,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6961A5F-F8EA-4989-8112-A0ACE51D011E}">
   <sheetPr codeName="Hoja1"/>
-  <dimension ref="A1:D182"/>
+  <dimension ref="A1:D183"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="37" style="2" customWidth="1"/>
@@ -4866,6 +4875,17 @@
       </c>
       <c r="C182" s="2" t="s">
         <v>648</v>
+      </c>
+    </row>
+    <row r="183" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A183" s="2" t="s">
+        <v>649</v>
+      </c>
+      <c r="B183" s="2" t="s">
+        <v>650</v>
+      </c>
+      <c r="C183" s="2" t="s">
+        <v>651</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fixed the fucking keypads jaja.
</commit_message>
<xml_diff>
--- a/Translations/Translations.xlsx
+++ b/Translations/Translations.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programacion\MelonLoader\FS_LevelEditor\Translations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB786E76-A019-42D4-8F79-498282CA4782}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0A6E2F4-67F3-47B1-8A7C-2F63188C131C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{F5C22481-FF1A-482C-BF7E-EB5A7718AF49}"/>
+    <workbookView xWindow="8430" yWindow="1410" windowWidth="28800" windowHeight="15345" xr2:uid="{F5C22481-FF1A-482C-BF7E-EB5A7718AF49}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1343" uniqueCount="652">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1352" uniqueCount="660">
   <si>
     <t>ID</t>
   </si>
@@ -1994,6 +1994,30 @@
   </si>
   <si>
     <t>Romper Al Evadir</t>
+  </si>
+  <si>
+    <t>LeaveOnIncorrect</t>
+  </si>
+  <si>
+    <t>Leave On Incorrect</t>
+  </si>
+  <si>
+    <t>Salir Al Fallar</t>
+  </si>
+  <si>
+    <t>Alternative</t>
+  </si>
+  <si>
+    <t>Alternativo</t>
+  </si>
+  <si>
+    <t>AlternativeComb</t>
+  </si>
+  <si>
+    <t>Alternative Keycode</t>
+  </si>
+  <si>
+    <t>Código Alternativo</t>
   </si>
 </sst>
 </file>
@@ -2393,7 +2417,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6961A5F-F8EA-4989-8112-A0ACE51D011E}">
   <sheetPr codeName="Hoja1"/>
-  <dimension ref="A1:D183"/>
+  <dimension ref="A1:D186"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="37" style="2" customWidth="1"/>
@@ -4886,6 +4910,39 @@
       </c>
       <c r="C183" s="2" t="s">
         <v>651</v>
+      </c>
+    </row>
+    <row r="184" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A184" s="2" t="s">
+        <v>652</v>
+      </c>
+      <c r="B184" s="2" t="s">
+        <v>653</v>
+      </c>
+      <c r="C184" s="2" t="s">
+        <v>654</v>
+      </c>
+    </row>
+    <row r="185" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A185" s="2" t="s">
+        <v>655</v>
+      </c>
+      <c r="B185" s="2" t="s">
+        <v>655</v>
+      </c>
+      <c r="C185" s="2" t="s">
+        <v>656</v>
+      </c>
+    </row>
+    <row r="186" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A186" s="2" t="s">
+        <v>657</v>
+      </c>
+      <c r="B186" s="2" t="s">
+        <v>658</v>
+      </c>
+      <c r="C186" s="2" t="s">
+        <v>659</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
ADDED FIRST WORKING VERSION OF SEQUENCERS.
</commit_message>
<xml_diff>
--- a/Translations/Translations.xlsx
+++ b/Translations/Translations.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programacion\MelonLoader\FS_LevelEditor\Translations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0A6E2F4-67F3-47B1-8A7C-2F63188C131C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0347AFAC-FBB2-4652-82AA-1B30737B79F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8430" yWindow="1410" windowWidth="28800" windowHeight="15345" xr2:uid="{F5C22481-FF1A-482C-BF7E-EB5A7718AF49}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{F5C22481-FF1A-482C-BF7E-EB5A7718AF49}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1352" uniqueCount="660">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1361" uniqueCount="669">
   <si>
     <t>ID</t>
   </si>
@@ -2018,6 +2018,33 @@
   </si>
   <si>
     <t>Código Alternativo</t>
+  </si>
+  <si>
+    <t>object.SEQUENCE</t>
+  </si>
+  <si>
+    <t>Sequencer</t>
+  </si>
+  <si>
+    <t>Secuenciador</t>
+  </si>
+  <si>
+    <t>object.SEQUENCE_WAYPOINT</t>
+  </si>
+  <si>
+    <t>Sequencer Step</t>
+  </si>
+  <si>
+    <t>Etapa del Secuenciador</t>
+  </si>
+  <si>
+    <t>AddSequencerWaypoint</t>
+  </si>
+  <si>
+    <t>+ Add Sequencer Step</t>
+  </si>
+  <si>
+    <t>+ Añadir Etapa del Secuenciador</t>
   </si>
 </sst>
 </file>
@@ -2417,7 +2444,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6961A5F-F8EA-4989-8112-A0ACE51D011E}">
   <sheetPr codeName="Hoja1"/>
-  <dimension ref="A1:D186"/>
+  <dimension ref="A1:D189"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="37" style="2" customWidth="1"/>
@@ -3236,1713 +3263,1746 @@
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" s="2" t="s">
-        <v>69</v>
+        <v>660</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>69</v>
+        <v>661</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="D59" s="2" t="s">
-        <v>364</v>
+        <v>662</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
-        <v>443</v>
+        <v>663</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>443</v>
+        <v>664</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>601</v>
-      </c>
-      <c r="D60" s="2" t="s">
-        <v>552</v>
+        <v>665</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61" s="2" t="s">
-        <v>456</v>
+        <v>69</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>456</v>
+        <v>69</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>456</v>
+        <v>101</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>457</v>
+        <v>364</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" s="2" t="s">
-        <v>105</v>
+        <v>443</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>2</v>
+        <v>443</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>102</v>
+        <v>601</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>365</v>
+        <v>552</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63" s="2" t="s">
-        <v>106</v>
+        <v>456</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>3</v>
+        <v>456</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>103</v>
+        <v>456</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>366</v>
+        <v>457</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" s="2" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A65" s="2" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>111</v>
+        <v>3</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="D65" s="2" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66" s="2" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>112</v>
+        <v>4</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>113</v>
+        <v>104</v>
       </c>
       <c r="D66" s="2" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A67" s="2" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>116</v>
+        <v>109</v>
       </c>
       <c r="D67" s="2" t="s">
-        <v>368</v>
+        <v>365</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A68" s="2" t="s">
-        <v>117</v>
+        <v>110</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>119</v>
+        <v>112</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>120</v>
+        <v>113</v>
       </c>
       <c r="D68" s="2" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A69" s="2" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="D69" s="2" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A70" s="2" t="s">
-        <v>445</v>
+        <v>117</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>446</v>
+        <v>119</v>
       </c>
       <c r="C70" s="2" t="s">
-        <v>459</v>
+        <v>120</v>
       </c>
       <c r="D70" s="2" t="s">
-        <v>447</v>
+        <v>369</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A71" s="2" t="s">
-        <v>512</v>
+        <v>118</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>513</v>
+        <v>122</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>602</v>
+        <v>121</v>
       </c>
       <c r="D71" s="2" t="s">
-        <v>514</v>
+        <v>370</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A72" s="2" t="s">
-        <v>518</v>
+        <v>445</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>519</v>
+        <v>446</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>603</v>
+        <v>459</v>
       </c>
       <c r="D72" s="2" t="s">
-        <v>520</v>
+        <v>447</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A73" s="2" t="s">
-        <v>521</v>
+        <v>512</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>522</v>
+        <v>513</v>
       </c>
       <c r="C73" s="2" t="s">
-        <v>604</v>
+        <v>602</v>
       </c>
       <c r="D73" s="2" t="s">
-        <v>523</v>
+        <v>514</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A74" s="2" t="s">
-        <v>532</v>
+        <v>518</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>533</v>
+        <v>519</v>
       </c>
       <c r="C74" s="2" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="D74" s="2" t="s">
-        <v>534</v>
+        <v>520</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A75" s="2" t="s">
-        <v>537</v>
+        <v>521</v>
       </c>
       <c r="B75" s="2" t="s">
-        <v>535</v>
+        <v>522</v>
       </c>
       <c r="C75" s="2" t="s">
-        <v>606</v>
+        <v>604</v>
       </c>
       <c r="D75" s="2" t="s">
-        <v>536</v>
+        <v>523</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A76" s="2" t="s">
-        <v>154</v>
+        <v>532</v>
       </c>
       <c r="B76" s="2" t="s">
-        <v>155</v>
+        <v>533</v>
       </c>
       <c r="C76" s="2" t="s">
-        <v>156</v>
+        <v>605</v>
       </c>
       <c r="D76" s="2" t="s">
-        <v>371</v>
+        <v>534</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A77" s="2" t="s">
-        <v>164</v>
+        <v>537</v>
       </c>
       <c r="B77" s="2" t="s">
-        <v>165</v>
+        <v>535</v>
       </c>
       <c r="C77" s="2" t="s">
-        <v>166</v>
+        <v>606</v>
       </c>
       <c r="D77" s="2" t="s">
-        <v>372</v>
+        <v>536</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A78" s="2" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="B78" s="2" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="C78" s="2" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="D78" s="2" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A79" s="2" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="B79" s="2" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="C79" s="2" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="D79" s="2" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
-        <v>141</v>
+        <v>157</v>
       </c>
       <c r="B80" s="2" t="s">
-        <v>142</v>
+        <v>158</v>
       </c>
       <c r="C80" s="2" t="s">
-        <v>143</v>
+        <v>159</v>
       </c>
       <c r="D80" s="2" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="81" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A81" s="2" t="s">
-        <v>144</v>
+        <v>167</v>
       </c>
       <c r="B81" s="2" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="C81" s="2" t="s">
-        <v>145</v>
+        <v>169</v>
       </c>
       <c r="D81" s="2" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A82" s="2" t="s">
-        <v>153</v>
+        <v>141</v>
       </c>
       <c r="B82" s="2" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="C82" s="2" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="D82" s="2" t="s">
-        <v>328</v>
-      </c>
-    </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A83" s="2" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="B83" s="2" t="s">
-        <v>148</v>
+        <v>163</v>
       </c>
       <c r="C83" s="2" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="D83" s="2" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A84" s="2" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="B84" s="2" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="C84" s="2" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="D84" s="2" t="s">
-        <v>378</v>
+        <v>328</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A85" s="2" t="s">
-        <v>172</v>
+        <v>147</v>
       </c>
       <c r="B85" s="2" t="s">
-        <v>170</v>
+        <v>148</v>
       </c>
       <c r="C85" s="2" t="s">
-        <v>171</v>
+        <v>149</v>
       </c>
       <c r="D85" s="2" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A86" s="2" t="s">
-        <v>173</v>
+        <v>150</v>
       </c>
       <c r="B86" s="2" t="s">
-        <v>174</v>
+        <v>151</v>
       </c>
       <c r="C86" s="2" t="s">
-        <v>175</v>
+        <v>152</v>
       </c>
       <c r="D86" s="2" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A87" s="2" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="B87" s="2" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
       <c r="C87" s="2" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="D87" s="2" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A88" s="2" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
       <c r="B88" s="2" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="C88" s="2" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="D88" s="2" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A89" s="2" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="B89" s="2" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="C89" s="2" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="D89" s="2" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A90" s="2" t="s">
-        <v>243</v>
+        <v>178</v>
       </c>
       <c r="B90" s="2" t="s">
-        <v>243</v>
+        <v>178</v>
       </c>
       <c r="C90" s="2" t="s">
-        <v>95</v>
+        <v>179</v>
       </c>
       <c r="D90" s="2" t="s">
-        <v>384</v>
-      </c>
-    </row>
-    <row r="91" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A91" s="2" t="s">
-        <v>138</v>
-      </c>
-      <c r="B91" s="1" t="s">
-        <v>140</v>
+        <v>180</v>
+      </c>
+      <c r="B91" s="2" t="s">
+        <v>180</v>
       </c>
       <c r="C91" s="2" t="s">
-        <v>139</v>
+        <v>181</v>
       </c>
       <c r="D91" s="2" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A92" s="2" t="s">
-        <v>182</v>
+        <v>243</v>
       </c>
       <c r="B92" s="2" t="s">
-        <v>183</v>
+        <v>243</v>
       </c>
       <c r="C92" s="2" t="s">
-        <v>183</v>
+        <v>95</v>
       </c>
       <c r="D92" s="2" t="s">
-        <v>386</v>
-      </c>
-    </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.25">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="93" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A93" s="2" t="s">
-        <v>184</v>
-      </c>
-      <c r="B93" s="2" t="s">
-        <v>184</v>
+        <v>138</v>
+      </c>
+      <c r="B93" s="1" t="s">
+        <v>140</v>
       </c>
       <c r="C93" s="2" t="s">
-        <v>185</v>
+        <v>139</v>
       </c>
       <c r="D93" s="2" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A94" s="2" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="B94" s="2" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="C94" s="2" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="D94" s="2" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A95" s="2" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="B95" s="2" t="s">
-        <v>525</v>
+        <v>184</v>
       </c>
       <c r="C95" s="2" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="D95" s="2" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A96" s="2" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="B96" s="2" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="C96" s="2" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="D96" s="2" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A97" s="2" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="B97" s="2" t="s">
-        <v>193</v>
+        <v>525</v>
       </c>
       <c r="C97" s="2" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="D97" s="2" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A98" s="2" t="s">
-        <v>434</v>
-      </c>
-      <c r="B98" s="4" t="s">
-        <v>435</v>
-      </c>
-      <c r="C98" s="4" t="s">
-        <v>436</v>
-      </c>
-      <c r="D98" s="4" t="s">
-        <v>591</v>
+        <v>190</v>
+      </c>
+      <c r="B98" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="C98" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="D98" s="2" t="s">
+        <v>390</v>
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A99" s="2" t="s">
-        <v>437</v>
-      </c>
-      <c r="B99" s="4" t="s">
-        <v>438</v>
-      </c>
-      <c r="C99" s="4" t="s">
-        <v>439</v>
-      </c>
-      <c r="D99" s="4" t="s">
-        <v>592</v>
+        <v>192</v>
+      </c>
+      <c r="B99" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="C99" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="D99" s="2" t="s">
+        <v>391</v>
       </c>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A100" s="2" t="s">
-        <v>473</v>
+        <v>434</v>
       </c>
       <c r="B100" s="4" t="s">
-        <v>590</v>
+        <v>435</v>
       </c>
       <c r="C100" s="4" t="s">
-        <v>474</v>
+        <v>436</v>
       </c>
       <c r="D100" s="4" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A101" s="2" t="s">
-        <v>195</v>
-      </c>
-      <c r="B101" s="2" t="s">
-        <v>196</v>
-      </c>
-      <c r="C101" s="2" t="s">
-        <v>197</v>
-      </c>
-      <c r="D101" s="2" t="s">
-        <v>392</v>
+        <v>437</v>
+      </c>
+      <c r="B101" s="4" t="s">
+        <v>438</v>
+      </c>
+      <c r="C101" s="4" t="s">
+        <v>439</v>
+      </c>
+      <c r="D101" s="4" t="s">
+        <v>592</v>
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A102" s="2" t="s">
-        <v>198</v>
-      </c>
-      <c r="B102" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="C102" s="2" t="s">
-        <v>200</v>
-      </c>
-      <c r="D102" s="2" t="s">
-        <v>393</v>
+        <v>473</v>
+      </c>
+      <c r="B102" s="4" t="s">
+        <v>590</v>
+      </c>
+      <c r="C102" s="4" t="s">
+        <v>474</v>
+      </c>
+      <c r="D102" s="4" t="s">
+        <v>593</v>
       </c>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A103" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
       <c r="B103" s="2" t="s">
-        <v>201</v>
+        <v>196</v>
       </c>
       <c r="C103" s="2" t="s">
-        <v>202</v>
+        <v>197</v>
       </c>
       <c r="D103" s="2" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A104" s="2" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
       <c r="B104" s="2" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="C104" s="2" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="D104" s="2" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A105" s="2" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="B105" s="2" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="C105" s="2" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="D105" s="2" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A106" s="2" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="B106" s="2" t="s">
-        <v>207</v>
+        <v>203</v>
       </c>
       <c r="C106" s="2" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
       <c r="D106" s="2" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A107" s="2" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="B107" s="2" t="s">
-        <v>210</v>
+        <v>205</v>
       </c>
       <c r="C107" s="2" t="s">
-        <v>211</v>
+        <v>205</v>
       </c>
       <c r="D107" s="2" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A108" s="2" t="s">
-        <v>212</v>
+        <v>206</v>
       </c>
       <c r="B108" s="2" t="s">
-        <v>213</v>
+        <v>207</v>
       </c>
       <c r="C108" s="2" t="s">
-        <v>214</v>
+        <v>208</v>
       </c>
       <c r="D108" s="2" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A109" s="2" t="s">
-        <v>215</v>
+        <v>209</v>
       </c>
       <c r="B109" s="2" t="s">
-        <v>216</v>
+        <v>210</v>
       </c>
       <c r="C109" s="2" t="s">
-        <v>217</v>
+        <v>211</v>
       </c>
       <c r="D109" s="2" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A110" s="2" t="s">
-        <v>220</v>
+        <v>212</v>
       </c>
       <c r="B110" s="2" t="s">
-        <v>219</v>
+        <v>213</v>
       </c>
       <c r="C110" s="2" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
       <c r="D110" s="2" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A111" s="2" t="s">
-        <v>292</v>
+        <v>215</v>
       </c>
       <c r="B111" s="2" t="s">
-        <v>292</v>
+        <v>216</v>
       </c>
       <c r="C111" s="2" t="s">
-        <v>293</v>
+        <v>217</v>
       </c>
       <c r="D111" s="2" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A112" s="2" t="s">
-        <v>294</v>
+        <v>220</v>
       </c>
       <c r="B112" s="2" t="s">
-        <v>295</v>
+        <v>219</v>
       </c>
       <c r="C112" s="2" t="s">
-        <v>296</v>
+        <v>218</v>
       </c>
       <c r="D112" s="2" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A113" s="2" t="s">
-        <v>297</v>
+        <v>292</v>
       </c>
       <c r="B113" s="2" t="s">
-        <v>298</v>
+        <v>292</v>
       </c>
       <c r="C113" s="2" t="s">
-        <v>299</v>
+        <v>293</v>
       </c>
       <c r="D113" s="2" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A114" s="2" t="s">
-        <v>221</v>
+        <v>294</v>
       </c>
       <c r="B114" s="2" t="s">
-        <v>221</v>
+        <v>295</v>
       </c>
       <c r="C114" s="2" t="s">
-        <v>222</v>
+        <v>296</v>
       </c>
       <c r="D114" s="2" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A115" s="2" t="s">
-        <v>223</v>
+        <v>297</v>
       </c>
       <c r="B115" s="2" t="s">
-        <v>224</v>
+        <v>298</v>
       </c>
       <c r="C115" s="2" t="s">
-        <v>225</v>
+        <v>299</v>
       </c>
       <c r="D115" s="2" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A116" s="2" t="s">
-        <v>226</v>
+        <v>221</v>
       </c>
       <c r="B116" s="2" t="s">
-        <v>227</v>
+        <v>221</v>
       </c>
       <c r="C116" s="2" t="s">
-        <v>228</v>
+        <v>222</v>
       </c>
       <c r="D116" s="2" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A117" s="2" t="s">
-        <v>229</v>
+        <v>223</v>
       </c>
       <c r="B117" s="2" t="s">
-        <v>229</v>
+        <v>224</v>
       </c>
       <c r="C117" s="2" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="D117" s="2" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A118" s="2" t="s">
-        <v>230</v>
+        <v>226</v>
       </c>
       <c r="B118" s="2" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="C118" s="2" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="D118" s="2" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
     </row>
     <row r="119" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A119" s="2" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="B119" s="2" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="C119" s="2" t="s">
-        <v>233</v>
+        <v>229</v>
       </c>
       <c r="D119" s="2" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A120" s="2" t="s">
-        <v>234</v>
+        <v>230</v>
       </c>
       <c r="B120" s="2" t="s">
-        <v>235</v>
+        <v>230</v>
       </c>
       <c r="C120" s="2" t="s">
-        <v>236</v>
+        <v>231</v>
       </c>
       <c r="D120" s="2" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A121" s="2" t="s">
-        <v>237</v>
+        <v>232</v>
       </c>
       <c r="B121" s="2" t="s">
-        <v>238</v>
+        <v>232</v>
       </c>
       <c r="C121" s="2" t="s">
-        <v>239</v>
+        <v>233</v>
       </c>
       <c r="D121" s="2" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A122" s="2" t="s">
-        <v>300</v>
+        <v>234</v>
       </c>
       <c r="B122" s="2" t="s">
-        <v>301</v>
+        <v>235</v>
       </c>
       <c r="C122" s="2" t="s">
-        <v>302</v>
+        <v>236</v>
       </c>
       <c r="D122" s="2" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
     </row>
     <row r="123" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A123" s="2" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="B123" s="2" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="C123" s="2" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="D123" s="2" t="s">
-        <v>414</v>
+        <v>412</v>
       </c>
     </row>
     <row r="124" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A124" s="2" t="s">
-        <v>244</v>
+        <v>300</v>
       </c>
       <c r="B124" s="2" t="s">
-        <v>252</v>
+        <v>301</v>
       </c>
       <c r="C124" s="2" t="s">
-        <v>251</v>
+        <v>302</v>
       </c>
       <c r="D124" s="2" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
     </row>
     <row r="125" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A125" s="2" t="s">
-        <v>245</v>
+        <v>240</v>
       </c>
       <c r="B125" s="2" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="C125" s="2" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="D125" s="2" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
     </row>
     <row r="126" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A126" s="2" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="B126" s="2" t="s">
-        <v>247</v>
+        <v>252</v>
       </c>
       <c r="C126" s="2" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="D126" s="2" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
     </row>
     <row r="127" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A127" s="2" t="s">
-        <v>249</v>
+        <v>245</v>
       </c>
       <c r="B127" s="2" t="s">
-        <v>249</v>
+        <v>245</v>
       </c>
       <c r="C127" s="2" t="s">
-        <v>250</v>
+        <v>246</v>
       </c>
       <c r="D127" s="2" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
     </row>
     <row r="128" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A128" s="2" t="s">
-        <v>253</v>
+        <v>247</v>
       </c>
       <c r="B128" s="2" t="s">
-        <v>254</v>
+        <v>247</v>
       </c>
       <c r="C128" s="2" t="s">
-        <v>255</v>
+        <v>248</v>
       </c>
       <c r="D128" s="2" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
     </row>
     <row r="129" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A129" s="2" t="s">
-        <v>256</v>
+        <v>249</v>
       </c>
       <c r="B129" s="2" t="s">
-        <v>257</v>
+        <v>249</v>
       </c>
       <c r="C129" s="2" t="s">
-        <v>258</v>
+        <v>250</v>
       </c>
       <c r="D129" s="2" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
     </row>
     <row r="130" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A130" s="2" t="s">
-        <v>259</v>
+        <v>253</v>
       </c>
       <c r="B130" s="2" t="s">
-        <v>260</v>
+        <v>254</v>
       </c>
       <c r="C130" s="2" t="s">
-        <v>261</v>
+        <v>255</v>
       </c>
       <c r="D130" s="2" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
     </row>
     <row r="131" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A131" s="2" t="s">
-        <v>262</v>
+        <v>256</v>
       </c>
       <c r="B131" s="2" t="s">
-        <v>263</v>
+        <v>257</v>
       </c>
       <c r="C131" s="2" t="s">
-        <v>264</v>
+        <v>258</v>
       </c>
       <c r="D131" s="2" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
     </row>
     <row r="132" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A132" s="2" t="s">
-        <v>265</v>
+        <v>259</v>
       </c>
       <c r="B132" s="2" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="C132" s="2" t="s">
-        <v>265</v>
+        <v>261</v>
       </c>
       <c r="D132" s="2" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
     </row>
     <row r="133" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A133" s="2" t="s">
-        <v>266</v>
+        <v>262</v>
       </c>
       <c r="B133" s="2" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
       <c r="C133" s="2" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="D133" s="2" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
     </row>
     <row r="134" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A134" s="2" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="B134" s="2" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="C134" s="2" t="s">
-        <v>269</v>
+        <v>265</v>
       </c>
       <c r="D134" s="2" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
     </row>
     <row r="135" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A135" s="2" t="s">
-        <v>270</v>
+        <v>266</v>
       </c>
       <c r="B135" s="2" t="s">
-        <v>270</v>
+        <v>266</v>
       </c>
       <c r="C135" s="2" t="s">
-        <v>273</v>
+        <v>267</v>
       </c>
       <c r="D135" s="2" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
     </row>
     <row r="136" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A136" s="2" t="s">
+        <v>268</v>
+      </c>
+      <c r="B136" s="2" t="s">
+        <v>268</v>
+      </c>
+      <c r="C136" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="D136" s="2" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="137" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A137" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="B137" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="C137" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="D137" s="2" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="138" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A138" s="2" t="s">
         <v>271</v>
       </c>
-      <c r="B136" s="2" t="s">
+      <c r="B138" s="2" t="s">
         <v>271</v>
       </c>
-      <c r="C136" s="2" t="s">
+      <c r="C138" s="2" t="s">
         <v>272</v>
       </c>
-      <c r="D136" s="2" t="s">
+      <c r="D138" s="2" t="s">
         <v>427</v>
       </c>
     </row>
-    <row r="137" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A137" s="2" t="s">
+    <row r="139" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A139" s="2" t="s">
         <v>274</v>
       </c>
-      <c r="B137" s="2" t="s">
+      <c r="B139" s="2" t="s">
         <v>276</v>
       </c>
-      <c r="C137" s="2" t="s">
+      <c r="C139" s="2" t="s">
         <v>279</v>
       </c>
     </row>
-    <row r="138" spans="1:4" ht="45" x14ac:dyDescent="0.25">
-      <c r="A138" s="2" t="s">
+    <row r="140" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="A140" s="2" t="s">
         <v>275</v>
       </c>
-      <c r="B138" s="2" t="s">
+      <c r="B140" s="2" t="s">
         <v>277</v>
       </c>
-      <c r="C138" s="2" t="s">
+      <c r="C140" s="2" t="s">
         <v>278</v>
       </c>
     </row>
-    <row r="139" spans="1:4" ht="75" x14ac:dyDescent="0.25">
-      <c r="A139" s="2" t="s">
+    <row r="141" spans="1:4" ht="75" x14ac:dyDescent="0.25">
+      <c r="A141" s="2" t="s">
         <v>289</v>
       </c>
-      <c r="B139" s="2" t="s">
+      <c r="B141" s="2" t="s">
         <v>290</v>
       </c>
-      <c r="C139" s="2" t="s">
+      <c r="C141" s="2" t="s">
         <v>291</v>
-      </c>
-    </row>
-    <row r="140" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A140" s="2" t="s">
-        <v>306</v>
-      </c>
-      <c r="B140" s="2" t="s">
-        <v>307</v>
-      </c>
-      <c r="C140" s="2" t="s">
-        <v>308</v>
-      </c>
-      <c r="D140" s="2" t="s">
-        <v>428</v>
-      </c>
-    </row>
-    <row r="141" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A141" s="2" t="s">
-        <v>309</v>
-      </c>
-      <c r="B141" s="2" t="s">
-        <v>311</v>
-      </c>
-      <c r="C141" s="2" t="s">
-        <v>312</v>
-      </c>
-      <c r="D141" s="2" t="s">
-        <v>429</v>
       </c>
     </row>
     <row r="142" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A142" s="2" t="s">
-        <v>310</v>
+        <v>306</v>
       </c>
       <c r="B142" s="2" t="s">
-        <v>314</v>
+        <v>307</v>
       </c>
       <c r="C142" s="2" t="s">
-        <v>313</v>
+        <v>308</v>
       </c>
       <c r="D142" s="2" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
     </row>
     <row r="143" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A143" s="2" t="s">
-        <v>315</v>
+        <v>309</v>
       </c>
       <c r="B143" s="2" t="s">
-        <v>315</v>
+        <v>311</v>
       </c>
       <c r="C143" s="2" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="D143" s="2" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
     </row>
     <row r="144" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A144" s="2" t="s">
-        <v>317</v>
+        <v>310</v>
       </c>
       <c r="B144" s="2" t="s">
-        <v>318</v>
+        <v>314</v>
       </c>
       <c r="C144" s="2" t="s">
-        <v>460</v>
+        <v>313</v>
       </c>
       <c r="D144" s="2" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
     </row>
     <row r="145" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A145" s="2" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="B145" s="2" t="s">
-        <v>320</v>
+        <v>315</v>
       </c>
       <c r="C145" s="2" t="s">
-        <v>461</v>
+        <v>316</v>
       </c>
       <c r="D145" s="2" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
     </row>
     <row r="146" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A146" s="2" t="s">
-        <v>448</v>
+        <v>317</v>
       </c>
       <c r="B146" s="2" t="s">
-        <v>448</v>
+        <v>318</v>
       </c>
       <c r="C146" s="2" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
       <c r="D146" s="2" t="s">
-        <v>345</v>
+        <v>432</v>
       </c>
     </row>
     <row r="147" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A147" s="2" t="s">
-        <v>449</v>
+        <v>319</v>
       </c>
       <c r="B147" s="2" t="s">
-        <v>450</v>
+        <v>320</v>
       </c>
       <c r="C147" s="2" t="s">
-        <v>463</v>
+        <v>461</v>
       </c>
       <c r="D147" s="2" t="s">
-        <v>451</v>
+        <v>433</v>
       </c>
     </row>
     <row r="148" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A148" s="2" t="s">
-        <v>475</v>
+        <v>448</v>
       </c>
       <c r="B148" s="2" t="s">
-        <v>476</v>
+        <v>448</v>
       </c>
       <c r="C148" s="2" t="s">
-        <v>619</v>
+        <v>462</v>
       </c>
       <c r="D148" s="2" t="s">
-        <v>569</v>
+        <v>345</v>
       </c>
     </row>
     <row r="149" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A149" s="2" t="s">
-        <v>478</v>
+        <v>449</v>
       </c>
       <c r="B149" s="2" t="s">
-        <v>524</v>
+        <v>450</v>
       </c>
       <c r="C149" s="2" t="s">
-        <v>479</v>
+        <v>463</v>
       </c>
       <c r="D149" s="2" t="s">
-        <v>568</v>
+        <v>451</v>
       </c>
     </row>
     <row r="150" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A150" s="2" t="s">
-        <v>480</v>
+        <v>475</v>
       </c>
       <c r="B150" s="2" t="s">
-        <v>481</v>
+        <v>476</v>
       </c>
       <c r="C150" s="2" t="s">
-        <v>482</v>
+        <v>619</v>
       </c>
       <c r="D150" s="2" t="s">
-        <v>567</v>
+        <v>569</v>
       </c>
     </row>
     <row r="151" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A151" s="2" t="s">
-        <v>483</v>
+        <v>478</v>
       </c>
       <c r="B151" s="2" t="s">
-        <v>484</v>
+        <v>524</v>
       </c>
       <c r="C151" s="2" t="s">
-        <v>485</v>
+        <v>479</v>
       </c>
       <c r="D151" s="2" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
     </row>
     <row r="152" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A152" s="2" t="s">
-        <v>486</v>
+        <v>480</v>
       </c>
       <c r="B152" s="2" t="s">
-        <v>487</v>
+        <v>481</v>
       </c>
       <c r="C152" s="2" t="s">
-        <v>488</v>
+        <v>482</v>
       </c>
       <c r="D152" s="2" t="s">
-        <v>565</v>
+        <v>567</v>
       </c>
     </row>
     <row r="153" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A153" s="2" t="s">
-        <v>489</v>
+        <v>483</v>
       </c>
       <c r="B153" s="2" t="s">
-        <v>490</v>
+        <v>484</v>
       </c>
       <c r="C153" s="2" t="s">
-        <v>491</v>
+        <v>485</v>
       </c>
       <c r="D153" s="2" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
     </row>
     <row r="154" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A154" s="2" t="s">
-        <v>538</v>
+        <v>486</v>
       </c>
       <c r="B154" s="2" t="s">
-        <v>538</v>
+        <v>487</v>
       </c>
       <c r="C154" s="2" t="s">
-        <v>607</v>
+        <v>488</v>
       </c>
       <c r="D154" s="2" t="s">
-        <v>539</v>
+        <v>565</v>
       </c>
     </row>
     <row r="155" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A155" s="2" t="s">
-        <v>540</v>
+        <v>489</v>
       </c>
       <c r="B155" s="2" t="s">
-        <v>541</v>
+        <v>490</v>
       </c>
       <c r="C155" s="2" t="s">
-        <v>608</v>
+        <v>491</v>
       </c>
       <c r="D155" s="2" t="s">
-        <v>542</v>
+        <v>564</v>
       </c>
     </row>
     <row r="156" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A156" s="2" t="s">
-        <v>492</v>
+        <v>538</v>
       </c>
       <c r="B156" s="2" t="s">
-        <v>493</v>
+        <v>538</v>
       </c>
       <c r="C156" s="2" t="s">
-        <v>494</v>
+        <v>607</v>
       </c>
       <c r="D156" s="2" t="s">
-        <v>563</v>
+        <v>539</v>
       </c>
     </row>
     <row r="157" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A157" s="2" t="s">
-        <v>495</v>
+        <v>540</v>
       </c>
       <c r="B157" s="2" t="s">
-        <v>496</v>
+        <v>541</v>
       </c>
       <c r="C157" s="2" t="s">
-        <v>497</v>
+        <v>608</v>
       </c>
       <c r="D157" s="2" t="s">
-        <v>562</v>
+        <v>542</v>
       </c>
     </row>
     <row r="158" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A158" s="2" t="s">
-        <v>498</v>
+        <v>492</v>
       </c>
       <c r="B158" s="2" t="s">
-        <v>499</v>
+        <v>493</v>
       </c>
       <c r="C158" s="2" t="s">
-        <v>500</v>
+        <v>494</v>
       </c>
       <c r="D158" s="2" t="s">
-        <v>561</v>
+        <v>563</v>
       </c>
     </row>
     <row r="159" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A159" s="2" t="s">
-        <v>501</v>
+        <v>495</v>
       </c>
       <c r="B159" s="2" t="s">
-        <v>501</v>
+        <v>496</v>
       </c>
       <c r="C159" s="2" t="s">
-        <v>502</v>
+        <v>497</v>
       </c>
       <c r="D159" s="2" t="s">
-        <v>560</v>
+        <v>562</v>
       </c>
     </row>
     <row r="160" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A160" s="2" t="s">
-        <v>503</v>
+        <v>498</v>
       </c>
       <c r="B160" s="2" t="s">
-        <v>503</v>
+        <v>499</v>
       </c>
       <c r="C160" s="2" t="s">
-        <v>504</v>
+        <v>500</v>
       </c>
       <c r="D160" s="2" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
     </row>
     <row r="161" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A161" s="2" t="s">
-        <v>505</v>
+        <v>501</v>
       </c>
       <c r="B161" s="2" t="s">
-        <v>505</v>
+        <v>501</v>
       </c>
       <c r="C161" s="2" t="s">
-        <v>506</v>
+        <v>502</v>
       </c>
       <c r="D161" s="2" t="s">
-        <v>558</v>
+        <v>560</v>
       </c>
     </row>
     <row r="162" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A162" s="2" t="s">
-        <v>507</v>
+        <v>503</v>
       </c>
       <c r="B162" s="2" t="s">
-        <v>507</v>
+        <v>503</v>
       </c>
       <c r="C162" s="2" t="s">
-        <v>508</v>
+        <v>504</v>
       </c>
       <c r="D162" s="2" t="s">
-        <v>557</v>
+        <v>559</v>
       </c>
     </row>
     <row r="163" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A163" s="2" t="s">
-        <v>570</v>
+        <v>505</v>
       </c>
       <c r="B163" s="2" t="s">
-        <v>571</v>
+        <v>505</v>
       </c>
       <c r="C163" s="2" t="s">
-        <v>609</v>
+        <v>506</v>
+      </c>
+      <c r="D163" s="2" t="s">
+        <v>558</v>
       </c>
     </row>
     <row r="164" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A164" s="2" t="s">
-        <v>572</v>
+        <v>507</v>
       </c>
       <c r="B164" s="2" t="s">
-        <v>573</v>
+        <v>507</v>
       </c>
       <c r="C164" s="2" t="s">
-        <v>610</v>
+        <v>508</v>
+      </c>
+      <c r="D164" s="2" t="s">
+        <v>557</v>
       </c>
     </row>
     <row r="165" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A165" s="2" t="s">
-        <v>574</v>
+        <v>570</v>
       </c>
       <c r="B165" s="2" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C165" s="2" t="s">
-        <v>611</v>
+        <v>609</v>
       </c>
     </row>
     <row r="166" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A166" s="2" t="s">
-        <v>576</v>
+        <v>572</v>
       </c>
       <c r="B166" s="2" t="s">
-        <v>577</v>
+        <v>573</v>
       </c>
       <c r="C166" s="2" t="s">
-        <v>612</v>
+        <v>610</v>
       </c>
     </row>
     <row r="167" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A167" s="2" t="s">
-        <v>578</v>
+        <v>574</v>
       </c>
       <c r="B167" s="2" t="s">
-        <v>579</v>
+        <v>575</v>
       </c>
       <c r="C167" s="2" t="s">
-        <v>613</v>
+        <v>611</v>
       </c>
     </row>
     <row r="168" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A168" s="2" t="s">
-        <v>580</v>
+        <v>576</v>
       </c>
       <c r="B168" s="2" t="s">
-        <v>581</v>
+        <v>577</v>
       </c>
       <c r="C168" s="2" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
     </row>
     <row r="169" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A169" s="2" t="s">
-        <v>582</v>
+        <v>578</v>
       </c>
       <c r="B169" s="2" t="s">
-        <v>583</v>
+        <v>579</v>
       </c>
       <c r="C169" s="2" t="s">
-        <v>615</v>
+        <v>613</v>
       </c>
     </row>
     <row r="170" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A170" s="2" t="s">
-        <v>584</v>
+        <v>580</v>
       </c>
       <c r="B170" s="2" t="s">
-        <v>585</v>
+        <v>581</v>
       </c>
       <c r="C170" s="2" t="s">
-        <v>616</v>
+        <v>614</v>
       </c>
     </row>
     <row r="171" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A171" s="2" t="s">
-        <v>586</v>
+        <v>582</v>
       </c>
       <c r="B171" s="2" t="s">
-        <v>587</v>
+        <v>583</v>
       </c>
       <c r="C171" s="2" t="s">
-        <v>617</v>
+        <v>615</v>
       </c>
     </row>
     <row r="172" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A172" s="2" t="s">
-        <v>588</v>
+        <v>584</v>
       </c>
       <c r="B172" s="2" t="s">
-        <v>589</v>
+        <v>585</v>
       </c>
       <c r="C172" s="2" t="s">
-        <v>618</v>
+        <v>616</v>
       </c>
     </row>
     <row r="173" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A173" s="2" t="s">
-        <v>620</v>
+        <v>586</v>
       </c>
       <c r="B173" s="2" t="s">
-        <v>621</v>
+        <v>587</v>
       </c>
       <c r="C173" s="2" t="s">
-        <v>622</v>
+        <v>617</v>
       </c>
     </row>
     <row r="174" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A174" s="2" t="s">
-        <v>623</v>
+        <v>588</v>
       </c>
       <c r="B174" s="2" t="s">
-        <v>623</v>
+        <v>589</v>
       </c>
       <c r="C174" s="2" t="s">
-        <v>624</v>
+        <v>618</v>
       </c>
     </row>
     <row r="175" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A175" s="2" t="s">
-        <v>625</v>
+        <v>620</v>
       </c>
       <c r="B175" s="2" t="s">
-        <v>625</v>
+        <v>621</v>
       </c>
       <c r="C175" s="2" t="s">
-        <v>627</v>
+        <v>622</v>
       </c>
     </row>
     <row r="176" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A176" s="2" t="s">
-        <v>626</v>
+        <v>623</v>
       </c>
       <c r="B176" s="2" t="s">
-        <v>626</v>
+        <v>623</v>
       </c>
       <c r="C176" s="2" t="s">
-        <v>628</v>
+        <v>624</v>
       </c>
     </row>
     <row r="177" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A177" s="2" t="s">
-        <v>629</v>
+        <v>625</v>
       </c>
       <c r="B177" s="2" t="s">
-        <v>630</v>
+        <v>625</v>
       </c>
       <c r="C177" s="2" t="s">
-        <v>631</v>
+        <v>627</v>
       </c>
     </row>
     <row r="178" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A178" s="2" t="s">
-        <v>632</v>
-      </c>
-      <c r="B178" s="4" t="s">
-        <v>633</v>
-      </c>
-      <c r="C178" s="4" t="s">
-        <v>634</v>
+        <v>626</v>
+      </c>
+      <c r="B178" s="2" t="s">
+        <v>626</v>
+      </c>
+      <c r="C178" s="2" t="s">
+        <v>628</v>
       </c>
     </row>
     <row r="179" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A179" s="2" t="s">
-        <v>638</v>
+        <v>629</v>
       </c>
       <c r="B179" s="2" t="s">
-        <v>639</v>
+        <v>630</v>
       </c>
       <c r="C179" s="2" t="s">
-        <v>640</v>
+        <v>631</v>
       </c>
     </row>
     <row r="180" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A180" s="2" t="s">
-        <v>641</v>
-      </c>
-      <c r="B180" s="2" t="s">
-        <v>641</v>
-      </c>
-      <c r="C180" s="2" t="s">
-        <v>642</v>
+        <v>632</v>
+      </c>
+      <c r="B180" s="4" t="s">
+        <v>633</v>
+      </c>
+      <c r="C180" s="4" t="s">
+        <v>634</v>
       </c>
     </row>
     <row r="181" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A181" s="2" t="s">
-        <v>643</v>
+        <v>638</v>
       </c>
       <c r="B181" s="2" t="s">
-        <v>644</v>
+        <v>639</v>
       </c>
       <c r="C181" s="2" t="s">
-        <v>645</v>
+        <v>640</v>
       </c>
     </row>
     <row r="182" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A182" s="2" t="s">
-        <v>646</v>
+        <v>641</v>
       </c>
       <c r="B182" s="2" t="s">
-        <v>647</v>
+        <v>641</v>
       </c>
       <c r="C182" s="2" t="s">
-        <v>648</v>
+        <v>642</v>
       </c>
     </row>
     <row r="183" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A183" s="2" t="s">
-        <v>649</v>
+        <v>643</v>
       </c>
       <c r="B183" s="2" t="s">
-        <v>650</v>
+        <v>644</v>
       </c>
       <c r="C183" s="2" t="s">
-        <v>651</v>
+        <v>645</v>
       </c>
     </row>
     <row r="184" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A184" s="2" t="s">
-        <v>652</v>
+        <v>646</v>
       </c>
       <c r="B184" s="2" t="s">
-        <v>653</v>
+        <v>647</v>
       </c>
       <c r="C184" s="2" t="s">
-        <v>654</v>
+        <v>648</v>
       </c>
     </row>
     <row r="185" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A185" s="2" t="s">
-        <v>655</v>
+        <v>649</v>
       </c>
       <c r="B185" s="2" t="s">
-        <v>655</v>
+        <v>650</v>
       </c>
       <c r="C185" s="2" t="s">
-        <v>656</v>
+        <v>651</v>
       </c>
     </row>
     <row r="186" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A186" s="2" t="s">
+        <v>652</v>
+      </c>
+      <c r="B186" s="2" t="s">
+        <v>653</v>
+      </c>
+      <c r="C186" s="2" t="s">
+        <v>654</v>
+      </c>
+    </row>
+    <row r="187" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A187" s="2" t="s">
+        <v>655</v>
+      </c>
+      <c r="B187" s="2" t="s">
+        <v>655</v>
+      </c>
+      <c r="C187" s="2" t="s">
+        <v>656</v>
+      </c>
+    </row>
+    <row r="188" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A188" s="2" t="s">
         <v>657</v>
       </c>
-      <c r="B186" s="2" t="s">
+      <c r="B188" s="2" t="s">
         <v>658</v>
       </c>
-      <c r="C186" s="2" t="s">
+      <c r="C188" s="2" t="s">
         <v>659</v>
+      </c>
+    </row>
+    <row r="189" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A189" s="2" t="s">
+        <v>666</v>
+      </c>
+      <c r="B189" s="4" t="s">
+        <v>667</v>
+      </c>
+      <c r="C189" s="4" t="s">
+        <v>668</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Sequencer Screen props translations.
</commit_message>
<xml_diff>
--- a/Translations/Translations.xlsx
+++ b/Translations/Translations.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programacion\MelonLoader\FS_LevelEditor\Translations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDC413F5-AC47-4D87-B9ED-808FEB158956}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{672CC127-6C57-4707-8ED0-AFF4E2583862}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{F5C22481-FF1A-482C-BF7E-EB5A7718AF49}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1364" uniqueCount="672">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1373" uniqueCount="681">
   <si>
     <t>ID</t>
   </si>
@@ -2054,6 +2054,33 @@
   </si>
   <si>
     <t>Al Completar</t>
+  </si>
+  <si>
+    <t>object.SEQUENCE_SCREEN</t>
+  </si>
+  <si>
+    <t>Sequence Screen</t>
+  </si>
+  <si>
+    <t>Pantalla del Secuenciador</t>
+  </si>
+  <si>
+    <t>SequencerID</t>
+  </si>
+  <si>
+    <t>Sequencer ID</t>
+  </si>
+  <si>
+    <t>ID del Secuenciador</t>
+  </si>
+  <si>
+    <t>InvertDisplayOrder</t>
+  </si>
+  <si>
+    <t>Invert Display Order</t>
+  </si>
+  <si>
+    <t>Invertir Orden</t>
   </si>
 </sst>
 </file>
@@ -2453,7 +2480,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6961A5F-F8EA-4989-8112-A0ACE51D011E}">
   <sheetPr codeName="Hoja1"/>
-  <dimension ref="A1:D190"/>
+  <dimension ref="A1:D193"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="37" style="2" customWidth="1"/>
@@ -3294,1735 +3321,1768 @@
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61" s="2" t="s">
-        <v>69</v>
+        <v>672</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>69</v>
+        <v>673</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="D61" s="2" t="s">
-        <v>364</v>
+        <v>674</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" s="2" t="s">
-        <v>443</v>
+        <v>69</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>443</v>
+        <v>69</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>601</v>
+        <v>101</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>552</v>
+        <v>364</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63" s="2" t="s">
-        <v>456</v>
+        <v>443</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>456</v>
+        <v>443</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>456</v>
+        <v>601</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>457</v>
+        <v>552</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" s="2" t="s">
-        <v>105</v>
+        <v>456</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>2</v>
+        <v>456</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>102</v>
+        <v>456</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>365</v>
+        <v>457</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A65" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D65" s="2" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D66" s="2" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A67" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>111</v>
+        <v>4</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="D67" s="2" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A68" s="2" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="D68" s="2" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A69" s="2" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="D69" s="2" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A70" s="2" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="C70" s="2" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="D70" s="2" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A71" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D71" s="2" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A72" s="2" t="s">
-        <v>445</v>
+        <v>118</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>446</v>
+        <v>122</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>459</v>
+        <v>121</v>
       </c>
       <c r="D72" s="2" t="s">
-        <v>447</v>
+        <v>370</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A73" s="2" t="s">
-        <v>512</v>
+        <v>445</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>513</v>
+        <v>446</v>
       </c>
       <c r="C73" s="2" t="s">
-        <v>602</v>
+        <v>459</v>
       </c>
       <c r="D73" s="2" t="s">
-        <v>514</v>
+        <v>447</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A74" s="2" t="s">
-        <v>518</v>
+        <v>512</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>519</v>
+        <v>513</v>
       </c>
       <c r="C74" s="2" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="D74" s="2" t="s">
-        <v>520</v>
+        <v>514</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A75" s="2" t="s">
-        <v>521</v>
+        <v>518</v>
       </c>
       <c r="B75" s="2" t="s">
-        <v>522</v>
+        <v>519</v>
       </c>
       <c r="C75" s="2" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="D75" s="2" t="s">
-        <v>523</v>
+        <v>520</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A76" s="2" t="s">
-        <v>532</v>
+        <v>521</v>
       </c>
       <c r="B76" s="2" t="s">
-        <v>533</v>
+        <v>522</v>
       </c>
       <c r="C76" s="2" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="D76" s="2" t="s">
-        <v>534</v>
+        <v>523</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A77" s="2" t="s">
-        <v>537</v>
+        <v>532</v>
       </c>
       <c r="B77" s="2" t="s">
-        <v>535</v>
+        <v>533</v>
       </c>
       <c r="C77" s="2" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="D77" s="2" t="s">
-        <v>536</v>
+        <v>534</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A78" s="2" t="s">
-        <v>154</v>
+        <v>537</v>
       </c>
       <c r="B78" s="2" t="s">
-        <v>155</v>
+        <v>535</v>
       </c>
       <c r="C78" s="2" t="s">
-        <v>156</v>
+        <v>606</v>
       </c>
       <c r="D78" s="2" t="s">
-        <v>371</v>
+        <v>536</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A79" s="2" t="s">
-        <v>164</v>
+        <v>154</v>
       </c>
       <c r="B79" s="2" t="s">
-        <v>165</v>
+        <v>155</v>
       </c>
       <c r="C79" s="2" t="s">
-        <v>166</v>
+        <v>156</v>
       </c>
       <c r="D79" s="2" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
-        <v>157</v>
+        <v>164</v>
       </c>
       <c r="B80" s="2" t="s">
-        <v>158</v>
+        <v>165</v>
       </c>
       <c r="C80" s="2" t="s">
-        <v>159</v>
+        <v>166</v>
       </c>
       <c r="D80" s="2" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A81" s="2" t="s">
-        <v>167</v>
+        <v>157</v>
       </c>
       <c r="B81" s="2" t="s">
-        <v>168</v>
+        <v>158</v>
       </c>
       <c r="C81" s="2" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="D81" s="2" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A82" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="B82" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="C82" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="D82" s="2" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A83" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="B82" s="2" t="s">
+      <c r="B83" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="C82" s="2" t="s">
+      <c r="C83" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="D82" s="2" t="s">
+      <c r="D83" s="2" t="s">
         <v>375</v>
       </c>
     </row>
-    <row r="83" spans="1:4" ht="45" x14ac:dyDescent="0.25">
-      <c r="A83" s="2" t="s">
+    <row r="84" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="A84" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="B83" s="2" t="s">
+      <c r="B84" s="2" t="s">
         <v>163</v>
       </c>
-      <c r="C83" s="2" t="s">
+      <c r="C84" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="D83" s="2" t="s">
+      <c r="D84" s="2" t="s">
         <v>376</v>
-      </c>
-    </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A84" s="2" t="s">
-        <v>153</v>
-      </c>
-      <c r="B84" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="C84" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="D84" s="2" t="s">
-        <v>328</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A85" s="2" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="B85" s="2" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="C85" s="2" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="D85" s="2" t="s">
-        <v>377</v>
+        <v>328</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A86" s="2" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="B86" s="2" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="C86" s="2" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="D86" s="2" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A87" s="2" t="s">
-        <v>172</v>
+        <v>150</v>
       </c>
       <c r="B87" s="2" t="s">
-        <v>170</v>
+        <v>151</v>
       </c>
       <c r="C87" s="2" t="s">
-        <v>171</v>
+        <v>152</v>
       </c>
       <c r="D87" s="2" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A88" s="2" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B88" s="2" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="C88" s="2" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="D88" s="2" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A89" s="2" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="B89" s="2" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="C89" s="2" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="D89" s="2" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A90" s="2" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="B90" s="2" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="C90" s="2" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="D90" s="2" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A91" s="2" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="B91" s="2" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="C91" s="2" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="D91" s="2" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A92" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="B92" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="C92" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="D92" s="2" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="93" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A93" s="2" t="s">
         <v>243</v>
       </c>
-      <c r="B92" s="2" t="s">
+      <c r="B93" s="2" t="s">
         <v>243</v>
       </c>
-      <c r="C92" s="2" t="s">
+      <c r="C93" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="D92" s="2" t="s">
+      <c r="D93" s="2" t="s">
         <v>384</v>
       </c>
     </row>
-    <row r="93" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A93" s="2" t="s">
+    <row r="94" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A94" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="B93" s="1" t="s">
+      <c r="B94" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="C93" s="2" t="s">
+      <c r="C94" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="D93" s="2" t="s">
+      <c r="D94" s="2" t="s">
         <v>385</v>
-      </c>
-    </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A94" s="2" t="s">
-        <v>182</v>
-      </c>
-      <c r="B94" s="2" t="s">
-        <v>183</v>
-      </c>
-      <c r="C94" s="2" t="s">
-        <v>183</v>
-      </c>
-      <c r="D94" s="2" t="s">
-        <v>386</v>
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A95" s="2" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="B95" s="2" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C95" s="2" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="D95" s="2" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A96" s="2" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="B96" s="2" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="C96" s="2" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="D96" s="2" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A97" s="2" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="B97" s="2" t="s">
-        <v>525</v>
+        <v>186</v>
       </c>
       <c r="C97" s="2" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="D97" s="2" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A98" s="2" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="B98" s="2" t="s">
-        <v>190</v>
+        <v>525</v>
       </c>
       <c r="C98" s="2" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="D98" s="2" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A99" s="2" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="B99" s="2" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="C99" s="2" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="D99" s="2" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A100" s="2" t="s">
-        <v>434</v>
-      </c>
-      <c r="B100" s="4" t="s">
-        <v>435</v>
-      </c>
-      <c r="C100" s="4" t="s">
-        <v>436</v>
-      </c>
-      <c r="D100" s="4" t="s">
-        <v>591</v>
+        <v>192</v>
+      </c>
+      <c r="B100" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="C100" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="D100" s="2" t="s">
+        <v>391</v>
       </c>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A101" s="2" t="s">
-        <v>437</v>
+        <v>434</v>
       </c>
       <c r="B101" s="4" t="s">
-        <v>438</v>
+        <v>435</v>
       </c>
       <c r="C101" s="4" t="s">
-        <v>439</v>
+        <v>436</v>
       </c>
       <c r="D101" s="4" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A102" s="2" t="s">
-        <v>473</v>
+        <v>437</v>
       </c>
       <c r="B102" s="4" t="s">
-        <v>590</v>
+        <v>438</v>
       </c>
       <c r="C102" s="4" t="s">
-        <v>474</v>
+        <v>439</v>
       </c>
       <c r="D102" s="4" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A103" s="2" t="s">
-        <v>195</v>
-      </c>
-      <c r="B103" s="2" t="s">
-        <v>196</v>
-      </c>
-      <c r="C103" s="2" t="s">
-        <v>197</v>
-      </c>
-      <c r="D103" s="2" t="s">
-        <v>392</v>
+        <v>473</v>
+      </c>
+      <c r="B103" s="4" t="s">
+        <v>590</v>
+      </c>
+      <c r="C103" s="4" t="s">
+        <v>474</v>
+      </c>
+      <c r="D103" s="4" t="s">
+        <v>593</v>
       </c>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A104" s="2" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="B104" s="2" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="C104" s="2" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="D104" s="2" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A105" s="2" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="B105" s="2" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="C105" s="2" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="D105" s="2" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A106" s="2" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="B106" s="2" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="C106" s="2" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="D106" s="2" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A107" s="2" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="B107" s="2" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="C107" s="2" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="D107" s="2" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A108" s="2" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B108" s="2" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="C108" s="2" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="D108" s="2" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A109" s="2" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="B109" s="2" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="C109" s="2" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="D109" s="2" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A110" s="2" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="B110" s="2" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="C110" s="2" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="D110" s="2" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A111" s="2" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="B111" s="2" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="C111" s="2" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="D111" s="2" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A112" s="2" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="B112" s="2" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="C112" s="2" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="D112" s="2" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A113" s="2" t="s">
-        <v>292</v>
+        <v>220</v>
       </c>
       <c r="B113" s="2" t="s">
-        <v>292</v>
+        <v>219</v>
       </c>
       <c r="C113" s="2" t="s">
-        <v>293</v>
+        <v>218</v>
       </c>
       <c r="D113" s="2" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A114" s="2" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="B114" s="2" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="C114" s="2" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
       <c r="D114" s="2" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A115" s="2" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
       <c r="B115" s="2" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="C115" s="2" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="D115" s="2" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A116" s="2" t="s">
-        <v>221</v>
+        <v>297</v>
       </c>
       <c r="B116" s="2" t="s">
-        <v>221</v>
+        <v>298</v>
       </c>
       <c r="C116" s="2" t="s">
-        <v>222</v>
+        <v>299</v>
       </c>
       <c r="D116" s="2" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A117" s="2" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="B117" s="2" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="C117" s="2" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="D117" s="2" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A118" s="2" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="B118" s="2" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="C118" s="2" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="D118" s="2" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
     </row>
     <row r="119" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A119" s="2" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="B119" s="2" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="C119" s="2" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="D119" s="2" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A120" s="2" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B120" s="2" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="C120" s="2" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="D120" s="2" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A121" s="2" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="B121" s="2" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="C121" s="2" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="D121" s="2" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A122" s="2" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="B122" s="2" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="C122" s="2" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="D122" s="2" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
     </row>
     <row r="123" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A123" s="2" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="B123" s="2" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="C123" s="2" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="D123" s="2" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
     </row>
     <row r="124" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A124" s="2" t="s">
-        <v>300</v>
+        <v>237</v>
       </c>
       <c r="B124" s="2" t="s">
-        <v>301</v>
+        <v>238</v>
       </c>
       <c r="C124" s="2" t="s">
-        <v>302</v>
+        <v>239</v>
       </c>
       <c r="D124" s="2" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
     </row>
     <row r="125" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A125" s="2" t="s">
-        <v>240</v>
+        <v>300</v>
       </c>
       <c r="B125" s="2" t="s">
-        <v>241</v>
+        <v>301</v>
       </c>
       <c r="C125" s="2" t="s">
-        <v>242</v>
+        <v>302</v>
       </c>
       <c r="D125" s="2" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
     </row>
     <row r="126" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A126" s="2" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="B126" s="2" t="s">
-        <v>252</v>
+        <v>241</v>
       </c>
       <c r="C126" s="2" t="s">
-        <v>251</v>
+        <v>242</v>
       </c>
       <c r="D126" s="2" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="127" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A127" s="2" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B127" s="2" t="s">
-        <v>245</v>
+        <v>252</v>
       </c>
       <c r="C127" s="2" t="s">
-        <v>246</v>
+        <v>251</v>
       </c>
       <c r="D127" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
     </row>
     <row r="128" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A128" s="2" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="B128" s="2" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="C128" s="2" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="D128" s="2" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
     </row>
     <row r="129" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A129" s="2" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="B129" s="2" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="C129" s="2" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="D129" s="2" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
     </row>
     <row r="130" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A130" s="2" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="B130" s="2" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="C130" s="2" t="s">
-        <v>255</v>
+        <v>250</v>
       </c>
       <c r="D130" s="2" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
     </row>
     <row r="131" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A131" s="2" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="B131" s="2" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="C131" s="2" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="D131" s="2" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
     </row>
     <row r="132" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A132" s="2" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="B132" s="2" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="C132" s="2" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="D132" s="2" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
     </row>
     <row r="133" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A133" s="2" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="B133" s="2" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="C133" s="2" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="D133" s="2" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="134" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A134" s="2" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="B134" s="2" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="C134" s="2" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="D134" s="2" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
     </row>
     <row r="135" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A135" s="2" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="B135" s="2" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="C135" s="2" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="D135" s="2" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
     </row>
     <row r="136" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A136" s="2" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="B136" s="2" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="C136" s="2" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="D136" s="2" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
     </row>
     <row r="137" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A137" s="2" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="B137" s="2" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="C137" s="2" t="s">
-        <v>273</v>
+        <v>269</v>
       </c>
       <c r="D137" s="2" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
     </row>
     <row r="138" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A138" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="B138" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="C138" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="D138" s="2" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="139" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A139" s="2" t="s">
         <v>271</v>
       </c>
-      <c r="B138" s="2" t="s">
+      <c r="B139" s="2" t="s">
         <v>271</v>
       </c>
-      <c r="C138" s="2" t="s">
+      <c r="C139" s="2" t="s">
         <v>272</v>
       </c>
-      <c r="D138" s="2" t="s">
+      <c r="D139" s="2" t="s">
         <v>427</v>
       </c>
     </row>
-    <row r="139" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A139" s="2" t="s">
+    <row r="140" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A140" s="2" t="s">
         <v>274</v>
       </c>
-      <c r="B139" s="2" t="s">
+      <c r="B140" s="2" t="s">
         <v>276</v>
       </c>
-      <c r="C139" s="2" t="s">
+      <c r="C140" s="2" t="s">
         <v>279</v>
       </c>
     </row>
-    <row r="140" spans="1:4" ht="45" x14ac:dyDescent="0.25">
-      <c r="A140" s="2" t="s">
+    <row r="141" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="A141" s="2" t="s">
         <v>275</v>
       </c>
-      <c r="B140" s="2" t="s">
+      <c r="B141" s="2" t="s">
         <v>277</v>
       </c>
-      <c r="C140" s="2" t="s">
+      <c r="C141" s="2" t="s">
         <v>278</v>
       </c>
     </row>
-    <row r="141" spans="1:4" ht="75" x14ac:dyDescent="0.25">
-      <c r="A141" s="2" t="s">
+    <row r="142" spans="1:4" ht="75" x14ac:dyDescent="0.25">
+      <c r="A142" s="2" t="s">
         <v>289</v>
       </c>
-      <c r="B141" s="2" t="s">
+      <c r="B142" s="2" t="s">
         <v>290</v>
       </c>
-      <c r="C141" s="2" t="s">
+      <c r="C142" s="2" t="s">
         <v>291</v>
-      </c>
-    </row>
-    <row r="142" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A142" s="2" t="s">
-        <v>306</v>
-      </c>
-      <c r="B142" s="2" t="s">
-        <v>307</v>
-      </c>
-      <c r="C142" s="2" t="s">
-        <v>308</v>
-      </c>
-      <c r="D142" s="2" t="s">
-        <v>428</v>
       </c>
     </row>
     <row r="143" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A143" s="2" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
       <c r="B143" s="2" t="s">
-        <v>311</v>
+        <v>307</v>
       </c>
       <c r="C143" s="2" t="s">
-        <v>312</v>
+        <v>308</v>
       </c>
       <c r="D143" s="2" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
     </row>
     <row r="144" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A144" s="2" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="B144" s="2" t="s">
-        <v>314</v>
+        <v>311</v>
       </c>
       <c r="C144" s="2" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="D144" s="2" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
     </row>
     <row r="145" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A145" s="2" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="B145" s="2" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="C145" s="2" t="s">
-        <v>316</v>
+        <v>313</v>
       </c>
       <c r="D145" s="2" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
     </row>
     <row r="146" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A146" s="2" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="B146" s="2" t="s">
-        <v>318</v>
+        <v>315</v>
       </c>
       <c r="C146" s="2" t="s">
-        <v>460</v>
+        <v>316</v>
       </c>
       <c r="D146" s="2" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
     </row>
     <row r="147" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A147" s="2" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="B147" s="2" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="C147" s="2" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="D147" s="2" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
     </row>
     <row r="148" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A148" s="2" t="s">
-        <v>448</v>
+        <v>319</v>
       </c>
       <c r="B148" s="2" t="s">
-        <v>448</v>
+        <v>320</v>
       </c>
       <c r="C148" s="2" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="D148" s="2" t="s">
-        <v>345</v>
+        <v>433</v>
       </c>
     </row>
     <row r="149" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A149" s="2" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="B149" s="2" t="s">
-        <v>450</v>
+        <v>448</v>
       </c>
       <c r="C149" s="2" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="D149" s="2" t="s">
-        <v>451</v>
+        <v>345</v>
       </c>
     </row>
     <row r="150" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A150" s="2" t="s">
-        <v>475</v>
+        <v>449</v>
       </c>
       <c r="B150" s="2" t="s">
-        <v>476</v>
+        <v>450</v>
       </c>
       <c r="C150" s="2" t="s">
-        <v>619</v>
+        <v>463</v>
       </c>
       <c r="D150" s="2" t="s">
-        <v>569</v>
+        <v>451</v>
       </c>
     </row>
     <row r="151" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A151" s="2" t="s">
-        <v>478</v>
+        <v>475</v>
       </c>
       <c r="B151" s="2" t="s">
-        <v>524</v>
+        <v>476</v>
       </c>
       <c r="C151" s="2" t="s">
-        <v>479</v>
+        <v>619</v>
       </c>
       <c r="D151" s="2" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
     </row>
     <row r="152" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A152" s="2" t="s">
-        <v>480</v>
+        <v>478</v>
       </c>
       <c r="B152" s="2" t="s">
-        <v>481</v>
+        <v>524</v>
       </c>
       <c r="C152" s="2" t="s">
-        <v>482</v>
+        <v>479</v>
       </c>
       <c r="D152" s="2" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
     </row>
     <row r="153" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A153" s="2" t="s">
-        <v>483</v>
+        <v>480</v>
       </c>
       <c r="B153" s="2" t="s">
-        <v>484</v>
+        <v>481</v>
       </c>
       <c r="C153" s="2" t="s">
-        <v>485</v>
+        <v>482</v>
       </c>
       <c r="D153" s="2" t="s">
-        <v>566</v>
+        <v>567</v>
       </c>
     </row>
     <row r="154" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A154" s="2" t="s">
-        <v>486</v>
+        <v>483</v>
       </c>
       <c r="B154" s="2" t="s">
-        <v>487</v>
+        <v>484</v>
       </c>
       <c r="C154" s="2" t="s">
-        <v>488</v>
+        <v>485</v>
       </c>
       <c r="D154" s="2" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
     </row>
     <row r="155" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A155" s="2" t="s">
-        <v>489</v>
+        <v>486</v>
       </c>
       <c r="B155" s="2" t="s">
-        <v>490</v>
+        <v>487</v>
       </c>
       <c r="C155" s="2" t="s">
-        <v>491</v>
+        <v>488</v>
       </c>
       <c r="D155" s="2" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
     </row>
     <row r="156" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A156" s="2" t="s">
-        <v>538</v>
+        <v>489</v>
       </c>
       <c r="B156" s="2" t="s">
-        <v>538</v>
+        <v>490</v>
       </c>
       <c r="C156" s="2" t="s">
-        <v>607</v>
+        <v>491</v>
       </c>
       <c r="D156" s="2" t="s">
-        <v>539</v>
+        <v>564</v>
       </c>
     </row>
     <row r="157" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A157" s="2" t="s">
-        <v>540</v>
+        <v>538</v>
       </c>
       <c r="B157" s="2" t="s">
-        <v>541</v>
+        <v>538</v>
       </c>
       <c r="C157" s="2" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="D157" s="2" t="s">
-        <v>542</v>
+        <v>539</v>
       </c>
     </row>
     <row r="158" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A158" s="2" t="s">
-        <v>492</v>
+        <v>540</v>
       </c>
       <c r="B158" s="2" t="s">
-        <v>493</v>
+        <v>541</v>
       </c>
       <c r="C158" s="2" t="s">
-        <v>494</v>
+        <v>608</v>
       </c>
       <c r="D158" s="2" t="s">
-        <v>563</v>
+        <v>542</v>
       </c>
     </row>
     <row r="159" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A159" s="2" t="s">
-        <v>495</v>
+        <v>492</v>
       </c>
       <c r="B159" s="2" t="s">
-        <v>496</v>
+        <v>493</v>
       </c>
       <c r="C159" s="2" t="s">
-        <v>497</v>
+        <v>494</v>
       </c>
       <c r="D159" s="2" t="s">
-        <v>562</v>
+        <v>563</v>
       </c>
     </row>
     <row r="160" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A160" s="2" t="s">
-        <v>498</v>
+        <v>495</v>
       </c>
       <c r="B160" s="2" t="s">
-        <v>499</v>
+        <v>496</v>
       </c>
       <c r="C160" s="2" t="s">
-        <v>500</v>
+        <v>497</v>
       </c>
       <c r="D160" s="2" t="s">
-        <v>561</v>
+        <v>562</v>
       </c>
     </row>
     <row r="161" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A161" s="2" t="s">
-        <v>501</v>
+        <v>498</v>
       </c>
       <c r="B161" s="2" t="s">
-        <v>501</v>
+        <v>499</v>
       </c>
       <c r="C161" s="2" t="s">
-        <v>502</v>
+        <v>500</v>
       </c>
       <c r="D161" s="2" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
     </row>
     <row r="162" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A162" s="2" t="s">
-        <v>503</v>
+        <v>501</v>
       </c>
       <c r="B162" s="2" t="s">
-        <v>503</v>
+        <v>501</v>
       </c>
       <c r="C162" s="2" t="s">
-        <v>504</v>
+        <v>502</v>
       </c>
       <c r="D162" s="2" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
     </row>
     <row r="163" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A163" s="2" t="s">
-        <v>505</v>
+        <v>503</v>
       </c>
       <c r="B163" s="2" t="s">
-        <v>505</v>
+        <v>503</v>
       </c>
       <c r="C163" s="2" t="s">
-        <v>506</v>
+        <v>504</v>
       </c>
       <c r="D163" s="2" t="s">
-        <v>558</v>
+        <v>559</v>
       </c>
     </row>
     <row r="164" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A164" s="2" t="s">
-        <v>507</v>
+        <v>505</v>
       </c>
       <c r="B164" s="2" t="s">
-        <v>507</v>
+        <v>505</v>
       </c>
       <c r="C164" s="2" t="s">
-        <v>508</v>
+        <v>506</v>
       </c>
       <c r="D164" s="2" t="s">
-        <v>557</v>
+        <v>558</v>
       </c>
     </row>
     <row r="165" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A165" s="2" t="s">
-        <v>570</v>
+        <v>507</v>
       </c>
       <c r="B165" s="2" t="s">
-        <v>571</v>
+        <v>507</v>
       </c>
       <c r="C165" s="2" t="s">
-        <v>609</v>
+        <v>508</v>
+      </c>
+      <c r="D165" s="2" t="s">
+        <v>557</v>
       </c>
     </row>
     <row r="166" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A166" s="2" t="s">
-        <v>572</v>
+        <v>570</v>
       </c>
       <c r="B166" s="2" t="s">
-        <v>573</v>
+        <v>571</v>
       </c>
       <c r="C166" s="2" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
     </row>
     <row r="167" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A167" s="2" t="s">
-        <v>574</v>
+        <v>572</v>
       </c>
       <c r="B167" s="2" t="s">
-        <v>575</v>
+        <v>573</v>
       </c>
       <c r="C167" s="2" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
     </row>
     <row r="168" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A168" s="2" t="s">
-        <v>576</v>
+        <v>574</v>
       </c>
       <c r="B168" s="2" t="s">
-        <v>577</v>
+        <v>575</v>
       </c>
       <c r="C168" s="2" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
     </row>
     <row r="169" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A169" s="2" t="s">
-        <v>578</v>
+        <v>576</v>
       </c>
       <c r="B169" s="2" t="s">
-        <v>579</v>
+        <v>577</v>
       </c>
       <c r="C169" s="2" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
     </row>
     <row r="170" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A170" s="2" t="s">
-        <v>580</v>
+        <v>578</v>
       </c>
       <c r="B170" s="2" t="s">
-        <v>581</v>
+        <v>579</v>
       </c>
       <c r="C170" s="2" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
     </row>
     <row r="171" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A171" s="2" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
       <c r="B171" s="2" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="C171" s="2" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
     </row>
     <row r="172" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A172" s="2" t="s">
-        <v>584</v>
+        <v>582</v>
       </c>
       <c r="B172" s="2" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="C172" s="2" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
     </row>
     <row r="173" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A173" s="2" t="s">
-        <v>586</v>
+        <v>584</v>
       </c>
       <c r="B173" s="2" t="s">
-        <v>587</v>
+        <v>585</v>
       </c>
       <c r="C173" s="2" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
     </row>
     <row r="174" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A174" s="2" t="s">
-        <v>588</v>
+        <v>586</v>
       </c>
       <c r="B174" s="2" t="s">
-        <v>589</v>
+        <v>587</v>
       </c>
       <c r="C174" s="2" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
     </row>
     <row r="175" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A175" s="2" t="s">
-        <v>620</v>
+        <v>588</v>
       </c>
       <c r="B175" s="2" t="s">
-        <v>621</v>
+        <v>589</v>
       </c>
       <c r="C175" s="2" t="s">
-        <v>622</v>
+        <v>618</v>
       </c>
     </row>
     <row r="176" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A176" s="2" t="s">
-        <v>623</v>
+        <v>620</v>
       </c>
       <c r="B176" s="2" t="s">
-        <v>623</v>
+        <v>621</v>
       </c>
       <c r="C176" s="2" t="s">
-        <v>624</v>
+        <v>622</v>
       </c>
     </row>
     <row r="177" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A177" s="2" t="s">
-        <v>625</v>
+        <v>623</v>
       </c>
       <c r="B177" s="2" t="s">
-        <v>625</v>
+        <v>623</v>
       </c>
       <c r="C177" s="2" t="s">
-        <v>627</v>
+        <v>624</v>
       </c>
     </row>
     <row r="178" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A178" s="2" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="B178" s="2" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="C178" s="2" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
     </row>
     <row r="179" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A179" s="2" t="s">
-        <v>629</v>
+        <v>626</v>
       </c>
       <c r="B179" s="2" t="s">
-        <v>630</v>
+        <v>626</v>
       </c>
       <c r="C179" s="2" t="s">
-        <v>631</v>
+        <v>628</v>
       </c>
     </row>
     <row r="180" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A180" s="2" t="s">
-        <v>632</v>
-      </c>
-      <c r="B180" s="4" t="s">
-        <v>633</v>
-      </c>
-      <c r="C180" s="4" t="s">
-        <v>634</v>
+        <v>629</v>
+      </c>
+      <c r="B180" s="2" t="s">
+        <v>630</v>
+      </c>
+      <c r="C180" s="2" t="s">
+        <v>631</v>
       </c>
     </row>
     <row r="181" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A181" s="2" t="s">
-        <v>638</v>
-      </c>
-      <c r="B181" s="2" t="s">
-        <v>639</v>
-      </c>
-      <c r="C181" s="2" t="s">
-        <v>640</v>
+        <v>632</v>
+      </c>
+      <c r="B181" s="4" t="s">
+        <v>633</v>
+      </c>
+      <c r="C181" s="4" t="s">
+        <v>634</v>
       </c>
     </row>
     <row r="182" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A182" s="2" t="s">
-        <v>641</v>
+        <v>638</v>
       </c>
       <c r="B182" s="2" t="s">
-        <v>641</v>
+        <v>639</v>
       </c>
       <c r="C182" s="2" t="s">
-        <v>642</v>
+        <v>640</v>
       </c>
     </row>
     <row r="183" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A183" s="2" t="s">
-        <v>643</v>
+        <v>641</v>
       </c>
       <c r="B183" s="2" t="s">
-        <v>644</v>
+        <v>641</v>
       </c>
       <c r="C183" s="2" t="s">
-        <v>645</v>
+        <v>642</v>
       </c>
     </row>
     <row r="184" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A184" s="2" t="s">
-        <v>646</v>
+        <v>643</v>
       </c>
       <c r="B184" s="2" t="s">
-        <v>647</v>
+        <v>644</v>
       </c>
       <c r="C184" s="2" t="s">
-        <v>648</v>
+        <v>645</v>
       </c>
     </row>
     <row r="185" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A185" s="2" t="s">
-        <v>649</v>
+        <v>646</v>
       </c>
       <c r="B185" s="2" t="s">
-        <v>650</v>
+        <v>647</v>
       </c>
       <c r="C185" s="2" t="s">
-        <v>651</v>
+        <v>648</v>
       </c>
     </row>
     <row r="186" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A186" s="2" t="s">
-        <v>652</v>
+        <v>649</v>
       </c>
       <c r="B186" s="2" t="s">
-        <v>653</v>
+        <v>650</v>
       </c>
       <c r="C186" s="2" t="s">
-        <v>654</v>
+        <v>651</v>
       </c>
     </row>
     <row r="187" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A187" s="2" t="s">
-        <v>655</v>
+        <v>652</v>
       </c>
       <c r="B187" s="2" t="s">
-        <v>655</v>
+        <v>653</v>
       </c>
       <c r="C187" s="2" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
     </row>
     <row r="188" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A188" s="2" t="s">
-        <v>657</v>
+        <v>655</v>
       </c>
       <c r="B188" s="2" t="s">
-        <v>658</v>
+        <v>655</v>
       </c>
       <c r="C188" s="2" t="s">
-        <v>659</v>
+        <v>656</v>
       </c>
     </row>
     <row r="189" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A189" s="2" t="s">
-        <v>666</v>
-      </c>
-      <c r="B189" s="4" t="s">
-        <v>667</v>
-      </c>
-      <c r="C189" s="4" t="s">
-        <v>668</v>
+        <v>657</v>
+      </c>
+      <c r="B189" s="2" t="s">
+        <v>658</v>
+      </c>
+      <c r="C189" s="2" t="s">
+        <v>659</v>
       </c>
     </row>
     <row r="190" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A190" s="2" t="s">
+        <v>666</v>
+      </c>
+      <c r="B190" s="4" t="s">
+        <v>667</v>
+      </c>
+      <c r="C190" s="4" t="s">
+        <v>668</v>
+      </c>
+    </row>
+    <row r="191" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A191" s="2" t="s">
         <v>669</v>
       </c>
-      <c r="B190" s="2" t="s">
+      <c r="B191" s="2" t="s">
         <v>670</v>
       </c>
-      <c r="C190" s="2" t="s">
+      <c r="C191" s="2" t="s">
         <v>671</v>
+      </c>
+    </row>
+    <row r="192" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A192" s="2" t="s">
+        <v>675</v>
+      </c>
+      <c r="B192" s="2" t="s">
+        <v>676</v>
+      </c>
+      <c r="C192" s="2" t="s">
+        <v>677</v>
+      </c>
+    </row>
+    <row r="193" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A193" s="2" t="s">
+        <v>678</v>
+      </c>
+      <c r="B193" s="2" t="s">
+        <v>679</v>
+      </c>
+      <c r="C193" s="2" t="s">
+        <v>680</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added "Use Numbers" for Sequencer Screens!
</commit_message>
<xml_diff>
--- a/Translations/Translations.xlsx
+++ b/Translations/Translations.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programacion\MelonLoader\FS_LevelEditor\Translations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{672CC127-6C57-4707-8ED0-AFF4E2583862}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5362AEC0-C36B-47CC-A96A-FFFF04E6DEA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{F5C22481-FF1A-482C-BF7E-EB5A7718AF49}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1373" uniqueCount="681">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1376" uniqueCount="684">
   <si>
     <t>ID</t>
   </si>
@@ -2081,6 +2081,15 @@
   </si>
   <si>
     <t>Invertir Orden</t>
+  </si>
+  <si>
+    <t>UseNumbers</t>
+  </si>
+  <si>
+    <t>Use Numbers</t>
+  </si>
+  <si>
+    <t>Usar Números</t>
   </si>
 </sst>
 </file>
@@ -2480,7 +2489,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6961A5F-F8EA-4989-8112-A0ACE51D011E}">
   <sheetPr codeName="Hoja1"/>
-  <dimension ref="A1:D193"/>
+  <dimension ref="A1:D194"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="37" style="2" customWidth="1"/>
@@ -5083,6 +5092,17 @@
       </c>
       <c r="C193" s="2" t="s">
         <v>680</v>
+      </c>
+    </row>
+    <row r="194" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A194" s="2" t="s">
+        <v>681</v>
+      </c>
+      <c r="B194" s="2" t="s">
+        <v>682</v>
+      </c>
+      <c r="C194" s="2" t="s">
+        <v>683</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added translations for Add To Group.
</commit_message>
<xml_diff>
--- a/Translations/Translations.xlsx
+++ b/Translations/Translations.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programacion\MelonLoader\FS_LevelEditor\Translations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0FA98B1-0562-4517-BD30-3676E19621A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4CF435F8-E214-45EF-8B95-054A40CC1DFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{F5C22481-FF1A-482C-BF7E-EB5A7718AF49}"/>
   </bookViews>
   <sheets>
-    <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
+    <sheet name="Translations" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029" calcMode="manual"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1382" uniqueCount="690">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1406" uniqueCount="713">
   <si>
     <t>ID</t>
   </si>
@@ -2108,6 +2108,75 @@
   </si>
   <si>
     <t>Permitir Modo Debug</t>
+  </si>
+  <si>
+    <t>AddToGroupButton</t>
+  </si>
+  <si>
+    <t>AddToGroupTitle</t>
+  </si>
+  <si>
+    <t>AddToNewGroup</t>
+  </si>
+  <si>
+    <t>AddToExistingGroup</t>
+  </si>
+  <si>
+    <t>+ Add To Group</t>
+  </si>
+  <si>
+    <t>+ Add To Existing Group</t>
+  </si>
+  <si>
+    <t>+ Add To New Group</t>
+  </si>
+  <si>
+    <t>Add To Group</t>
+  </si>
+  <si>
+    <t>Groups</t>
+  </si>
+  <si>
+    <t>GroupsTitle</t>
+  </si>
+  <si>
+    <t>SelectAll</t>
+  </si>
+  <si>
+    <t>DeleteGroup</t>
+  </si>
+  <si>
+    <t>Select All</t>
+  </si>
+  <si>
+    <t>Delete Group</t>
+  </si>
+  <si>
+    <t>+ Añadir A Grupo</t>
+  </si>
+  <si>
+    <t>+ Añadir A Grupo Existente</t>
+  </si>
+  <si>
+    <t>+ Añadir A Grupo Nuevo</t>
+  </si>
+  <si>
+    <t>Grupos</t>
+  </si>
+  <si>
+    <t>Seleccionar Todo</t>
+  </si>
+  <si>
+    <t>Eliminar Grupo</t>
+  </si>
+  <si>
+    <t>Añadir A Grupo</t>
+  </si>
+  <si>
+    <t>Group</t>
+  </si>
+  <si>
+    <t>Grupo</t>
   </si>
 </sst>
 </file>
@@ -2507,7 +2576,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6961A5F-F8EA-4989-8112-A0ACE51D011E}">
   <sheetPr codeName="Hoja1"/>
-  <dimension ref="A1:D196"/>
+  <dimension ref="A1:D204"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="37" style="2" customWidth="1"/>
@@ -5143,6 +5212,94 @@
       </c>
       <c r="C196" s="2" t="s">
         <v>689</v>
+      </c>
+    </row>
+    <row r="197" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A197" s="2" t="s">
+        <v>690</v>
+      </c>
+      <c r="B197" s="4" t="s">
+        <v>694</v>
+      </c>
+      <c r="C197" s="4" t="s">
+        <v>704</v>
+      </c>
+    </row>
+    <row r="198" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A198" s="2" t="s">
+        <v>691</v>
+      </c>
+      <c r="B198" s="2" t="s">
+        <v>697</v>
+      </c>
+      <c r="C198" s="2" t="s">
+        <v>710</v>
+      </c>
+    </row>
+    <row r="199" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A199" s="2" t="s">
+        <v>693</v>
+      </c>
+      <c r="B199" s="4" t="s">
+        <v>695</v>
+      </c>
+      <c r="C199" s="4" t="s">
+        <v>705</v>
+      </c>
+    </row>
+    <row r="200" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A200" s="2" t="s">
+        <v>692</v>
+      </c>
+      <c r="B200" s="4" t="s">
+        <v>696</v>
+      </c>
+      <c r="C200" s="4" t="s">
+        <v>706</v>
+      </c>
+    </row>
+    <row r="201" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A201" s="2" t="s">
+        <v>699</v>
+      </c>
+      <c r="B201" s="2" t="s">
+        <v>698</v>
+      </c>
+      <c r="C201" s="2" t="s">
+        <v>707</v>
+      </c>
+    </row>
+    <row r="202" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A202" s="2" t="s">
+        <v>700</v>
+      </c>
+      <c r="B202" s="2" t="s">
+        <v>702</v>
+      </c>
+      <c r="C202" s="2" t="s">
+        <v>708</v>
+      </c>
+    </row>
+    <row r="203" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A203" s="2" t="s">
+        <v>701</v>
+      </c>
+      <c r="B203" s="2" t="s">
+        <v>703</v>
+      </c>
+      <c r="C203" s="2" t="s">
+        <v>709</v>
+      </c>
+    </row>
+    <row r="204" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A204" s="2" t="s">
+        <v>711</v>
+      </c>
+      <c r="B204" s="2" t="s">
+        <v>711</v>
+      </c>
+      <c r="C204" s="2" t="s">
+        <v>712</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added Remove From Group button.
</commit_message>
<xml_diff>
--- a/Translations/Translations.xlsx
+++ b/Translations/Translations.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programacion\MelonLoader\FS_LevelEditor\Translations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4CF435F8-E214-45EF-8B95-054A40CC1DFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A09C027C-5775-4AFE-958C-D2720FD8422A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{F5C22481-FF1A-482C-BF7E-EB5A7718AF49}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1406" uniqueCount="713">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1409" uniqueCount="716">
   <si>
     <t>ID</t>
   </si>
@@ -2177,6 +2177,15 @@
   </si>
   <si>
     <t>Grupo</t>
+  </si>
+  <si>
+    <t>RemoveFromGroup</t>
+  </si>
+  <si>
+    <t>Remove From Group</t>
+  </si>
+  <si>
+    <t>Eliminar Del Grupo</t>
   </si>
 </sst>
 </file>
@@ -2576,7 +2585,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6961A5F-F8EA-4989-8112-A0ACE51D011E}">
   <sheetPr codeName="Hoja1"/>
-  <dimension ref="A1:D204"/>
+  <dimension ref="A1:D205"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="37" style="2" customWidth="1"/>
@@ -5300,6 +5309,17 @@
       </c>
       <c r="C204" s="2" t="s">
         <v>712</v>
+      </c>
+    </row>
+    <row r="205" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A205" s="2" t="s">
+        <v>713</v>
+      </c>
+      <c r="B205" s="2" t="s">
+        <v>714</v>
+      </c>
+      <c r="C205" s="2" t="s">
+        <v>715</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added "When Reached" events for global waypoints.
</commit_message>
<xml_diff>
--- a/Translations/Translations.xlsx
+++ b/Translations/Translations.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programacion\MelonLoader\FS_LevelEditor\Translations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A09C027C-5775-4AFE-958C-D2720FD8422A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B4C6FB0-0B0A-45BD-8E31-82C54564B04B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{F5C22481-FF1A-482C-BF7E-EB5A7718AF49}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1409" uniqueCount="716">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1415" uniqueCount="722">
   <si>
     <t>ID</t>
   </si>
@@ -2186,6 +2186,24 @@
   </si>
   <si>
     <t>Eliminar Del Grupo</t>
+  </si>
+  <si>
+    <t>StopHere</t>
+  </si>
+  <si>
+    <t>Stop Here</t>
+  </si>
+  <si>
+    <t>Parar Aquí</t>
+  </si>
+  <si>
+    <t>events.WhenReached</t>
+  </si>
+  <si>
+    <t>When Reached</t>
+  </si>
+  <si>
+    <t>Al Ser Alcanzado</t>
   </si>
 </sst>
 </file>
@@ -2585,7 +2603,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6961A5F-F8EA-4989-8112-A0ACE51D011E}">
   <sheetPr codeName="Hoja1"/>
-  <dimension ref="A1:D205"/>
+  <dimension ref="A1:D207"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="37" style="2" customWidth="1"/>
@@ -5320,6 +5338,28 @@
       </c>
       <c r="C205" s="2" t="s">
         <v>715</v>
+      </c>
+    </row>
+    <row r="206" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A206" s="2" t="s">
+        <v>716</v>
+      </c>
+      <c r="B206" s="2" t="s">
+        <v>717</v>
+      </c>
+      <c r="C206" s="2" t="s">
+        <v>718</v>
+      </c>
+    </row>
+    <row r="207" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A207" s="2" t="s">
+        <v>719</v>
+      </c>
+      <c r="B207" s="2" t="s">
+        <v>720</v>
+      </c>
+      <c r="C207" s="2" t="s">
+        <v>721</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added power cores (still no power slot yet).
</commit_message>
<xml_diff>
--- a/Translations/Translations.xlsx
+++ b/Translations/Translations.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programacion\MelonLoader\FS_LevelEditor\Translations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B4C6FB0-0B0A-45BD-8E31-82C54564B04B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1528DA4C-287B-4FC8-9C1C-C925C8734DFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{F5C22481-FF1A-482C-BF7E-EB5A7718AF49}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1415" uniqueCount="722">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1418" uniqueCount="725">
   <si>
     <t>ID</t>
   </si>
@@ -2204,6 +2204,15 @@
   </si>
   <si>
     <t>Al Ser Alcanzado</t>
+  </si>
+  <si>
+    <t>object.POWER_CORE</t>
+  </si>
+  <si>
+    <t>Power Core</t>
+  </si>
+  <si>
+    <t>Núcleo de Energía</t>
   </si>
 </sst>
 </file>
@@ -2603,7 +2612,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6961A5F-F8EA-4989-8112-A0ACE51D011E}">
   <sheetPr codeName="Hoja1"/>
-  <dimension ref="A1:D207"/>
+  <dimension ref="A1:D208"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="37" style="2" customWidth="1"/>
@@ -3455,1910 +3464,1921 @@
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" s="2" t="s">
-        <v>69</v>
+        <v>722</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>69</v>
+        <v>723</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="D62" s="2" t="s">
-        <v>364</v>
+        <v>724</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63" s="2" t="s">
-        <v>443</v>
+        <v>69</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>443</v>
+        <v>69</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>601</v>
+        <v>101</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>552</v>
+        <v>364</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" s="2" t="s">
-        <v>456</v>
+        <v>443</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>456</v>
+        <v>443</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>456</v>
+        <v>601</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>457</v>
+        <v>552</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A65" s="2" t="s">
-        <v>105</v>
+        <v>456</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>2</v>
+        <v>456</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>102</v>
+        <v>456</v>
       </c>
       <c r="D65" s="2" t="s">
-        <v>365</v>
+        <v>457</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D66" s="2" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A67" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D67" s="2" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A68" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>111</v>
+        <v>4</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="D68" s="2" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A69" s="2" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="D69" s="2" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A70" s="2" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="C70" s="2" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="D70" s="2" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A71" s="2" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="D71" s="2" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A72" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D72" s="2" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A73" s="2" t="s">
-        <v>445</v>
+        <v>118</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>446</v>
+        <v>122</v>
       </c>
       <c r="C73" s="2" t="s">
-        <v>459</v>
+        <v>121</v>
       </c>
       <c r="D73" s="2" t="s">
-        <v>447</v>
+        <v>370</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A74" s="2" t="s">
-        <v>512</v>
+        <v>445</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>513</v>
+        <v>446</v>
       </c>
       <c r="C74" s="2" t="s">
-        <v>602</v>
+        <v>459</v>
       </c>
       <c r="D74" s="2" t="s">
-        <v>514</v>
+        <v>447</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A75" s="2" t="s">
-        <v>518</v>
+        <v>512</v>
       </c>
       <c r="B75" s="2" t="s">
-        <v>519</v>
+        <v>513</v>
       </c>
       <c r="C75" s="2" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="D75" s="2" t="s">
-        <v>520</v>
+        <v>514</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A76" s="2" t="s">
-        <v>521</v>
+        <v>518</v>
       </c>
       <c r="B76" s="2" t="s">
-        <v>522</v>
+        <v>519</v>
       </c>
       <c r="C76" s="2" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="D76" s="2" t="s">
-        <v>523</v>
+        <v>520</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A77" s="2" t="s">
-        <v>532</v>
+        <v>521</v>
       </c>
       <c r="B77" s="2" t="s">
-        <v>533</v>
+        <v>522</v>
       </c>
       <c r="C77" s="2" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="D77" s="2" t="s">
-        <v>534</v>
+        <v>523</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A78" s="2" t="s">
-        <v>537</v>
+        <v>532</v>
       </c>
       <c r="B78" s="2" t="s">
-        <v>535</v>
+        <v>533</v>
       </c>
       <c r="C78" s="2" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="D78" s="2" t="s">
-        <v>536</v>
+        <v>534</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A79" s="2" t="s">
-        <v>154</v>
+        <v>537</v>
       </c>
       <c r="B79" s="2" t="s">
-        <v>155</v>
+        <v>535</v>
       </c>
       <c r="C79" s="2" t="s">
-        <v>156</v>
+        <v>606</v>
       </c>
       <c r="D79" s="2" t="s">
-        <v>371</v>
+        <v>536</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
-        <v>164</v>
+        <v>154</v>
       </c>
       <c r="B80" s="2" t="s">
-        <v>165</v>
+        <v>155</v>
       </c>
       <c r="C80" s="2" t="s">
-        <v>166</v>
+        <v>156</v>
       </c>
       <c r="D80" s="2" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A81" s="2" t="s">
-        <v>157</v>
+        <v>164</v>
       </c>
       <c r="B81" s="2" t="s">
-        <v>158</v>
+        <v>165</v>
       </c>
       <c r="C81" s="2" t="s">
-        <v>159</v>
+        <v>166</v>
       </c>
       <c r="D81" s="2" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A82" s="2" t="s">
-        <v>167</v>
+        <v>157</v>
       </c>
       <c r="B82" s="2" t="s">
-        <v>168</v>
+        <v>158</v>
       </c>
       <c r="C82" s="2" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="D82" s="2" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A83" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="B83" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="C83" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="D83" s="2" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A84" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="B83" s="2" t="s">
+      <c r="B84" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="C83" s="2" t="s">
+      <c r="C84" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="D83" s="2" t="s">
+      <c r="D84" s="2" t="s">
         <v>375</v>
       </c>
     </row>
-    <row r="84" spans="1:4" ht="45" x14ac:dyDescent="0.25">
-      <c r="A84" s="2" t="s">
+    <row r="85" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="A85" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="B84" s="2" t="s">
+      <c r="B85" s="2" t="s">
         <v>163</v>
       </c>
-      <c r="C84" s="2" t="s">
+      <c r="C85" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="D84" s="2" t="s">
+      <c r="D85" s="2" t="s">
         <v>376</v>
-      </c>
-    </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A85" s="2" t="s">
-        <v>153</v>
-      </c>
-      <c r="B85" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="C85" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="D85" s="2" t="s">
-        <v>328</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A86" s="2" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="B86" s="2" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="C86" s="2" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="D86" s="2" t="s">
-        <v>377</v>
+        <v>328</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A87" s="2" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="B87" s="2" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="C87" s="2" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="D87" s="2" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A88" s="2" t="s">
-        <v>172</v>
+        <v>150</v>
       </c>
       <c r="B88" s="2" t="s">
-        <v>170</v>
+        <v>151</v>
       </c>
       <c r="C88" s="2" t="s">
-        <v>171</v>
+        <v>152</v>
       </c>
       <c r="D88" s="2" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A89" s="2" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B89" s="2" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="C89" s="2" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="D89" s="2" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A90" s="2" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="B90" s="2" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="C90" s="2" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="D90" s="2" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A91" s="2" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="B91" s="2" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="C91" s="2" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="D91" s="2" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A92" s="2" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="B92" s="2" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="C92" s="2" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="D92" s="2" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A93" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="B93" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="C93" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="D93" s="2" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A94" s="2" t="s">
         <v>243</v>
       </c>
-      <c r="B93" s="2" t="s">
+      <c r="B94" s="2" t="s">
         <v>243</v>
       </c>
-      <c r="C93" s="2" t="s">
+      <c r="C94" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="D93" s="2" t="s">
+      <c r="D94" s="2" t="s">
         <v>384</v>
       </c>
     </row>
-    <row r="94" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A94" s="2" t="s">
+    <row r="95" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A95" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="B94" s="1" t="s">
+      <c r="B95" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="C94" s="2" t="s">
+      <c r="C95" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="D94" s="2" t="s">
+      <c r="D95" s="2" t="s">
         <v>385</v>
-      </c>
-    </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A95" s="2" t="s">
-        <v>182</v>
-      </c>
-      <c r="B95" s="2" t="s">
-        <v>183</v>
-      </c>
-      <c r="C95" s="2" t="s">
-        <v>183</v>
-      </c>
-      <c r="D95" s="2" t="s">
-        <v>386</v>
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A96" s="2" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="B96" s="2" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C96" s="2" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="D96" s="2" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A97" s="2" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="B97" s="2" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="C97" s="2" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="D97" s="2" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A98" s="2" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="B98" s="2" t="s">
-        <v>525</v>
+        <v>186</v>
       </c>
       <c r="C98" s="2" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="D98" s="2" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A99" s="2" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="B99" s="2" t="s">
-        <v>190</v>
+        <v>525</v>
       </c>
       <c r="C99" s="2" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="D99" s="2" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A100" s="2" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="B100" s="2" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="C100" s="2" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="D100" s="2" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A101" s="2" t="s">
-        <v>434</v>
-      </c>
-      <c r="B101" s="4" t="s">
-        <v>435</v>
-      </c>
-      <c r="C101" s="4" t="s">
-        <v>436</v>
-      </c>
-      <c r="D101" s="4" t="s">
-        <v>591</v>
+        <v>192</v>
+      </c>
+      <c r="B101" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="C101" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="D101" s="2" t="s">
+        <v>391</v>
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A102" s="2" t="s">
-        <v>437</v>
+        <v>434</v>
       </c>
       <c r="B102" s="4" t="s">
-        <v>438</v>
+        <v>435</v>
       </c>
       <c r="C102" s="4" t="s">
-        <v>439</v>
+        <v>436</v>
       </c>
       <c r="D102" s="4" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A103" s="2" t="s">
-        <v>473</v>
+        <v>437</v>
       </c>
       <c r="B103" s="4" t="s">
-        <v>590</v>
+        <v>438</v>
       </c>
       <c r="C103" s="4" t="s">
-        <v>474</v>
+        <v>439</v>
       </c>
       <c r="D103" s="4" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A104" s="2" t="s">
-        <v>195</v>
-      </c>
-      <c r="B104" s="2" t="s">
-        <v>196</v>
-      </c>
-      <c r="C104" s="2" t="s">
-        <v>197</v>
-      </c>
-      <c r="D104" s="2" t="s">
-        <v>392</v>
+        <v>473</v>
+      </c>
+      <c r="B104" s="4" t="s">
+        <v>590</v>
+      </c>
+      <c r="C104" s="4" t="s">
+        <v>474</v>
+      </c>
+      <c r="D104" s="4" t="s">
+        <v>593</v>
       </c>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A105" s="2" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="B105" s="2" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="C105" s="2" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="D105" s="2" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A106" s="2" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="B106" s="2" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="C106" s="2" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="D106" s="2" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A107" s="2" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="B107" s="2" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="C107" s="2" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="D107" s="2" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A108" s="2" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="B108" s="2" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="C108" s="2" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="D108" s="2" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A109" s="2" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B109" s="2" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="C109" s="2" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="D109" s="2" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A110" s="2" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="B110" s="2" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="C110" s="2" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="D110" s="2" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A111" s="2" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="B111" s="2" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="C111" s="2" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="D111" s="2" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A112" s="2" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="B112" s="2" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="C112" s="2" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="D112" s="2" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A113" s="2" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="B113" s="2" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="C113" s="2" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="D113" s="2" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A114" s="2" t="s">
-        <v>292</v>
+        <v>220</v>
       </c>
       <c r="B114" s="2" t="s">
-        <v>292</v>
+        <v>219</v>
       </c>
       <c r="C114" s="2" t="s">
-        <v>293</v>
+        <v>218</v>
       </c>
       <c r="D114" s="2" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A115" s="2" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="B115" s="2" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="C115" s="2" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
       <c r="D115" s="2" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A116" s="2" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
       <c r="B116" s="2" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="C116" s="2" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="D116" s="2" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A117" s="2" t="s">
-        <v>221</v>
+        <v>297</v>
       </c>
       <c r="B117" s="2" t="s">
-        <v>221</v>
+        <v>298</v>
       </c>
       <c r="C117" s="2" t="s">
-        <v>222</v>
+        <v>299</v>
       </c>
       <c r="D117" s="2" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A118" s="2" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="B118" s="2" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="C118" s="2" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="D118" s="2" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="119" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A119" s="2" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="B119" s="2" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="C119" s="2" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="D119" s="2" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A120" s="2" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="B120" s="2" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="C120" s="2" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="D120" s="2" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A121" s="2" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B121" s="2" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="C121" s="2" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="D121" s="2" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A122" s="2" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="B122" s="2" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="C122" s="2" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="D122" s="2" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
     </row>
     <row r="123" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A123" s="2" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="B123" s="2" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="C123" s="2" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="D123" s="2" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
     </row>
     <row r="124" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A124" s="2" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="B124" s="2" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="C124" s="2" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="D124" s="2" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
     </row>
     <row r="125" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A125" s="2" t="s">
-        <v>300</v>
+        <v>237</v>
       </c>
       <c r="B125" s="2" t="s">
-        <v>301</v>
+        <v>238</v>
       </c>
       <c r="C125" s="2" t="s">
-        <v>302</v>
+        <v>239</v>
       </c>
       <c r="D125" s="2" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
     </row>
     <row r="126" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A126" s="2" t="s">
-        <v>240</v>
+        <v>300</v>
       </c>
       <c r="B126" s="2" t="s">
-        <v>241</v>
+        <v>301</v>
       </c>
       <c r="C126" s="2" t="s">
-        <v>242</v>
+        <v>302</v>
       </c>
       <c r="D126" s="2" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
     </row>
     <row r="127" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A127" s="2" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="B127" s="2" t="s">
-        <v>252</v>
+        <v>241</v>
       </c>
       <c r="C127" s="2" t="s">
-        <v>251</v>
+        <v>242</v>
       </c>
       <c r="D127" s="2" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="128" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A128" s="2" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B128" s="2" t="s">
-        <v>245</v>
+        <v>252</v>
       </c>
       <c r="C128" s="2" t="s">
-        <v>246</v>
+        <v>251</v>
       </c>
       <c r="D128" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
     </row>
     <row r="129" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A129" s="2" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="B129" s="2" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="C129" s="2" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="D129" s="2" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
     </row>
     <row r="130" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A130" s="2" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="B130" s="2" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="C130" s="2" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="D130" s="2" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
     </row>
     <row r="131" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A131" s="2" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="B131" s="2" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="C131" s="2" t="s">
-        <v>255</v>
+        <v>250</v>
       </c>
       <c r="D131" s="2" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
     </row>
     <row r="132" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A132" s="2" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="B132" s="2" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="C132" s="2" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="D132" s="2" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
     </row>
     <row r="133" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A133" s="2" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="B133" s="2" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="C133" s="2" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="D133" s="2" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
     </row>
     <row r="134" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A134" s="2" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="B134" s="2" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="C134" s="2" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="D134" s="2" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="135" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A135" s="2" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="B135" s="2" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="C135" s="2" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="D135" s="2" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
     </row>
     <row r="136" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A136" s="2" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="B136" s="2" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="C136" s="2" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="D136" s="2" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
     </row>
     <row r="137" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A137" s="2" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="B137" s="2" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="C137" s="2" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="D137" s="2" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
     </row>
     <row r="138" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A138" s="2" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="B138" s="2" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="C138" s="2" t="s">
-        <v>273</v>
+        <v>269</v>
       </c>
       <c r="D138" s="2" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
     </row>
     <row r="139" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A139" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="B139" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="C139" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="D139" s="2" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="140" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A140" s="2" t="s">
         <v>271</v>
       </c>
-      <c r="B139" s="2" t="s">
+      <c r="B140" s="2" t="s">
         <v>271</v>
       </c>
-      <c r="C139" s="2" t="s">
+      <c r="C140" s="2" t="s">
         <v>272</v>
       </c>
-      <c r="D139" s="2" t="s">
+      <c r="D140" s="2" t="s">
         <v>427</v>
       </c>
     </row>
-    <row r="140" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A140" s="2" t="s">
+    <row r="141" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A141" s="2" t="s">
         <v>274</v>
       </c>
-      <c r="B140" s="2" t="s">
+      <c r="B141" s="2" t="s">
         <v>276</v>
       </c>
-      <c r="C140" s="2" t="s">
+      <c r="C141" s="2" t="s">
         <v>279</v>
       </c>
     </row>
-    <row r="141" spans="1:4" ht="45" x14ac:dyDescent="0.25">
-      <c r="A141" s="2" t="s">
+    <row r="142" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="A142" s="2" t="s">
         <v>275</v>
       </c>
-      <c r="B141" s="2" t="s">
+      <c r="B142" s="2" t="s">
         <v>277</v>
       </c>
-      <c r="C141" s="2" t="s">
+      <c r="C142" s="2" t="s">
         <v>278</v>
       </c>
     </row>
-    <row r="142" spans="1:4" ht="75" x14ac:dyDescent="0.25">
-      <c r="A142" s="2" t="s">
+    <row r="143" spans="1:4" ht="75" x14ac:dyDescent="0.25">
+      <c r="A143" s="2" t="s">
         <v>289</v>
       </c>
-      <c r="B142" s="2" t="s">
+      <c r="B143" s="2" t="s">
         <v>290</v>
       </c>
-      <c r="C142" s="2" t="s">
+      <c r="C143" s="2" t="s">
         <v>291</v>
-      </c>
-    </row>
-    <row r="143" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A143" s="2" t="s">
-        <v>306</v>
-      </c>
-      <c r="B143" s="2" t="s">
-        <v>307</v>
-      </c>
-      <c r="C143" s="2" t="s">
-        <v>308</v>
-      </c>
-      <c r="D143" s="2" t="s">
-        <v>428</v>
       </c>
     </row>
     <row r="144" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A144" s="2" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
       <c r="B144" s="2" t="s">
-        <v>311</v>
+        <v>307</v>
       </c>
       <c r="C144" s="2" t="s">
-        <v>312</v>
+        <v>308</v>
       </c>
       <c r="D144" s="2" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
     </row>
     <row r="145" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A145" s="2" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="B145" s="2" t="s">
-        <v>314</v>
+        <v>311</v>
       </c>
       <c r="C145" s="2" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="D145" s="2" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
     </row>
     <row r="146" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A146" s="2" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="B146" s="2" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="C146" s="2" t="s">
-        <v>316</v>
+        <v>313</v>
       </c>
       <c r="D146" s="2" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
     </row>
     <row r="147" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A147" s="2" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="B147" s="2" t="s">
-        <v>318</v>
+        <v>315</v>
       </c>
       <c r="C147" s="2" t="s">
-        <v>460</v>
+        <v>316</v>
       </c>
       <c r="D147" s="2" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
     </row>
     <row r="148" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A148" s="2" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="B148" s="2" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="C148" s="2" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="D148" s="2" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
     </row>
     <row r="149" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A149" s="2" t="s">
-        <v>448</v>
+        <v>319</v>
       </c>
       <c r="B149" s="2" t="s">
-        <v>448</v>
+        <v>320</v>
       </c>
       <c r="C149" s="2" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="D149" s="2" t="s">
-        <v>345</v>
+        <v>433</v>
       </c>
     </row>
     <row r="150" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A150" s="2" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="B150" s="2" t="s">
-        <v>450</v>
+        <v>448</v>
       </c>
       <c r="C150" s="2" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="D150" s="2" t="s">
-        <v>451</v>
+        <v>345</v>
       </c>
     </row>
     <row r="151" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A151" s="2" t="s">
-        <v>475</v>
+        <v>449</v>
       </c>
       <c r="B151" s="2" t="s">
-        <v>476</v>
+        <v>450</v>
       </c>
       <c r="C151" s="2" t="s">
-        <v>619</v>
+        <v>463</v>
       </c>
       <c r="D151" s="2" t="s">
-        <v>569</v>
+        <v>451</v>
       </c>
     </row>
     <row r="152" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A152" s="2" t="s">
-        <v>478</v>
+        <v>475</v>
       </c>
       <c r="B152" s="2" t="s">
-        <v>524</v>
+        <v>476</v>
       </c>
       <c r="C152" s="2" t="s">
-        <v>479</v>
+        <v>619</v>
       </c>
       <c r="D152" s="2" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
     </row>
     <row r="153" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A153" s="2" t="s">
-        <v>480</v>
+        <v>478</v>
       </c>
       <c r="B153" s="2" t="s">
-        <v>481</v>
+        <v>524</v>
       </c>
       <c r="C153" s="2" t="s">
-        <v>482</v>
+        <v>479</v>
       </c>
       <c r="D153" s="2" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
     </row>
     <row r="154" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A154" s="2" t="s">
-        <v>483</v>
+        <v>480</v>
       </c>
       <c r="B154" s="2" t="s">
-        <v>484</v>
+        <v>481</v>
       </c>
       <c r="C154" s="2" t="s">
-        <v>485</v>
+        <v>482</v>
       </c>
       <c r="D154" s="2" t="s">
-        <v>566</v>
+        <v>567</v>
       </c>
     </row>
     <row r="155" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A155" s="2" t="s">
-        <v>486</v>
+        <v>483</v>
       </c>
       <c r="B155" s="2" t="s">
-        <v>487</v>
+        <v>484</v>
       </c>
       <c r="C155" s="2" t="s">
-        <v>488</v>
+        <v>485</v>
       </c>
       <c r="D155" s="2" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
     </row>
     <row r="156" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A156" s="2" t="s">
-        <v>489</v>
+        <v>486</v>
       </c>
       <c r="B156" s="2" t="s">
-        <v>490</v>
+        <v>487</v>
       </c>
       <c r="C156" s="2" t="s">
-        <v>491</v>
+        <v>488</v>
       </c>
       <c r="D156" s="2" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
     </row>
     <row r="157" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A157" s="2" t="s">
-        <v>538</v>
+        <v>489</v>
       </c>
       <c r="B157" s="2" t="s">
-        <v>538</v>
+        <v>490</v>
       </c>
       <c r="C157" s="2" t="s">
-        <v>607</v>
+        <v>491</v>
       </c>
       <c r="D157" s="2" t="s">
-        <v>539</v>
+        <v>564</v>
       </c>
     </row>
     <row r="158" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A158" s="2" t="s">
-        <v>540</v>
+        <v>538</v>
       </c>
       <c r="B158" s="2" t="s">
-        <v>541</v>
+        <v>538</v>
       </c>
       <c r="C158" s="2" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="D158" s="2" t="s">
-        <v>542</v>
+        <v>539</v>
       </c>
     </row>
     <row r="159" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A159" s="2" t="s">
-        <v>492</v>
+        <v>540</v>
       </c>
       <c r="B159" s="2" t="s">
-        <v>493</v>
+        <v>541</v>
       </c>
       <c r="C159" s="2" t="s">
-        <v>494</v>
+        <v>608</v>
       </c>
       <c r="D159" s="2" t="s">
-        <v>563</v>
+        <v>542</v>
       </c>
     </row>
     <row r="160" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A160" s="2" t="s">
-        <v>495</v>
+        <v>492</v>
       </c>
       <c r="B160" s="2" t="s">
-        <v>496</v>
+        <v>493</v>
       </c>
       <c r="C160" s="2" t="s">
-        <v>497</v>
+        <v>494</v>
       </c>
       <c r="D160" s="2" t="s">
-        <v>562</v>
+        <v>563</v>
       </c>
     </row>
     <row r="161" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A161" s="2" t="s">
-        <v>498</v>
+        <v>495</v>
       </c>
       <c r="B161" s="2" t="s">
-        <v>499</v>
+        <v>496</v>
       </c>
       <c r="C161" s="2" t="s">
-        <v>500</v>
+        <v>497</v>
       </c>
       <c r="D161" s="2" t="s">
-        <v>561</v>
+        <v>562</v>
       </c>
     </row>
     <row r="162" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A162" s="2" t="s">
-        <v>501</v>
+        <v>498</v>
       </c>
       <c r="B162" s="2" t="s">
-        <v>501</v>
+        <v>499</v>
       </c>
       <c r="C162" s="2" t="s">
-        <v>502</v>
+        <v>500</v>
       </c>
       <c r="D162" s="2" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
     </row>
     <row r="163" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A163" s="2" t="s">
-        <v>503</v>
+        <v>501</v>
       </c>
       <c r="B163" s="2" t="s">
-        <v>503</v>
+        <v>501</v>
       </c>
       <c r="C163" s="2" t="s">
-        <v>504</v>
+        <v>502</v>
       </c>
       <c r="D163" s="2" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
     </row>
     <row r="164" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A164" s="2" t="s">
-        <v>505</v>
+        <v>503</v>
       </c>
       <c r="B164" s="2" t="s">
-        <v>505</v>
+        <v>503</v>
       </c>
       <c r="C164" s="2" t="s">
-        <v>506</v>
+        <v>504</v>
       </c>
       <c r="D164" s="2" t="s">
-        <v>558</v>
+        <v>559</v>
       </c>
     </row>
     <row r="165" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A165" s="2" t="s">
-        <v>507</v>
+        <v>505</v>
       </c>
       <c r="B165" s="2" t="s">
-        <v>507</v>
+        <v>505</v>
       </c>
       <c r="C165" s="2" t="s">
-        <v>508</v>
+        <v>506</v>
       </c>
       <c r="D165" s="2" t="s">
-        <v>557</v>
+        <v>558</v>
       </c>
     </row>
     <row r="166" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A166" s="2" t="s">
-        <v>570</v>
+        <v>507</v>
       </c>
       <c r="B166" s="2" t="s">
-        <v>571</v>
+        <v>507</v>
       </c>
       <c r="C166" s="2" t="s">
-        <v>609</v>
+        <v>508</v>
+      </c>
+      <c r="D166" s="2" t="s">
+        <v>557</v>
       </c>
     </row>
     <row r="167" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A167" s="2" t="s">
-        <v>572</v>
+        <v>570</v>
       </c>
       <c r="B167" s="2" t="s">
-        <v>573</v>
+        <v>571</v>
       </c>
       <c r="C167" s="2" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
     </row>
     <row r="168" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A168" s="2" t="s">
-        <v>574</v>
+        <v>572</v>
       </c>
       <c r="B168" s="2" t="s">
-        <v>575</v>
+        <v>573</v>
       </c>
       <c r="C168" s="2" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
     </row>
     <row r="169" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A169" s="2" t="s">
-        <v>576</v>
+        <v>574</v>
       </c>
       <c r="B169" s="2" t="s">
-        <v>577</v>
+        <v>575</v>
       </c>
       <c r="C169" s="2" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
     </row>
     <row r="170" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A170" s="2" t="s">
-        <v>578</v>
+        <v>576</v>
       </c>
       <c r="B170" s="2" t="s">
-        <v>579</v>
+        <v>577</v>
       </c>
       <c r="C170" s="2" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
     </row>
     <row r="171" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A171" s="2" t="s">
-        <v>580</v>
+        <v>578</v>
       </c>
       <c r="B171" s="2" t="s">
-        <v>581</v>
+        <v>579</v>
       </c>
       <c r="C171" s="2" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
     </row>
     <row r="172" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A172" s="2" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
       <c r="B172" s="2" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="C172" s="2" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
     </row>
     <row r="173" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A173" s="2" t="s">
-        <v>584</v>
+        <v>582</v>
       </c>
       <c r="B173" s="2" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="C173" s="2" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
     </row>
     <row r="174" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A174" s="2" t="s">
-        <v>586</v>
+        <v>584</v>
       </c>
       <c r="B174" s="2" t="s">
-        <v>587</v>
+        <v>585</v>
       </c>
       <c r="C174" s="2" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
     </row>
     <row r="175" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A175" s="2" t="s">
-        <v>588</v>
+        <v>586</v>
       </c>
       <c r="B175" s="2" t="s">
-        <v>589</v>
+        <v>587</v>
       </c>
       <c r="C175" s="2" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
     </row>
     <row r="176" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A176" s="2" t="s">
-        <v>620</v>
+        <v>588</v>
       </c>
       <c r="B176" s="2" t="s">
-        <v>621</v>
+        <v>589</v>
       </c>
       <c r="C176" s="2" t="s">
-        <v>622</v>
+        <v>618</v>
       </c>
     </row>
     <row r="177" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A177" s="2" t="s">
-        <v>623</v>
+        <v>620</v>
       </c>
       <c r="B177" s="2" t="s">
-        <v>623</v>
+        <v>621</v>
       </c>
       <c r="C177" s="2" t="s">
-        <v>624</v>
+        <v>622</v>
       </c>
     </row>
     <row r="178" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A178" s="2" t="s">
-        <v>625</v>
+        <v>623</v>
       </c>
       <c r="B178" s="2" t="s">
-        <v>625</v>
+        <v>623</v>
       </c>
       <c r="C178" s="2" t="s">
-        <v>627</v>
+        <v>624</v>
       </c>
     </row>
     <row r="179" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A179" s="2" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="B179" s="2" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="C179" s="2" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
     </row>
     <row r="180" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A180" s="2" t="s">
-        <v>629</v>
+        <v>626</v>
       </c>
       <c r="B180" s="2" t="s">
-        <v>630</v>
+        <v>626</v>
       </c>
       <c r="C180" s="2" t="s">
-        <v>631</v>
+        <v>628</v>
       </c>
     </row>
     <row r="181" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A181" s="2" t="s">
-        <v>632</v>
-      </c>
-      <c r="B181" s="4" t="s">
-        <v>633</v>
-      </c>
-      <c r="C181" s="4" t="s">
-        <v>634</v>
+        <v>629</v>
+      </c>
+      <c r="B181" s="2" t="s">
+        <v>630</v>
+      </c>
+      <c r="C181" s="2" t="s">
+        <v>631</v>
       </c>
     </row>
     <row r="182" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A182" s="2" t="s">
-        <v>638</v>
-      </c>
-      <c r="B182" s="2" t="s">
-        <v>639</v>
-      </c>
-      <c r="C182" s="2" t="s">
-        <v>640</v>
+        <v>632</v>
+      </c>
+      <c r="B182" s="4" t="s">
+        <v>633</v>
+      </c>
+      <c r="C182" s="4" t="s">
+        <v>634</v>
       </c>
     </row>
     <row r="183" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A183" s="2" t="s">
-        <v>641</v>
+        <v>638</v>
       </c>
       <c r="B183" s="2" t="s">
-        <v>641</v>
+        <v>639</v>
       </c>
       <c r="C183" s="2" t="s">
-        <v>642</v>
+        <v>640</v>
       </c>
     </row>
     <row r="184" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A184" s="2" t="s">
-        <v>643</v>
+        <v>641</v>
       </c>
       <c r="B184" s="2" t="s">
-        <v>644</v>
+        <v>641</v>
       </c>
       <c r="C184" s="2" t="s">
-        <v>645</v>
+        <v>642</v>
       </c>
     </row>
     <row r="185" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A185" s="2" t="s">
-        <v>646</v>
+        <v>643</v>
       </c>
       <c r="B185" s="2" t="s">
-        <v>647</v>
+        <v>644</v>
       </c>
       <c r="C185" s="2" t="s">
-        <v>648</v>
+        <v>645</v>
       </c>
     </row>
     <row r="186" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A186" s="2" t="s">
-        <v>649</v>
+        <v>646</v>
       </c>
       <c r="B186" s="2" t="s">
-        <v>650</v>
+        <v>647</v>
       </c>
       <c r="C186" s="2" t="s">
-        <v>651</v>
+        <v>648</v>
       </c>
     </row>
     <row r="187" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A187" s="2" t="s">
-        <v>652</v>
+        <v>649</v>
       </c>
       <c r="B187" s="2" t="s">
-        <v>653</v>
+        <v>650</v>
       </c>
       <c r="C187" s="2" t="s">
-        <v>654</v>
+        <v>651</v>
       </c>
     </row>
     <row r="188" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A188" s="2" t="s">
-        <v>655</v>
+        <v>652</v>
       </c>
       <c r="B188" s="2" t="s">
-        <v>655</v>
+        <v>653</v>
       </c>
       <c r="C188" s="2" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
     </row>
     <row r="189" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A189" s="2" t="s">
-        <v>657</v>
+        <v>655</v>
       </c>
       <c r="B189" s="2" t="s">
-        <v>658</v>
+        <v>655</v>
       </c>
       <c r="C189" s="2" t="s">
-        <v>659</v>
+        <v>656</v>
       </c>
     </row>
     <row r="190" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A190" s="2" t="s">
-        <v>666</v>
-      </c>
-      <c r="B190" s="4" t="s">
-        <v>667</v>
-      </c>
-      <c r="C190" s="4" t="s">
-        <v>668</v>
+        <v>657</v>
+      </c>
+      <c r="B190" s="2" t="s">
+        <v>658</v>
+      </c>
+      <c r="C190" s="2" t="s">
+        <v>659</v>
       </c>
     </row>
     <row r="191" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A191" s="2" t="s">
-        <v>669</v>
-      </c>
-      <c r="B191" s="2" t="s">
-        <v>670</v>
-      </c>
-      <c r="C191" s="2" t="s">
-        <v>671</v>
+        <v>666</v>
+      </c>
+      <c r="B191" s="4" t="s">
+        <v>667</v>
+      </c>
+      <c r="C191" s="4" t="s">
+        <v>668</v>
       </c>
     </row>
     <row r="192" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A192" s="2" t="s">
-        <v>675</v>
+        <v>669</v>
       </c>
       <c r="B192" s="2" t="s">
-        <v>676</v>
+        <v>670</v>
       </c>
       <c r="C192" s="2" t="s">
-        <v>677</v>
+        <v>671</v>
       </c>
     </row>
     <row r="193" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A193" s="2" t="s">
-        <v>678</v>
+        <v>675</v>
       </c>
       <c r="B193" s="2" t="s">
-        <v>679</v>
+        <v>676</v>
       </c>
       <c r="C193" s="2" t="s">
-        <v>680</v>
+        <v>677</v>
       </c>
     </row>
     <row r="194" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A194" s="2" t="s">
-        <v>681</v>
+        <v>678</v>
       </c>
       <c r="B194" s="2" t="s">
-        <v>682</v>
+        <v>679</v>
       </c>
       <c r="C194" s="2" t="s">
-        <v>683</v>
+        <v>680</v>
       </c>
     </row>
     <row r="195" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A195" s="2" t="s">
-        <v>684</v>
+        <v>681</v>
       </c>
       <c r="B195" s="2" t="s">
-        <v>685</v>
+        <v>682</v>
       </c>
       <c r="C195" s="2" t="s">
-        <v>686</v>
+        <v>683</v>
       </c>
     </row>
     <row r="196" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A196" s="2" t="s">
-        <v>687</v>
+        <v>684</v>
       </c>
       <c r="B196" s="2" t="s">
-        <v>688</v>
+        <v>685</v>
       </c>
       <c r="C196" s="2" t="s">
-        <v>689</v>
+        <v>686</v>
       </c>
     </row>
     <row r="197" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A197" s="2" t="s">
-        <v>690</v>
-      </c>
-      <c r="B197" s="4" t="s">
-        <v>694</v>
-      </c>
-      <c r="C197" s="4" t="s">
-        <v>704</v>
+        <v>687</v>
+      </c>
+      <c r="B197" s="2" t="s">
+        <v>688</v>
+      </c>
+      <c r="C197" s="2" t="s">
+        <v>689</v>
       </c>
     </row>
     <row r="198" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A198" s="2" t="s">
-        <v>691</v>
-      </c>
-      <c r="B198" s="2" t="s">
-        <v>697</v>
-      </c>
-      <c r="C198" s="2" t="s">
-        <v>710</v>
+        <v>690</v>
+      </c>
+      <c r="B198" s="4" t="s">
+        <v>694</v>
+      </c>
+      <c r="C198" s="4" t="s">
+        <v>704</v>
       </c>
     </row>
     <row r="199" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A199" s="2" t="s">
-        <v>693</v>
-      </c>
-      <c r="B199" s="4" t="s">
-        <v>695</v>
-      </c>
-      <c r="C199" s="4" t="s">
-        <v>705</v>
+        <v>691</v>
+      </c>
+      <c r="B199" s="2" t="s">
+        <v>697</v>
+      </c>
+      <c r="C199" s="2" t="s">
+        <v>710</v>
       </c>
     </row>
     <row r="200" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A200" s="2" t="s">
-        <v>692</v>
+        <v>693</v>
       </c>
       <c r="B200" s="4" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
       <c r="C200" s="4" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
     </row>
     <row r="201" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A201" s="2" t="s">
-        <v>699</v>
-      </c>
-      <c r="B201" s="2" t="s">
-        <v>698</v>
-      </c>
-      <c r="C201" s="2" t="s">
-        <v>707</v>
+        <v>692</v>
+      </c>
+      <c r="B201" s="4" t="s">
+        <v>696</v>
+      </c>
+      <c r="C201" s="4" t="s">
+        <v>706</v>
       </c>
     </row>
     <row r="202" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A202" s="2" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="B202" s="2" t="s">
-        <v>702</v>
+        <v>698</v>
       </c>
       <c r="C202" s="2" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
     </row>
     <row r="203" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A203" s="2" t="s">
-        <v>701</v>
+        <v>700</v>
       </c>
       <c r="B203" s="2" t="s">
-        <v>703</v>
+        <v>702</v>
       </c>
       <c r="C203" s="2" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
     </row>
     <row r="204" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A204" s="2" t="s">
-        <v>711</v>
+        <v>701</v>
       </c>
       <c r="B204" s="2" t="s">
-        <v>711</v>
+        <v>703</v>
       </c>
       <c r="C204" s="2" t="s">
-        <v>712</v>
+        <v>709</v>
       </c>
     </row>
     <row r="205" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A205" s="2" t="s">
-        <v>713</v>
+        <v>711</v>
       </c>
       <c r="B205" s="2" t="s">
-        <v>714</v>
+        <v>711</v>
       </c>
       <c r="C205" s="2" t="s">
-        <v>715</v>
+        <v>712</v>
       </c>
     </row>
     <row r="206" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A206" s="2" t="s">
-        <v>716</v>
+        <v>713</v>
       </c>
       <c r="B206" s="2" t="s">
-        <v>717</v>
+        <v>714</v>
       </c>
       <c r="C206" s="2" t="s">
-        <v>718</v>
+        <v>715</v>
       </c>
     </row>
     <row r="207" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A207" s="2" t="s">
+        <v>716</v>
+      </c>
+      <c r="B207" s="2" t="s">
+        <v>717</v>
+      </c>
+      <c r="C207" s="2" t="s">
+        <v>718</v>
+      </c>
+    </row>
+    <row r="208" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A208" s="2" t="s">
         <v>719</v>
       </c>
-      <c r="B207" s="2" t="s">
+      <c r="B208" s="2" t="s">
         <v>720</v>
       </c>
-      <c r="C207" s="2" t="s">
+      <c r="C208" s="2" t="s">
         <v>721</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Added Power Slots (useless for now, no events yet).
</commit_message>
<xml_diff>
--- a/Translations/Translations.xlsx
+++ b/Translations/Translations.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programacion\MelonLoader\FS_LevelEditor\Translations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1528DA4C-287B-4FC8-9C1C-C925C8734DFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB352B10-965D-4524-9151-D1CF1499DFD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{F5C22481-FF1A-482C-BF7E-EB5A7718AF49}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1418" uniqueCount="725">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1421" uniqueCount="728">
   <si>
     <t>ID</t>
   </si>
@@ -2213,6 +2213,15 @@
   </si>
   <si>
     <t>Núcleo de Energía</t>
+  </si>
+  <si>
+    <t>object.POWER_SLOT</t>
+  </si>
+  <si>
+    <t>Power Slot</t>
+  </si>
+  <si>
+    <t>Entrada de Energía</t>
   </si>
 </sst>
 </file>
@@ -2612,7 +2621,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6961A5F-F8EA-4989-8112-A0ACE51D011E}">
   <sheetPr codeName="Hoja1"/>
-  <dimension ref="A1:D208"/>
+  <dimension ref="A1:D209"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="37" style="2" customWidth="1"/>
@@ -3475,1910 +3484,1921 @@
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63" s="2" t="s">
-        <v>69</v>
+        <v>725</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>69</v>
+        <v>726</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="D63" s="2" t="s">
-        <v>364</v>
+        <v>727</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" s="2" t="s">
-        <v>443</v>
+        <v>69</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>443</v>
+        <v>69</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>601</v>
+        <v>101</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>552</v>
+        <v>364</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A65" s="2" t="s">
-        <v>456</v>
+        <v>443</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>456</v>
+        <v>443</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>456</v>
+        <v>601</v>
       </c>
       <c r="D65" s="2" t="s">
-        <v>457</v>
+        <v>552</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66" s="2" t="s">
-        <v>105</v>
+        <v>456</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>2</v>
+        <v>456</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>102</v>
+        <v>456</v>
       </c>
       <c r="D66" s="2" t="s">
-        <v>365</v>
+        <v>457</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A67" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D67" s="2" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A68" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D68" s="2" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A69" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>111</v>
+        <v>4</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="D69" s="2" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A70" s="2" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C70" s="2" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="D70" s="2" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A71" s="2" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="D71" s="2" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A72" s="2" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="D72" s="2" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A73" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="C73" s="2" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D73" s="2" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A74" s="2" t="s">
-        <v>445</v>
+        <v>118</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>446</v>
+        <v>122</v>
       </c>
       <c r="C74" s="2" t="s">
-        <v>459</v>
+        <v>121</v>
       </c>
       <c r="D74" s="2" t="s">
-        <v>447</v>
+        <v>370</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A75" s="2" t="s">
-        <v>512</v>
+        <v>445</v>
       </c>
       <c r="B75" s="2" t="s">
-        <v>513</v>
+        <v>446</v>
       </c>
       <c r="C75" s="2" t="s">
-        <v>602</v>
+        <v>459</v>
       </c>
       <c r="D75" s="2" t="s">
-        <v>514</v>
+        <v>447</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A76" s="2" t="s">
-        <v>518</v>
+        <v>512</v>
       </c>
       <c r="B76" s="2" t="s">
-        <v>519</v>
+        <v>513</v>
       </c>
       <c r="C76" s="2" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="D76" s="2" t="s">
-        <v>520</v>
+        <v>514</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A77" s="2" t="s">
-        <v>521</v>
+        <v>518</v>
       </c>
       <c r="B77" s="2" t="s">
-        <v>522</v>
+        <v>519</v>
       </c>
       <c r="C77" s="2" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="D77" s="2" t="s">
-        <v>523</v>
+        <v>520</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A78" s="2" t="s">
-        <v>532</v>
+        <v>521</v>
       </c>
       <c r="B78" s="2" t="s">
-        <v>533</v>
+        <v>522</v>
       </c>
       <c r="C78" s="2" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="D78" s="2" t="s">
-        <v>534</v>
+        <v>523</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A79" s="2" t="s">
-        <v>537</v>
+        <v>532</v>
       </c>
       <c r="B79" s="2" t="s">
-        <v>535</v>
+        <v>533</v>
       </c>
       <c r="C79" s="2" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="D79" s="2" t="s">
-        <v>536</v>
+        <v>534</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
-        <v>154</v>
+        <v>537</v>
       </c>
       <c r="B80" s="2" t="s">
-        <v>155</v>
+        <v>535</v>
       </c>
       <c r="C80" s="2" t="s">
-        <v>156</v>
+        <v>606</v>
       </c>
       <c r="D80" s="2" t="s">
-        <v>371</v>
+        <v>536</v>
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A81" s="2" t="s">
-        <v>164</v>
+        <v>154</v>
       </c>
       <c r="B81" s="2" t="s">
-        <v>165</v>
+        <v>155</v>
       </c>
       <c r="C81" s="2" t="s">
-        <v>166</v>
+        <v>156</v>
       </c>
       <c r="D81" s="2" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A82" s="2" t="s">
-        <v>157</v>
+        <v>164</v>
       </c>
       <c r="B82" s="2" t="s">
-        <v>158</v>
+        <v>165</v>
       </c>
       <c r="C82" s="2" t="s">
-        <v>159</v>
+        <v>166</v>
       </c>
       <c r="D82" s="2" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A83" s="2" t="s">
-        <v>167</v>
+        <v>157</v>
       </c>
       <c r="B83" s="2" t="s">
-        <v>168</v>
+        <v>158</v>
       </c>
       <c r="C83" s="2" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="D83" s="2" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A84" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="B84" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="C84" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="D84" s="2" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A85" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="B84" s="2" t="s">
+      <c r="B85" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="C84" s="2" t="s">
+      <c r="C85" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="D84" s="2" t="s">
+      <c r="D85" s="2" t="s">
         <v>375</v>
       </c>
     </row>
-    <row r="85" spans="1:4" ht="45" x14ac:dyDescent="0.25">
-      <c r="A85" s="2" t="s">
+    <row r="86" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="A86" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="B85" s="2" t="s">
+      <c r="B86" s="2" t="s">
         <v>163</v>
       </c>
-      <c r="C85" s="2" t="s">
+      <c r="C86" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="D85" s="2" t="s">
+      <c r="D86" s="2" t="s">
         <v>376</v>
-      </c>
-    </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A86" s="2" t="s">
-        <v>153</v>
-      </c>
-      <c r="B86" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="C86" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="D86" s="2" t="s">
-        <v>328</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A87" s="2" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="B87" s="2" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="C87" s="2" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="D87" s="2" t="s">
-        <v>377</v>
+        <v>328</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A88" s="2" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="B88" s="2" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="C88" s="2" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="D88" s="2" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A89" s="2" t="s">
-        <v>172</v>
+        <v>150</v>
       </c>
       <c r="B89" s="2" t="s">
-        <v>170</v>
+        <v>151</v>
       </c>
       <c r="C89" s="2" t="s">
-        <v>171</v>
+        <v>152</v>
       </c>
       <c r="D89" s="2" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A90" s="2" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B90" s="2" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="C90" s="2" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="D90" s="2" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A91" s="2" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="B91" s="2" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="C91" s="2" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="D91" s="2" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A92" s="2" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="B92" s="2" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="C92" s="2" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="D92" s="2" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A93" s="2" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="B93" s="2" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="C93" s="2" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="D93" s="2" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A94" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="B94" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="C94" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="D94" s="2" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="95" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A95" s="2" t="s">
         <v>243</v>
       </c>
-      <c r="B94" s="2" t="s">
+      <c r="B95" s="2" t="s">
         <v>243</v>
       </c>
-      <c r="C94" s="2" t="s">
+      <c r="C95" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="D94" s="2" t="s">
+      <c r="D95" s="2" t="s">
         <v>384</v>
       </c>
     </row>
-    <row r="95" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A95" s="2" t="s">
+    <row r="96" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A96" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="B95" s="1" t="s">
+      <c r="B96" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="C95" s="2" t="s">
+      <c r="C96" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="D95" s="2" t="s">
+      <c r="D96" s="2" t="s">
         <v>385</v>
-      </c>
-    </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A96" s="2" t="s">
-        <v>182</v>
-      </c>
-      <c r="B96" s="2" t="s">
-        <v>183</v>
-      </c>
-      <c r="C96" s="2" t="s">
-        <v>183</v>
-      </c>
-      <c r="D96" s="2" t="s">
-        <v>386</v>
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A97" s="2" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="B97" s="2" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C97" s="2" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="D97" s="2" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A98" s="2" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="B98" s="2" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="C98" s="2" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="D98" s="2" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A99" s="2" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="B99" s="2" t="s">
-        <v>525</v>
+        <v>186</v>
       </c>
       <c r="C99" s="2" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="D99" s="2" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A100" s="2" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="B100" s="2" t="s">
-        <v>190</v>
+        <v>525</v>
       </c>
       <c r="C100" s="2" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="D100" s="2" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A101" s="2" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="B101" s="2" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="C101" s="2" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="D101" s="2" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A102" s="2" t="s">
-        <v>434</v>
-      </c>
-      <c r="B102" s="4" t="s">
-        <v>435</v>
-      </c>
-      <c r="C102" s="4" t="s">
-        <v>436</v>
-      </c>
-      <c r="D102" s="4" t="s">
-        <v>591</v>
+        <v>192</v>
+      </c>
+      <c r="B102" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="C102" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="D102" s="2" t="s">
+        <v>391</v>
       </c>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A103" s="2" t="s">
-        <v>437</v>
+        <v>434</v>
       </c>
       <c r="B103" s="4" t="s">
-        <v>438</v>
+        <v>435</v>
       </c>
       <c r="C103" s="4" t="s">
-        <v>439</v>
+        <v>436</v>
       </c>
       <c r="D103" s="4" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A104" s="2" t="s">
-        <v>473</v>
+        <v>437</v>
       </c>
       <c r="B104" s="4" t="s">
-        <v>590</v>
+        <v>438</v>
       </c>
       <c r="C104" s="4" t="s">
-        <v>474</v>
+        <v>439</v>
       </c>
       <c r="D104" s="4" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A105" s="2" t="s">
-        <v>195</v>
-      </c>
-      <c r="B105" s="2" t="s">
-        <v>196</v>
-      </c>
-      <c r="C105" s="2" t="s">
-        <v>197</v>
-      </c>
-      <c r="D105" s="2" t="s">
-        <v>392</v>
+        <v>473</v>
+      </c>
+      <c r="B105" s="4" t="s">
+        <v>590</v>
+      </c>
+      <c r="C105" s="4" t="s">
+        <v>474</v>
+      </c>
+      <c r="D105" s="4" t="s">
+        <v>593</v>
       </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A106" s="2" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="B106" s="2" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="C106" s="2" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="D106" s="2" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A107" s="2" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="B107" s="2" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="C107" s="2" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="D107" s="2" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A108" s="2" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="B108" s="2" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="C108" s="2" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="D108" s="2" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A109" s="2" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="B109" s="2" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="C109" s="2" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="D109" s="2" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A110" s="2" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B110" s="2" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="C110" s="2" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="D110" s="2" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A111" s="2" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="B111" s="2" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="C111" s="2" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="D111" s="2" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A112" s="2" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="B112" s="2" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="C112" s="2" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="D112" s="2" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A113" s="2" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="B113" s="2" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="C113" s="2" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="D113" s="2" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A114" s="2" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="B114" s="2" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="C114" s="2" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="D114" s="2" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A115" s="2" t="s">
-        <v>292</v>
+        <v>220</v>
       </c>
       <c r="B115" s="2" t="s">
-        <v>292</v>
+        <v>219</v>
       </c>
       <c r="C115" s="2" t="s">
-        <v>293</v>
+        <v>218</v>
       </c>
       <c r="D115" s="2" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A116" s="2" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="B116" s="2" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="C116" s="2" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
       <c r="D116" s="2" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A117" s="2" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
       <c r="B117" s="2" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="C117" s="2" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="D117" s="2" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A118" s="2" t="s">
-        <v>221</v>
+        <v>297</v>
       </c>
       <c r="B118" s="2" t="s">
-        <v>221</v>
+        <v>298</v>
       </c>
       <c r="C118" s="2" t="s">
-        <v>222</v>
+        <v>299</v>
       </c>
       <c r="D118" s="2" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
     </row>
     <row r="119" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A119" s="2" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="B119" s="2" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="C119" s="2" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="D119" s="2" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A120" s="2" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="B120" s="2" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="C120" s="2" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="D120" s="2" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A121" s="2" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="B121" s="2" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="C121" s="2" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="D121" s="2" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A122" s="2" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B122" s="2" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="C122" s="2" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="D122" s="2" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
     </row>
     <row r="123" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A123" s="2" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="B123" s="2" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="C123" s="2" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="D123" s="2" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
     </row>
     <row r="124" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A124" s="2" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="B124" s="2" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="C124" s="2" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="D124" s="2" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
     </row>
     <row r="125" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A125" s="2" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="B125" s="2" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="C125" s="2" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="D125" s="2" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
     </row>
     <row r="126" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A126" s="2" t="s">
-        <v>300</v>
+        <v>237</v>
       </c>
       <c r="B126" s="2" t="s">
-        <v>301</v>
+        <v>238</v>
       </c>
       <c r="C126" s="2" t="s">
-        <v>302</v>
+        <v>239</v>
       </c>
       <c r="D126" s="2" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
     </row>
     <row r="127" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A127" s="2" t="s">
-        <v>240</v>
+        <v>300</v>
       </c>
       <c r="B127" s="2" t="s">
-        <v>241</v>
+        <v>301</v>
       </c>
       <c r="C127" s="2" t="s">
-        <v>242</v>
+        <v>302</v>
       </c>
       <c r="D127" s="2" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
     </row>
     <row r="128" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A128" s="2" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="B128" s="2" t="s">
-        <v>252</v>
+        <v>241</v>
       </c>
       <c r="C128" s="2" t="s">
-        <v>251</v>
+        <v>242</v>
       </c>
       <c r="D128" s="2" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="129" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A129" s="2" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B129" s="2" t="s">
-        <v>245</v>
+        <v>252</v>
       </c>
       <c r="C129" s="2" t="s">
-        <v>246</v>
+        <v>251</v>
       </c>
       <c r="D129" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
     </row>
     <row r="130" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A130" s="2" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="B130" s="2" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="C130" s="2" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="D130" s="2" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
     </row>
     <row r="131" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A131" s="2" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="B131" s="2" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="C131" s="2" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="D131" s="2" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
     </row>
     <row r="132" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A132" s="2" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="B132" s="2" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="C132" s="2" t="s">
-        <v>255</v>
+        <v>250</v>
       </c>
       <c r="D132" s="2" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
     </row>
     <row r="133" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A133" s="2" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="B133" s="2" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="C133" s="2" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="D133" s="2" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
     </row>
     <row r="134" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A134" s="2" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="B134" s="2" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="C134" s="2" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="D134" s="2" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
     </row>
     <row r="135" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A135" s="2" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="B135" s="2" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="C135" s="2" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="D135" s="2" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="136" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A136" s="2" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="B136" s="2" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="C136" s="2" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="D136" s="2" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
     </row>
     <row r="137" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A137" s="2" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="B137" s="2" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="C137" s="2" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="D137" s="2" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
     </row>
     <row r="138" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A138" s="2" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="B138" s="2" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="C138" s="2" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="D138" s="2" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
     </row>
     <row r="139" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A139" s="2" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="B139" s="2" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="C139" s="2" t="s">
-        <v>273</v>
+        <v>269</v>
       </c>
       <c r="D139" s="2" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
     </row>
     <row r="140" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A140" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="B140" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="C140" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="D140" s="2" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="141" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A141" s="2" t="s">
         <v>271</v>
       </c>
-      <c r="B140" s="2" t="s">
+      <c r="B141" s="2" t="s">
         <v>271</v>
       </c>
-      <c r="C140" s="2" t="s">
+      <c r="C141" s="2" t="s">
         <v>272</v>
       </c>
-      <c r="D140" s="2" t="s">
+      <c r="D141" s="2" t="s">
         <v>427</v>
       </c>
     </row>
-    <row r="141" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A141" s="2" t="s">
+    <row r="142" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A142" s="2" t="s">
         <v>274</v>
       </c>
-      <c r="B141" s="2" t="s">
+      <c r="B142" s="2" t="s">
         <v>276</v>
       </c>
-      <c r="C141" s="2" t="s">
+      <c r="C142" s="2" t="s">
         <v>279</v>
       </c>
     </row>
-    <row r="142" spans="1:4" ht="45" x14ac:dyDescent="0.25">
-      <c r="A142" s="2" t="s">
+    <row r="143" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="A143" s="2" t="s">
         <v>275</v>
       </c>
-      <c r="B142" s="2" t="s">
+      <c r="B143" s="2" t="s">
         <v>277</v>
       </c>
-      <c r="C142" s="2" t="s">
+      <c r="C143" s="2" t="s">
         <v>278</v>
       </c>
     </row>
-    <row r="143" spans="1:4" ht="75" x14ac:dyDescent="0.25">
-      <c r="A143" s="2" t="s">
+    <row r="144" spans="1:4" ht="75" x14ac:dyDescent="0.25">
+      <c r="A144" s="2" t="s">
         <v>289</v>
       </c>
-      <c r="B143" s="2" t="s">
+      <c r="B144" s="2" t="s">
         <v>290</v>
       </c>
-      <c r="C143" s="2" t="s">
+      <c r="C144" s="2" t="s">
         <v>291</v>
-      </c>
-    </row>
-    <row r="144" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A144" s="2" t="s">
-        <v>306</v>
-      </c>
-      <c r="B144" s="2" t="s">
-        <v>307</v>
-      </c>
-      <c r="C144" s="2" t="s">
-        <v>308</v>
-      </c>
-      <c r="D144" s="2" t="s">
-        <v>428</v>
       </c>
     </row>
     <row r="145" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A145" s="2" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
       <c r="B145" s="2" t="s">
-        <v>311</v>
+        <v>307</v>
       </c>
       <c r="C145" s="2" t="s">
-        <v>312</v>
+        <v>308</v>
       </c>
       <c r="D145" s="2" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
     </row>
     <row r="146" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A146" s="2" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="B146" s="2" t="s">
-        <v>314</v>
+        <v>311</v>
       </c>
       <c r="C146" s="2" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="D146" s="2" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
     </row>
     <row r="147" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A147" s="2" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="B147" s="2" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="C147" s="2" t="s">
-        <v>316</v>
+        <v>313</v>
       </c>
       <c r="D147" s="2" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
     </row>
     <row r="148" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A148" s="2" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="B148" s="2" t="s">
-        <v>318</v>
+        <v>315</v>
       </c>
       <c r="C148" s="2" t="s">
-        <v>460</v>
+        <v>316</v>
       </c>
       <c r="D148" s="2" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
     </row>
     <row r="149" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A149" s="2" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="B149" s="2" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="C149" s="2" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="D149" s="2" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
     </row>
     <row r="150" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A150" s="2" t="s">
-        <v>448</v>
+        <v>319</v>
       </c>
       <c r="B150" s="2" t="s">
-        <v>448</v>
+        <v>320</v>
       </c>
       <c r="C150" s="2" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="D150" s="2" t="s">
-        <v>345</v>
+        <v>433</v>
       </c>
     </row>
     <row r="151" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A151" s="2" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="B151" s="2" t="s">
-        <v>450</v>
+        <v>448</v>
       </c>
       <c r="C151" s="2" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="D151" s="2" t="s">
-        <v>451</v>
+        <v>345</v>
       </c>
     </row>
     <row r="152" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A152" s="2" t="s">
-        <v>475</v>
+        <v>449</v>
       </c>
       <c r="B152" s="2" t="s">
-        <v>476</v>
+        <v>450</v>
       </c>
       <c r="C152" s="2" t="s">
-        <v>619</v>
+        <v>463</v>
       </c>
       <c r="D152" s="2" t="s">
-        <v>569</v>
+        <v>451</v>
       </c>
     </row>
     <row r="153" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A153" s="2" t="s">
-        <v>478</v>
+        <v>475</v>
       </c>
       <c r="B153" s="2" t="s">
-        <v>524</v>
+        <v>476</v>
       </c>
       <c r="C153" s="2" t="s">
-        <v>479</v>
+        <v>619</v>
       </c>
       <c r="D153" s="2" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
     </row>
     <row r="154" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A154" s="2" t="s">
-        <v>480</v>
+        <v>478</v>
       </c>
       <c r="B154" s="2" t="s">
-        <v>481</v>
+        <v>524</v>
       </c>
       <c r="C154" s="2" t="s">
-        <v>482</v>
+        <v>479</v>
       </c>
       <c r="D154" s="2" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
     </row>
     <row r="155" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A155" s="2" t="s">
-        <v>483</v>
+        <v>480</v>
       </c>
       <c r="B155" s="2" t="s">
-        <v>484</v>
+        <v>481</v>
       </c>
       <c r="C155" s="2" t="s">
-        <v>485</v>
+        <v>482</v>
       </c>
       <c r="D155" s="2" t="s">
-        <v>566</v>
+        <v>567</v>
       </c>
     </row>
     <row r="156" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A156" s="2" t="s">
-        <v>486</v>
+        <v>483</v>
       </c>
       <c r="B156" s="2" t="s">
-        <v>487</v>
+        <v>484</v>
       </c>
       <c r="C156" s="2" t="s">
-        <v>488</v>
+        <v>485</v>
       </c>
       <c r="D156" s="2" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
     </row>
     <row r="157" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A157" s="2" t="s">
-        <v>489</v>
+        <v>486</v>
       </c>
       <c r="B157" s="2" t="s">
-        <v>490</v>
+        <v>487</v>
       </c>
       <c r="C157" s="2" t="s">
-        <v>491</v>
+        <v>488</v>
       </c>
       <c r="D157" s="2" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
     </row>
     <row r="158" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A158" s="2" t="s">
-        <v>538</v>
+        <v>489</v>
       </c>
       <c r="B158" s="2" t="s">
-        <v>538</v>
+        <v>490</v>
       </c>
       <c r="C158" s="2" t="s">
-        <v>607</v>
+        <v>491</v>
       </c>
       <c r="D158" s="2" t="s">
-        <v>539</v>
+        <v>564</v>
       </c>
     </row>
     <row r="159" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A159" s="2" t="s">
-        <v>540</v>
+        <v>538</v>
       </c>
       <c r="B159" s="2" t="s">
-        <v>541</v>
+        <v>538</v>
       </c>
       <c r="C159" s="2" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="D159" s="2" t="s">
-        <v>542</v>
+        <v>539</v>
       </c>
     </row>
     <row r="160" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A160" s="2" t="s">
-        <v>492</v>
+        <v>540</v>
       </c>
       <c r="B160" s="2" t="s">
-        <v>493</v>
+        <v>541</v>
       </c>
       <c r="C160" s="2" t="s">
-        <v>494</v>
+        <v>608</v>
       </c>
       <c r="D160" s="2" t="s">
-        <v>563</v>
+        <v>542</v>
       </c>
     </row>
     <row r="161" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A161" s="2" t="s">
-        <v>495</v>
+        <v>492</v>
       </c>
       <c r="B161" s="2" t="s">
-        <v>496</v>
+        <v>493</v>
       </c>
       <c r="C161" s="2" t="s">
-        <v>497</v>
+        <v>494</v>
       </c>
       <c r="D161" s="2" t="s">
-        <v>562</v>
+        <v>563</v>
       </c>
     </row>
     <row r="162" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A162" s="2" t="s">
-        <v>498</v>
+        <v>495</v>
       </c>
       <c r="B162" s="2" t="s">
-        <v>499</v>
+        <v>496</v>
       </c>
       <c r="C162" s="2" t="s">
-        <v>500</v>
+        <v>497</v>
       </c>
       <c r="D162" s="2" t="s">
-        <v>561</v>
+        <v>562</v>
       </c>
     </row>
     <row r="163" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A163" s="2" t="s">
-        <v>501</v>
+        <v>498</v>
       </c>
       <c r="B163" s="2" t="s">
-        <v>501</v>
+        <v>499</v>
       </c>
       <c r="C163" s="2" t="s">
-        <v>502</v>
+        <v>500</v>
       </c>
       <c r="D163" s="2" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
     </row>
     <row r="164" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A164" s="2" t="s">
-        <v>503</v>
+        <v>501</v>
       </c>
       <c r="B164" s="2" t="s">
-        <v>503</v>
+        <v>501</v>
       </c>
       <c r="C164" s="2" t="s">
-        <v>504</v>
+        <v>502</v>
       </c>
       <c r="D164" s="2" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
     </row>
     <row r="165" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A165" s="2" t="s">
-        <v>505</v>
+        <v>503</v>
       </c>
       <c r="B165" s="2" t="s">
-        <v>505</v>
+        <v>503</v>
       </c>
       <c r="C165" s="2" t="s">
-        <v>506</v>
+        <v>504</v>
       </c>
       <c r="D165" s="2" t="s">
-        <v>558</v>
+        <v>559</v>
       </c>
     </row>
     <row r="166" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A166" s="2" t="s">
-        <v>507</v>
+        <v>505</v>
       </c>
       <c r="B166" s="2" t="s">
-        <v>507</v>
+        <v>505</v>
       </c>
       <c r="C166" s="2" t="s">
-        <v>508</v>
+        <v>506</v>
       </c>
       <c r="D166" s="2" t="s">
-        <v>557</v>
+        <v>558</v>
       </c>
     </row>
     <row r="167" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A167" s="2" t="s">
-        <v>570</v>
+        <v>507</v>
       </c>
       <c r="B167" s="2" t="s">
-        <v>571</v>
+        <v>507</v>
       </c>
       <c r="C167" s="2" t="s">
-        <v>609</v>
+        <v>508</v>
+      </c>
+      <c r="D167" s="2" t="s">
+        <v>557</v>
       </c>
     </row>
     <row r="168" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A168" s="2" t="s">
-        <v>572</v>
+        <v>570</v>
       </c>
       <c r="B168" s="2" t="s">
-        <v>573</v>
+        <v>571</v>
       </c>
       <c r="C168" s="2" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
     </row>
     <row r="169" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A169" s="2" t="s">
-        <v>574</v>
+        <v>572</v>
       </c>
       <c r="B169" s="2" t="s">
-        <v>575</v>
+        <v>573</v>
       </c>
       <c r="C169" s="2" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
     </row>
     <row r="170" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A170" s="2" t="s">
-        <v>576</v>
+        <v>574</v>
       </c>
       <c r="B170" s="2" t="s">
-        <v>577</v>
+        <v>575</v>
       </c>
       <c r="C170" s="2" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
     </row>
     <row r="171" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A171" s="2" t="s">
-        <v>578</v>
+        <v>576</v>
       </c>
       <c r="B171" s="2" t="s">
-        <v>579</v>
+        <v>577</v>
       </c>
       <c r="C171" s="2" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
     </row>
     <row r="172" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A172" s="2" t="s">
-        <v>580</v>
+        <v>578</v>
       </c>
       <c r="B172" s="2" t="s">
-        <v>581</v>
+        <v>579</v>
       </c>
       <c r="C172" s="2" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
     </row>
     <row r="173" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A173" s="2" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
       <c r="B173" s="2" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="C173" s="2" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
     </row>
     <row r="174" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A174" s="2" t="s">
-        <v>584</v>
+        <v>582</v>
       </c>
       <c r="B174" s="2" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="C174" s="2" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
     </row>
     <row r="175" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A175" s="2" t="s">
-        <v>586</v>
+        <v>584</v>
       </c>
       <c r="B175" s="2" t="s">
-        <v>587</v>
+        <v>585</v>
       </c>
       <c r="C175" s="2" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
     </row>
     <row r="176" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A176" s="2" t="s">
-        <v>588</v>
+        <v>586</v>
       </c>
       <c r="B176" s="2" t="s">
-        <v>589</v>
+        <v>587</v>
       </c>
       <c r="C176" s="2" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
     </row>
     <row r="177" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A177" s="2" t="s">
-        <v>620</v>
+        <v>588</v>
       </c>
       <c r="B177" s="2" t="s">
-        <v>621</v>
+        <v>589</v>
       </c>
       <c r="C177" s="2" t="s">
-        <v>622</v>
+        <v>618</v>
       </c>
     </row>
     <row r="178" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A178" s="2" t="s">
-        <v>623</v>
+        <v>620</v>
       </c>
       <c r="B178" s="2" t="s">
-        <v>623</v>
+        <v>621</v>
       </c>
       <c r="C178" s="2" t="s">
-        <v>624</v>
+        <v>622</v>
       </c>
     </row>
     <row r="179" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A179" s="2" t="s">
-        <v>625</v>
+        <v>623</v>
       </c>
       <c r="B179" s="2" t="s">
-        <v>625</v>
+        <v>623</v>
       </c>
       <c r="C179" s="2" t="s">
-        <v>627</v>
+        <v>624</v>
       </c>
     </row>
     <row r="180" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A180" s="2" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="B180" s="2" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="C180" s="2" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
     </row>
     <row r="181" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A181" s="2" t="s">
-        <v>629</v>
+        <v>626</v>
       </c>
       <c r="B181" s="2" t="s">
-        <v>630</v>
+        <v>626</v>
       </c>
       <c r="C181" s="2" t="s">
-        <v>631</v>
+        <v>628</v>
       </c>
     </row>
     <row r="182" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A182" s="2" t="s">
-        <v>632</v>
-      </c>
-      <c r="B182" s="4" t="s">
-        <v>633</v>
-      </c>
-      <c r="C182" s="4" t="s">
-        <v>634</v>
+        <v>629</v>
+      </c>
+      <c r="B182" s="2" t="s">
+        <v>630</v>
+      </c>
+      <c r="C182" s="2" t="s">
+        <v>631</v>
       </c>
     </row>
     <row r="183" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A183" s="2" t="s">
-        <v>638</v>
-      </c>
-      <c r="B183" s="2" t="s">
-        <v>639</v>
-      </c>
-      <c r="C183" s="2" t="s">
-        <v>640</v>
+        <v>632</v>
+      </c>
+      <c r="B183" s="4" t="s">
+        <v>633</v>
+      </c>
+      <c r="C183" s="4" t="s">
+        <v>634</v>
       </c>
     </row>
     <row r="184" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A184" s="2" t="s">
-        <v>641</v>
+        <v>638</v>
       </c>
       <c r="B184" s="2" t="s">
-        <v>641</v>
+        <v>639</v>
       </c>
       <c r="C184" s="2" t="s">
-        <v>642</v>
+        <v>640</v>
       </c>
     </row>
     <row r="185" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A185" s="2" t="s">
-        <v>643</v>
+        <v>641</v>
       </c>
       <c r="B185" s="2" t="s">
-        <v>644</v>
+        <v>641</v>
       </c>
       <c r="C185" s="2" t="s">
-        <v>645</v>
+        <v>642</v>
       </c>
     </row>
     <row r="186" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A186" s="2" t="s">
-        <v>646</v>
+        <v>643</v>
       </c>
       <c r="B186" s="2" t="s">
-        <v>647</v>
+        <v>644</v>
       </c>
       <c r="C186" s="2" t="s">
-        <v>648</v>
+        <v>645</v>
       </c>
     </row>
     <row r="187" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A187" s="2" t="s">
-        <v>649</v>
+        <v>646</v>
       </c>
       <c r="B187" s="2" t="s">
-        <v>650</v>
+        <v>647</v>
       </c>
       <c r="C187" s="2" t="s">
-        <v>651</v>
+        <v>648</v>
       </c>
     </row>
     <row r="188" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A188" s="2" t="s">
-        <v>652</v>
+        <v>649</v>
       </c>
       <c r="B188" s="2" t="s">
-        <v>653</v>
+        <v>650</v>
       </c>
       <c r="C188" s="2" t="s">
-        <v>654</v>
+        <v>651</v>
       </c>
     </row>
     <row r="189" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A189" s="2" t="s">
-        <v>655</v>
+        <v>652</v>
       </c>
       <c r="B189" s="2" t="s">
-        <v>655</v>
+        <v>653</v>
       </c>
       <c r="C189" s="2" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
     </row>
     <row r="190" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A190" s="2" t="s">
-        <v>657</v>
+        <v>655</v>
       </c>
       <c r="B190" s="2" t="s">
-        <v>658</v>
+        <v>655</v>
       </c>
       <c r="C190" s="2" t="s">
-        <v>659</v>
+        <v>656</v>
       </c>
     </row>
     <row r="191" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A191" s="2" t="s">
-        <v>666</v>
-      </c>
-      <c r="B191" s="4" t="s">
-        <v>667</v>
-      </c>
-      <c r="C191" s="4" t="s">
-        <v>668</v>
+        <v>657</v>
+      </c>
+      <c r="B191" s="2" t="s">
+        <v>658</v>
+      </c>
+      <c r="C191" s="2" t="s">
+        <v>659</v>
       </c>
     </row>
     <row r="192" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A192" s="2" t="s">
-        <v>669</v>
-      </c>
-      <c r="B192" s="2" t="s">
-        <v>670</v>
-      </c>
-      <c r="C192" s="2" t="s">
-        <v>671</v>
+        <v>666</v>
+      </c>
+      <c r="B192" s="4" t="s">
+        <v>667</v>
+      </c>
+      <c r="C192" s="4" t="s">
+        <v>668</v>
       </c>
     </row>
     <row r="193" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A193" s="2" t="s">
-        <v>675</v>
+        <v>669</v>
       </c>
       <c r="B193" s="2" t="s">
-        <v>676</v>
+        <v>670</v>
       </c>
       <c r="C193" s="2" t="s">
-        <v>677</v>
+        <v>671</v>
       </c>
     </row>
     <row r="194" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A194" s="2" t="s">
-        <v>678</v>
+        <v>675</v>
       </c>
       <c r="B194" s="2" t="s">
-        <v>679</v>
+        <v>676</v>
       </c>
       <c r="C194" s="2" t="s">
-        <v>680</v>
+        <v>677</v>
       </c>
     </row>
     <row r="195" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A195" s="2" t="s">
-        <v>681</v>
+        <v>678</v>
       </c>
       <c r="B195" s="2" t="s">
-        <v>682</v>
+        <v>679</v>
       </c>
       <c r="C195" s="2" t="s">
-        <v>683</v>
+        <v>680</v>
       </c>
     </row>
     <row r="196" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A196" s="2" t="s">
-        <v>684</v>
+        <v>681</v>
       </c>
       <c r="B196" s="2" t="s">
-        <v>685</v>
+        <v>682</v>
       </c>
       <c r="C196" s="2" t="s">
-        <v>686</v>
+        <v>683</v>
       </c>
     </row>
     <row r="197" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A197" s="2" t="s">
-        <v>687</v>
+        <v>684</v>
       </c>
       <c r="B197" s="2" t="s">
-        <v>688</v>
+        <v>685</v>
       </c>
       <c r="C197" s="2" t="s">
-        <v>689</v>
+        <v>686</v>
       </c>
     </row>
     <row r="198" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A198" s="2" t="s">
-        <v>690</v>
-      </c>
-      <c r="B198" s="4" t="s">
-        <v>694</v>
-      </c>
-      <c r="C198" s="4" t="s">
-        <v>704</v>
+        <v>687</v>
+      </c>
+      <c r="B198" s="2" t="s">
+        <v>688</v>
+      </c>
+      <c r="C198" s="2" t="s">
+        <v>689</v>
       </c>
     </row>
     <row r="199" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A199" s="2" t="s">
-        <v>691</v>
-      </c>
-      <c r="B199" s="2" t="s">
-        <v>697</v>
-      </c>
-      <c r="C199" s="2" t="s">
-        <v>710</v>
+        <v>690</v>
+      </c>
+      <c r="B199" s="4" t="s">
+        <v>694</v>
+      </c>
+      <c r="C199" s="4" t="s">
+        <v>704</v>
       </c>
     </row>
     <row r="200" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A200" s="2" t="s">
-        <v>693</v>
-      </c>
-      <c r="B200" s="4" t="s">
-        <v>695</v>
-      </c>
-      <c r="C200" s="4" t="s">
-        <v>705</v>
+        <v>691</v>
+      </c>
+      <c r="B200" s="2" t="s">
+        <v>697</v>
+      </c>
+      <c r="C200" s="2" t="s">
+        <v>710</v>
       </c>
     </row>
     <row r="201" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A201" s="2" t="s">
-        <v>692</v>
+        <v>693</v>
       </c>
       <c r="B201" s="4" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
       <c r="C201" s="4" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
     </row>
     <row r="202" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A202" s="2" t="s">
-        <v>699</v>
-      </c>
-      <c r="B202" s="2" t="s">
-        <v>698</v>
-      </c>
-      <c r="C202" s="2" t="s">
-        <v>707</v>
+        <v>692</v>
+      </c>
+      <c r="B202" s="4" t="s">
+        <v>696</v>
+      </c>
+      <c r="C202" s="4" t="s">
+        <v>706</v>
       </c>
     </row>
     <row r="203" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A203" s="2" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="B203" s="2" t="s">
-        <v>702</v>
+        <v>698</v>
       </c>
       <c r="C203" s="2" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
     </row>
     <row r="204" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A204" s="2" t="s">
-        <v>701</v>
+        <v>700</v>
       </c>
       <c r="B204" s="2" t="s">
-        <v>703</v>
+        <v>702</v>
       </c>
       <c r="C204" s="2" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
     </row>
     <row r="205" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A205" s="2" t="s">
-        <v>711</v>
+        <v>701</v>
       </c>
       <c r="B205" s="2" t="s">
-        <v>711</v>
+        <v>703</v>
       </c>
       <c r="C205" s="2" t="s">
-        <v>712</v>
+        <v>709</v>
       </c>
     </row>
     <row r="206" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A206" s="2" t="s">
-        <v>713</v>
+        <v>711</v>
       </c>
       <c r="B206" s="2" t="s">
-        <v>714</v>
+        <v>711</v>
       </c>
       <c r="C206" s="2" t="s">
-        <v>715</v>
+        <v>712</v>
       </c>
     </row>
     <row r="207" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A207" s="2" t="s">
-        <v>716</v>
+        <v>713</v>
       </c>
       <c r="B207" s="2" t="s">
-        <v>717</v>
+        <v>714</v>
       </c>
       <c r="C207" s="2" t="s">
-        <v>718</v>
+        <v>715</v>
       </c>
     </row>
     <row r="208" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A208" s="2" t="s">
+        <v>716</v>
+      </c>
+      <c r="B208" s="2" t="s">
+        <v>717</v>
+      </c>
+      <c r="C208" s="2" t="s">
+        <v>718</v>
+      </c>
+    </row>
+    <row r="209" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A209" s="2" t="s">
         <v>719</v>
       </c>
-      <c r="B208" s="2" t="s">
+      <c r="B209" s="2" t="s">
         <v>720</v>
       </c>
-      <c r="C208" s="2" t="s">
+      <c r="C209" s="2" t="s">
         <v>721</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Added "Execute Events If Inside" and "Execute Events If Despawned" for triggers.
</commit_message>
<xml_diff>
--- a/Translations/Translations.xlsx
+++ b/Translations/Translations.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programacion\MelonLoader\FS_LevelEditor\Translations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB352B10-965D-4524-9151-D1CF1499DFD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8FB2823-C575-4BDD-8BB9-A216691A3669}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{F5C22481-FF1A-482C-BF7E-EB5A7718AF49}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1421" uniqueCount="728">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1433" uniqueCount="740">
   <si>
     <t>ID</t>
   </si>
@@ -2222,6 +2222,42 @@
   </si>
   <si>
     <t>Entrada de Energía</t>
+  </si>
+  <si>
+    <t>ExecIfInsideTooltip</t>
+  </si>
+  <si>
+    <t>Executes the [b]On Enter[/b] events when the trigger is [i]spawned[/i] while the player is [b]already inside.[/b]</t>
+  </si>
+  <si>
+    <t>ExecIfDespawnedTooltip</t>
+  </si>
+  <si>
+    <t>Executes the [b]On Exit[/b] events when the trigger is [i]despawned[/i] while the player is [b]still inside.[/b]</t>
+  </si>
+  <si>
+    <t>ExecIfInside</t>
+  </si>
+  <si>
+    <t>Execute Events If Inside</t>
+  </si>
+  <si>
+    <t>ExecIfDespawned</t>
+  </si>
+  <si>
+    <t>Execute Events If Despawned</t>
+  </si>
+  <si>
+    <t>Ejecutar Eventos Si Está Adentro</t>
+  </si>
+  <si>
+    <t>Ejecutar Eventos Si Está Desactivado</t>
+  </si>
+  <si>
+    <t>Ejecuta los eventos [b]Al Entrar[/b] cuando el trigger se [i]activa[/i] mientras el jugador [b]ya está adentro.[/b]</t>
+  </si>
+  <si>
+    <t>Ejecuta los eventos [b]Al Salir[/b] cuando el trigger se [i]desactiva[/i] mientras el jugador [b]sigue adentro.[/b]</t>
   </si>
 </sst>
 </file>
@@ -2621,7 +2657,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6961A5F-F8EA-4989-8112-A0ACE51D011E}">
   <sheetPr codeName="Hoja1"/>
-  <dimension ref="A1:D209"/>
+  <dimension ref="A1:D213"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="37" style="2" customWidth="1"/>
@@ -5400,6 +5436,50 @@
       </c>
       <c r="C209" s="2" t="s">
         <v>721</v>
+      </c>
+    </row>
+    <row r="210" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A210" s="2" t="s">
+        <v>732</v>
+      </c>
+      <c r="B210" s="2" t="s">
+        <v>733</v>
+      </c>
+      <c r="C210" s="2" t="s">
+        <v>736</v>
+      </c>
+    </row>
+    <row r="211" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A211" s="2" t="s">
+        <v>734</v>
+      </c>
+      <c r="B211" s="2" t="s">
+        <v>735</v>
+      </c>
+      <c r="C211" s="2" t="s">
+        <v>737</v>
+      </c>
+    </row>
+    <row r="212" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A212" s="2" t="s">
+        <v>728</v>
+      </c>
+      <c r="B212" s="2" t="s">
+        <v>729</v>
+      </c>
+      <c r="C212" s="2" t="s">
+        <v>738</v>
+      </c>
+    </row>
+    <row r="213" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A213" s="2" t="s">
+        <v>730</v>
+      </c>
+      <c r="B213" s="2" t="s">
+        <v>731</v>
+      </c>
+      <c r="C213" s="2" t="s">
+        <v>739</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added "On Insert" translation for Power Slots.
</commit_message>
<xml_diff>
--- a/Translations/Translations.xlsx
+++ b/Translations/Translations.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programacion\MelonLoader\FS_LevelEditor\Translations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8FB2823-C575-4BDD-8BB9-A216691A3669}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6191E90-3161-47AF-AFA2-8D96590A7A7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{F5C22481-FF1A-482C-BF7E-EB5A7718AF49}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1433" uniqueCount="740">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1436" uniqueCount="743">
   <si>
     <t>ID</t>
   </si>
@@ -2258,6 +2258,15 @@
   </si>
   <si>
     <t>Ejecuta los eventos [b]Al Salir[/b] cuando el trigger se [i]desactiva[/i] mientras el jugador [b]sigue adentro.[/b]</t>
+  </si>
+  <si>
+    <t>events.OnInsert</t>
+  </si>
+  <si>
+    <t>On Insert</t>
+  </si>
+  <si>
+    <t>Al Insertar</t>
   </si>
 </sst>
 </file>
@@ -2657,7 +2666,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6961A5F-F8EA-4989-8112-A0ACE51D011E}">
   <sheetPr codeName="Hoja1"/>
-  <dimension ref="A1:D213"/>
+  <dimension ref="A1:D214"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="37" style="2" customWidth="1"/>
@@ -3769,1716 +3778,1727 @@
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A81" s="2" t="s">
-        <v>154</v>
+        <v>740</v>
       </c>
       <c r="B81" s="2" t="s">
-        <v>155</v>
+        <v>741</v>
       </c>
       <c r="C81" s="2" t="s">
-        <v>156</v>
-      </c>
-      <c r="D81" s="2" t="s">
-        <v>371</v>
+        <v>742</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A82" s="2" t="s">
-        <v>164</v>
+        <v>154</v>
       </c>
       <c r="B82" s="2" t="s">
-        <v>165</v>
+        <v>155</v>
       </c>
       <c r="C82" s="2" t="s">
-        <v>166</v>
+        <v>156</v>
       </c>
       <c r="D82" s="2" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A83" s="2" t="s">
-        <v>157</v>
+        <v>164</v>
       </c>
       <c r="B83" s="2" t="s">
-        <v>158</v>
+        <v>165</v>
       </c>
       <c r="C83" s="2" t="s">
-        <v>159</v>
+        <v>166</v>
       </c>
       <c r="D83" s="2" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A84" s="2" t="s">
-        <v>167</v>
+        <v>157</v>
       </c>
       <c r="B84" s="2" t="s">
-        <v>168</v>
+        <v>158</v>
       </c>
       <c r="C84" s="2" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="D84" s="2" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A85" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="B85" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="C85" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="D85" s="2" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A86" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="B85" s="2" t="s">
+      <c r="B86" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="C85" s="2" t="s">
+      <c r="C86" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="D85" s="2" t="s">
+      <c r="D86" s="2" t="s">
         <v>375</v>
       </c>
     </row>
-    <row r="86" spans="1:4" ht="45" x14ac:dyDescent="0.25">
-      <c r="A86" s="2" t="s">
+    <row r="87" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="A87" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="B86" s="2" t="s">
+      <c r="B87" s="2" t="s">
         <v>163</v>
       </c>
-      <c r="C86" s="2" t="s">
+      <c r="C87" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="D86" s="2" t="s">
+      <c r="D87" s="2" t="s">
         <v>376</v>
-      </c>
-    </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A87" s="2" t="s">
-        <v>153</v>
-      </c>
-      <c r="B87" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="C87" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="D87" s="2" t="s">
-        <v>328</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A88" s="2" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="B88" s="2" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="C88" s="2" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="D88" s="2" t="s">
-        <v>377</v>
+        <v>328</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A89" s="2" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="B89" s="2" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="C89" s="2" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="D89" s="2" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A90" s="2" t="s">
-        <v>172</v>
+        <v>150</v>
       </c>
       <c r="B90" s="2" t="s">
-        <v>170</v>
+        <v>151</v>
       </c>
       <c r="C90" s="2" t="s">
-        <v>171</v>
+        <v>152</v>
       </c>
       <c r="D90" s="2" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A91" s="2" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B91" s="2" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="C91" s="2" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="D91" s="2" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A92" s="2" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="B92" s="2" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="C92" s="2" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="D92" s="2" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A93" s="2" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="B93" s="2" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="C93" s="2" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="D93" s="2" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A94" s="2" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="B94" s="2" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="C94" s="2" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="D94" s="2" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A95" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="B95" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="C95" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="D95" s="2" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="96" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A96" s="2" t="s">
         <v>243</v>
       </c>
-      <c r="B95" s="2" t="s">
+      <c r="B96" s="2" t="s">
         <v>243</v>
       </c>
-      <c r="C95" s="2" t="s">
+      <c r="C96" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="D95" s="2" t="s">
+      <c r="D96" s="2" t="s">
         <v>384</v>
       </c>
     </row>
-    <row r="96" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A96" s="2" t="s">
+    <row r="97" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A97" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="B96" s="1" t="s">
+      <c r="B97" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="C96" s="2" t="s">
+      <c r="C97" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="D96" s="2" t="s">
+      <c r="D97" s="2" t="s">
         <v>385</v>
-      </c>
-    </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A97" s="2" t="s">
-        <v>182</v>
-      </c>
-      <c r="B97" s="2" t="s">
-        <v>183</v>
-      </c>
-      <c r="C97" s="2" t="s">
-        <v>183</v>
-      </c>
-      <c r="D97" s="2" t="s">
-        <v>386</v>
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A98" s="2" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="B98" s="2" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C98" s="2" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="D98" s="2" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A99" s="2" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="B99" s="2" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="C99" s="2" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="D99" s="2" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A100" s="2" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="B100" s="2" t="s">
-        <v>525</v>
+        <v>186</v>
       </c>
       <c r="C100" s="2" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="D100" s="2" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A101" s="2" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="B101" s="2" t="s">
-        <v>190</v>
+        <v>525</v>
       </c>
       <c r="C101" s="2" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="D101" s="2" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A102" s="2" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="B102" s="2" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="C102" s="2" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="D102" s="2" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A103" s="2" t="s">
-        <v>434</v>
-      </c>
-      <c r="B103" s="4" t="s">
-        <v>435</v>
-      </c>
-      <c r="C103" s="4" t="s">
-        <v>436</v>
-      </c>
-      <c r="D103" s="4" t="s">
-        <v>591</v>
+        <v>192</v>
+      </c>
+      <c r="B103" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="C103" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="D103" s="2" t="s">
+        <v>391</v>
       </c>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A104" s="2" t="s">
-        <v>437</v>
+        <v>434</v>
       </c>
       <c r="B104" s="4" t="s">
-        <v>438</v>
+        <v>435</v>
       </c>
       <c r="C104" s="4" t="s">
-        <v>439</v>
+        <v>436</v>
       </c>
       <c r="D104" s="4" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A105" s="2" t="s">
-        <v>473</v>
+        <v>437</v>
       </c>
       <c r="B105" s="4" t="s">
-        <v>590</v>
+        <v>438</v>
       </c>
       <c r="C105" s="4" t="s">
-        <v>474</v>
+        <v>439</v>
       </c>
       <c r="D105" s="4" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A106" s="2" t="s">
-        <v>195</v>
-      </c>
-      <c r="B106" s="2" t="s">
-        <v>196</v>
-      </c>
-      <c r="C106" s="2" t="s">
-        <v>197</v>
-      </c>
-      <c r="D106" s="2" t="s">
-        <v>392</v>
+        <v>473</v>
+      </c>
+      <c r="B106" s="4" t="s">
+        <v>590</v>
+      </c>
+      <c r="C106" s="4" t="s">
+        <v>474</v>
+      </c>
+      <c r="D106" s="4" t="s">
+        <v>593</v>
       </c>
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A107" s="2" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="B107" s="2" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="C107" s="2" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="D107" s="2" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A108" s="2" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="B108" s="2" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="C108" s="2" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="D108" s="2" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A109" s="2" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="B109" s="2" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="C109" s="2" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="D109" s="2" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A110" s="2" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="B110" s="2" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="C110" s="2" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="D110" s="2" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A111" s="2" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B111" s="2" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="C111" s="2" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="D111" s="2" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A112" s="2" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="B112" s="2" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="C112" s="2" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="D112" s="2" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A113" s="2" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="B113" s="2" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="C113" s="2" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="D113" s="2" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A114" s="2" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="B114" s="2" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="C114" s="2" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="D114" s="2" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A115" s="2" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="B115" s="2" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="C115" s="2" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="D115" s="2" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A116" s="2" t="s">
-        <v>292</v>
+        <v>220</v>
       </c>
       <c r="B116" s="2" t="s">
-        <v>292</v>
+        <v>219</v>
       </c>
       <c r="C116" s="2" t="s">
-        <v>293</v>
+        <v>218</v>
       </c>
       <c r="D116" s="2" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A117" s="2" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="B117" s="2" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="C117" s="2" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
       <c r="D117" s="2" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A118" s="2" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
       <c r="B118" s="2" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="C118" s="2" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="D118" s="2" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
     </row>
     <row r="119" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A119" s="2" t="s">
-        <v>221</v>
+        <v>297</v>
       </c>
       <c r="B119" s="2" t="s">
-        <v>221</v>
+        <v>298</v>
       </c>
       <c r="C119" s="2" t="s">
-        <v>222</v>
+        <v>299</v>
       </c>
       <c r="D119" s="2" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A120" s="2" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="B120" s="2" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="C120" s="2" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="D120" s="2" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A121" s="2" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="B121" s="2" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="C121" s="2" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="D121" s="2" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A122" s="2" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="B122" s="2" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="C122" s="2" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="D122" s="2" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
     </row>
     <row r="123" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A123" s="2" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B123" s="2" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="C123" s="2" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="D123" s="2" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
     </row>
     <row r="124" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A124" s="2" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="B124" s="2" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="C124" s="2" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="D124" s="2" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
     </row>
     <row r="125" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A125" s="2" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="B125" s="2" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="C125" s="2" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="D125" s="2" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
     </row>
     <row r="126" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A126" s="2" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="B126" s="2" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="C126" s="2" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="D126" s="2" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
     </row>
     <row r="127" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A127" s="2" t="s">
-        <v>300</v>
+        <v>237</v>
       </c>
       <c r="B127" s="2" t="s">
-        <v>301</v>
+        <v>238</v>
       </c>
       <c r="C127" s="2" t="s">
-        <v>302</v>
+        <v>239</v>
       </c>
       <c r="D127" s="2" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
     </row>
     <row r="128" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A128" s="2" t="s">
-        <v>240</v>
+        <v>300</v>
       </c>
       <c r="B128" s="2" t="s">
-        <v>241</v>
+        <v>301</v>
       </c>
       <c r="C128" s="2" t="s">
-        <v>242</v>
+        <v>302</v>
       </c>
       <c r="D128" s="2" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
     </row>
     <row r="129" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A129" s="2" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="B129" s="2" t="s">
-        <v>252</v>
+        <v>241</v>
       </c>
       <c r="C129" s="2" t="s">
-        <v>251</v>
+        <v>242</v>
       </c>
       <c r="D129" s="2" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="130" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A130" s="2" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B130" s="2" t="s">
-        <v>245</v>
+        <v>252</v>
       </c>
       <c r="C130" s="2" t="s">
-        <v>246</v>
+        <v>251</v>
       </c>
       <c r="D130" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
     </row>
     <row r="131" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A131" s="2" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="B131" s="2" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="C131" s="2" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="D131" s="2" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
     </row>
     <row r="132" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A132" s="2" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="B132" s="2" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="C132" s="2" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="D132" s="2" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
     </row>
     <row r="133" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A133" s="2" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="B133" s="2" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="C133" s="2" t="s">
-        <v>255</v>
+        <v>250</v>
       </c>
       <c r="D133" s="2" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
     </row>
     <row r="134" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A134" s="2" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="B134" s="2" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="C134" s="2" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="D134" s="2" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
     </row>
     <row r="135" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A135" s="2" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="B135" s="2" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="C135" s="2" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="D135" s="2" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
     </row>
     <row r="136" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A136" s="2" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="B136" s="2" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="C136" s="2" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="D136" s="2" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="137" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A137" s="2" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="B137" s="2" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="C137" s="2" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="D137" s="2" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
     </row>
     <row r="138" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A138" s="2" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="B138" s="2" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="C138" s="2" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="D138" s="2" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
     </row>
     <row r="139" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A139" s="2" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="B139" s="2" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="C139" s="2" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="D139" s="2" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
     </row>
     <row r="140" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A140" s="2" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="B140" s="2" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="C140" s="2" t="s">
-        <v>273</v>
+        <v>269</v>
       </c>
       <c r="D140" s="2" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
     </row>
     <row r="141" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A141" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="B141" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="C141" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="D141" s="2" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="142" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A142" s="2" t="s">
         <v>271</v>
       </c>
-      <c r="B141" s="2" t="s">
+      <c r="B142" s="2" t="s">
         <v>271</v>
       </c>
-      <c r="C141" s="2" t="s">
+      <c r="C142" s="2" t="s">
         <v>272</v>
       </c>
-      <c r="D141" s="2" t="s">
+      <c r="D142" s="2" t="s">
         <v>427</v>
       </c>
     </row>
-    <row r="142" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A142" s="2" t="s">
+    <row r="143" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A143" s="2" t="s">
         <v>274</v>
       </c>
-      <c r="B142" s="2" t="s">
+      <c r="B143" s="2" t="s">
         <v>276</v>
       </c>
-      <c r="C142" s="2" t="s">
+      <c r="C143" s="2" t="s">
         <v>279</v>
       </c>
     </row>
-    <row r="143" spans="1:4" ht="45" x14ac:dyDescent="0.25">
-      <c r="A143" s="2" t="s">
+    <row r="144" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="A144" s="2" t="s">
         <v>275</v>
       </c>
-      <c r="B143" s="2" t="s">
+      <c r="B144" s="2" t="s">
         <v>277</v>
       </c>
-      <c r="C143" s="2" t="s">
+      <c r="C144" s="2" t="s">
         <v>278</v>
       </c>
     </row>
-    <row r="144" spans="1:4" ht="75" x14ac:dyDescent="0.25">
-      <c r="A144" s="2" t="s">
+    <row r="145" spans="1:4" ht="75" x14ac:dyDescent="0.25">
+      <c r="A145" s="2" t="s">
         <v>289</v>
       </c>
-      <c r="B144" s="2" t="s">
+      <c r="B145" s="2" t="s">
         <v>290</v>
       </c>
-      <c r="C144" s="2" t="s">
+      <c r="C145" s="2" t="s">
         <v>291</v>
-      </c>
-    </row>
-    <row r="145" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A145" s="2" t="s">
-        <v>306</v>
-      </c>
-      <c r="B145" s="2" t="s">
-        <v>307</v>
-      </c>
-      <c r="C145" s="2" t="s">
-        <v>308</v>
-      </c>
-      <c r="D145" s="2" t="s">
-        <v>428</v>
       </c>
     </row>
     <row r="146" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A146" s="2" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
       <c r="B146" s="2" t="s">
-        <v>311</v>
+        <v>307</v>
       </c>
       <c r="C146" s="2" t="s">
-        <v>312</v>
+        <v>308</v>
       </c>
       <c r="D146" s="2" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
     </row>
     <row r="147" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A147" s="2" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="B147" s="2" t="s">
-        <v>314</v>
+        <v>311</v>
       </c>
       <c r="C147" s="2" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="D147" s="2" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
     </row>
     <row r="148" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A148" s="2" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="B148" s="2" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="C148" s="2" t="s">
-        <v>316</v>
+        <v>313</v>
       </c>
       <c r="D148" s="2" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
     </row>
     <row r="149" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A149" s="2" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="B149" s="2" t="s">
-        <v>318</v>
+        <v>315</v>
       </c>
       <c r="C149" s="2" t="s">
-        <v>460</v>
+        <v>316</v>
       </c>
       <c r="D149" s="2" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
     </row>
     <row r="150" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A150" s="2" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="B150" s="2" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="C150" s="2" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="D150" s="2" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
     </row>
     <row r="151" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A151" s="2" t="s">
-        <v>448</v>
+        <v>319</v>
       </c>
       <c r="B151" s="2" t="s">
-        <v>448</v>
+        <v>320</v>
       </c>
       <c r="C151" s="2" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="D151" s="2" t="s">
-        <v>345</v>
+        <v>433</v>
       </c>
     </row>
     <row r="152" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A152" s="2" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="B152" s="2" t="s">
-        <v>450</v>
+        <v>448</v>
       </c>
       <c r="C152" s="2" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="D152" s="2" t="s">
-        <v>451</v>
+        <v>345</v>
       </c>
     </row>
     <row r="153" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A153" s="2" t="s">
-        <v>475</v>
+        <v>449</v>
       </c>
       <c r="B153" s="2" t="s">
-        <v>476</v>
+        <v>450</v>
       </c>
       <c r="C153" s="2" t="s">
-        <v>619</v>
+        <v>463</v>
       </c>
       <c r="D153" s="2" t="s">
-        <v>569</v>
+        <v>451</v>
       </c>
     </row>
     <row r="154" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A154" s="2" t="s">
-        <v>478</v>
+        <v>475</v>
       </c>
       <c r="B154" s="2" t="s">
-        <v>524</v>
+        <v>476</v>
       </c>
       <c r="C154" s="2" t="s">
-        <v>479</v>
+        <v>619</v>
       </c>
       <c r="D154" s="2" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
     </row>
     <row r="155" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A155" s="2" t="s">
-        <v>480</v>
+        <v>478</v>
       </c>
       <c r="B155" s="2" t="s">
-        <v>481</v>
+        <v>524</v>
       </c>
       <c r="C155" s="2" t="s">
-        <v>482</v>
+        <v>479</v>
       </c>
       <c r="D155" s="2" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
     </row>
     <row r="156" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A156" s="2" t="s">
-        <v>483</v>
+        <v>480</v>
       </c>
       <c r="B156" s="2" t="s">
-        <v>484</v>
+        <v>481</v>
       </c>
       <c r="C156" s="2" t="s">
-        <v>485</v>
+        <v>482</v>
       </c>
       <c r="D156" s="2" t="s">
-        <v>566</v>
+        <v>567</v>
       </c>
     </row>
     <row r="157" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A157" s="2" t="s">
-        <v>486</v>
+        <v>483</v>
       </c>
       <c r="B157" s="2" t="s">
-        <v>487</v>
+        <v>484</v>
       </c>
       <c r="C157" s="2" t="s">
-        <v>488</v>
+        <v>485</v>
       </c>
       <c r="D157" s="2" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
     </row>
     <row r="158" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A158" s="2" t="s">
-        <v>489</v>
+        <v>486</v>
       </c>
       <c r="B158" s="2" t="s">
-        <v>490</v>
+        <v>487</v>
       </c>
       <c r="C158" s="2" t="s">
-        <v>491</v>
+        <v>488</v>
       </c>
       <c r="D158" s="2" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
     </row>
     <row r="159" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A159" s="2" t="s">
-        <v>538</v>
+        <v>489</v>
       </c>
       <c r="B159" s="2" t="s">
-        <v>538</v>
+        <v>490</v>
       </c>
       <c r="C159" s="2" t="s">
-        <v>607</v>
+        <v>491</v>
       </c>
       <c r="D159" s="2" t="s">
-        <v>539</v>
+        <v>564</v>
       </c>
     </row>
     <row r="160" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A160" s="2" t="s">
-        <v>540</v>
+        <v>538</v>
       </c>
       <c r="B160" s="2" t="s">
-        <v>541</v>
+        <v>538</v>
       </c>
       <c r="C160" s="2" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="D160" s="2" t="s">
-        <v>542</v>
+        <v>539</v>
       </c>
     </row>
     <row r="161" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A161" s="2" t="s">
-        <v>492</v>
+        <v>540</v>
       </c>
       <c r="B161" s="2" t="s">
-        <v>493</v>
+        <v>541</v>
       </c>
       <c r="C161" s="2" t="s">
-        <v>494</v>
+        <v>608</v>
       </c>
       <c r="D161" s="2" t="s">
-        <v>563</v>
+        <v>542</v>
       </c>
     </row>
     <row r="162" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A162" s="2" t="s">
-        <v>495</v>
+        <v>492</v>
       </c>
       <c r="B162" s="2" t="s">
-        <v>496</v>
+        <v>493</v>
       </c>
       <c r="C162" s="2" t="s">
-        <v>497</v>
+        <v>494</v>
       </c>
       <c r="D162" s="2" t="s">
-        <v>562</v>
+        <v>563</v>
       </c>
     </row>
     <row r="163" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A163" s="2" t="s">
-        <v>498</v>
+        <v>495</v>
       </c>
       <c r="B163" s="2" t="s">
-        <v>499</v>
+        <v>496</v>
       </c>
       <c r="C163" s="2" t="s">
-        <v>500</v>
+        <v>497</v>
       </c>
       <c r="D163" s="2" t="s">
-        <v>561</v>
+        <v>562</v>
       </c>
     </row>
     <row r="164" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A164" s="2" t="s">
-        <v>501</v>
+        <v>498</v>
       </c>
       <c r="B164" s="2" t="s">
-        <v>501</v>
+        <v>499</v>
       </c>
       <c r="C164" s="2" t="s">
-        <v>502</v>
+        <v>500</v>
       </c>
       <c r="D164" s="2" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
     </row>
     <row r="165" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A165" s="2" t="s">
-        <v>503</v>
+        <v>501</v>
       </c>
       <c r="B165" s="2" t="s">
-        <v>503</v>
+        <v>501</v>
       </c>
       <c r="C165" s="2" t="s">
-        <v>504</v>
+        <v>502</v>
       </c>
       <c r="D165" s="2" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
     </row>
     <row r="166" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A166" s="2" t="s">
-        <v>505</v>
+        <v>503</v>
       </c>
       <c r="B166" s="2" t="s">
-        <v>505</v>
+        <v>503</v>
       </c>
       <c r="C166" s="2" t="s">
-        <v>506</v>
+        <v>504</v>
       </c>
       <c r="D166" s="2" t="s">
-        <v>558</v>
+        <v>559</v>
       </c>
     </row>
     <row r="167" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A167" s="2" t="s">
-        <v>507</v>
+        <v>505</v>
       </c>
       <c r="B167" s="2" t="s">
-        <v>507</v>
+        <v>505</v>
       </c>
       <c r="C167" s="2" t="s">
-        <v>508</v>
+        <v>506</v>
       </c>
       <c r="D167" s="2" t="s">
-        <v>557</v>
+        <v>558</v>
       </c>
     </row>
     <row r="168" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A168" s="2" t="s">
-        <v>570</v>
+        <v>507</v>
       </c>
       <c r="B168" s="2" t="s">
-        <v>571</v>
+        <v>507</v>
       </c>
       <c r="C168" s="2" t="s">
-        <v>609</v>
+        <v>508</v>
+      </c>
+      <c r="D168" s="2" t="s">
+        <v>557</v>
       </c>
     </row>
     <row r="169" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A169" s="2" t="s">
-        <v>572</v>
+        <v>570</v>
       </c>
       <c r="B169" s="2" t="s">
-        <v>573</v>
+        <v>571</v>
       </c>
       <c r="C169" s="2" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
     </row>
     <row r="170" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A170" s="2" t="s">
-        <v>574</v>
+        <v>572</v>
       </c>
       <c r="B170" s="2" t="s">
-        <v>575</v>
+        <v>573</v>
       </c>
       <c r="C170" s="2" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
     </row>
     <row r="171" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A171" s="2" t="s">
-        <v>576</v>
+        <v>574</v>
       </c>
       <c r="B171" s="2" t="s">
-        <v>577</v>
+        <v>575</v>
       </c>
       <c r="C171" s="2" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
     </row>
     <row r="172" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A172" s="2" t="s">
-        <v>578</v>
+        <v>576</v>
       </c>
       <c r="B172" s="2" t="s">
-        <v>579</v>
+        <v>577</v>
       </c>
       <c r="C172" s="2" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
     </row>
     <row r="173" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A173" s="2" t="s">
-        <v>580</v>
+        <v>578</v>
       </c>
       <c r="B173" s="2" t="s">
-        <v>581</v>
+        <v>579</v>
       </c>
       <c r="C173" s="2" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
     </row>
     <row r="174" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A174" s="2" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
       <c r="B174" s="2" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="C174" s="2" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
     </row>
     <row r="175" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A175" s="2" t="s">
-        <v>584</v>
+        <v>582</v>
       </c>
       <c r="B175" s="2" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="C175" s="2" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
     </row>
     <row r="176" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A176" s="2" t="s">
-        <v>586</v>
+        <v>584</v>
       </c>
       <c r="B176" s="2" t="s">
-        <v>587</v>
+        <v>585</v>
       </c>
       <c r="C176" s="2" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
     </row>
     <row r="177" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A177" s="2" t="s">
-        <v>588</v>
+        <v>586</v>
       </c>
       <c r="B177" s="2" t="s">
-        <v>589</v>
+        <v>587</v>
       </c>
       <c r="C177" s="2" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
     </row>
     <row r="178" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A178" s="2" t="s">
-        <v>620</v>
+        <v>588</v>
       </c>
       <c r="B178" s="2" t="s">
-        <v>621</v>
+        <v>589</v>
       </c>
       <c r="C178" s="2" t="s">
-        <v>622</v>
+        <v>618</v>
       </c>
     </row>
     <row r="179" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A179" s="2" t="s">
-        <v>623</v>
+        <v>620</v>
       </c>
       <c r="B179" s="2" t="s">
-        <v>623</v>
+        <v>621</v>
       </c>
       <c r="C179" s="2" t="s">
-        <v>624</v>
+        <v>622</v>
       </c>
     </row>
     <row r="180" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A180" s="2" t="s">
-        <v>625</v>
+        <v>623</v>
       </c>
       <c r="B180" s="2" t="s">
-        <v>625</v>
+        <v>623</v>
       </c>
       <c r="C180" s="2" t="s">
-        <v>627</v>
+        <v>624</v>
       </c>
     </row>
     <row r="181" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A181" s="2" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="B181" s="2" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="C181" s="2" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
     </row>
     <row r="182" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A182" s="2" t="s">
-        <v>629</v>
+        <v>626</v>
       </c>
       <c r="B182" s="2" t="s">
-        <v>630</v>
+        <v>626</v>
       </c>
       <c r="C182" s="2" t="s">
-        <v>631</v>
+        <v>628</v>
       </c>
     </row>
     <row r="183" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A183" s="2" t="s">
-        <v>632</v>
-      </c>
-      <c r="B183" s="4" t="s">
-        <v>633</v>
-      </c>
-      <c r="C183" s="4" t="s">
-        <v>634</v>
+        <v>629</v>
+      </c>
+      <c r="B183" s="2" t="s">
+        <v>630</v>
+      </c>
+      <c r="C183" s="2" t="s">
+        <v>631</v>
       </c>
     </row>
     <row r="184" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A184" s="2" t="s">
-        <v>638</v>
-      </c>
-      <c r="B184" s="2" t="s">
-        <v>639</v>
-      </c>
-      <c r="C184" s="2" t="s">
-        <v>640</v>
+        <v>632</v>
+      </c>
+      <c r="B184" s="4" t="s">
+        <v>633</v>
+      </c>
+      <c r="C184" s="4" t="s">
+        <v>634</v>
       </c>
     </row>
     <row r="185" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A185" s="2" t="s">
-        <v>641</v>
+        <v>638</v>
       </c>
       <c r="B185" s="2" t="s">
-        <v>641</v>
+        <v>639</v>
       </c>
       <c r="C185" s="2" t="s">
-        <v>642</v>
+        <v>640</v>
       </c>
     </row>
     <row r="186" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A186" s="2" t="s">
-        <v>643</v>
+        <v>641</v>
       </c>
       <c r="B186" s="2" t="s">
-        <v>644</v>
+        <v>641</v>
       </c>
       <c r="C186" s="2" t="s">
-        <v>645</v>
+        <v>642</v>
       </c>
     </row>
     <row r="187" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A187" s="2" t="s">
-        <v>646</v>
+        <v>643</v>
       </c>
       <c r="B187" s="2" t="s">
-        <v>647</v>
+        <v>644</v>
       </c>
       <c r="C187" s="2" t="s">
-        <v>648</v>
+        <v>645</v>
       </c>
     </row>
     <row r="188" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A188" s="2" t="s">
-        <v>649</v>
+        <v>646</v>
       </c>
       <c r="B188" s="2" t="s">
-        <v>650</v>
+        <v>647</v>
       </c>
       <c r="C188" s="2" t="s">
-        <v>651</v>
+        <v>648</v>
       </c>
     </row>
     <row r="189" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A189" s="2" t="s">
-        <v>652</v>
+        <v>649</v>
       </c>
       <c r="B189" s="2" t="s">
-        <v>653</v>
+        <v>650</v>
       </c>
       <c r="C189" s="2" t="s">
-        <v>654</v>
+        <v>651</v>
       </c>
     </row>
     <row r="190" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A190" s="2" t="s">
-        <v>655</v>
+        <v>652</v>
       </c>
       <c r="B190" s="2" t="s">
-        <v>655</v>
+        <v>653</v>
       </c>
       <c r="C190" s="2" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
     </row>
     <row r="191" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A191" s="2" t="s">
-        <v>657</v>
+        <v>655</v>
       </c>
       <c r="B191" s="2" t="s">
-        <v>658</v>
+        <v>655</v>
       </c>
       <c r="C191" s="2" t="s">
-        <v>659</v>
+        <v>656</v>
       </c>
     </row>
     <row r="192" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A192" s="2" t="s">
-        <v>666</v>
-      </c>
-      <c r="B192" s="4" t="s">
-        <v>667</v>
-      </c>
-      <c r="C192" s="4" t="s">
-        <v>668</v>
+        <v>657</v>
+      </c>
+      <c r="B192" s="2" t="s">
+        <v>658</v>
+      </c>
+      <c r="C192" s="2" t="s">
+        <v>659</v>
       </c>
     </row>
     <row r="193" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A193" s="2" t="s">
-        <v>669</v>
-      </c>
-      <c r="B193" s="2" t="s">
-        <v>670</v>
-      </c>
-      <c r="C193" s="2" t="s">
-        <v>671</v>
+        <v>666</v>
+      </c>
+      <c r="B193" s="4" t="s">
+        <v>667</v>
+      </c>
+      <c r="C193" s="4" t="s">
+        <v>668</v>
       </c>
     </row>
     <row r="194" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A194" s="2" t="s">
-        <v>675</v>
+        <v>669</v>
       </c>
       <c r="B194" s="2" t="s">
-        <v>676</v>
+        <v>670</v>
       </c>
       <c r="C194" s="2" t="s">
-        <v>677</v>
+        <v>671</v>
       </c>
     </row>
     <row r="195" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A195" s="2" t="s">
-        <v>678</v>
+        <v>675</v>
       </c>
       <c r="B195" s="2" t="s">
-        <v>679</v>
+        <v>676</v>
       </c>
       <c r="C195" s="2" t="s">
-        <v>680</v>
+        <v>677</v>
       </c>
     </row>
     <row r="196" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A196" s="2" t="s">
-        <v>681</v>
+        <v>678</v>
       </c>
       <c r="B196" s="2" t="s">
-        <v>682</v>
+        <v>679</v>
       </c>
       <c r="C196" s="2" t="s">
-        <v>683</v>
+        <v>680</v>
       </c>
     </row>
     <row r="197" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A197" s="2" t="s">
-        <v>684</v>
+        <v>681</v>
       </c>
       <c r="B197" s="2" t="s">
-        <v>685</v>
+        <v>682</v>
       </c>
       <c r="C197" s="2" t="s">
-        <v>686</v>
+        <v>683</v>
       </c>
     </row>
     <row r="198" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A198" s="2" t="s">
-        <v>687</v>
+        <v>684</v>
       </c>
       <c r="B198" s="2" t="s">
-        <v>688</v>
+        <v>685</v>
       </c>
       <c r="C198" s="2" t="s">
-        <v>689</v>
+        <v>686</v>
       </c>
     </row>
     <row r="199" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A199" s="2" t="s">
-        <v>690</v>
-      </c>
-      <c r="B199" s="4" t="s">
-        <v>694</v>
-      </c>
-      <c r="C199" s="4" t="s">
-        <v>704</v>
+        <v>687</v>
+      </c>
+      <c r="B199" s="2" t="s">
+        <v>688</v>
+      </c>
+      <c r="C199" s="2" t="s">
+        <v>689</v>
       </c>
     </row>
     <row r="200" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A200" s="2" t="s">
-        <v>691</v>
-      </c>
-      <c r="B200" s="2" t="s">
-        <v>697</v>
-      </c>
-      <c r="C200" s="2" t="s">
-        <v>710</v>
+        <v>690</v>
+      </c>
+      <c r="B200" s="4" t="s">
+        <v>694</v>
+      </c>
+      <c r="C200" s="4" t="s">
+        <v>704</v>
       </c>
     </row>
     <row r="201" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A201" s="2" t="s">
-        <v>693</v>
-      </c>
-      <c r="B201" s="4" t="s">
-        <v>695</v>
-      </c>
-      <c r="C201" s="4" t="s">
-        <v>705</v>
+        <v>691</v>
+      </c>
+      <c r="B201" s="2" t="s">
+        <v>697</v>
+      </c>
+      <c r="C201" s="2" t="s">
+        <v>710</v>
       </c>
     </row>
     <row r="202" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A202" s="2" t="s">
-        <v>692</v>
+        <v>693</v>
       </c>
       <c r="B202" s="4" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
       <c r="C202" s="4" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
     </row>
     <row r="203" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A203" s="2" t="s">
-        <v>699</v>
-      </c>
-      <c r="B203" s="2" t="s">
-        <v>698</v>
-      </c>
-      <c r="C203" s="2" t="s">
-        <v>707</v>
+        <v>692</v>
+      </c>
+      <c r="B203" s="4" t="s">
+        <v>696</v>
+      </c>
+      <c r="C203" s="4" t="s">
+        <v>706</v>
       </c>
     </row>
     <row r="204" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A204" s="2" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="B204" s="2" t="s">
-        <v>702</v>
+        <v>698</v>
       </c>
       <c r="C204" s="2" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
     </row>
     <row r="205" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A205" s="2" t="s">
-        <v>701</v>
+        <v>700</v>
       </c>
       <c r="B205" s="2" t="s">
-        <v>703</v>
+        <v>702</v>
       </c>
       <c r="C205" s="2" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
     </row>
     <row r="206" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A206" s="2" t="s">
-        <v>711</v>
+        <v>701</v>
       </c>
       <c r="B206" s="2" t="s">
-        <v>711</v>
+        <v>703</v>
       </c>
       <c r="C206" s="2" t="s">
-        <v>712</v>
+        <v>709</v>
       </c>
     </row>
     <row r="207" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A207" s="2" t="s">
-        <v>713</v>
+        <v>711</v>
       </c>
       <c r="B207" s="2" t="s">
-        <v>714</v>
+        <v>711</v>
       </c>
       <c r="C207" s="2" t="s">
-        <v>715</v>
+        <v>712</v>
       </c>
     </row>
     <row r="208" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A208" s="2" t="s">
-        <v>716</v>
+        <v>713</v>
       </c>
       <c r="B208" s="2" t="s">
-        <v>717</v>
+        <v>714</v>
       </c>
       <c r="C208" s="2" t="s">
-        <v>718</v>
+        <v>715</v>
       </c>
     </row>
     <row r="209" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A209" s="2" t="s">
-        <v>719</v>
+        <v>716</v>
       </c>
       <c r="B209" s="2" t="s">
-        <v>720</v>
+        <v>717</v>
       </c>
       <c r="C209" s="2" t="s">
-        <v>721</v>
+        <v>718</v>
       </c>
     </row>
     <row r="210" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A210" s="2" t="s">
-        <v>732</v>
+        <v>719</v>
       </c>
       <c r="B210" s="2" t="s">
-        <v>733</v>
+        <v>720</v>
       </c>
       <c r="C210" s="2" t="s">
-        <v>736</v>
+        <v>721</v>
       </c>
     </row>
     <row r="211" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A211" s="2" t="s">
+        <v>732</v>
+      </c>
+      <c r="B211" s="2" t="s">
+        <v>733</v>
+      </c>
+      <c r="C211" s="2" t="s">
+        <v>736</v>
+      </c>
+    </row>
+    <row r="212" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A212" s="2" t="s">
         <v>734</v>
       </c>
-      <c r="B211" s="2" t="s">
+      <c r="B212" s="2" t="s">
         <v>735</v>
       </c>
-      <c r="C211" s="2" t="s">
+      <c r="C212" s="2" t="s">
         <v>737</v>
-      </c>
-    </row>
-    <row r="212" spans="1:3" ht="45" x14ac:dyDescent="0.25">
-      <c r="A212" s="2" t="s">
-        <v>728</v>
-      </c>
-      <c r="B212" s="2" t="s">
-        <v>729</v>
-      </c>
-      <c r="C212" s="2" t="s">
-        <v>738</v>
       </c>
     </row>
     <row r="213" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A213" s="2" t="s">
+        <v>728</v>
+      </c>
+      <c r="B213" s="2" t="s">
+        <v>729</v>
+      </c>
+      <c r="C213" s="2" t="s">
+        <v>738</v>
+      </c>
+    </row>
+    <row r="214" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A214" s="2" t="s">
         <v>730</v>
       </c>
-      <c r="B213" s="2" t="s">
+      <c r="B214" s="2" t="s">
         <v>731</v>
       </c>
-      <c r="C213" s="2" t="s">
+      <c r="C214" s="2" t="s">
         <v>739</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Added translation for "canBeUsed" on switches.
</commit_message>
<xml_diff>
--- a/Translations/Translations.xlsx
+++ b/Translations/Translations.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programacion\MelonLoader\FS_LevelEditor\Translations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6191E90-3161-47AF-AFA2-8D96590A7A7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08401188-9007-404E-9EB5-82E3577E19F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{F5C22481-FF1A-482C-BF7E-EB5A7718AF49}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1436" uniqueCount="743">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1439" uniqueCount="745">
   <si>
     <t>ID</t>
   </si>
@@ -2267,13 +2267,19 @@
   </si>
   <si>
     <t>Al Insertar</t>
+  </si>
+  <si>
+    <t>canBeUsed</t>
+  </si>
+  <si>
+    <t>Usable</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2291,6 +2297,14 @@
     </font>
     <font>
       <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -2337,7 +2351,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -2349,6 +2363,9 @@
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2666,7 +2683,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6961A5F-F8EA-4989-8112-A0ACE51D011E}">
   <sheetPr codeName="Hoja1"/>
-  <dimension ref="A1:D214"/>
+  <dimension ref="A1:D217"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="37" style="2" customWidth="1"/>
@@ -5501,6 +5518,20 @@
       <c r="C214" s="2" t="s">
         <v>739</v>
       </c>
+    </row>
+    <row r="215" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A215" s="2" t="s">
+        <v>743</v>
+      </c>
+      <c r="B215" s="2" t="s">
+        <v>744</v>
+      </c>
+      <c r="C215" s="2" t="s">
+        <v>744</v>
+      </c>
+    </row>
+    <row r="217" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A217" s="5"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>

</xml_diff>

<commit_message>
Added "Destroy Cubes" property for laser fields.
</commit_message>
<xml_diff>
--- a/Translations/Translations.xlsx
+++ b/Translations/Translations.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programacion\MelonLoader\FS_LevelEditor\Translations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08401188-9007-404E-9EB5-82E3577E19F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26A09B9C-D8E5-47C1-B46B-DE4EBA2103A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{F5C22481-FF1A-482C-BF7E-EB5A7718AF49}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1439" uniqueCount="745">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1442" uniqueCount="748">
   <si>
     <t>ID</t>
   </si>
@@ -2273,6 +2273,15 @@
   </si>
   <si>
     <t>Usable</t>
+  </si>
+  <si>
+    <t>DestroyCubes</t>
+  </si>
+  <si>
+    <t>Destroy Cubes</t>
+  </si>
+  <si>
+    <t>Destruir Cubos</t>
   </si>
 </sst>
 </file>
@@ -5530,6 +5539,17 @@
         <v>744</v>
       </c>
     </row>
+    <row r="216" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A216" s="2" t="s">
+        <v>745</v>
+      </c>
+      <c r="B216" s="2" t="s">
+        <v>746</v>
+      </c>
+      <c r="C216" s="2" t="s">
+        <v>747</v>
+      </c>
+    </row>
     <row r="217" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A217" s="5"/>
     </row>

</xml_diff>

<commit_message>
Implemented primitive upgrade terminals.
</commit_message>
<xml_diff>
--- a/Translations/Translations.xlsx
+++ b/Translations/Translations.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programacion\MelonLoader\FS_LevelEditor\Translations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26A09B9C-D8E5-47C1-B46B-DE4EBA2103A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBD89AB5-FC0B-4A1E-9873-73A12E7F3EAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{F5C22481-FF1A-482C-BF7E-EB5A7718AF49}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1442" uniqueCount="748">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1445" uniqueCount="751">
   <si>
     <t>ID</t>
   </si>
@@ -2282,6 +2282,15 @@
   </si>
   <si>
     <t>Destruir Cubos</t>
+  </si>
+  <si>
+    <t>object.UPGRADE_TERMINAL</t>
+  </si>
+  <si>
+    <t>Upgrade Terminal</t>
+  </si>
+  <si>
+    <t>Terminal de Mejora</t>
   </si>
 </sst>
 </file>
@@ -3566,1992 +3575,2001 @@
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" s="2" t="s">
-        <v>69</v>
+        <v>748</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>69</v>
+        <v>749</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="D64" s="2" t="s">
-        <v>364</v>
-      </c>
+        <v>750</v>
+      </c>
+      <c r="D64" s="5"/>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A65" s="2" t="s">
-        <v>443</v>
+        <v>69</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>443</v>
+        <v>69</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>601</v>
+        <v>101</v>
       </c>
       <c r="D65" s="2" t="s">
-        <v>552</v>
+        <v>364</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66" s="2" t="s">
-        <v>456</v>
+        <v>443</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>456</v>
+        <v>443</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>456</v>
+        <v>601</v>
       </c>
       <c r="D66" s="2" t="s">
-        <v>457</v>
+        <v>552</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A67" s="2" t="s">
-        <v>105</v>
+        <v>456</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>2</v>
+        <v>456</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>102</v>
+        <v>456</v>
       </c>
       <c r="D67" s="2" t="s">
-        <v>365</v>
+        <v>457</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A68" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D68" s="2" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A69" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D69" s="2" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A70" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>111</v>
+        <v>4</v>
       </c>
       <c r="C70" s="2" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="D70" s="2" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A71" s="2" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="D71" s="2" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A72" s="2" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="D72" s="2" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A73" s="2" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="C73" s="2" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="D73" s="2" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A74" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="C74" s="2" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D74" s="2" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A75" s="2" t="s">
-        <v>445</v>
+        <v>118</v>
       </c>
       <c r="B75" s="2" t="s">
-        <v>446</v>
+        <v>122</v>
       </c>
       <c r="C75" s="2" t="s">
-        <v>459</v>
+        <v>121</v>
       </c>
       <c r="D75" s="2" t="s">
-        <v>447</v>
+        <v>370</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A76" s="2" t="s">
-        <v>512</v>
+        <v>445</v>
       </c>
       <c r="B76" s="2" t="s">
-        <v>513</v>
+        <v>446</v>
       </c>
       <c r="C76" s="2" t="s">
-        <v>602</v>
+        <v>459</v>
       </c>
       <c r="D76" s="2" t="s">
-        <v>514</v>
+        <v>447</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A77" s="2" t="s">
-        <v>518</v>
+        <v>512</v>
       </c>
       <c r="B77" s="2" t="s">
-        <v>519</v>
+        <v>513</v>
       </c>
       <c r="C77" s="2" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="D77" s="2" t="s">
-        <v>520</v>
+        <v>514</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A78" s="2" t="s">
-        <v>521</v>
+        <v>518</v>
       </c>
       <c r="B78" s="2" t="s">
-        <v>522</v>
+        <v>519</v>
       </c>
       <c r="C78" s="2" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="D78" s="2" t="s">
-        <v>523</v>
+        <v>520</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A79" s="2" t="s">
-        <v>532</v>
+        <v>521</v>
       </c>
       <c r="B79" s="2" t="s">
-        <v>533</v>
+        <v>522</v>
       </c>
       <c r="C79" s="2" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="D79" s="2" t="s">
-        <v>534</v>
+        <v>523</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
-        <v>537</v>
+        <v>532</v>
       </c>
       <c r="B80" s="2" t="s">
-        <v>535</v>
+        <v>533</v>
       </c>
       <c r="C80" s="2" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="D80" s="2" t="s">
-        <v>536</v>
+        <v>534</v>
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A81" s="2" t="s">
-        <v>740</v>
+        <v>537</v>
       </c>
       <c r="B81" s="2" t="s">
-        <v>741</v>
+        <v>535</v>
       </c>
       <c r="C81" s="2" t="s">
-        <v>742</v>
+        <v>606</v>
+      </c>
+      <c r="D81" s="2" t="s">
+        <v>536</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A82" s="2" t="s">
-        <v>154</v>
+        <v>740</v>
       </c>
       <c r="B82" s="2" t="s">
-        <v>155</v>
+        <v>741</v>
       </c>
       <c r="C82" s="2" t="s">
-        <v>156</v>
-      </c>
-      <c r="D82" s="2" t="s">
-        <v>371</v>
+        <v>742</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A83" s="2" t="s">
-        <v>164</v>
+        <v>154</v>
       </c>
       <c r="B83" s="2" t="s">
-        <v>165</v>
+        <v>155</v>
       </c>
       <c r="C83" s="2" t="s">
-        <v>166</v>
+        <v>156</v>
       </c>
       <c r="D83" s="2" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A84" s="2" t="s">
-        <v>157</v>
+        <v>164</v>
       </c>
       <c r="B84" s="2" t="s">
-        <v>158</v>
+        <v>165</v>
       </c>
       <c r="C84" s="2" t="s">
-        <v>159</v>
+        <v>166</v>
       </c>
       <c r="D84" s="2" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A85" s="2" t="s">
-        <v>167</v>
+        <v>157</v>
       </c>
       <c r="B85" s="2" t="s">
-        <v>168</v>
+        <v>158</v>
       </c>
       <c r="C85" s="2" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="D85" s="2" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A86" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="B86" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="C86" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="D86" s="2" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A87" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="B86" s="2" t="s">
+      <c r="B87" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="C86" s="2" t="s">
+      <c r="C87" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="D86" s="2" t="s">
+      <c r="D87" s="2" t="s">
         <v>375</v>
       </c>
     </row>
-    <row r="87" spans="1:4" ht="45" x14ac:dyDescent="0.25">
-      <c r="A87" s="2" t="s">
+    <row r="88" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="A88" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="B87" s="2" t="s">
+      <c r="B88" s="2" t="s">
         <v>163</v>
       </c>
-      <c r="C87" s="2" t="s">
+      <c r="C88" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="D87" s="2" t="s">
+      <c r="D88" s="2" t="s">
         <v>376</v>
-      </c>
-    </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A88" s="2" t="s">
-        <v>153</v>
-      </c>
-      <c r="B88" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="C88" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="D88" s="2" t="s">
-        <v>328</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A89" s="2" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="B89" s="2" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="C89" s="2" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="D89" s="2" t="s">
-        <v>377</v>
+        <v>328</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A90" s="2" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="B90" s="2" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="C90" s="2" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="D90" s="2" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A91" s="2" t="s">
-        <v>172</v>
+        <v>150</v>
       </c>
       <c r="B91" s="2" t="s">
-        <v>170</v>
+        <v>151</v>
       </c>
       <c r="C91" s="2" t="s">
-        <v>171</v>
+        <v>152</v>
       </c>
       <c r="D91" s="2" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A92" s="2" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B92" s="2" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="C92" s="2" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="D92" s="2" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A93" s="2" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="B93" s="2" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="C93" s="2" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="D93" s="2" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A94" s="2" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="B94" s="2" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="C94" s="2" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="D94" s="2" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A95" s="2" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="B95" s="2" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="C95" s="2" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="D95" s="2" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A96" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="B96" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="C96" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="D96" s="2" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A97" s="2" t="s">
         <v>243</v>
       </c>
-      <c r="B96" s="2" t="s">
+      <c r="B97" s="2" t="s">
         <v>243</v>
       </c>
-      <c r="C96" s="2" t="s">
+      <c r="C97" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="D96" s="2" t="s">
+      <c r="D97" s="2" t="s">
         <v>384</v>
       </c>
     </row>
-    <row r="97" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A97" s="2" t="s">
+    <row r="98" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A98" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="B97" s="1" t="s">
+      <c r="B98" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="C97" s="2" t="s">
+      <c r="C98" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="D97" s="2" t="s">
+      <c r="D98" s="2" t="s">
         <v>385</v>
-      </c>
-    </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A98" s="2" t="s">
-        <v>182</v>
-      </c>
-      <c r="B98" s="2" t="s">
-        <v>183</v>
-      </c>
-      <c r="C98" s="2" t="s">
-        <v>183</v>
-      </c>
-      <c r="D98" s="2" t="s">
-        <v>386</v>
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A99" s="2" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="B99" s="2" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C99" s="2" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="D99" s="2" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A100" s="2" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="B100" s="2" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="C100" s="2" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="D100" s="2" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A101" s="2" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="B101" s="2" t="s">
-        <v>525</v>
+        <v>186</v>
       </c>
       <c r="C101" s="2" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="D101" s="2" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A102" s="2" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="B102" s="2" t="s">
-        <v>190</v>
+        <v>525</v>
       </c>
       <c r="C102" s="2" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="D102" s="2" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A103" s="2" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="B103" s="2" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="C103" s="2" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="D103" s="2" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A104" s="2" t="s">
-        <v>434</v>
-      </c>
-      <c r="B104" s="4" t="s">
-        <v>435</v>
-      </c>
-      <c r="C104" s="4" t="s">
-        <v>436</v>
-      </c>
-      <c r="D104" s="4" t="s">
-        <v>591</v>
+        <v>192</v>
+      </c>
+      <c r="B104" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="C104" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="D104" s="2" t="s">
+        <v>391</v>
       </c>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A105" s="2" t="s">
-        <v>437</v>
+        <v>434</v>
       </c>
       <c r="B105" s="4" t="s">
-        <v>438</v>
+        <v>435</v>
       </c>
       <c r="C105" s="4" t="s">
-        <v>439</v>
+        <v>436</v>
       </c>
       <c r="D105" s="4" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A106" s="2" t="s">
-        <v>473</v>
+        <v>437</v>
       </c>
       <c r="B106" s="4" t="s">
-        <v>590</v>
+        <v>438</v>
       </c>
       <c r="C106" s="4" t="s">
-        <v>474</v>
+        <v>439</v>
       </c>
       <c r="D106" s="4" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A107" s="2" t="s">
-        <v>195</v>
-      </c>
-      <c r="B107" s="2" t="s">
-        <v>196</v>
-      </c>
-      <c r="C107" s="2" t="s">
-        <v>197</v>
-      </c>
-      <c r="D107" s="2" t="s">
-        <v>392</v>
+        <v>473</v>
+      </c>
+      <c r="B107" s="4" t="s">
+        <v>590</v>
+      </c>
+      <c r="C107" s="4" t="s">
+        <v>474</v>
+      </c>
+      <c r="D107" s="4" t="s">
+        <v>593</v>
       </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A108" s="2" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="B108" s="2" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="C108" s="2" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="D108" s="2" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A109" s="2" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="B109" s="2" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="C109" s="2" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="D109" s="2" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A110" s="2" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="B110" s="2" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="C110" s="2" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="D110" s="2" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A111" s="2" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="B111" s="2" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="C111" s="2" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="D111" s="2" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A112" s="2" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B112" s="2" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="C112" s="2" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="D112" s="2" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A113" s="2" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="B113" s="2" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="C113" s="2" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="D113" s="2" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A114" s="2" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="B114" s="2" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="C114" s="2" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="D114" s="2" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A115" s="2" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="B115" s="2" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="C115" s="2" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="D115" s="2" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A116" s="2" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="B116" s="2" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="C116" s="2" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="D116" s="2" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A117" s="2" t="s">
-        <v>292</v>
+        <v>220</v>
       </c>
       <c r="B117" s="2" t="s">
-        <v>292</v>
+        <v>219</v>
       </c>
       <c r="C117" s="2" t="s">
-        <v>293</v>
+        <v>218</v>
       </c>
       <c r="D117" s="2" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A118" s="2" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="B118" s="2" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="C118" s="2" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
       <c r="D118" s="2" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
     </row>
     <row r="119" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A119" s="2" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
       <c r="B119" s="2" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="C119" s="2" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="D119" s="2" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A120" s="2" t="s">
-        <v>221</v>
+        <v>297</v>
       </c>
       <c r="B120" s="2" t="s">
-        <v>221</v>
+        <v>298</v>
       </c>
       <c r="C120" s="2" t="s">
-        <v>222</v>
+        <v>299</v>
       </c>
       <c r="D120" s="2" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A121" s="2" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="B121" s="2" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="C121" s="2" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="D121" s="2" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A122" s="2" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="B122" s="2" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="C122" s="2" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="D122" s="2" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
     </row>
     <row r="123" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A123" s="2" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="B123" s="2" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="C123" s="2" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="D123" s="2" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
     </row>
     <row r="124" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A124" s="2" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B124" s="2" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="C124" s="2" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="D124" s="2" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
     </row>
     <row r="125" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A125" s="2" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="B125" s="2" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="C125" s="2" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="D125" s="2" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
     </row>
     <row r="126" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A126" s="2" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="B126" s="2" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="C126" s="2" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="D126" s="2" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
     </row>
     <row r="127" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A127" s="2" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="B127" s="2" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="C127" s="2" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="D127" s="2" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
     </row>
     <row r="128" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A128" s="2" t="s">
-        <v>300</v>
+        <v>237</v>
       </c>
       <c r="B128" s="2" t="s">
-        <v>301</v>
+        <v>238</v>
       </c>
       <c r="C128" s="2" t="s">
-        <v>302</v>
+        <v>239</v>
       </c>
       <c r="D128" s="2" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
     </row>
     <row r="129" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A129" s="2" t="s">
-        <v>240</v>
+        <v>300</v>
       </c>
       <c r="B129" s="2" t="s">
-        <v>241</v>
+        <v>301</v>
       </c>
       <c r="C129" s="2" t="s">
-        <v>242</v>
+        <v>302</v>
       </c>
       <c r="D129" s="2" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
     </row>
     <row r="130" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A130" s="2" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="B130" s="2" t="s">
-        <v>252</v>
+        <v>241</v>
       </c>
       <c r="C130" s="2" t="s">
-        <v>251</v>
+        <v>242</v>
       </c>
       <c r="D130" s="2" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="131" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A131" s="2" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B131" s="2" t="s">
-        <v>245</v>
+        <v>252</v>
       </c>
       <c r="C131" s="2" t="s">
-        <v>246</v>
+        <v>251</v>
       </c>
       <c r="D131" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
     </row>
     <row r="132" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A132" s="2" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="B132" s="2" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="C132" s="2" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="D132" s="2" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
     </row>
     <row r="133" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A133" s="2" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="B133" s="2" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="C133" s="2" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="D133" s="2" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
     </row>
     <row r="134" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A134" s="2" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="B134" s="2" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="C134" s="2" t="s">
-        <v>255</v>
+        <v>250</v>
       </c>
       <c r="D134" s="2" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
     </row>
     <row r="135" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A135" s="2" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="B135" s="2" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="C135" s="2" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="D135" s="2" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
     </row>
     <row r="136" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A136" s="2" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="B136" s="2" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="C136" s="2" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="D136" s="2" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
     </row>
     <row r="137" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A137" s="2" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="B137" s="2" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="C137" s="2" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="D137" s="2" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="138" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A138" s="2" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="B138" s="2" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="C138" s="2" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="D138" s="2" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
     </row>
     <row r="139" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A139" s="2" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="B139" s="2" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="C139" s="2" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="D139" s="2" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
     </row>
     <row r="140" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A140" s="2" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="B140" s="2" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="C140" s="2" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="D140" s="2" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
     </row>
     <row r="141" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A141" s="2" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="B141" s="2" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="C141" s="2" t="s">
-        <v>273</v>
+        <v>269</v>
       </c>
       <c r="D141" s="2" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
     </row>
     <row r="142" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A142" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="B142" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="C142" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="D142" s="2" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="143" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A143" s="2" t="s">
         <v>271</v>
       </c>
-      <c r="B142" s="2" t="s">
+      <c r="B143" s="2" t="s">
         <v>271</v>
       </c>
-      <c r="C142" s="2" t="s">
+      <c r="C143" s="2" t="s">
         <v>272</v>
       </c>
-      <c r="D142" s="2" t="s">
+      <c r="D143" s="2" t="s">
         <v>427</v>
       </c>
     </row>
-    <row r="143" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A143" s="2" t="s">
+    <row r="144" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A144" s="2" t="s">
         <v>274</v>
       </c>
-      <c r="B143" s="2" t="s">
+      <c r="B144" s="2" t="s">
         <v>276</v>
       </c>
-      <c r="C143" s="2" t="s">
+      <c r="C144" s="2" t="s">
         <v>279</v>
       </c>
     </row>
-    <row r="144" spans="1:4" ht="45" x14ac:dyDescent="0.25">
-      <c r="A144" s="2" t="s">
+    <row r="145" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="A145" s="2" t="s">
         <v>275</v>
       </c>
-      <c r="B144" s="2" t="s">
+      <c r="B145" s="2" t="s">
         <v>277</v>
       </c>
-      <c r="C144" s="2" t="s">
+      <c r="C145" s="2" t="s">
         <v>278</v>
       </c>
     </row>
-    <row r="145" spans="1:4" ht="75" x14ac:dyDescent="0.25">
-      <c r="A145" s="2" t="s">
+    <row r="146" spans="1:4" ht="75" x14ac:dyDescent="0.25">
+      <c r="A146" s="2" t="s">
         <v>289</v>
       </c>
-      <c r="B145" s="2" t="s">
+      <c r="B146" s="2" t="s">
         <v>290</v>
       </c>
-      <c r="C145" s="2" t="s">
+      <c r="C146" s="2" t="s">
         <v>291</v>
-      </c>
-    </row>
-    <row r="146" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A146" s="2" t="s">
-        <v>306</v>
-      </c>
-      <c r="B146" s="2" t="s">
-        <v>307</v>
-      </c>
-      <c r="C146" s="2" t="s">
-        <v>308</v>
-      </c>
-      <c r="D146" s="2" t="s">
-        <v>428</v>
       </c>
     </row>
     <row r="147" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A147" s="2" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
       <c r="B147" s="2" t="s">
-        <v>311</v>
+        <v>307</v>
       </c>
       <c r="C147" s="2" t="s">
-        <v>312</v>
+        <v>308</v>
       </c>
       <c r="D147" s="2" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
     </row>
     <row r="148" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A148" s="2" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="B148" s="2" t="s">
-        <v>314</v>
+        <v>311</v>
       </c>
       <c r="C148" s="2" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="D148" s="2" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
     </row>
     <row r="149" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A149" s="2" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="B149" s="2" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="C149" s="2" t="s">
-        <v>316</v>
+        <v>313</v>
       </c>
       <c r="D149" s="2" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
     </row>
     <row r="150" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A150" s="2" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="B150" s="2" t="s">
-        <v>318</v>
+        <v>315</v>
       </c>
       <c r="C150" s="2" t="s">
-        <v>460</v>
+        <v>316</v>
       </c>
       <c r="D150" s="2" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
     </row>
     <row r="151" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A151" s="2" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="B151" s="2" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="C151" s="2" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="D151" s="2" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
     </row>
     <row r="152" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A152" s="2" t="s">
-        <v>448</v>
+        <v>319</v>
       </c>
       <c r="B152" s="2" t="s">
-        <v>448</v>
+        <v>320</v>
       </c>
       <c r="C152" s="2" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="D152" s="2" t="s">
-        <v>345</v>
+        <v>433</v>
       </c>
     </row>
     <row r="153" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A153" s="2" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="B153" s="2" t="s">
-        <v>450</v>
+        <v>448</v>
       </c>
       <c r="C153" s="2" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="D153" s="2" t="s">
-        <v>451</v>
+        <v>345</v>
       </c>
     </row>
     <row r="154" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A154" s="2" t="s">
-        <v>475</v>
+        <v>449</v>
       </c>
       <c r="B154" s="2" t="s">
-        <v>476</v>
+        <v>450</v>
       </c>
       <c r="C154" s="2" t="s">
-        <v>619</v>
+        <v>463</v>
       </c>
       <c r="D154" s="2" t="s">
-        <v>569</v>
+        <v>451</v>
       </c>
     </row>
     <row r="155" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A155" s="2" t="s">
-        <v>478</v>
+        <v>475</v>
       </c>
       <c r="B155" s="2" t="s">
-        <v>524</v>
+        <v>476</v>
       </c>
       <c r="C155" s="2" t="s">
-        <v>479</v>
+        <v>619</v>
       </c>
       <c r="D155" s="2" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
     </row>
     <row r="156" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A156" s="2" t="s">
-        <v>480</v>
+        <v>478</v>
       </c>
       <c r="B156" s="2" t="s">
-        <v>481</v>
+        <v>524</v>
       </c>
       <c r="C156" s="2" t="s">
-        <v>482</v>
+        <v>479</v>
       </c>
       <c r="D156" s="2" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
     </row>
     <row r="157" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A157" s="2" t="s">
-        <v>483</v>
+        <v>480</v>
       </c>
       <c r="B157" s="2" t="s">
-        <v>484</v>
+        <v>481</v>
       </c>
       <c r="C157" s="2" t="s">
-        <v>485</v>
+        <v>482</v>
       </c>
       <c r="D157" s="2" t="s">
-        <v>566</v>
+        <v>567</v>
       </c>
     </row>
     <row r="158" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A158" s="2" t="s">
-        <v>486</v>
+        <v>483</v>
       </c>
       <c r="B158" s="2" t="s">
-        <v>487</v>
+        <v>484</v>
       </c>
       <c r="C158" s="2" t="s">
-        <v>488</v>
+        <v>485</v>
       </c>
       <c r="D158" s="2" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
     </row>
     <row r="159" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A159" s="2" t="s">
-        <v>489</v>
+        <v>486</v>
       </c>
       <c r="B159" s="2" t="s">
-        <v>490</v>
+        <v>487</v>
       </c>
       <c r="C159" s="2" t="s">
-        <v>491</v>
+        <v>488</v>
       </c>
       <c r="D159" s="2" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
     </row>
     <row r="160" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A160" s="2" t="s">
-        <v>538</v>
+        <v>489</v>
       </c>
       <c r="B160" s="2" t="s">
-        <v>538</v>
+        <v>490</v>
       </c>
       <c r="C160" s="2" t="s">
-        <v>607</v>
+        <v>491</v>
       </c>
       <c r="D160" s="2" t="s">
-        <v>539</v>
+        <v>564</v>
       </c>
     </row>
     <row r="161" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A161" s="2" t="s">
-        <v>540</v>
+        <v>538</v>
       </c>
       <c r="B161" s="2" t="s">
-        <v>541</v>
+        <v>538</v>
       </c>
       <c r="C161" s="2" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="D161" s="2" t="s">
-        <v>542</v>
+        <v>539</v>
       </c>
     </row>
     <row r="162" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A162" s="2" t="s">
-        <v>492</v>
+        <v>540</v>
       </c>
       <c r="B162" s="2" t="s">
-        <v>493</v>
+        <v>541</v>
       </c>
       <c r="C162" s="2" t="s">
-        <v>494</v>
+        <v>608</v>
       </c>
       <c r="D162" s="2" t="s">
-        <v>563</v>
+        <v>542</v>
       </c>
     </row>
     <row r="163" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A163" s="2" t="s">
-        <v>495</v>
+        <v>492</v>
       </c>
       <c r="B163" s="2" t="s">
-        <v>496</v>
+        <v>493</v>
       </c>
       <c r="C163" s="2" t="s">
-        <v>497</v>
+        <v>494</v>
       </c>
       <c r="D163" s="2" t="s">
-        <v>562</v>
+        <v>563</v>
       </c>
     </row>
     <row r="164" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A164" s="2" t="s">
-        <v>498</v>
+        <v>495</v>
       </c>
       <c r="B164" s="2" t="s">
-        <v>499</v>
+        <v>496</v>
       </c>
       <c r="C164" s="2" t="s">
-        <v>500</v>
+        <v>497</v>
       </c>
       <c r="D164" s="2" t="s">
-        <v>561</v>
+        <v>562</v>
       </c>
     </row>
     <row r="165" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A165" s="2" t="s">
-        <v>501</v>
+        <v>498</v>
       </c>
       <c r="B165" s="2" t="s">
-        <v>501</v>
+        <v>499</v>
       </c>
       <c r="C165" s="2" t="s">
-        <v>502</v>
+        <v>500</v>
       </c>
       <c r="D165" s="2" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
     </row>
     <row r="166" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A166" s="2" t="s">
-        <v>503</v>
+        <v>501</v>
       </c>
       <c r="B166" s="2" t="s">
-        <v>503</v>
+        <v>501</v>
       </c>
       <c r="C166" s="2" t="s">
-        <v>504</v>
+        <v>502</v>
       </c>
       <c r="D166" s="2" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
     </row>
     <row r="167" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A167" s="2" t="s">
-        <v>505</v>
+        <v>503</v>
       </c>
       <c r="B167" s="2" t="s">
-        <v>505</v>
+        <v>503</v>
       </c>
       <c r="C167" s="2" t="s">
-        <v>506</v>
+        <v>504</v>
       </c>
       <c r="D167" s="2" t="s">
-        <v>558</v>
+        <v>559</v>
       </c>
     </row>
     <row r="168" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A168" s="2" t="s">
-        <v>507</v>
+        <v>505</v>
       </c>
       <c r="B168" s="2" t="s">
-        <v>507</v>
+        <v>505</v>
       </c>
       <c r="C168" s="2" t="s">
-        <v>508</v>
+        <v>506</v>
       </c>
       <c r="D168" s="2" t="s">
-        <v>557</v>
+        <v>558</v>
       </c>
     </row>
     <row r="169" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A169" s="2" t="s">
-        <v>570</v>
+        <v>507</v>
       </c>
       <c r="B169" s="2" t="s">
-        <v>571</v>
+        <v>507</v>
       </c>
       <c r="C169" s="2" t="s">
-        <v>609</v>
+        <v>508</v>
+      </c>
+      <c r="D169" s="2" t="s">
+        <v>557</v>
       </c>
     </row>
     <row r="170" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A170" s="2" t="s">
-        <v>572</v>
+        <v>570</v>
       </c>
       <c r="B170" s="2" t="s">
-        <v>573</v>
+        <v>571</v>
       </c>
       <c r="C170" s="2" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
     </row>
     <row r="171" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A171" s="2" t="s">
-        <v>574</v>
+        <v>572</v>
       </c>
       <c r="B171" s="2" t="s">
-        <v>575</v>
+        <v>573</v>
       </c>
       <c r="C171" s="2" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
     </row>
     <row r="172" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A172" s="2" t="s">
-        <v>576</v>
+        <v>574</v>
       </c>
       <c r="B172" s="2" t="s">
-        <v>577</v>
+        <v>575</v>
       </c>
       <c r="C172" s="2" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
     </row>
     <row r="173" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A173" s="2" t="s">
-        <v>578</v>
+        <v>576</v>
       </c>
       <c r="B173" s="2" t="s">
-        <v>579</v>
+        <v>577</v>
       </c>
       <c r="C173" s="2" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
     </row>
     <row r="174" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A174" s="2" t="s">
-        <v>580</v>
+        <v>578</v>
       </c>
       <c r="B174" s="2" t="s">
-        <v>581</v>
+        <v>579</v>
       </c>
       <c r="C174" s="2" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
     </row>
     <row r="175" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A175" s="2" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
       <c r="B175" s="2" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="C175" s="2" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
     </row>
     <row r="176" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A176" s="2" t="s">
-        <v>584</v>
+        <v>582</v>
       </c>
       <c r="B176" s="2" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="C176" s="2" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
     </row>
     <row r="177" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A177" s="2" t="s">
-        <v>586</v>
+        <v>584</v>
       </c>
       <c r="B177" s="2" t="s">
-        <v>587</v>
+        <v>585</v>
       </c>
       <c r="C177" s="2" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
     </row>
     <row r="178" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A178" s="2" t="s">
-        <v>588</v>
+        <v>586</v>
       </c>
       <c r="B178" s="2" t="s">
-        <v>589</v>
+        <v>587</v>
       </c>
       <c r="C178" s="2" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
     </row>
     <row r="179" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A179" s="2" t="s">
-        <v>620</v>
+        <v>588</v>
       </c>
       <c r="B179" s="2" t="s">
-        <v>621</v>
+        <v>589</v>
       </c>
       <c r="C179" s="2" t="s">
-        <v>622</v>
+        <v>618</v>
       </c>
     </row>
     <row r="180" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A180" s="2" t="s">
-        <v>623</v>
+        <v>620</v>
       </c>
       <c r="B180" s="2" t="s">
-        <v>623</v>
+        <v>621</v>
       </c>
       <c r="C180" s="2" t="s">
-        <v>624</v>
+        <v>622</v>
       </c>
     </row>
     <row r="181" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A181" s="2" t="s">
-        <v>625</v>
+        <v>623</v>
       </c>
       <c r="B181" s="2" t="s">
-        <v>625</v>
+        <v>623</v>
       </c>
       <c r="C181" s="2" t="s">
-        <v>627</v>
+        <v>624</v>
       </c>
     </row>
     <row r="182" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A182" s="2" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="B182" s="2" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="C182" s="2" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
     </row>
     <row r="183" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A183" s="2" t="s">
-        <v>629</v>
+        <v>626</v>
       </c>
       <c r="B183" s="2" t="s">
-        <v>630</v>
+        <v>626</v>
       </c>
       <c r="C183" s="2" t="s">
-        <v>631</v>
+        <v>628</v>
       </c>
     </row>
     <row r="184" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A184" s="2" t="s">
-        <v>632</v>
-      </c>
-      <c r="B184" s="4" t="s">
-        <v>633</v>
-      </c>
-      <c r="C184" s="4" t="s">
-        <v>634</v>
+        <v>629</v>
+      </c>
+      <c r="B184" s="2" t="s">
+        <v>630</v>
+      </c>
+      <c r="C184" s="2" t="s">
+        <v>631</v>
       </c>
     </row>
     <row r="185" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A185" s="2" t="s">
-        <v>638</v>
-      </c>
-      <c r="B185" s="2" t="s">
-        <v>639</v>
-      </c>
-      <c r="C185" s="2" t="s">
-        <v>640</v>
+        <v>632</v>
+      </c>
+      <c r="B185" s="4" t="s">
+        <v>633</v>
+      </c>
+      <c r="C185" s="4" t="s">
+        <v>634</v>
       </c>
     </row>
     <row r="186" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A186" s="2" t="s">
-        <v>641</v>
+        <v>638</v>
       </c>
       <c r="B186" s="2" t="s">
-        <v>641</v>
+        <v>639</v>
       </c>
       <c r="C186" s="2" t="s">
-        <v>642</v>
+        <v>640</v>
       </c>
     </row>
     <row r="187" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A187" s="2" t="s">
-        <v>643</v>
+        <v>641</v>
       </c>
       <c r="B187" s="2" t="s">
-        <v>644</v>
+        <v>641</v>
       </c>
       <c r="C187" s="2" t="s">
-        <v>645</v>
+        <v>642</v>
       </c>
     </row>
     <row r="188" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A188" s="2" t="s">
-        <v>646</v>
+        <v>643</v>
       </c>
       <c r="B188" s="2" t="s">
-        <v>647</v>
+        <v>644</v>
       </c>
       <c r="C188" s="2" t="s">
-        <v>648</v>
+        <v>645</v>
       </c>
     </row>
     <row r="189" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A189" s="2" t="s">
-        <v>649</v>
+        <v>646</v>
       </c>
       <c r="B189" s="2" t="s">
-        <v>650</v>
+        <v>647</v>
       </c>
       <c r="C189" s="2" t="s">
-        <v>651</v>
+        <v>648</v>
       </c>
     </row>
     <row r="190" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A190" s="2" t="s">
-        <v>652</v>
+        <v>649</v>
       </c>
       <c r="B190" s="2" t="s">
-        <v>653</v>
+        <v>650</v>
       </c>
       <c r="C190" s="2" t="s">
-        <v>654</v>
+        <v>651</v>
       </c>
     </row>
     <row r="191" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A191" s="2" t="s">
-        <v>655</v>
+        <v>652</v>
       </c>
       <c r="B191" s="2" t="s">
-        <v>655</v>
+        <v>653</v>
       </c>
       <c r="C191" s="2" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
     </row>
     <row r="192" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A192" s="2" t="s">
-        <v>657</v>
+        <v>655</v>
       </c>
       <c r="B192" s="2" t="s">
-        <v>658</v>
+        <v>655</v>
       </c>
       <c r="C192" s="2" t="s">
-        <v>659</v>
+        <v>656</v>
       </c>
     </row>
     <row r="193" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A193" s="2" t="s">
-        <v>666</v>
-      </c>
-      <c r="B193" s="4" t="s">
-        <v>667</v>
-      </c>
-      <c r="C193" s="4" t="s">
-        <v>668</v>
+        <v>657</v>
+      </c>
+      <c r="B193" s="2" t="s">
+        <v>658</v>
+      </c>
+      <c r="C193" s="2" t="s">
+        <v>659</v>
       </c>
     </row>
     <row r="194" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A194" s="2" t="s">
-        <v>669</v>
-      </c>
-      <c r="B194" s="2" t="s">
-        <v>670</v>
-      </c>
-      <c r="C194" s="2" t="s">
-        <v>671</v>
+        <v>666</v>
+      </c>
+      <c r="B194" s="4" t="s">
+        <v>667</v>
+      </c>
+      <c r="C194" s="4" t="s">
+        <v>668</v>
       </c>
     </row>
     <row r="195" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A195" s="2" t="s">
-        <v>675</v>
+        <v>669</v>
       </c>
       <c r="B195" s="2" t="s">
-        <v>676</v>
+        <v>670</v>
       </c>
       <c r="C195" s="2" t="s">
-        <v>677</v>
+        <v>671</v>
       </c>
     </row>
     <row r="196" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A196" s="2" t="s">
-        <v>678</v>
+        <v>675</v>
       </c>
       <c r="B196" s="2" t="s">
-        <v>679</v>
+        <v>676</v>
       </c>
       <c r="C196" s="2" t="s">
-        <v>680</v>
+        <v>677</v>
       </c>
     </row>
     <row r="197" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A197" s="2" t="s">
-        <v>681</v>
+        <v>678</v>
       </c>
       <c r="B197" s="2" t="s">
-        <v>682</v>
+        <v>679</v>
       </c>
       <c r="C197" s="2" t="s">
-        <v>683</v>
+        <v>680</v>
       </c>
     </row>
     <row r="198" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A198" s="2" t="s">
-        <v>684</v>
+        <v>681</v>
       </c>
       <c r="B198" s="2" t="s">
-        <v>685</v>
+        <v>682</v>
       </c>
       <c r="C198" s="2" t="s">
-        <v>686</v>
+        <v>683</v>
       </c>
     </row>
     <row r="199" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A199" s="2" t="s">
-        <v>687</v>
+        <v>684</v>
       </c>
       <c r="B199" s="2" t="s">
-        <v>688</v>
+        <v>685</v>
       </c>
       <c r="C199" s="2" t="s">
-        <v>689</v>
+        <v>686</v>
       </c>
     </row>
     <row r="200" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A200" s="2" t="s">
-        <v>690</v>
-      </c>
-      <c r="B200" s="4" t="s">
-        <v>694</v>
-      </c>
-      <c r="C200" s="4" t="s">
-        <v>704</v>
+        <v>687</v>
+      </c>
+      <c r="B200" s="2" t="s">
+        <v>688</v>
+      </c>
+      <c r="C200" s="2" t="s">
+        <v>689</v>
       </c>
     </row>
     <row r="201" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A201" s="2" t="s">
-        <v>691</v>
-      </c>
-      <c r="B201" s="2" t="s">
-        <v>697</v>
-      </c>
-      <c r="C201" s="2" t="s">
-        <v>710</v>
+        <v>690</v>
+      </c>
+      <c r="B201" s="4" t="s">
+        <v>694</v>
+      </c>
+      <c r="C201" s="4" t="s">
+        <v>704</v>
       </c>
     </row>
     <row r="202" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A202" s="2" t="s">
-        <v>693</v>
-      </c>
-      <c r="B202" s="4" t="s">
-        <v>695</v>
-      </c>
-      <c r="C202" s="4" t="s">
-        <v>705</v>
+        <v>691</v>
+      </c>
+      <c r="B202" s="2" t="s">
+        <v>697</v>
+      </c>
+      <c r="C202" s="2" t="s">
+        <v>710</v>
       </c>
     </row>
     <row r="203" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A203" s="2" t="s">
-        <v>692</v>
+        <v>693</v>
       </c>
       <c r="B203" s="4" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
       <c r="C203" s="4" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
     </row>
     <row r="204" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A204" s="2" t="s">
-        <v>699</v>
-      </c>
-      <c r="B204" s="2" t="s">
-        <v>698</v>
-      </c>
-      <c r="C204" s="2" t="s">
-        <v>707</v>
+        <v>692</v>
+      </c>
+      <c r="B204" s="4" t="s">
+        <v>696</v>
+      </c>
+      <c r="C204" s="4" t="s">
+        <v>706</v>
       </c>
     </row>
     <row r="205" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A205" s="2" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="B205" s="2" t="s">
-        <v>702</v>
+        <v>698</v>
       </c>
       <c r="C205" s="2" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
     </row>
     <row r="206" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A206" s="2" t="s">
-        <v>701</v>
+        <v>700</v>
       </c>
       <c r="B206" s="2" t="s">
-        <v>703</v>
+        <v>702</v>
       </c>
       <c r="C206" s="2" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
     </row>
     <row r="207" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A207" s="2" t="s">
-        <v>711</v>
+        <v>701</v>
       </c>
       <c r="B207" s="2" t="s">
-        <v>711</v>
+        <v>703</v>
       </c>
       <c r="C207" s="2" t="s">
-        <v>712</v>
+        <v>709</v>
       </c>
     </row>
     <row r="208" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A208" s="2" t="s">
-        <v>713</v>
+        <v>711</v>
       </c>
       <c r="B208" s="2" t="s">
-        <v>714</v>
+        <v>711</v>
       </c>
       <c r="C208" s="2" t="s">
-        <v>715</v>
+        <v>712</v>
       </c>
     </row>
     <row r="209" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A209" s="2" t="s">
-        <v>716</v>
+        <v>713</v>
       </c>
       <c r="B209" s="2" t="s">
-        <v>717</v>
+        <v>714</v>
       </c>
       <c r="C209" s="2" t="s">
-        <v>718</v>
+        <v>715</v>
       </c>
     </row>
     <row r="210" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A210" s="2" t="s">
-        <v>719</v>
+        <v>716</v>
       </c>
       <c r="B210" s="2" t="s">
-        <v>720</v>
+        <v>717</v>
       </c>
       <c r="C210" s="2" t="s">
-        <v>721</v>
+        <v>718</v>
       </c>
     </row>
     <row r="211" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A211" s="2" t="s">
-        <v>732</v>
+        <v>719</v>
       </c>
       <c r="B211" s="2" t="s">
-        <v>733</v>
+        <v>720</v>
       </c>
       <c r="C211" s="2" t="s">
-        <v>736</v>
+        <v>721</v>
       </c>
     </row>
     <row r="212" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A212" s="2" t="s">
+        <v>732</v>
+      </c>
+      <c r="B212" s="2" t="s">
+        <v>733</v>
+      </c>
+      <c r="C212" s="2" t="s">
+        <v>736</v>
+      </c>
+    </row>
+    <row r="213" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A213" s="2" t="s">
         <v>734</v>
       </c>
-      <c r="B212" s="2" t="s">
+      <c r="B213" s="2" t="s">
         <v>735</v>
       </c>
-      <c r="C212" s="2" t="s">
+      <c r="C213" s="2" t="s">
         <v>737</v>
-      </c>
-    </row>
-    <row r="213" spans="1:3" ht="45" x14ac:dyDescent="0.25">
-      <c r="A213" s="2" t="s">
-        <v>728</v>
-      </c>
-      <c r="B213" s="2" t="s">
-        <v>729</v>
-      </c>
-      <c r="C213" s="2" t="s">
-        <v>738</v>
       </c>
     </row>
     <row r="214" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A214" s="2" t="s">
+        <v>728</v>
+      </c>
+      <c r="B214" s="2" t="s">
+        <v>729</v>
+      </c>
+      <c r="C214" s="2" t="s">
+        <v>738</v>
+      </c>
+    </row>
+    <row r="215" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A215" s="2" t="s">
         <v>730</v>
       </c>
-      <c r="B214" s="2" t="s">
+      <c r="B215" s="2" t="s">
         <v>731</v>
       </c>
-      <c r="C214" s="2" t="s">
+      <c r="C215" s="2" t="s">
         <v>739</v>
-      </c>
-    </row>
-    <row r="215" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A215" s="2" t="s">
-        <v>743</v>
-      </c>
-      <c r="B215" s="2" t="s">
-        <v>744</v>
-      </c>
-      <c r="C215" s="2" t="s">
-        <v>744</v>
       </c>
     </row>
     <row r="216" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A216" s="2" t="s">
+        <v>743</v>
+      </c>
+      <c r="B216" s="2" t="s">
+        <v>744</v>
+      </c>
+      <c r="C216" s="2" t="s">
+        <v>744</v>
+      </c>
+    </row>
+    <row r="217" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A217" s="2" t="s">
         <v>745</v>
       </c>
-      <c r="B216" s="2" t="s">
+      <c r="B217" s="2" t="s">
         <v>746</v>
       </c>
-      <c r="C216" s="2" t="s">
+      <c r="C217" s="2" t="s">
         <v>747</v>
       </c>
-    </row>
-    <row r="217" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A217" s="5"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>

</xml_diff>

<commit_message>
Added "Find Object" ui.
</commit_message>
<xml_diff>
--- a/Translations/Translations.xlsx
+++ b/Translations/Translations.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programacion\MelonLoader\FS_LevelEditor\Translations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBD89AB5-FC0B-4A1E-9873-73A12E7F3EAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{853E5F13-460F-47DE-BF62-F26A27F8D94C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{F5C22481-FF1A-482C-BF7E-EB5A7718AF49}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1445" uniqueCount="751">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1457" uniqueCount="763">
   <si>
     <t>ID</t>
   </si>
@@ -2291,6 +2291,42 @@
   </si>
   <si>
     <t>Terminal de Mejora</t>
+  </si>
+  <si>
+    <t>FindObject</t>
+  </si>
+  <si>
+    <t>Find Object</t>
+  </si>
+  <si>
+    <t>Encontrar Objeto</t>
+  </si>
+  <si>
+    <t>SelectObject</t>
+  </si>
+  <si>
+    <t>Select Object</t>
+  </si>
+  <si>
+    <t>Seleccionar Objeto</t>
+  </si>
+  <si>
+    <t>SelectAllObjects</t>
+  </si>
+  <si>
+    <t>Select All Objects</t>
+  </si>
+  <si>
+    <t>Seleccionar Todos los Objetos</t>
+  </si>
+  <si>
+    <t>EnterAnObjectName</t>
+  </si>
+  <si>
+    <t>Enter an object name...</t>
+  </si>
+  <si>
+    <t>Introduce el nombre de un objeto...</t>
   </si>
 </sst>
 </file>
@@ -2701,7 +2737,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6961A5F-F8EA-4989-8112-A0ACE51D011E}">
   <sheetPr codeName="Hoja1"/>
-  <dimension ref="A1:D217"/>
+  <dimension ref="A1:D221"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="37" style="2" customWidth="1"/>
@@ -5569,6 +5605,50 @@
       </c>
       <c r="C217" s="2" t="s">
         <v>747</v>
+      </c>
+    </row>
+    <row r="218" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A218" s="2" t="s">
+        <v>751</v>
+      </c>
+      <c r="B218" s="2" t="s">
+        <v>752</v>
+      </c>
+      <c r="C218" s="2" t="s">
+        <v>753</v>
+      </c>
+    </row>
+    <row r="219" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A219" s="2" t="s">
+        <v>754</v>
+      </c>
+      <c r="B219" s="2" t="s">
+        <v>755</v>
+      </c>
+      <c r="C219" s="2" t="s">
+        <v>756</v>
+      </c>
+    </row>
+    <row r="220" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A220" s="2" t="s">
+        <v>757</v>
+      </c>
+      <c r="B220" s="2" t="s">
+        <v>758</v>
+      </c>
+      <c r="C220" s="2" t="s">
+        <v>759</v>
+      </c>
+    </row>
+    <row r="221" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A221" s="2" t="s">
+        <v>760</v>
+      </c>
+      <c r="B221" s="2" t="s">
+        <v>761</v>
+      </c>
+      <c r="C221" s="2" t="s">
+        <v>762</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added a tooltip for the new power slot initial state prop + REAL tooltip for "Rotate Player" for death triggers respawn points.
</commit_message>
<xml_diff>
--- a/Translations/Translations.xlsx
+++ b/Translations/Translations.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programacion\MelonLoader\FS_LevelEditor\Translations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{853E5F13-460F-47DE-BF62-F26A27F8D94C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{744FF6CA-2AC2-4CEA-BE26-8BBB4380EFA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{F5C22481-FF1A-482C-BF7E-EB5A7718AF49}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1457" uniqueCount="763">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1463" uniqueCount="769">
   <si>
     <t>ID</t>
   </si>
@@ -2327,6 +2327,24 @@
   </si>
   <si>
     <t>Introduce el nombre de un objeto...</t>
+  </si>
+  <si>
+    <t>RotatePlayerTooltip</t>
+  </si>
+  <si>
+    <t>Should the player rotate where this respawn point is looking at?</t>
+  </si>
+  <si>
+    <t>¿Debería rotar el jugador a donde el punto de reaparición está mirando?</t>
+  </si>
+  <si>
+    <t>PowerSlotInitialStateTooltip</t>
+  </si>
+  <si>
+    <t>[b][FFFF00]WARNING:[-][/b] Setting this to [00FF00][i]ACTIVATED[/i][-] will create a new [i]Power Core[/i] in the level when it starts.</t>
+  </si>
+  <si>
+    <t>[b][FFFF00]ADVERTENCIA:[-][/b] Poner esto en [00FF00][i]ACTIVADO[/i][-] creará un nuevo [i]Núcleo de Energía[/i] en el nivel cuando este empiece.</t>
   </si>
 </sst>
 </file>
@@ -2737,7 +2755,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6961A5F-F8EA-4989-8112-A0ACE51D011E}">
   <sheetPr codeName="Hoja1"/>
-  <dimension ref="A1:D221"/>
+  <dimension ref="A1:D223"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="37" style="2" customWidth="1"/>
@@ -5649,6 +5667,28 @@
       </c>
       <c r="C221" s="2" t="s">
         <v>762</v>
+      </c>
+    </row>
+    <row r="222" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A222" s="2" t="s">
+        <v>763</v>
+      </c>
+      <c r="B222" s="2" t="s">
+        <v>764</v>
+      </c>
+      <c r="C222" s="2" t="s">
+        <v>765</v>
+      </c>
+    </row>
+    <row r="223" spans="1:3" ht="60" x14ac:dyDescent="0.25">
+      <c r="A223" s="2" t="s">
+        <v>766</v>
+      </c>
+      <c r="B223" s="2" t="s">
+        <v>767</v>
+      </c>
+      <c r="C223" s="2" t="s">
+        <v>768</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added carries player as a toggle for the objects with waypoints!
</commit_message>
<xml_diff>
--- a/Translations/Translations.xlsx
+++ b/Translations/Translations.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programacion\MelonLoader\FS_LevelEditor\Translations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{744FF6CA-2AC2-4CEA-BE26-8BBB4380EFA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79C2AAB1-A132-48A7-A205-E7B354737615}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{F5C22481-FF1A-482C-BF7E-EB5A7718AF49}"/>
+    <workbookView xWindow="4635" yWindow="4635" windowWidth="28800" windowHeight="15345" xr2:uid="{F5C22481-FF1A-482C-BF7E-EB5A7718AF49}"/>
   </bookViews>
   <sheets>
     <sheet name="Translations" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1463" uniqueCount="769">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1466" uniqueCount="771">
   <si>
     <t>ID</t>
   </si>
@@ -2345,6 +2345,12 @@
   </si>
   <si>
     <t>[b][FFFF00]ADVERTENCIA:[-][/b] Poner esto en [00FF00][i]ACTIVADO[/i][-] creará un nuevo [i]Núcleo de Energía[/i] en el nivel cuando este empiece.</t>
+  </si>
+  <si>
+    <t>CarriesPlayer</t>
+  </si>
+  <si>
+    <t>Carries Player</t>
   </si>
 </sst>
 </file>
@@ -2755,7 +2761,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6961A5F-F8EA-4989-8112-A0ACE51D011E}">
   <sheetPr codeName="Hoja1"/>
-  <dimension ref="A1:D223"/>
+  <dimension ref="A1:D224"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="37" style="2" customWidth="1"/>
@@ -5689,6 +5695,17 @@
       </c>
       <c r="C223" s="2" t="s">
         <v>768</v>
+      </c>
+    </row>
+    <row r="224" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A224" s="2" t="s">
+        <v>769</v>
+      </c>
+      <c r="B224" s="2" t="s">
+        <v>770</v>
+      </c>
+      <c r="C224" s="2" t="s">
+        <v>770</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added a tooltip for the target object field in the events ui, so new uses can see what they can do with it.
</commit_message>
<xml_diff>
--- a/Translations/Translations.xlsx
+++ b/Translations/Translations.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programacion\MelonLoader\FS_LevelEditor\Translations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{082C49EC-1E22-4CA9-B8A6-32DE4A43DAAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E38A61CD-CC1A-4F1F-AEE6-1C6350B2B393}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{F5C22481-FF1A-482C-BF7E-EB5A7718AF49}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1469" uniqueCount="774">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1471" uniqueCount="776">
   <si>
     <t>ID</t>
   </si>
@@ -2360,6 +2360,19 @@
   </si>
   <si>
     <t>Árbol de Navidad</t>
+  </si>
+  <si>
+    <t>EventsTargetObjectFieldTooltip</t>
+  </si>
+  <si>
+    <t>The [b]Target Object Field[/b] supports the following syntaxes:
+- [b]Objects:[/b] [FFFF00]TYPE ID[-] Example: [00FFFF]Ground 12[-].
+- [b]Player:[/b] Access to Player options.
+- [b]Taser:[/b] Access to Taser options.
+- [b]Jetpack:[/b] Access to Jetpack options.
+- [b]Objectives:[/b] [00FFFF]Obj_[-][FFFF00]OBJECTIVE TEXT[-] Example: [00FFFF]Obj_Find a way out[-].
+- [b]Wait:[/b] [00FFFF]Wait[-] [FFFF00]Xs or Xms[-] Example: [00FFFF]Wait 3s[-].
+- [b]Groups:[/b] [00FFFF]Group[-] [FFFF00]ID[-] Example: [00FFFF]Group 2[-].</t>
   </si>
 </sst>
 </file>
@@ -2770,7 +2783,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6961A5F-F8EA-4989-8112-A0ACE51D011E}">
   <sheetPr codeName="Hoja1"/>
-  <dimension ref="A1:D225"/>
+  <dimension ref="A1:D226"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="37" style="2" customWidth="1"/>
@@ -5726,6 +5739,14 @@
       </c>
       <c r="C225" s="2" t="s">
         <v>770</v>
+      </c>
+    </row>
+    <row r="226" spans="1:3" ht="225" x14ac:dyDescent="0.25">
+      <c r="A226" s="2" t="s">
+        <v>774</v>
+      </c>
+      <c r="B226" s="2" t="s">
+        <v>775</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fixed On Teleport events not having a translation.
</commit_message>
<xml_diff>
--- a/Translations/Translations.xlsx
+++ b/Translations/Translations.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programacion\MelonLoader\FS_LevelEditor\Translations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E38A61CD-CC1A-4F1F-AEE6-1C6350B2B393}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17CFF239-3AF0-4A43-9265-150185C4E1D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{F5C22481-FF1A-482C-BF7E-EB5A7718AF49}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1471" uniqueCount="776">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1474" uniqueCount="779">
   <si>
     <t>ID</t>
   </si>
@@ -2373,6 +2373,15 @@
 - [b]Objectives:[/b] [00FFFF]Obj_[-][FFFF00]OBJECTIVE TEXT[-] Example: [00FFFF]Obj_Find a way out[-].
 - [b]Wait:[/b] [00FFFF]Wait[-] [FFFF00]Xs or Xms[-] Example: [00FFFF]Wait 3s[-].
 - [b]Groups:[/b] [00FFFF]Group[-] [FFFF00]ID[-] Example: [00FFFF]Group 2[-].</t>
+  </si>
+  <si>
+    <t>events.OnTeleport</t>
+  </si>
+  <si>
+    <t>On Teleport</t>
+  </si>
+  <si>
+    <t>Al Teletransportar</t>
   </si>
 </sst>
 </file>
@@ -2783,7 +2792,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6961A5F-F8EA-4989-8112-A0ACE51D011E}">
   <sheetPr codeName="Hoja1"/>
-  <dimension ref="A1:D226"/>
+  <dimension ref="A1:D227"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="37" style="2" customWidth="1"/>
@@ -3929,1823 +3938,1834 @@
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A84" s="2" t="s">
-        <v>154</v>
+        <v>776</v>
       </c>
       <c r="B84" s="2" t="s">
-        <v>155</v>
+        <v>777</v>
       </c>
       <c r="C84" s="2" t="s">
-        <v>156</v>
-      </c>
-      <c r="D84" s="2" t="s">
-        <v>371</v>
+        <v>778</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A85" s="2" t="s">
-        <v>164</v>
+        <v>154</v>
       </c>
       <c r="B85" s="2" t="s">
-        <v>165</v>
+        <v>155</v>
       </c>
       <c r="C85" s="2" t="s">
-        <v>166</v>
+        <v>156</v>
       </c>
       <c r="D85" s="2" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A86" s="2" t="s">
-        <v>157</v>
+        <v>164</v>
       </c>
       <c r="B86" s="2" t="s">
-        <v>158</v>
+        <v>165</v>
       </c>
       <c r="C86" s="2" t="s">
-        <v>159</v>
+        <v>166</v>
       </c>
       <c r="D86" s="2" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A87" s="2" t="s">
-        <v>167</v>
+        <v>157</v>
       </c>
       <c r="B87" s="2" t="s">
-        <v>168</v>
+        <v>158</v>
       </c>
       <c r="C87" s="2" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="D87" s="2" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A88" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="B88" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="C88" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="D88" s="2" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A89" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="B88" s="2" t="s">
+      <c r="B89" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="C88" s="2" t="s">
+      <c r="C89" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="D88" s="2" t="s">
+      <c r="D89" s="2" t="s">
         <v>375</v>
       </c>
     </row>
-    <row r="89" spans="1:4" ht="45" x14ac:dyDescent="0.25">
-      <c r="A89" s="2" t="s">
+    <row r="90" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="A90" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="B89" s="2" t="s">
+      <c r="B90" s="2" t="s">
         <v>163</v>
       </c>
-      <c r="C89" s="2" t="s">
+      <c r="C90" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="D89" s="2" t="s">
+      <c r="D90" s="2" t="s">
         <v>376</v>
-      </c>
-    </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A90" s="2" t="s">
-        <v>153</v>
-      </c>
-      <c r="B90" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="C90" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="D90" s="2" t="s">
-        <v>328</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A91" s="2" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="B91" s="2" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="C91" s="2" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="D91" s="2" t="s">
-        <v>377</v>
+        <v>328</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A92" s="2" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="B92" s="2" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="C92" s="2" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="D92" s="2" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A93" s="2" t="s">
-        <v>172</v>
+        <v>150</v>
       </c>
       <c r="B93" s="2" t="s">
-        <v>170</v>
+        <v>151</v>
       </c>
       <c r="C93" s="2" t="s">
-        <v>171</v>
+        <v>152</v>
       </c>
       <c r="D93" s="2" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A94" s="2" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B94" s="2" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="C94" s="2" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="D94" s="2" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A95" s="2" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="B95" s="2" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="C95" s="2" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="D95" s="2" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A96" s="2" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="B96" s="2" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="C96" s="2" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="D96" s="2" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A97" s="2" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="B97" s="2" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="C97" s="2" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="D97" s="2" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A98" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="B98" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="C98" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="D98" s="2" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A99" s="2" t="s">
         <v>243</v>
       </c>
-      <c r="B98" s="2" t="s">
+      <c r="B99" s="2" t="s">
         <v>243</v>
       </c>
-      <c r="C98" s="2" t="s">
+      <c r="C99" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="D98" s="2" t="s">
+      <c r="D99" s="2" t="s">
         <v>384</v>
       </c>
     </row>
-    <row r="99" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A99" s="2" t="s">
+    <row r="100" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A100" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="B99" s="1" t="s">
+      <c r="B100" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="C99" s="2" t="s">
+      <c r="C100" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="D99" s="2" t="s">
+      <c r="D100" s="2" t="s">
         <v>385</v>
-      </c>
-    </row>
-    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A100" s="2" t="s">
-        <v>182</v>
-      </c>
-      <c r="B100" s="2" t="s">
-        <v>183</v>
-      </c>
-      <c r="C100" s="2" t="s">
-        <v>183</v>
-      </c>
-      <c r="D100" s="2" t="s">
-        <v>386</v>
       </c>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A101" s="2" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="B101" s="2" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C101" s="2" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="D101" s="2" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A102" s="2" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="B102" s="2" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="C102" s="2" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="D102" s="2" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A103" s="2" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="B103" s="2" t="s">
-        <v>525</v>
+        <v>186</v>
       </c>
       <c r="C103" s="2" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="D103" s="2" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A104" s="2" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="B104" s="2" t="s">
-        <v>190</v>
+        <v>525</v>
       </c>
       <c r="C104" s="2" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="D104" s="2" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A105" s="2" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="B105" s="2" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="C105" s="2" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="D105" s="2" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A106" s="2" t="s">
-        <v>434</v>
-      </c>
-      <c r="B106" s="4" t="s">
-        <v>435</v>
-      </c>
-      <c r="C106" s="4" t="s">
-        <v>436</v>
-      </c>
-      <c r="D106" s="4" t="s">
-        <v>591</v>
+        <v>192</v>
+      </c>
+      <c r="B106" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="C106" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="D106" s="2" t="s">
+        <v>391</v>
       </c>
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A107" s="2" t="s">
-        <v>437</v>
+        <v>434</v>
       </c>
       <c r="B107" s="4" t="s">
-        <v>438</v>
+        <v>435</v>
       </c>
       <c r="C107" s="4" t="s">
-        <v>439</v>
+        <v>436</v>
       </c>
       <c r="D107" s="4" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A108" s="2" t="s">
-        <v>473</v>
+        <v>437</v>
       </c>
       <c r="B108" s="4" t="s">
-        <v>590</v>
+        <v>438</v>
       </c>
       <c r="C108" s="4" t="s">
-        <v>474</v>
+        <v>439</v>
       </c>
       <c r="D108" s="4" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A109" s="2" t="s">
-        <v>195</v>
-      </c>
-      <c r="B109" s="2" t="s">
-        <v>196</v>
-      </c>
-      <c r="C109" s="2" t="s">
-        <v>197</v>
-      </c>
-      <c r="D109" s="2" t="s">
-        <v>392</v>
+        <v>473</v>
+      </c>
+      <c r="B109" s="4" t="s">
+        <v>590</v>
+      </c>
+      <c r="C109" s="4" t="s">
+        <v>474</v>
+      </c>
+      <c r="D109" s="4" t="s">
+        <v>593</v>
       </c>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A110" s="2" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="B110" s="2" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="C110" s="2" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="D110" s="2" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A111" s="2" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="B111" s="2" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="C111" s="2" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="D111" s="2" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A112" s="2" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="B112" s="2" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="C112" s="2" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="D112" s="2" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A113" s="2" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="B113" s="2" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="C113" s="2" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="D113" s="2" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A114" s="2" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B114" s="2" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="C114" s="2" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="D114" s="2" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A115" s="2" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="B115" s="2" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="C115" s="2" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="D115" s="2" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A116" s="2" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="B116" s="2" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="C116" s="2" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="D116" s="2" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A117" s="2" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="B117" s="2" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="C117" s="2" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="D117" s="2" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A118" s="2" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="B118" s="2" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="C118" s="2" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="D118" s="2" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
     </row>
     <row r="119" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A119" s="2" t="s">
-        <v>292</v>
+        <v>220</v>
       </c>
       <c r="B119" s="2" t="s">
-        <v>292</v>
+        <v>219</v>
       </c>
       <c r="C119" s="2" t="s">
-        <v>293</v>
+        <v>218</v>
       </c>
       <c r="D119" s="2" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A120" s="2" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="B120" s="2" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="C120" s="2" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
       <c r="D120" s="2" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A121" s="2" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
       <c r="B121" s="2" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="C121" s="2" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="D121" s="2" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A122" s="2" t="s">
-        <v>221</v>
+        <v>297</v>
       </c>
       <c r="B122" s="2" t="s">
-        <v>221</v>
+        <v>298</v>
       </c>
       <c r="C122" s="2" t="s">
-        <v>222</v>
+        <v>299</v>
       </c>
       <c r="D122" s="2" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
     </row>
     <row r="123" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A123" s="2" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="B123" s="2" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="C123" s="2" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="D123" s="2" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="124" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A124" s="2" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="B124" s="2" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="C124" s="2" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="D124" s="2" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
     </row>
     <row r="125" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A125" s="2" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="B125" s="2" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="C125" s="2" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="D125" s="2" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
     </row>
     <row r="126" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A126" s="2" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B126" s="2" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="C126" s="2" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="D126" s="2" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
     </row>
     <row r="127" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A127" s="2" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="B127" s="2" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="C127" s="2" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="D127" s="2" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
     </row>
     <row r="128" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A128" s="2" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="B128" s="2" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="C128" s="2" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="D128" s="2" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
     </row>
     <row r="129" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A129" s="2" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="B129" s="2" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="C129" s="2" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="D129" s="2" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
     </row>
     <row r="130" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A130" s="2" t="s">
-        <v>300</v>
+        <v>237</v>
       </c>
       <c r="B130" s="2" t="s">
-        <v>301</v>
+        <v>238</v>
       </c>
       <c r="C130" s="2" t="s">
-        <v>302</v>
+        <v>239</v>
       </c>
       <c r="D130" s="2" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
     </row>
     <row r="131" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A131" s="2" t="s">
-        <v>240</v>
+        <v>300</v>
       </c>
       <c r="B131" s="2" t="s">
-        <v>241</v>
+        <v>301</v>
       </c>
       <c r="C131" s="2" t="s">
-        <v>242</v>
+        <v>302</v>
       </c>
       <c r="D131" s="2" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
     </row>
     <row r="132" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A132" s="2" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="B132" s="2" t="s">
-        <v>252</v>
+        <v>241</v>
       </c>
       <c r="C132" s="2" t="s">
-        <v>251</v>
+        <v>242</v>
       </c>
       <c r="D132" s="2" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="133" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A133" s="2" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B133" s="2" t="s">
-        <v>245</v>
+        <v>252</v>
       </c>
       <c r="C133" s="2" t="s">
-        <v>246</v>
+        <v>251</v>
       </c>
       <c r="D133" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
     </row>
     <row r="134" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A134" s="2" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="B134" s="2" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="C134" s="2" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="D134" s="2" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
     </row>
     <row r="135" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A135" s="2" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="B135" s="2" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="C135" s="2" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="D135" s="2" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
     </row>
     <row r="136" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A136" s="2" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="B136" s="2" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="C136" s="2" t="s">
-        <v>255</v>
+        <v>250</v>
       </c>
       <c r="D136" s="2" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
     </row>
     <row r="137" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A137" s="2" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="B137" s="2" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="C137" s="2" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="D137" s="2" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
     </row>
     <row r="138" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A138" s="2" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="B138" s="2" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="C138" s="2" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="D138" s="2" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
     </row>
     <row r="139" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A139" s="2" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="B139" s="2" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="C139" s="2" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="D139" s="2" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="140" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A140" s="2" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="B140" s="2" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="C140" s="2" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="D140" s="2" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
     </row>
     <row r="141" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A141" s="2" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="B141" s="2" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="C141" s="2" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="D141" s="2" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
     </row>
     <row r="142" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A142" s="2" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="B142" s="2" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="C142" s="2" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="D142" s="2" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
     </row>
     <row r="143" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A143" s="2" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="B143" s="2" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="C143" s="2" t="s">
-        <v>273</v>
+        <v>269</v>
       </c>
       <c r="D143" s="2" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
     </row>
     <row r="144" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A144" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="B144" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="C144" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="D144" s="2" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="145" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A145" s="2" t="s">
         <v>271</v>
       </c>
-      <c r="B144" s="2" t="s">
+      <c r="B145" s="2" t="s">
         <v>271</v>
       </c>
-      <c r="C144" s="2" t="s">
+      <c r="C145" s="2" t="s">
         <v>272</v>
       </c>
-      <c r="D144" s="2" t="s">
+      <c r="D145" s="2" t="s">
         <v>427</v>
       </c>
     </row>
-    <row r="145" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A145" s="2" t="s">
+    <row r="146" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A146" s="2" t="s">
         <v>274</v>
       </c>
-      <c r="B145" s="2" t="s">
+      <c r="B146" s="2" t="s">
         <v>276</v>
       </c>
-      <c r="C145" s="2" t="s">
+      <c r="C146" s="2" t="s">
         <v>279</v>
       </c>
     </row>
-    <row r="146" spans="1:4" ht="45" x14ac:dyDescent="0.25">
-      <c r="A146" s="2" t="s">
+    <row r="147" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="A147" s="2" t="s">
         <v>275</v>
       </c>
-      <c r="B146" s="2" t="s">
+      <c r="B147" s="2" t="s">
         <v>277</v>
       </c>
-      <c r="C146" s="2" t="s">
+      <c r="C147" s="2" t="s">
         <v>278</v>
       </c>
     </row>
-    <row r="147" spans="1:4" ht="75" x14ac:dyDescent="0.25">
-      <c r="A147" s="2" t="s">
+    <row r="148" spans="1:4" ht="75" x14ac:dyDescent="0.25">
+      <c r="A148" s="2" t="s">
         <v>289</v>
       </c>
-      <c r="B147" s="2" t="s">
+      <c r="B148" s="2" t="s">
         <v>290</v>
       </c>
-      <c r="C147" s="2" t="s">
+      <c r="C148" s="2" t="s">
         <v>291</v>
-      </c>
-    </row>
-    <row r="148" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A148" s="2" t="s">
-        <v>306</v>
-      </c>
-      <c r="B148" s="2" t="s">
-        <v>307</v>
-      </c>
-      <c r="C148" s="2" t="s">
-        <v>308</v>
-      </c>
-      <c r="D148" s="2" t="s">
-        <v>428</v>
       </c>
     </row>
     <row r="149" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A149" s="2" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
       <c r="B149" s="2" t="s">
-        <v>311</v>
+        <v>307</v>
       </c>
       <c r="C149" s="2" t="s">
-        <v>312</v>
+        <v>308</v>
       </c>
       <c r="D149" s="2" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
     </row>
     <row r="150" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A150" s="2" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="B150" s="2" t="s">
-        <v>314</v>
+        <v>311</v>
       </c>
       <c r="C150" s="2" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="D150" s="2" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
     </row>
     <row r="151" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A151" s="2" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="B151" s="2" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="C151" s="2" t="s">
-        <v>316</v>
+        <v>313</v>
       </c>
       <c r="D151" s="2" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
     </row>
     <row r="152" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A152" s="2" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="B152" s="2" t="s">
-        <v>318</v>
+        <v>315</v>
       </c>
       <c r="C152" s="2" t="s">
-        <v>460</v>
+        <v>316</v>
       </c>
       <c r="D152" s="2" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
     </row>
     <row r="153" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A153" s="2" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="B153" s="2" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="C153" s="2" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="D153" s="2" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
     </row>
     <row r="154" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A154" s="2" t="s">
-        <v>448</v>
+        <v>319</v>
       </c>
       <c r="B154" s="2" t="s">
-        <v>448</v>
+        <v>320</v>
       </c>
       <c r="C154" s="2" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="D154" s="2" t="s">
-        <v>345</v>
+        <v>433</v>
       </c>
     </row>
     <row r="155" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A155" s="2" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="B155" s="2" t="s">
-        <v>450</v>
+        <v>448</v>
       </c>
       <c r="C155" s="2" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="D155" s="2" t="s">
-        <v>451</v>
+        <v>345</v>
       </c>
     </row>
     <row r="156" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A156" s="2" t="s">
-        <v>475</v>
+        <v>449</v>
       </c>
       <c r="B156" s="2" t="s">
-        <v>476</v>
+        <v>450</v>
       </c>
       <c r="C156" s="2" t="s">
-        <v>619</v>
+        <v>463</v>
       </c>
       <c r="D156" s="2" t="s">
-        <v>569</v>
+        <v>451</v>
       </c>
     </row>
     <row r="157" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A157" s="2" t="s">
-        <v>478</v>
+        <v>475</v>
       </c>
       <c r="B157" s="2" t="s">
-        <v>524</v>
+        <v>476</v>
       </c>
       <c r="C157" s="2" t="s">
-        <v>479</v>
+        <v>619</v>
       </c>
       <c r="D157" s="2" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
     </row>
     <row r="158" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A158" s="2" t="s">
-        <v>480</v>
+        <v>478</v>
       </c>
       <c r="B158" s="2" t="s">
-        <v>481</v>
+        <v>524</v>
       </c>
       <c r="C158" s="2" t="s">
-        <v>482</v>
+        <v>479</v>
       </c>
       <c r="D158" s="2" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
     </row>
     <row r="159" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A159" s="2" t="s">
-        <v>483</v>
+        <v>480</v>
       </c>
       <c r="B159" s="2" t="s">
-        <v>484</v>
+        <v>481</v>
       </c>
       <c r="C159" s="2" t="s">
-        <v>485</v>
+        <v>482</v>
       </c>
       <c r="D159" s="2" t="s">
-        <v>566</v>
+        <v>567</v>
       </c>
     </row>
     <row r="160" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A160" s="2" t="s">
-        <v>486</v>
+        <v>483</v>
       </c>
       <c r="B160" s="2" t="s">
-        <v>487</v>
+        <v>484</v>
       </c>
       <c r="C160" s="2" t="s">
-        <v>488</v>
+        <v>485</v>
       </c>
       <c r="D160" s="2" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
     </row>
     <row r="161" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A161" s="2" t="s">
-        <v>489</v>
+        <v>486</v>
       </c>
       <c r="B161" s="2" t="s">
-        <v>490</v>
+        <v>487</v>
       </c>
       <c r="C161" s="2" t="s">
-        <v>491</v>
+        <v>488</v>
       </c>
       <c r="D161" s="2" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
     </row>
     <row r="162" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A162" s="2" t="s">
-        <v>538</v>
+        <v>489</v>
       </c>
       <c r="B162" s="2" t="s">
-        <v>538</v>
+        <v>490</v>
       </c>
       <c r="C162" s="2" t="s">
-        <v>607</v>
+        <v>491</v>
       </c>
       <c r="D162" s="2" t="s">
-        <v>539</v>
+        <v>564</v>
       </c>
     </row>
     <row r="163" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A163" s="2" t="s">
-        <v>540</v>
+        <v>538</v>
       </c>
       <c r="B163" s="2" t="s">
-        <v>541</v>
+        <v>538</v>
       </c>
       <c r="C163" s="2" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="D163" s="2" t="s">
-        <v>542</v>
+        <v>539</v>
       </c>
     </row>
     <row r="164" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A164" s="2" t="s">
-        <v>492</v>
+        <v>540</v>
       </c>
       <c r="B164" s="2" t="s">
-        <v>493</v>
+        <v>541</v>
       </c>
       <c r="C164" s="2" t="s">
-        <v>494</v>
+        <v>608</v>
       </c>
       <c r="D164" s="2" t="s">
-        <v>563</v>
+        <v>542</v>
       </c>
     </row>
     <row r="165" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A165" s="2" t="s">
-        <v>495</v>
+        <v>492</v>
       </c>
       <c r="B165" s="2" t="s">
-        <v>496</v>
+        <v>493</v>
       </c>
       <c r="C165" s="2" t="s">
-        <v>497</v>
+        <v>494</v>
       </c>
       <c r="D165" s="2" t="s">
-        <v>562</v>
+        <v>563</v>
       </c>
     </row>
     <row r="166" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A166" s="2" t="s">
-        <v>498</v>
+        <v>495</v>
       </c>
       <c r="B166" s="2" t="s">
-        <v>499</v>
+        <v>496</v>
       </c>
       <c r="C166" s="2" t="s">
-        <v>500</v>
+        <v>497</v>
       </c>
       <c r="D166" s="2" t="s">
-        <v>561</v>
+        <v>562</v>
       </c>
     </row>
     <row r="167" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A167" s="2" t="s">
-        <v>501</v>
+        <v>498</v>
       </c>
       <c r="B167" s="2" t="s">
-        <v>501</v>
+        <v>499</v>
       </c>
       <c r="C167" s="2" t="s">
-        <v>502</v>
+        <v>500</v>
       </c>
       <c r="D167" s="2" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
     </row>
     <row r="168" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A168" s="2" t="s">
-        <v>503</v>
+        <v>501</v>
       </c>
       <c r="B168" s="2" t="s">
-        <v>503</v>
+        <v>501</v>
       </c>
       <c r="C168" s="2" t="s">
-        <v>504</v>
+        <v>502</v>
       </c>
       <c r="D168" s="2" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
     </row>
     <row r="169" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A169" s="2" t="s">
-        <v>505</v>
+        <v>503</v>
       </c>
       <c r="B169" s="2" t="s">
-        <v>505</v>
+        <v>503</v>
       </c>
       <c r="C169" s="2" t="s">
-        <v>506</v>
+        <v>504</v>
       </c>
       <c r="D169" s="2" t="s">
-        <v>558</v>
+        <v>559</v>
       </c>
     </row>
     <row r="170" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A170" s="2" t="s">
-        <v>507</v>
+        <v>505</v>
       </c>
       <c r="B170" s="2" t="s">
-        <v>507</v>
+        <v>505</v>
       </c>
       <c r="C170" s="2" t="s">
-        <v>508</v>
+        <v>506</v>
       </c>
       <c r="D170" s="2" t="s">
-        <v>557</v>
+        <v>558</v>
       </c>
     </row>
     <row r="171" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A171" s="2" t="s">
-        <v>570</v>
+        <v>507</v>
       </c>
       <c r="B171" s="2" t="s">
-        <v>571</v>
+        <v>507</v>
       </c>
       <c r="C171" s="2" t="s">
-        <v>609</v>
+        <v>508</v>
+      </c>
+      <c r="D171" s="2" t="s">
+        <v>557</v>
       </c>
     </row>
     <row r="172" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A172" s="2" t="s">
-        <v>572</v>
+        <v>570</v>
       </c>
       <c r="B172" s="2" t="s">
-        <v>573</v>
+        <v>571</v>
       </c>
       <c r="C172" s="2" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
     </row>
     <row r="173" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A173" s="2" t="s">
-        <v>574</v>
+        <v>572</v>
       </c>
       <c r="B173" s="2" t="s">
-        <v>575</v>
+        <v>573</v>
       </c>
       <c r="C173" s="2" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
     </row>
     <row r="174" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A174" s="2" t="s">
-        <v>576</v>
+        <v>574</v>
       </c>
       <c r="B174" s="2" t="s">
-        <v>577</v>
+        <v>575</v>
       </c>
       <c r="C174" s="2" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
     </row>
     <row r="175" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A175" s="2" t="s">
-        <v>578</v>
+        <v>576</v>
       </c>
       <c r="B175" s="2" t="s">
-        <v>579</v>
+        <v>577</v>
       </c>
       <c r="C175" s="2" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
     </row>
     <row r="176" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A176" s="2" t="s">
-        <v>580</v>
+        <v>578</v>
       </c>
       <c r="B176" s="2" t="s">
-        <v>581</v>
+        <v>579</v>
       </c>
       <c r="C176" s="2" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
     </row>
     <row r="177" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A177" s="2" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
       <c r="B177" s="2" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="C177" s="2" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
     </row>
     <row r="178" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A178" s="2" t="s">
-        <v>584</v>
+        <v>582</v>
       </c>
       <c r="B178" s="2" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="C178" s="2" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
     </row>
     <row r="179" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A179" s="2" t="s">
-        <v>586</v>
+        <v>584</v>
       </c>
       <c r="B179" s="2" t="s">
-        <v>587</v>
+        <v>585</v>
       </c>
       <c r="C179" s="2" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
     </row>
     <row r="180" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A180" s="2" t="s">
-        <v>588</v>
+        <v>586</v>
       </c>
       <c r="B180" s="2" t="s">
-        <v>589</v>
+        <v>587</v>
       </c>
       <c r="C180" s="2" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
     </row>
     <row r="181" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A181" s="2" t="s">
-        <v>620</v>
+        <v>588</v>
       </c>
       <c r="B181" s="2" t="s">
-        <v>621</v>
+        <v>589</v>
       </c>
       <c r="C181" s="2" t="s">
-        <v>622</v>
+        <v>618</v>
       </c>
     </row>
     <row r="182" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A182" s="2" t="s">
-        <v>623</v>
+        <v>620</v>
       </c>
       <c r="B182" s="2" t="s">
-        <v>623</v>
+        <v>621</v>
       </c>
       <c r="C182" s="2" t="s">
-        <v>624</v>
+        <v>622</v>
       </c>
     </row>
     <row r="183" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A183" s="2" t="s">
-        <v>625</v>
+        <v>623</v>
       </c>
       <c r="B183" s="2" t="s">
-        <v>625</v>
+        <v>623</v>
       </c>
       <c r="C183" s="2" t="s">
-        <v>627</v>
+        <v>624</v>
       </c>
     </row>
     <row r="184" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A184" s="2" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="B184" s="2" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="C184" s="2" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
     </row>
     <row r="185" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A185" s="2" t="s">
-        <v>629</v>
+        <v>626</v>
       </c>
       <c r="B185" s="2" t="s">
-        <v>630</v>
+        <v>626</v>
       </c>
       <c r="C185" s="2" t="s">
-        <v>631</v>
+        <v>628</v>
       </c>
     </row>
     <row r="186" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A186" s="2" t="s">
-        <v>632</v>
-      </c>
-      <c r="B186" s="4" t="s">
-        <v>633</v>
-      </c>
-      <c r="C186" s="4" t="s">
-        <v>634</v>
+        <v>629</v>
+      </c>
+      <c r="B186" s="2" t="s">
+        <v>630</v>
+      </c>
+      <c r="C186" s="2" t="s">
+        <v>631</v>
       </c>
     </row>
     <row r="187" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A187" s="2" t="s">
-        <v>638</v>
-      </c>
-      <c r="B187" s="2" t="s">
-        <v>639</v>
-      </c>
-      <c r="C187" s="2" t="s">
-        <v>640</v>
+        <v>632</v>
+      </c>
+      <c r="B187" s="4" t="s">
+        <v>633</v>
+      </c>
+      <c r="C187" s="4" t="s">
+        <v>634</v>
       </c>
     </row>
     <row r="188" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A188" s="2" t="s">
-        <v>641</v>
+        <v>638</v>
       </c>
       <c r="B188" s="2" t="s">
-        <v>641</v>
+        <v>639</v>
       </c>
       <c r="C188" s="2" t="s">
-        <v>642</v>
+        <v>640</v>
       </c>
     </row>
     <row r="189" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A189" s="2" t="s">
-        <v>643</v>
+        <v>641</v>
       </c>
       <c r="B189" s="2" t="s">
-        <v>644</v>
+        <v>641</v>
       </c>
       <c r="C189" s="2" t="s">
-        <v>645</v>
+        <v>642</v>
       </c>
     </row>
     <row r="190" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A190" s="2" t="s">
-        <v>646</v>
+        <v>643</v>
       </c>
       <c r="B190" s="2" t="s">
-        <v>647</v>
+        <v>644</v>
       </c>
       <c r="C190" s="2" t="s">
-        <v>648</v>
+        <v>645</v>
       </c>
     </row>
     <row r="191" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A191" s="2" t="s">
-        <v>649</v>
+        <v>646</v>
       </c>
       <c r="B191" s="2" t="s">
-        <v>650</v>
+        <v>647</v>
       </c>
       <c r="C191" s="2" t="s">
-        <v>651</v>
+        <v>648</v>
       </c>
     </row>
     <row r="192" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A192" s="2" t="s">
-        <v>652</v>
+        <v>649</v>
       </c>
       <c r="B192" s="2" t="s">
-        <v>653</v>
+        <v>650</v>
       </c>
       <c r="C192" s="2" t="s">
-        <v>654</v>
+        <v>651</v>
       </c>
     </row>
     <row r="193" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A193" s="2" t="s">
-        <v>655</v>
+        <v>652</v>
       </c>
       <c r="B193" s="2" t="s">
-        <v>655</v>
+        <v>653</v>
       </c>
       <c r="C193" s="2" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
     </row>
     <row r="194" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A194" s="2" t="s">
-        <v>657</v>
+        <v>655</v>
       </c>
       <c r="B194" s="2" t="s">
-        <v>658</v>
+        <v>655</v>
       </c>
       <c r="C194" s="2" t="s">
-        <v>659</v>
+        <v>656</v>
       </c>
     </row>
     <row r="195" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A195" s="2" t="s">
-        <v>666</v>
-      </c>
-      <c r="B195" s="4" t="s">
-        <v>667</v>
-      </c>
-      <c r="C195" s="4" t="s">
-        <v>668</v>
+        <v>657</v>
+      </c>
+      <c r="B195" s="2" t="s">
+        <v>658</v>
+      </c>
+      <c r="C195" s="2" t="s">
+        <v>659</v>
       </c>
     </row>
     <row r="196" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A196" s="2" t="s">
-        <v>669</v>
-      </c>
-      <c r="B196" s="2" t="s">
-        <v>670</v>
-      </c>
-      <c r="C196" s="2" t="s">
-        <v>671</v>
+        <v>666</v>
+      </c>
+      <c r="B196" s="4" t="s">
+        <v>667</v>
+      </c>
+      <c r="C196" s="4" t="s">
+        <v>668</v>
       </c>
     </row>
     <row r="197" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A197" s="2" t="s">
-        <v>675</v>
+        <v>669</v>
       </c>
       <c r="B197" s="2" t="s">
-        <v>676</v>
+        <v>670</v>
       </c>
       <c r="C197" s="2" t="s">
-        <v>677</v>
+        <v>671</v>
       </c>
     </row>
     <row r="198" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A198" s="2" t="s">
-        <v>678</v>
+        <v>675</v>
       </c>
       <c r="B198" s="2" t="s">
-        <v>679</v>
+        <v>676</v>
       </c>
       <c r="C198" s="2" t="s">
-        <v>680</v>
+        <v>677</v>
       </c>
     </row>
     <row r="199" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A199" s="2" t="s">
-        <v>681</v>
+        <v>678</v>
       </c>
       <c r="B199" s="2" t="s">
-        <v>682</v>
+        <v>679</v>
       </c>
       <c r="C199" s="2" t="s">
-        <v>683</v>
+        <v>680</v>
       </c>
     </row>
     <row r="200" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A200" s="2" t="s">
-        <v>684</v>
+        <v>681</v>
       </c>
       <c r="B200" s="2" t="s">
-        <v>685</v>
+        <v>682</v>
       </c>
       <c r="C200" s="2" t="s">
-        <v>686</v>
+        <v>683</v>
       </c>
     </row>
     <row r="201" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A201" s="2" t="s">
-        <v>687</v>
+        <v>684</v>
       </c>
       <c r="B201" s="2" t="s">
-        <v>688</v>
+        <v>685</v>
       </c>
       <c r="C201" s="2" t="s">
-        <v>689</v>
+        <v>686</v>
       </c>
     </row>
     <row r="202" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A202" s="2" t="s">
-        <v>690</v>
-      </c>
-      <c r="B202" s="4" t="s">
-        <v>694</v>
-      </c>
-      <c r="C202" s="4" t="s">
-        <v>704</v>
+        <v>687</v>
+      </c>
+      <c r="B202" s="2" t="s">
+        <v>688</v>
+      </c>
+      <c r="C202" s="2" t="s">
+        <v>689</v>
       </c>
     </row>
     <row r="203" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A203" s="2" t="s">
-        <v>691</v>
-      </c>
-      <c r="B203" s="2" t="s">
-        <v>697</v>
-      </c>
-      <c r="C203" s="2" t="s">
-        <v>710</v>
+        <v>690</v>
+      </c>
+      <c r="B203" s="4" t="s">
+        <v>694</v>
+      </c>
+      <c r="C203" s="4" t="s">
+        <v>704</v>
       </c>
     </row>
     <row r="204" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A204" s="2" t="s">
-        <v>693</v>
-      </c>
-      <c r="B204" s="4" t="s">
-        <v>695</v>
-      </c>
-      <c r="C204" s="4" t="s">
-        <v>705</v>
+        <v>691</v>
+      </c>
+      <c r="B204" s="2" t="s">
+        <v>697</v>
+      </c>
+      <c r="C204" s="2" t="s">
+        <v>710</v>
       </c>
     </row>
     <row r="205" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A205" s="2" t="s">
-        <v>692</v>
+        <v>693</v>
       </c>
       <c r="B205" s="4" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
       <c r="C205" s="4" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
     </row>
     <row r="206" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A206" s="2" t="s">
-        <v>699</v>
-      </c>
-      <c r="B206" s="2" t="s">
-        <v>698</v>
-      </c>
-      <c r="C206" s="2" t="s">
-        <v>707</v>
+        <v>692</v>
+      </c>
+      <c r="B206" s="4" t="s">
+        <v>696</v>
+      </c>
+      <c r="C206" s="4" t="s">
+        <v>706</v>
       </c>
     </row>
     <row r="207" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A207" s="2" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="B207" s="2" t="s">
-        <v>702</v>
+        <v>698</v>
       </c>
       <c r="C207" s="2" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
     </row>
     <row r="208" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A208" s="2" t="s">
-        <v>701</v>
+        <v>700</v>
       </c>
       <c r="B208" s="2" t="s">
-        <v>703</v>
+        <v>702</v>
       </c>
       <c r="C208" s="2" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
     </row>
     <row r="209" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A209" s="2" t="s">
-        <v>711</v>
+        <v>701</v>
       </c>
       <c r="B209" s="2" t="s">
-        <v>711</v>
+        <v>703</v>
       </c>
       <c r="C209" s="2" t="s">
-        <v>712</v>
+        <v>709</v>
       </c>
     </row>
     <row r="210" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A210" s="2" t="s">
-        <v>713</v>
+        <v>711</v>
       </c>
       <c r="B210" s="2" t="s">
-        <v>714</v>
+        <v>711</v>
       </c>
       <c r="C210" s="2" t="s">
-        <v>715</v>
+        <v>712</v>
       </c>
     </row>
     <row r="211" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A211" s="2" t="s">
-        <v>716</v>
+        <v>713</v>
       </c>
       <c r="B211" s="2" t="s">
-        <v>717</v>
+        <v>714</v>
       </c>
       <c r="C211" s="2" t="s">
-        <v>718</v>
+        <v>715</v>
       </c>
     </row>
     <row r="212" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A212" s="2" t="s">
-        <v>719</v>
+        <v>716</v>
       </c>
       <c r="B212" s="2" t="s">
-        <v>720</v>
+        <v>717</v>
       </c>
       <c r="C212" s="2" t="s">
-        <v>721</v>
+        <v>718</v>
       </c>
     </row>
     <row r="213" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A213" s="2" t="s">
-        <v>732</v>
+        <v>719</v>
       </c>
       <c r="B213" s="2" t="s">
-        <v>733</v>
+        <v>720</v>
       </c>
       <c r="C213" s="2" t="s">
-        <v>736</v>
+        <v>721</v>
       </c>
     </row>
     <row r="214" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A214" s="2" t="s">
+        <v>732</v>
+      </c>
+      <c r="B214" s="2" t="s">
+        <v>733</v>
+      </c>
+      <c r="C214" s="2" t="s">
+        <v>736</v>
+      </c>
+    </row>
+    <row r="215" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A215" s="2" t="s">
         <v>734</v>
       </c>
-      <c r="B214" s="2" t="s">
+      <c r="B215" s="2" t="s">
         <v>735</v>
       </c>
-      <c r="C214" s="2" t="s">
+      <c r="C215" s="2" t="s">
         <v>737</v>
-      </c>
-    </row>
-    <row r="215" spans="1:3" ht="45" x14ac:dyDescent="0.25">
-      <c r="A215" s="2" t="s">
-        <v>728</v>
-      </c>
-      <c r="B215" s="2" t="s">
-        <v>729</v>
-      </c>
-      <c r="C215" s="2" t="s">
-        <v>738</v>
       </c>
     </row>
     <row r="216" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A216" s="2" t="s">
+        <v>728</v>
+      </c>
+      <c r="B216" s="2" t="s">
+        <v>729</v>
+      </c>
+      <c r="C216" s="2" t="s">
+        <v>738</v>
+      </c>
+    </row>
+    <row r="217" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A217" s="2" t="s">
         <v>730</v>
       </c>
-      <c r="B216" s="2" t="s">
+      <c r="B217" s="2" t="s">
         <v>731</v>
       </c>
-      <c r="C216" s="2" t="s">
+      <c r="C217" s="2" t="s">
         <v>739</v>
-      </c>
-    </row>
-    <row r="217" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A217" s="2" t="s">
-        <v>743</v>
-      </c>
-      <c r="B217" s="2" t="s">
-        <v>744</v>
-      </c>
-      <c r="C217" s="2" t="s">
-        <v>744</v>
       </c>
     </row>
     <row r="218" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A218" s="2" t="s">
-        <v>745</v>
+        <v>743</v>
       </c>
       <c r="B218" s="2" t="s">
-        <v>746</v>
+        <v>744</v>
       </c>
       <c r="C218" s="2" t="s">
-        <v>747</v>
+        <v>744</v>
       </c>
     </row>
     <row r="219" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A219" s="2" t="s">
-        <v>751</v>
+        <v>745</v>
       </c>
       <c r="B219" s="2" t="s">
-        <v>752</v>
+        <v>746</v>
       </c>
       <c r="C219" s="2" t="s">
-        <v>753</v>
+        <v>747</v>
       </c>
     </row>
     <row r="220" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A220" s="2" t="s">
-        <v>754</v>
+        <v>751</v>
       </c>
       <c r="B220" s="2" t="s">
-        <v>755</v>
+        <v>752</v>
       </c>
       <c r="C220" s="2" t="s">
-        <v>756</v>
+        <v>753</v>
       </c>
     </row>
     <row r="221" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A221" s="2" t="s">
-        <v>757</v>
+        <v>754</v>
       </c>
       <c r="B221" s="2" t="s">
-        <v>758</v>
+        <v>755</v>
       </c>
       <c r="C221" s="2" t="s">
-        <v>759</v>
+        <v>756</v>
       </c>
     </row>
     <row r="222" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A222" s="2" t="s">
+        <v>757</v>
+      </c>
+      <c r="B222" s="2" t="s">
+        <v>758</v>
+      </c>
+      <c r="C222" s="2" t="s">
+        <v>759</v>
+      </c>
+    </row>
+    <row r="223" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A223" s="2" t="s">
         <v>760</v>
       </c>
-      <c r="B222" s="2" t="s">
+      <c r="B223" s="2" t="s">
         <v>761</v>
       </c>
-      <c r="C222" s="2" t="s">
+      <c r="C223" s="2" t="s">
         <v>762</v>
       </c>
     </row>
-    <row r="223" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A223" s="2" t="s">
+    <row r="224" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A224" s="2" t="s">
         <v>763</v>
       </c>
-      <c r="B223" s="2" t="s">
+      <c r="B224" s="2" t="s">
         <v>764</v>
       </c>
-      <c r="C223" s="2" t="s">
+      <c r="C224" s="2" t="s">
         <v>765</v>
       </c>
     </row>
-    <row r="224" spans="1:3" ht="60" x14ac:dyDescent="0.25">
-      <c r="A224" s="2" t="s">
+    <row r="225" spans="1:3" ht="60" x14ac:dyDescent="0.25">
+      <c r="A225" s="2" t="s">
         <v>766</v>
       </c>
-      <c r="B224" s="2" t="s">
+      <c r="B225" s="2" t="s">
         <v>767</v>
       </c>
-      <c r="C224" s="2" t="s">
+      <c r="C225" s="2" t="s">
         <v>768</v>
       </c>
     </row>
-    <row r="225" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A225" s="2" t="s">
+    <row r="226" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A226" s="2" t="s">
         <v>769</v>
       </c>
-      <c r="B225" s="2" t="s">
+      <c r="B226" s="2" t="s">
         <v>770</v>
       </c>
-      <c r="C225" s="2" t="s">
+      <c r="C226" s="2" t="s">
         <v>770</v>
       </c>
     </row>
-    <row r="226" spans="1:3" ht="225" x14ac:dyDescent="0.25">
-      <c r="A226" s="2" t="s">
+    <row r="227" spans="1:3" ht="225" x14ac:dyDescent="0.25">
+      <c r="A227" s="2" t="s">
         <v>774</v>
       </c>
-      <c r="B226" s="2" t="s">
+      <c r="B227" s="2" t="s">
         <v>775</v>
       </c>
     </row>

</xml_diff>

<commit_message>
ADDED DUMMY CHECKPOINTS!! Still experimental.
</commit_message>
<xml_diff>
--- a/Translations/Translations.xlsx
+++ b/Translations/Translations.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programacion\MelonLoader\FS_LevelEditor\Translations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17CFF239-3AF0-4A43-9265-150185C4E1D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{499E0310-3A6B-4531-90D8-D8321144CDE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{F5C22481-FF1A-482C-BF7E-EB5A7718AF49}"/>
   </bookViews>
@@ -30,15 +30,12 @@
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
     </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1474" uniqueCount="779">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1486" uniqueCount="791">
   <si>
     <t>ID</t>
   </si>
@@ -2382,6 +2379,42 @@
   </si>
   <si>
     <t>Al Teletransportar</t>
+  </si>
+  <si>
+    <t>object.DUMMY_CHECKPOINT</t>
+  </si>
+  <si>
+    <t>Dummy Checkpoint</t>
+  </si>
+  <si>
+    <t>Punto de Control Parcial</t>
+  </si>
+  <si>
+    <t>events.OnSave</t>
+  </si>
+  <si>
+    <t>On Save</t>
+  </si>
+  <si>
+    <t>Al Guardar</t>
+  </si>
+  <si>
+    <t>events.OnRespawn</t>
+  </si>
+  <si>
+    <t>On Respawn</t>
+  </si>
+  <si>
+    <t>Al Reaparecer</t>
+  </si>
+  <si>
+    <t>RespawnAnim</t>
+  </si>
+  <si>
+    <t>Respawn Animation</t>
+  </si>
+  <si>
+    <t>Animación de Reaparición</t>
   </si>
 </sst>
 </file>
@@ -2792,7 +2825,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6961A5F-F8EA-4989-8112-A0ACE51D011E}">
   <sheetPr codeName="Hoja1"/>
-  <dimension ref="A1:D227"/>
+  <dimension ref="A1:D231"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="37" style="2" customWidth="1"/>
@@ -3689,2084 +3722,2128 @@
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66" s="2" t="s">
-        <v>69</v>
+        <v>779</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>69</v>
+        <v>780</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="D66" s="2" t="s">
-        <v>364</v>
+        <v>781</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A67" s="2" t="s">
-        <v>443</v>
+        <v>69</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>443</v>
+        <v>69</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>601</v>
+        <v>101</v>
       </c>
       <c r="D67" s="2" t="s">
-        <v>552</v>
+        <v>364</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A68" s="2" t="s">
-        <v>456</v>
+        <v>443</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>456</v>
+        <v>443</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>456</v>
+        <v>601</v>
       </c>
       <c r="D68" s="2" t="s">
-        <v>457</v>
+        <v>552</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A69" s="2" t="s">
-        <v>105</v>
+        <v>456</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>2</v>
+        <v>456</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>102</v>
+        <v>456</v>
       </c>
       <c r="D69" s="2" t="s">
-        <v>365</v>
+        <v>457</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A70" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C70" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D70" s="2" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A71" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D71" s="2" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A72" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>111</v>
+        <v>4</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="D72" s="2" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A73" s="2" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C73" s="2" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="D73" s="2" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A74" s="2" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="C74" s="2" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="D74" s="2" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A75" s="2" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="B75" s="2" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="C75" s="2" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="D75" s="2" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A76" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B76" s="2" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="C76" s="2" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D76" s="2" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A77" s="2" t="s">
-        <v>445</v>
+        <v>118</v>
       </c>
       <c r="B77" s="2" t="s">
-        <v>446</v>
+        <v>122</v>
       </c>
       <c r="C77" s="2" t="s">
-        <v>459</v>
+        <v>121</v>
       </c>
       <c r="D77" s="2" t="s">
-        <v>447</v>
+        <v>370</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A78" s="2" t="s">
-        <v>512</v>
+        <v>445</v>
       </c>
       <c r="B78" s="2" t="s">
-        <v>513</v>
+        <v>446</v>
       </c>
       <c r="C78" s="2" t="s">
-        <v>602</v>
+        <v>459</v>
       </c>
       <c r="D78" s="2" t="s">
-        <v>514</v>
+        <v>447</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A79" s="2" t="s">
-        <v>518</v>
+        <v>512</v>
       </c>
       <c r="B79" s="2" t="s">
-        <v>519</v>
+        <v>513</v>
       </c>
       <c r="C79" s="2" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="D79" s="2" t="s">
-        <v>520</v>
+        <v>514</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
-        <v>521</v>
+        <v>518</v>
       </c>
       <c r="B80" s="2" t="s">
-        <v>522</v>
+        <v>519</v>
       </c>
       <c r="C80" s="2" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="D80" s="2" t="s">
-        <v>523</v>
+        <v>520</v>
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A81" s="2" t="s">
-        <v>532</v>
+        <v>521</v>
       </c>
       <c r="B81" s="2" t="s">
-        <v>533</v>
+        <v>522</v>
       </c>
       <c r="C81" s="2" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="D81" s="2" t="s">
-        <v>534</v>
+        <v>523</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A82" s="2" t="s">
-        <v>537</v>
+        <v>532</v>
       </c>
       <c r="B82" s="2" t="s">
-        <v>535</v>
+        <v>533</v>
       </c>
       <c r="C82" s="2" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="D82" s="2" t="s">
-        <v>536</v>
+        <v>534</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A83" s="2" t="s">
-        <v>740</v>
+        <v>537</v>
       </c>
       <c r="B83" s="2" t="s">
-        <v>741</v>
+        <v>535</v>
       </c>
       <c r="C83" s="2" t="s">
-        <v>742</v>
+        <v>606</v>
+      </c>
+      <c r="D83" s="2" t="s">
+        <v>536</v>
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A84" s="2" t="s">
-        <v>776</v>
+        <v>740</v>
       </c>
       <c r="B84" s="2" t="s">
-        <v>777</v>
+        <v>741</v>
       </c>
       <c r="C84" s="2" t="s">
-        <v>778</v>
+        <v>742</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A85" s="2" t="s">
-        <v>154</v>
+        <v>776</v>
       </c>
       <c r="B85" s="2" t="s">
-        <v>155</v>
+        <v>777</v>
       </c>
       <c r="C85" s="2" t="s">
-        <v>156</v>
-      </c>
-      <c r="D85" s="2" t="s">
-        <v>371</v>
+        <v>778</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A86" s="2" t="s">
-        <v>164</v>
+        <v>782</v>
       </c>
       <c r="B86" s="2" t="s">
-        <v>165</v>
+        <v>783</v>
       </c>
       <c r="C86" s="2" t="s">
-        <v>166</v>
-      </c>
-      <c r="D86" s="2" t="s">
-        <v>372</v>
+        <v>784</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A87" s="2" t="s">
-        <v>157</v>
+        <v>785</v>
       </c>
       <c r="B87" s="2" t="s">
-        <v>158</v>
+        <v>786</v>
       </c>
       <c r="C87" s="2" t="s">
-        <v>159</v>
-      </c>
-      <c r="D87" s="2" t="s">
-        <v>373</v>
+        <v>787</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A88" s="2" t="s">
-        <v>167</v>
+        <v>154</v>
       </c>
       <c r="B88" s="2" t="s">
-        <v>168</v>
+        <v>155</v>
       </c>
       <c r="C88" s="2" t="s">
-        <v>169</v>
+        <v>156</v>
       </c>
       <c r="D88" s="2" t="s">
-        <v>374</v>
+        <v>371</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A89" s="2" t="s">
-        <v>141</v>
+        <v>164</v>
       </c>
       <c r="B89" s="2" t="s">
-        <v>142</v>
+        <v>165</v>
       </c>
       <c r="C89" s="2" t="s">
-        <v>143</v>
+        <v>166</v>
       </c>
       <c r="D89" s="2" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="90" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A90" s="2" t="s">
-        <v>144</v>
+        <v>157</v>
       </c>
       <c r="B90" s="2" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="C90" s="2" t="s">
-        <v>145</v>
+        <v>159</v>
       </c>
       <c r="D90" s="2" t="s">
-        <v>376</v>
+        <v>373</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A91" s="2" t="s">
-        <v>153</v>
+        <v>167</v>
       </c>
       <c r="B91" s="2" t="s">
-        <v>146</v>
+        <v>168</v>
       </c>
       <c r="C91" s="2" t="s">
-        <v>146</v>
+        <v>169</v>
       </c>
       <c r="D91" s="2" t="s">
-        <v>328</v>
+        <v>374</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A92" s="2" t="s">
-        <v>147</v>
+        <v>141</v>
       </c>
       <c r="B92" s="2" t="s">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="C92" s="2" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
       <c r="D92" s="2" t="s">
-        <v>377</v>
-      </c>
-    </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.25">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="93" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A93" s="2" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="B93" s="2" t="s">
-        <v>151</v>
+        <v>163</v>
       </c>
       <c r="C93" s="2" t="s">
-        <v>152</v>
+        <v>145</v>
       </c>
       <c r="D93" s="2" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A94" s="2" t="s">
-        <v>172</v>
+        <v>153</v>
       </c>
       <c r="B94" s="2" t="s">
-        <v>170</v>
+        <v>146</v>
       </c>
       <c r="C94" s="2" t="s">
-        <v>171</v>
+        <v>146</v>
       </c>
       <c r="D94" s="2" t="s">
-        <v>379</v>
+        <v>328</v>
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A95" s="2" t="s">
-        <v>173</v>
+        <v>147</v>
       </c>
       <c r="B95" s="2" t="s">
-        <v>174</v>
+        <v>148</v>
       </c>
       <c r="C95" s="2" t="s">
-        <v>175</v>
+        <v>149</v>
       </c>
       <c r="D95" s="2" t="s">
-        <v>380</v>
+        <v>377</v>
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A96" s="2" t="s">
-        <v>176</v>
+        <v>150</v>
       </c>
       <c r="B96" s="2" t="s">
-        <v>176</v>
+        <v>151</v>
       </c>
       <c r="C96" s="2" t="s">
-        <v>177</v>
+        <v>152</v>
       </c>
       <c r="D96" s="2" t="s">
-        <v>381</v>
+        <v>378</v>
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A97" s="2" t="s">
-        <v>178</v>
+        <v>172</v>
       </c>
       <c r="B97" s="2" t="s">
-        <v>178</v>
+        <v>170</v>
       </c>
       <c r="C97" s="2" t="s">
-        <v>179</v>
+        <v>171</v>
       </c>
       <c r="D97" s="2" t="s">
-        <v>382</v>
+        <v>379</v>
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A98" s="2" t="s">
-        <v>180</v>
+        <v>173</v>
       </c>
       <c r="B98" s="2" t="s">
-        <v>180</v>
+        <v>174</v>
       </c>
       <c r="C98" s="2" t="s">
-        <v>181</v>
+        <v>175</v>
       </c>
       <c r="D98" s="2" t="s">
-        <v>383</v>
+        <v>380</v>
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A99" s="2" t="s">
-        <v>243</v>
+        <v>176</v>
       </c>
       <c r="B99" s="2" t="s">
-        <v>243</v>
+        <v>176</v>
       </c>
       <c r="C99" s="2" t="s">
-        <v>95</v>
+        <v>177</v>
       </c>
       <c r="D99" s="2" t="s">
-        <v>384</v>
-      </c>
-    </row>
-    <row r="100" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A100" s="2" t="s">
-        <v>138</v>
-      </c>
-      <c r="B100" s="1" t="s">
-        <v>140</v>
+        <v>178</v>
+      </c>
+      <c r="B100" s="2" t="s">
+        <v>178</v>
       </c>
       <c r="C100" s="2" t="s">
-        <v>139</v>
+        <v>179</v>
       </c>
       <c r="D100" s="2" t="s">
-        <v>385</v>
+        <v>382</v>
       </c>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A101" s="2" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="B101" s="2" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="C101" s="2" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="D101" s="2" t="s">
-        <v>386</v>
+        <v>383</v>
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A102" s="2" t="s">
-        <v>184</v>
+        <v>243</v>
       </c>
       <c r="B102" s="2" t="s">
-        <v>184</v>
+        <v>243</v>
       </c>
       <c r="C102" s="2" t="s">
-        <v>185</v>
+        <v>95</v>
       </c>
       <c r="D102" s="2" t="s">
-        <v>387</v>
-      </c>
-    </row>
-    <row r="103" spans="1:4" x14ac:dyDescent="0.25">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="103" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A103" s="2" t="s">
-        <v>186</v>
-      </c>
-      <c r="B103" s="2" t="s">
-        <v>186</v>
+        <v>138</v>
+      </c>
+      <c r="B103" s="1" t="s">
+        <v>140</v>
       </c>
       <c r="C103" s="2" t="s">
-        <v>187</v>
+        <v>139</v>
       </c>
       <c r="D103" s="2" t="s">
-        <v>388</v>
+        <v>385</v>
       </c>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A104" s="2" t="s">
-        <v>188</v>
+        <v>182</v>
       </c>
       <c r="B104" s="2" t="s">
-        <v>525</v>
+        <v>183</v>
       </c>
       <c r="C104" s="2" t="s">
-        <v>189</v>
+        <v>183</v>
       </c>
       <c r="D104" s="2" t="s">
-        <v>389</v>
+        <v>386</v>
       </c>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A105" s="2" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="B105" s="2" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="C105" s="2" t="s">
-        <v>191</v>
+        <v>185</v>
       </c>
       <c r="D105" s="2" t="s">
-        <v>390</v>
+        <v>387</v>
       </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A106" s="2" t="s">
-        <v>192</v>
+        <v>186</v>
       </c>
       <c r="B106" s="2" t="s">
-        <v>193</v>
+        <v>186</v>
       </c>
       <c r="C106" s="2" t="s">
-        <v>194</v>
+        <v>187</v>
       </c>
       <c r="D106" s="2" t="s">
-        <v>391</v>
+        <v>388</v>
       </c>
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A107" s="2" t="s">
-        <v>434</v>
-      </c>
-      <c r="B107" s="4" t="s">
-        <v>435</v>
-      </c>
-      <c r="C107" s="4" t="s">
-        <v>436</v>
-      </c>
-      <c r="D107" s="4" t="s">
-        <v>591</v>
+        <v>188</v>
+      </c>
+      <c r="B107" s="2" t="s">
+        <v>525</v>
+      </c>
+      <c r="C107" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="D107" s="2" t="s">
+        <v>389</v>
       </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A108" s="2" t="s">
-        <v>437</v>
-      </c>
-      <c r="B108" s="4" t="s">
-        <v>438</v>
-      </c>
-      <c r="C108" s="4" t="s">
-        <v>439</v>
-      </c>
-      <c r="D108" s="4" t="s">
-        <v>592</v>
+        <v>190</v>
+      </c>
+      <c r="B108" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="C108" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="D108" s="2" t="s">
+        <v>390</v>
       </c>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A109" s="2" t="s">
-        <v>473</v>
-      </c>
-      <c r="B109" s="4" t="s">
-        <v>590</v>
-      </c>
-      <c r="C109" s="4" t="s">
-        <v>474</v>
-      </c>
-      <c r="D109" s="4" t="s">
-        <v>593</v>
+        <v>192</v>
+      </c>
+      <c r="B109" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="C109" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="D109" s="2" t="s">
+        <v>391</v>
       </c>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A110" s="2" t="s">
-        <v>195</v>
-      </c>
-      <c r="B110" s="2" t="s">
-        <v>196</v>
-      </c>
-      <c r="C110" s="2" t="s">
-        <v>197</v>
-      </c>
-      <c r="D110" s="2" t="s">
-        <v>392</v>
+        <v>434</v>
+      </c>
+      <c r="B110" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="C110" s="4" t="s">
+        <v>436</v>
+      </c>
+      <c r="D110" s="4" t="s">
+        <v>591</v>
       </c>
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A111" s="2" t="s">
-        <v>198</v>
-      </c>
-      <c r="B111" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="C111" s="2" t="s">
-        <v>200</v>
-      </c>
-      <c r="D111" s="2" t="s">
-        <v>393</v>
+        <v>437</v>
+      </c>
+      <c r="B111" s="4" t="s">
+        <v>438</v>
+      </c>
+      <c r="C111" s="4" t="s">
+        <v>439</v>
+      </c>
+      <c r="D111" s="4" t="s">
+        <v>592</v>
       </c>
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A112" s="2" t="s">
-        <v>201</v>
-      </c>
-      <c r="B112" s="2" t="s">
-        <v>201</v>
-      </c>
-      <c r="C112" s="2" t="s">
-        <v>202</v>
-      </c>
-      <c r="D112" s="2" t="s">
-        <v>394</v>
+        <v>473</v>
+      </c>
+      <c r="B112" s="4" t="s">
+        <v>590</v>
+      </c>
+      <c r="C112" s="4" t="s">
+        <v>474</v>
+      </c>
+      <c r="D112" s="4" t="s">
+        <v>593</v>
       </c>
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A113" s="2" t="s">
-        <v>203</v>
+        <v>195</v>
       </c>
       <c r="B113" s="2" t="s">
-        <v>203</v>
+        <v>196</v>
       </c>
       <c r="C113" s="2" t="s">
-        <v>204</v>
+        <v>197</v>
       </c>
       <c r="D113" s="2" t="s">
-        <v>395</v>
+        <v>392</v>
       </c>
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A114" s="2" t="s">
-        <v>205</v>
+        <v>198</v>
       </c>
       <c r="B114" s="2" t="s">
-        <v>205</v>
+        <v>199</v>
       </c>
       <c r="C114" s="2" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
       <c r="D114" s="2" t="s">
-        <v>396</v>
+        <v>393</v>
       </c>
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A115" s="2" t="s">
-        <v>206</v>
+        <v>201</v>
       </c>
       <c r="B115" s="2" t="s">
-        <v>207</v>
+        <v>201</v>
       </c>
       <c r="C115" s="2" t="s">
-        <v>208</v>
+        <v>202</v>
       </c>
       <c r="D115" s="2" t="s">
-        <v>397</v>
+        <v>394</v>
       </c>
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A116" s="2" t="s">
-        <v>209</v>
+        <v>203</v>
       </c>
       <c r="B116" s="2" t="s">
-        <v>210</v>
+        <v>203</v>
       </c>
       <c r="C116" s="2" t="s">
-        <v>211</v>
+        <v>204</v>
       </c>
       <c r="D116" s="2" t="s">
-        <v>398</v>
+        <v>395</v>
       </c>
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A117" s="2" t="s">
-        <v>212</v>
+        <v>205</v>
       </c>
       <c r="B117" s="2" t="s">
-        <v>213</v>
+        <v>205</v>
       </c>
       <c r="C117" s="2" t="s">
-        <v>214</v>
+        <v>205</v>
       </c>
       <c r="D117" s="2" t="s">
-        <v>399</v>
+        <v>396</v>
       </c>
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A118" s="2" t="s">
-        <v>215</v>
+        <v>206</v>
       </c>
       <c r="B118" s="2" t="s">
-        <v>216</v>
+        <v>207</v>
       </c>
       <c r="C118" s="2" t="s">
-        <v>217</v>
+        <v>208</v>
       </c>
       <c r="D118" s="2" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
     </row>
     <row r="119" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A119" s="2" t="s">
-        <v>220</v>
+        <v>209</v>
       </c>
       <c r="B119" s="2" t="s">
-        <v>219</v>
+        <v>210</v>
       </c>
       <c r="C119" s="2" t="s">
-        <v>218</v>
+        <v>211</v>
       </c>
       <c r="D119" s="2" t="s">
-        <v>401</v>
+        <v>398</v>
       </c>
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A120" s="2" t="s">
-        <v>292</v>
+        <v>212</v>
       </c>
       <c r="B120" s="2" t="s">
-        <v>292</v>
+        <v>213</v>
       </c>
       <c r="C120" s="2" t="s">
-        <v>293</v>
+        <v>214</v>
       </c>
       <c r="D120" s="2" t="s">
-        <v>402</v>
+        <v>399</v>
       </c>
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A121" s="2" t="s">
-        <v>294</v>
+        <v>215</v>
       </c>
       <c r="B121" s="2" t="s">
-        <v>295</v>
+        <v>216</v>
       </c>
       <c r="C121" s="2" t="s">
-        <v>296</v>
+        <v>217</v>
       </c>
       <c r="D121" s="2" t="s">
-        <v>403</v>
+        <v>400</v>
       </c>
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A122" s="2" t="s">
-        <v>297</v>
+        <v>220</v>
       </c>
       <c r="B122" s="2" t="s">
-        <v>298</v>
+        <v>219</v>
       </c>
       <c r="C122" s="2" t="s">
-        <v>299</v>
+        <v>218</v>
       </c>
       <c r="D122" s="2" t="s">
-        <v>404</v>
+        <v>401</v>
       </c>
     </row>
     <row r="123" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A123" s="2" t="s">
-        <v>221</v>
+        <v>292</v>
       </c>
       <c r="B123" s="2" t="s">
-        <v>221</v>
+        <v>292</v>
       </c>
       <c r="C123" s="2" t="s">
-        <v>222</v>
+        <v>293</v>
       </c>
       <c r="D123" s="2" t="s">
-        <v>405</v>
+        <v>402</v>
       </c>
     </row>
     <row r="124" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A124" s="2" t="s">
-        <v>223</v>
+        <v>294</v>
       </c>
       <c r="B124" s="2" t="s">
-        <v>224</v>
+        <v>295</v>
       </c>
       <c r="C124" s="2" t="s">
-        <v>225</v>
+        <v>296</v>
       </c>
       <c r="D124" s="2" t="s">
-        <v>406</v>
+        <v>403</v>
       </c>
     </row>
     <row r="125" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A125" s="2" t="s">
-        <v>226</v>
+        <v>297</v>
       </c>
       <c r="B125" s="2" t="s">
-        <v>227</v>
+        <v>298</v>
       </c>
       <c r="C125" s="2" t="s">
-        <v>228</v>
+        <v>299</v>
       </c>
       <c r="D125" s="2" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
     </row>
     <row r="126" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A126" s="2" t="s">
-        <v>229</v>
+        <v>221</v>
       </c>
       <c r="B126" s="2" t="s">
-        <v>229</v>
+        <v>221</v>
       </c>
       <c r="C126" s="2" t="s">
-        <v>229</v>
+        <v>222</v>
       </c>
       <c r="D126" s="2" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
     </row>
     <row r="127" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A127" s="2" t="s">
-        <v>230</v>
+        <v>223</v>
       </c>
       <c r="B127" s="2" t="s">
-        <v>230</v>
+        <v>224</v>
       </c>
       <c r="C127" s="2" t="s">
-        <v>231</v>
+        <v>225</v>
       </c>
       <c r="D127" s="2" t="s">
-        <v>409</v>
+        <v>406</v>
       </c>
     </row>
     <row r="128" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A128" s="2" t="s">
-        <v>232</v>
+        <v>226</v>
       </c>
       <c r="B128" s="2" t="s">
-        <v>232</v>
+        <v>227</v>
       </c>
       <c r="C128" s="2" t="s">
-        <v>233</v>
+        <v>228</v>
       </c>
       <c r="D128" s="2" t="s">
-        <v>410</v>
+        <v>407</v>
       </c>
     </row>
     <row r="129" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A129" s="2" t="s">
-        <v>234</v>
+        <v>229</v>
       </c>
       <c r="B129" s="2" t="s">
-        <v>235</v>
+        <v>229</v>
       </c>
       <c r="C129" s="2" t="s">
-        <v>236</v>
+        <v>229</v>
       </c>
       <c r="D129" s="2" t="s">
-        <v>411</v>
+        <v>408</v>
       </c>
     </row>
     <row r="130" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A130" s="2" t="s">
-        <v>237</v>
+        <v>230</v>
       </c>
       <c r="B130" s="2" t="s">
-        <v>238</v>
+        <v>230</v>
       </c>
       <c r="C130" s="2" t="s">
-        <v>239</v>
+        <v>231</v>
       </c>
       <c r="D130" s="2" t="s">
-        <v>412</v>
+        <v>409</v>
       </c>
     </row>
     <row r="131" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A131" s="2" t="s">
-        <v>300</v>
+        <v>232</v>
       </c>
       <c r="B131" s="2" t="s">
-        <v>301</v>
+        <v>232</v>
       </c>
       <c r="C131" s="2" t="s">
-        <v>302</v>
+        <v>233</v>
       </c>
       <c r="D131" s="2" t="s">
-        <v>413</v>
+        <v>410</v>
       </c>
     </row>
     <row r="132" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A132" s="2" t="s">
-        <v>240</v>
+        <v>234</v>
       </c>
       <c r="B132" s="2" t="s">
-        <v>241</v>
+        <v>235</v>
       </c>
       <c r="C132" s="2" t="s">
-        <v>242</v>
+        <v>236</v>
       </c>
       <c r="D132" s="2" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="133" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A133" s="2" t="s">
-        <v>244</v>
+        <v>237</v>
       </c>
       <c r="B133" s="2" t="s">
-        <v>252</v>
+        <v>238</v>
       </c>
       <c r="C133" s="2" t="s">
-        <v>251</v>
+        <v>239</v>
       </c>
       <c r="D133" s="2" t="s">
-        <v>415</v>
+        <v>412</v>
       </c>
     </row>
     <row r="134" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A134" s="2" t="s">
-        <v>245</v>
+        <v>300</v>
       </c>
       <c r="B134" s="2" t="s">
-        <v>245</v>
+        <v>301</v>
       </c>
       <c r="C134" s="2" t="s">
-        <v>246</v>
+        <v>302</v>
       </c>
       <c r="D134" s="2" t="s">
-        <v>416</v>
+        <v>413</v>
       </c>
     </row>
     <row r="135" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A135" s="2" t="s">
-        <v>247</v>
+        <v>240</v>
       </c>
       <c r="B135" s="2" t="s">
-        <v>247</v>
+        <v>241</v>
       </c>
       <c r="C135" s="2" t="s">
-        <v>248</v>
+        <v>242</v>
       </c>
       <c r="D135" s="2" t="s">
-        <v>417</v>
+        <v>414</v>
       </c>
     </row>
     <row r="136" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A136" s="2" t="s">
-        <v>249</v>
+        <v>244</v>
       </c>
       <c r="B136" s="2" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="C136" s="2" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="D136" s="2" t="s">
-        <v>418</v>
+        <v>415</v>
       </c>
     </row>
     <row r="137" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A137" s="2" t="s">
-        <v>253</v>
+        <v>245</v>
       </c>
       <c r="B137" s="2" t="s">
-        <v>254</v>
+        <v>245</v>
       </c>
       <c r="C137" s="2" t="s">
-        <v>255</v>
+        <v>246</v>
       </c>
       <c r="D137" s="2" t="s">
-        <v>419</v>
+        <v>416</v>
       </c>
     </row>
     <row r="138" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A138" s="2" t="s">
-        <v>256</v>
+        <v>247</v>
       </c>
       <c r="B138" s="2" t="s">
-        <v>257</v>
+        <v>247</v>
       </c>
       <c r="C138" s="2" t="s">
-        <v>258</v>
+        <v>248</v>
       </c>
       <c r="D138" s="2" t="s">
-        <v>420</v>
+        <v>417</v>
       </c>
     </row>
     <row r="139" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A139" s="2" t="s">
-        <v>259</v>
+        <v>249</v>
       </c>
       <c r="B139" s="2" t="s">
-        <v>260</v>
+        <v>249</v>
       </c>
       <c r="C139" s="2" t="s">
-        <v>261</v>
+        <v>250</v>
       </c>
       <c r="D139" s="2" t="s">
-        <v>421</v>
+        <v>418</v>
       </c>
     </row>
     <row r="140" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A140" s="2" t="s">
-        <v>262</v>
+        <v>253</v>
       </c>
       <c r="B140" s="2" t="s">
-        <v>263</v>
+        <v>254</v>
       </c>
       <c r="C140" s="2" t="s">
-        <v>264</v>
+        <v>255</v>
       </c>
       <c r="D140" s="2" t="s">
-        <v>422</v>
+        <v>419</v>
       </c>
     </row>
     <row r="141" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A141" s="2" t="s">
-        <v>265</v>
+        <v>256</v>
       </c>
       <c r="B141" s="2" t="s">
-        <v>265</v>
+        <v>257</v>
       </c>
       <c r="C141" s="2" t="s">
-        <v>265</v>
+        <v>258</v>
       </c>
       <c r="D141" s="2" t="s">
-        <v>423</v>
+        <v>420</v>
       </c>
     </row>
     <row r="142" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A142" s="2" t="s">
-        <v>266</v>
+        <v>259</v>
       </c>
       <c r="B142" s="2" t="s">
-        <v>266</v>
+        <v>260</v>
       </c>
       <c r="C142" s="2" t="s">
-        <v>267</v>
+        <v>261</v>
       </c>
       <c r="D142" s="2" t="s">
-        <v>424</v>
+        <v>421</v>
       </c>
     </row>
     <row r="143" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A143" s="2" t="s">
-        <v>268</v>
+        <v>262</v>
       </c>
       <c r="B143" s="2" t="s">
-        <v>268</v>
+        <v>263</v>
       </c>
       <c r="C143" s="2" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="D143" s="2" t="s">
-        <v>425</v>
+        <v>422</v>
       </c>
     </row>
     <row r="144" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A144" s="2" t="s">
-        <v>270</v>
+        <v>265</v>
       </c>
       <c r="B144" s="2" t="s">
-        <v>270</v>
+        <v>265</v>
       </c>
       <c r="C144" s="2" t="s">
-        <v>273</v>
+        <v>265</v>
       </c>
       <c r="D144" s="2" t="s">
-        <v>426</v>
+        <v>423</v>
       </c>
     </row>
     <row r="145" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A145" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="B145" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="C145" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="D145" s="2" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="146" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A146" s="2" t="s">
+        <v>268</v>
+      </c>
+      <c r="B146" s="2" t="s">
+        <v>268</v>
+      </c>
+      <c r="C146" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="D146" s="2" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="147" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A147" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="B147" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="C147" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="D147" s="2" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="148" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A148" s="2" t="s">
         <v>271</v>
       </c>
-      <c r="B145" s="2" t="s">
+      <c r="B148" s="2" t="s">
         <v>271</v>
       </c>
-      <c r="C145" s="2" t="s">
+      <c r="C148" s="2" t="s">
         <v>272</v>
       </c>
-      <c r="D145" s="2" t="s">
+      <c r="D148" s="2" t="s">
         <v>427</v>
       </c>
     </row>
-    <row r="146" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A146" s="2" t="s">
+    <row r="149" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A149" s="2" t="s">
         <v>274</v>
       </c>
-      <c r="B146" s="2" t="s">
+      <c r="B149" s="2" t="s">
         <v>276</v>
       </c>
-      <c r="C146" s="2" t="s">
+      <c r="C149" s="2" t="s">
         <v>279</v>
       </c>
     </row>
-    <row r="147" spans="1:4" ht="45" x14ac:dyDescent="0.25">
-      <c r="A147" s="2" t="s">
+    <row r="150" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="A150" s="2" t="s">
         <v>275</v>
       </c>
-      <c r="B147" s="2" t="s">
+      <c r="B150" s="2" t="s">
         <v>277</v>
       </c>
-      <c r="C147" s="2" t="s">
+      <c r="C150" s="2" t="s">
         <v>278</v>
       </c>
     </row>
-    <row r="148" spans="1:4" ht="75" x14ac:dyDescent="0.25">
-      <c r="A148" s="2" t="s">
+    <row r="151" spans="1:4" ht="75" x14ac:dyDescent="0.25">
+      <c r="A151" s="2" t="s">
         <v>289</v>
       </c>
-      <c r="B148" s="2" t="s">
+      <c r="B151" s="2" t="s">
         <v>290</v>
       </c>
-      <c r="C148" s="2" t="s">
+      <c r="C151" s="2" t="s">
         <v>291</v>
-      </c>
-    </row>
-    <row r="149" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A149" s="2" t="s">
-        <v>306</v>
-      </c>
-      <c r="B149" s="2" t="s">
-        <v>307</v>
-      </c>
-      <c r="C149" s="2" t="s">
-        <v>308</v>
-      </c>
-      <c r="D149" s="2" t="s">
-        <v>428</v>
-      </c>
-    </row>
-    <row r="150" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A150" s="2" t="s">
-        <v>309</v>
-      </c>
-      <c r="B150" s="2" t="s">
-        <v>311</v>
-      </c>
-      <c r="C150" s="2" t="s">
-        <v>312</v>
-      </c>
-      <c r="D150" s="2" t="s">
-        <v>429</v>
-      </c>
-    </row>
-    <row r="151" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A151" s="2" t="s">
-        <v>310</v>
-      </c>
-      <c r="B151" s="2" t="s">
-        <v>314</v>
-      </c>
-      <c r="C151" s="2" t="s">
-        <v>313</v>
-      </c>
-      <c r="D151" s="2" t="s">
-        <v>430</v>
       </c>
     </row>
     <row r="152" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A152" s="2" t="s">
-        <v>315</v>
+        <v>306</v>
       </c>
       <c r="B152" s="2" t="s">
-        <v>315</v>
+        <v>307</v>
       </c>
       <c r="C152" s="2" t="s">
-        <v>316</v>
+        <v>308</v>
       </c>
       <c r="D152" s="2" t="s">
-        <v>431</v>
+        <v>428</v>
       </c>
     </row>
     <row r="153" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A153" s="2" t="s">
-        <v>317</v>
+        <v>309</v>
       </c>
       <c r="B153" s="2" t="s">
-        <v>318</v>
+        <v>311</v>
       </c>
       <c r="C153" s="2" t="s">
-        <v>460</v>
+        <v>312</v>
       </c>
       <c r="D153" s="2" t="s">
-        <v>432</v>
+        <v>429</v>
       </c>
     </row>
     <row r="154" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A154" s="2" t="s">
-        <v>319</v>
+        <v>310</v>
       </c>
       <c r="B154" s="2" t="s">
-        <v>320</v>
+        <v>314</v>
       </c>
       <c r="C154" s="2" t="s">
-        <v>461</v>
+        <v>313</v>
       </c>
       <c r="D154" s="2" t="s">
-        <v>433</v>
+        <v>430</v>
       </c>
     </row>
     <row r="155" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A155" s="2" t="s">
-        <v>448</v>
+        <v>315</v>
       </c>
       <c r="B155" s="2" t="s">
-        <v>448</v>
+        <v>315</v>
       </c>
       <c r="C155" s="2" t="s">
-        <v>462</v>
+        <v>316</v>
       </c>
       <c r="D155" s="2" t="s">
-        <v>345</v>
+        <v>431</v>
       </c>
     </row>
     <row r="156" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A156" s="2" t="s">
-        <v>449</v>
+        <v>317</v>
       </c>
       <c r="B156" s="2" t="s">
-        <v>450</v>
+        <v>318</v>
       </c>
       <c r="C156" s="2" t="s">
-        <v>463</v>
+        <v>460</v>
       </c>
       <c r="D156" s="2" t="s">
-        <v>451</v>
+        <v>432</v>
       </c>
     </row>
     <row r="157" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A157" s="2" t="s">
-        <v>475</v>
+        <v>319</v>
       </c>
       <c r="B157" s="2" t="s">
-        <v>476</v>
+        <v>320</v>
       </c>
       <c r="C157" s="2" t="s">
-        <v>619</v>
+        <v>461</v>
       </c>
       <c r="D157" s="2" t="s">
-        <v>569</v>
+        <v>433</v>
       </c>
     </row>
     <row r="158" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A158" s="2" t="s">
-        <v>478</v>
+        <v>448</v>
       </c>
       <c r="B158" s="2" t="s">
-        <v>524</v>
+        <v>448</v>
       </c>
       <c r="C158" s="2" t="s">
-        <v>479</v>
+        <v>462</v>
       </c>
       <c r="D158" s="2" t="s">
-        <v>568</v>
+        <v>345</v>
       </c>
     </row>
     <row r="159" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A159" s="2" t="s">
-        <v>480</v>
+        <v>449</v>
       </c>
       <c r="B159" s="2" t="s">
-        <v>481</v>
+        <v>450</v>
       </c>
       <c r="C159" s="2" t="s">
-        <v>482</v>
+        <v>463</v>
       </c>
       <c r="D159" s="2" t="s">
-        <v>567</v>
+        <v>451</v>
       </c>
     </row>
     <row r="160" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A160" s="2" t="s">
-        <v>483</v>
+        <v>475</v>
       </c>
       <c r="B160" s="2" t="s">
-        <v>484</v>
+        <v>476</v>
       </c>
       <c r="C160" s="2" t="s">
-        <v>485</v>
+        <v>619</v>
       </c>
       <c r="D160" s="2" t="s">
-        <v>566</v>
+        <v>569</v>
       </c>
     </row>
     <row r="161" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A161" s="2" t="s">
-        <v>486</v>
+        <v>478</v>
       </c>
       <c r="B161" s="2" t="s">
-        <v>487</v>
+        <v>524</v>
       </c>
       <c r="C161" s="2" t="s">
-        <v>488</v>
+        <v>479</v>
       </c>
       <c r="D161" s="2" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
     </row>
     <row r="162" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A162" s="2" t="s">
-        <v>489</v>
+        <v>480</v>
       </c>
       <c r="B162" s="2" t="s">
-        <v>490</v>
+        <v>481</v>
       </c>
       <c r="C162" s="2" t="s">
-        <v>491</v>
+        <v>482</v>
       </c>
       <c r="D162" s="2" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
     </row>
     <row r="163" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A163" s="2" t="s">
-        <v>538</v>
+        <v>483</v>
       </c>
       <c r="B163" s="2" t="s">
-        <v>538</v>
+        <v>484</v>
       </c>
       <c r="C163" s="2" t="s">
-        <v>607</v>
+        <v>485</v>
       </c>
       <c r="D163" s="2" t="s">
-        <v>539</v>
+        <v>566</v>
       </c>
     </row>
     <row r="164" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A164" s="2" t="s">
-        <v>540</v>
+        <v>486</v>
       </c>
       <c r="B164" s="2" t="s">
-        <v>541</v>
+        <v>487</v>
       </c>
       <c r="C164" s="2" t="s">
-        <v>608</v>
+        <v>488</v>
       </c>
       <c r="D164" s="2" t="s">
-        <v>542</v>
+        <v>565</v>
       </c>
     </row>
     <row r="165" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A165" s="2" t="s">
-        <v>492</v>
+        <v>489</v>
       </c>
       <c r="B165" s="2" t="s">
-        <v>493</v>
+        <v>490</v>
       </c>
       <c r="C165" s="2" t="s">
-        <v>494</v>
+        <v>491</v>
       </c>
       <c r="D165" s="2" t="s">
-        <v>563</v>
+        <v>564</v>
       </c>
     </row>
     <row r="166" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A166" s="2" t="s">
-        <v>495</v>
+        <v>538</v>
       </c>
       <c r="B166" s="2" t="s">
-        <v>496</v>
+        <v>538</v>
       </c>
       <c r="C166" s="2" t="s">
-        <v>497</v>
+        <v>607</v>
       </c>
       <c r="D166" s="2" t="s">
-        <v>562</v>
+        <v>539</v>
       </c>
     </row>
     <row r="167" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A167" s="2" t="s">
-        <v>498</v>
+        <v>540</v>
       </c>
       <c r="B167" s="2" t="s">
-        <v>499</v>
+        <v>541</v>
       </c>
       <c r="C167" s="2" t="s">
-        <v>500</v>
+        <v>608</v>
       </c>
       <c r="D167" s="2" t="s">
-        <v>561</v>
+        <v>542</v>
       </c>
     </row>
     <row r="168" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A168" s="2" t="s">
-        <v>501</v>
+        <v>492</v>
       </c>
       <c r="B168" s="2" t="s">
-        <v>501</v>
+        <v>493</v>
       </c>
       <c r="C168" s="2" t="s">
-        <v>502</v>
+        <v>494</v>
       </c>
       <c r="D168" s="2" t="s">
-        <v>560</v>
+        <v>563</v>
       </c>
     </row>
     <row r="169" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A169" s="2" t="s">
-        <v>503</v>
+        <v>495</v>
       </c>
       <c r="B169" s="2" t="s">
-        <v>503</v>
+        <v>496</v>
       </c>
       <c r="C169" s="2" t="s">
-        <v>504</v>
+        <v>497</v>
       </c>
       <c r="D169" s="2" t="s">
-        <v>559</v>
+        <v>562</v>
       </c>
     </row>
     <row r="170" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A170" s="2" t="s">
-        <v>505</v>
+        <v>498</v>
       </c>
       <c r="B170" s="2" t="s">
-        <v>505</v>
+        <v>499</v>
       </c>
       <c r="C170" s="2" t="s">
-        <v>506</v>
+        <v>500</v>
       </c>
       <c r="D170" s="2" t="s">
-        <v>558</v>
+        <v>561</v>
       </c>
     </row>
     <row r="171" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A171" s="2" t="s">
-        <v>507</v>
+        <v>501</v>
       </c>
       <c r="B171" s="2" t="s">
-        <v>507</v>
+        <v>501</v>
       </c>
       <c r="C171" s="2" t="s">
-        <v>508</v>
+        <v>502</v>
       </c>
       <c r="D171" s="2" t="s">
-        <v>557</v>
+        <v>560</v>
       </c>
     </row>
     <row r="172" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A172" s="2" t="s">
-        <v>570</v>
+        <v>503</v>
       </c>
       <c r="B172" s="2" t="s">
-        <v>571</v>
+        <v>503</v>
       </c>
       <c r="C172" s="2" t="s">
-        <v>609</v>
+        <v>504</v>
+      </c>
+      <c r="D172" s="2" t="s">
+        <v>559</v>
       </c>
     </row>
     <row r="173" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A173" s="2" t="s">
-        <v>572</v>
+        <v>505</v>
       </c>
       <c r="B173" s="2" t="s">
-        <v>573</v>
+        <v>505</v>
       </c>
       <c r="C173" s="2" t="s">
-        <v>610</v>
+        <v>506</v>
+      </c>
+      <c r="D173" s="2" t="s">
+        <v>558</v>
       </c>
     </row>
     <row r="174" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A174" s="2" t="s">
-        <v>574</v>
+        <v>507</v>
       </c>
       <c r="B174" s="2" t="s">
-        <v>575</v>
+        <v>507</v>
       </c>
       <c r="C174" s="2" t="s">
-        <v>611</v>
+        <v>508</v>
+      </c>
+      <c r="D174" s="2" t="s">
+        <v>557</v>
       </c>
     </row>
     <row r="175" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A175" s="2" t="s">
-        <v>576</v>
+        <v>570</v>
       </c>
       <c r="B175" s="2" t="s">
-        <v>577</v>
+        <v>571</v>
       </c>
       <c r="C175" s="2" t="s">
-        <v>612</v>
+        <v>609</v>
       </c>
     </row>
     <row r="176" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A176" s="2" t="s">
-        <v>578</v>
+        <v>572</v>
       </c>
       <c r="B176" s="2" t="s">
-        <v>579</v>
+        <v>573</v>
       </c>
       <c r="C176" s="2" t="s">
-        <v>613</v>
+        <v>610</v>
       </c>
     </row>
     <row r="177" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A177" s="2" t="s">
-        <v>580</v>
+        <v>574</v>
       </c>
       <c r="B177" s="2" t="s">
-        <v>581</v>
+        <v>575</v>
       </c>
       <c r="C177" s="2" t="s">
-        <v>614</v>
+        <v>611</v>
       </c>
     </row>
     <row r="178" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A178" s="2" t="s">
-        <v>582</v>
+        <v>576</v>
       </c>
       <c r="B178" s="2" t="s">
-        <v>583</v>
+        <v>577</v>
       </c>
       <c r="C178" s="2" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
     </row>
     <row r="179" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A179" s="2" t="s">
-        <v>584</v>
+        <v>578</v>
       </c>
       <c r="B179" s="2" t="s">
-        <v>585</v>
+        <v>579</v>
       </c>
       <c r="C179" s="2" t="s">
-        <v>616</v>
+        <v>613</v>
       </c>
     </row>
     <row r="180" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A180" s="2" t="s">
-        <v>586</v>
+        <v>580</v>
       </c>
       <c r="B180" s="2" t="s">
-        <v>587</v>
+        <v>581</v>
       </c>
       <c r="C180" s="2" t="s">
-        <v>617</v>
+        <v>614</v>
       </c>
     </row>
     <row r="181" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A181" s="2" t="s">
-        <v>588</v>
+        <v>582</v>
       </c>
       <c r="B181" s="2" t="s">
-        <v>589</v>
+        <v>583</v>
       </c>
       <c r="C181" s="2" t="s">
-        <v>618</v>
+        <v>615</v>
       </c>
     </row>
     <row r="182" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A182" s="2" t="s">
-        <v>620</v>
+        <v>584</v>
       </c>
       <c r="B182" s="2" t="s">
-        <v>621</v>
+        <v>585</v>
       </c>
       <c r="C182" s="2" t="s">
-        <v>622</v>
+        <v>616</v>
       </c>
     </row>
     <row r="183" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A183" s="2" t="s">
-        <v>623</v>
+        <v>586</v>
       </c>
       <c r="B183" s="2" t="s">
-        <v>623</v>
+        <v>587</v>
       </c>
       <c r="C183" s="2" t="s">
-        <v>624</v>
+        <v>617</v>
       </c>
     </row>
     <row r="184" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A184" s="2" t="s">
-        <v>625</v>
+        <v>588</v>
       </c>
       <c r="B184" s="2" t="s">
-        <v>625</v>
+        <v>589</v>
       </c>
       <c r="C184" s="2" t="s">
-        <v>627</v>
+        <v>618</v>
       </c>
     </row>
     <row r="185" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A185" s="2" t="s">
-        <v>626</v>
+        <v>620</v>
       </c>
       <c r="B185" s="2" t="s">
-        <v>626</v>
+        <v>621</v>
       </c>
       <c r="C185" s="2" t="s">
-        <v>628</v>
+        <v>622</v>
       </c>
     </row>
     <row r="186" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A186" s="2" t="s">
-        <v>629</v>
+        <v>623</v>
       </c>
       <c r="B186" s="2" t="s">
-        <v>630</v>
+        <v>623</v>
       </c>
       <c r="C186" s="2" t="s">
-        <v>631</v>
+        <v>624</v>
       </c>
     </row>
     <row r="187" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A187" s="2" t="s">
-        <v>632</v>
-      </c>
-      <c r="B187" s="4" t="s">
-        <v>633</v>
-      </c>
-      <c r="C187" s="4" t="s">
-        <v>634</v>
+        <v>625</v>
+      </c>
+      <c r="B187" s="2" t="s">
+        <v>625</v>
+      </c>
+      <c r="C187" s="2" t="s">
+        <v>627</v>
       </c>
     </row>
     <row r="188" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A188" s="2" t="s">
-        <v>638</v>
+        <v>626</v>
       </c>
       <c r="B188" s="2" t="s">
-        <v>639</v>
+        <v>626</v>
       </c>
       <c r="C188" s="2" t="s">
-        <v>640</v>
+        <v>628</v>
       </c>
     </row>
     <row r="189" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A189" s="2" t="s">
-        <v>641</v>
+        <v>629</v>
       </c>
       <c r="B189" s="2" t="s">
-        <v>641</v>
+        <v>630</v>
       </c>
       <c r="C189" s="2" t="s">
-        <v>642</v>
+        <v>631</v>
       </c>
     </row>
     <row r="190" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A190" s="2" t="s">
-        <v>643</v>
-      </c>
-      <c r="B190" s="2" t="s">
-        <v>644</v>
-      </c>
-      <c r="C190" s="2" t="s">
-        <v>645</v>
+        <v>632</v>
+      </c>
+      <c r="B190" s="4" t="s">
+        <v>633</v>
+      </c>
+      <c r="C190" s="4" t="s">
+        <v>634</v>
       </c>
     </row>
     <row r="191" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A191" s="2" t="s">
-        <v>646</v>
+        <v>638</v>
       </c>
       <c r="B191" s="2" t="s">
-        <v>647</v>
+        <v>639</v>
       </c>
       <c r="C191" s="2" t="s">
-        <v>648</v>
+        <v>640</v>
       </c>
     </row>
     <row r="192" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A192" s="2" t="s">
-        <v>649</v>
+        <v>641</v>
       </c>
       <c r="B192" s="2" t="s">
-        <v>650</v>
+        <v>641</v>
       </c>
       <c r="C192" s="2" t="s">
-        <v>651</v>
+        <v>642</v>
       </c>
     </row>
     <row r="193" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A193" s="2" t="s">
-        <v>652</v>
+        <v>643</v>
       </c>
       <c r="B193" s="2" t="s">
-        <v>653</v>
+        <v>644</v>
       </c>
       <c r="C193" s="2" t="s">
-        <v>654</v>
+        <v>645</v>
       </c>
     </row>
     <row r="194" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A194" s="2" t="s">
-        <v>655</v>
+        <v>646</v>
       </c>
       <c r="B194" s="2" t="s">
-        <v>655</v>
+        <v>647</v>
       </c>
       <c r="C194" s="2" t="s">
-        <v>656</v>
+        <v>648</v>
       </c>
     </row>
     <row r="195" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A195" s="2" t="s">
-        <v>657</v>
+        <v>649</v>
       </c>
       <c r="B195" s="2" t="s">
-        <v>658</v>
+        <v>650</v>
       </c>
       <c r="C195" s="2" t="s">
-        <v>659</v>
+        <v>651</v>
       </c>
     </row>
     <row r="196" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A196" s="2" t="s">
-        <v>666</v>
-      </c>
-      <c r="B196" s="4" t="s">
-        <v>667</v>
-      </c>
-      <c r="C196" s="4" t="s">
-        <v>668</v>
+        <v>652</v>
+      </c>
+      <c r="B196" s="2" t="s">
+        <v>653</v>
+      </c>
+      <c r="C196" s="2" t="s">
+        <v>654</v>
       </c>
     </row>
     <row r="197" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A197" s="2" t="s">
-        <v>669</v>
+        <v>655</v>
       </c>
       <c r="B197" s="2" t="s">
-        <v>670</v>
+        <v>655</v>
       </c>
       <c r="C197" s="2" t="s">
-        <v>671</v>
+        <v>656</v>
       </c>
     </row>
     <row r="198" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A198" s="2" t="s">
-        <v>675</v>
+        <v>657</v>
       </c>
       <c r="B198" s="2" t="s">
-        <v>676</v>
+        <v>658</v>
       </c>
       <c r="C198" s="2" t="s">
-        <v>677</v>
+        <v>659</v>
       </c>
     </row>
     <row r="199" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A199" s="2" t="s">
-        <v>678</v>
-      </c>
-      <c r="B199" s="2" t="s">
-        <v>679</v>
-      </c>
-      <c r="C199" s="2" t="s">
-        <v>680</v>
+        <v>666</v>
+      </c>
+      <c r="B199" s="4" t="s">
+        <v>667</v>
+      </c>
+      <c r="C199" s="4" t="s">
+        <v>668</v>
       </c>
     </row>
     <row r="200" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A200" s="2" t="s">
-        <v>681</v>
+        <v>669</v>
       </c>
       <c r="B200" s="2" t="s">
-        <v>682</v>
+        <v>670</v>
       </c>
       <c r="C200" s="2" t="s">
-        <v>683</v>
+        <v>671</v>
       </c>
     </row>
     <row r="201" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A201" s="2" t="s">
-        <v>684</v>
+        <v>675</v>
       </c>
       <c r="B201" s="2" t="s">
-        <v>685</v>
+        <v>676</v>
       </c>
       <c r="C201" s="2" t="s">
-        <v>686</v>
+        <v>677</v>
       </c>
     </row>
     <row r="202" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A202" s="2" t="s">
-        <v>687</v>
+        <v>678</v>
       </c>
       <c r="B202" s="2" t="s">
-        <v>688</v>
+        <v>679</v>
       </c>
       <c r="C202" s="2" t="s">
-        <v>689</v>
+        <v>680</v>
       </c>
     </row>
     <row r="203" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A203" s="2" t="s">
-        <v>690</v>
-      </c>
-      <c r="B203" s="4" t="s">
-        <v>694</v>
-      </c>
-      <c r="C203" s="4" t="s">
-        <v>704</v>
+        <v>681</v>
+      </c>
+      <c r="B203" s="2" t="s">
+        <v>682</v>
+      </c>
+      <c r="C203" s="2" t="s">
+        <v>683</v>
       </c>
     </row>
     <row r="204" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A204" s="2" t="s">
-        <v>691</v>
+        <v>684</v>
       </c>
       <c r="B204" s="2" t="s">
-        <v>697</v>
+        <v>685</v>
       </c>
       <c r="C204" s="2" t="s">
-        <v>710</v>
+        <v>686</v>
       </c>
     </row>
     <row r="205" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A205" s="2" t="s">
-        <v>693</v>
-      </c>
-      <c r="B205" s="4" t="s">
-        <v>695</v>
-      </c>
-      <c r="C205" s="4" t="s">
-        <v>705</v>
+        <v>687</v>
+      </c>
+      <c r="B205" s="2" t="s">
+        <v>688</v>
+      </c>
+      <c r="C205" s="2" t="s">
+        <v>689</v>
       </c>
     </row>
     <row r="206" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A206" s="2" t="s">
-        <v>692</v>
+        <v>690</v>
       </c>
       <c r="B206" s="4" t="s">
-        <v>696</v>
+        <v>694</v>
       </c>
       <c r="C206" s="4" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
     </row>
     <row r="207" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A207" s="2" t="s">
-        <v>699</v>
+        <v>691</v>
       </c>
       <c r="B207" s="2" t="s">
-        <v>698</v>
+        <v>697</v>
       </c>
       <c r="C207" s="2" t="s">
-        <v>707</v>
+        <v>710</v>
       </c>
     </row>
     <row r="208" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A208" s="2" t="s">
-        <v>700</v>
-      </c>
-      <c r="B208" s="2" t="s">
-        <v>702</v>
-      </c>
-      <c r="C208" s="2" t="s">
-        <v>708</v>
+        <v>693</v>
+      </c>
+      <c r="B208" s="4" t="s">
+        <v>695</v>
+      </c>
+      <c r="C208" s="4" t="s">
+        <v>705</v>
       </c>
     </row>
     <row r="209" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A209" s="2" t="s">
-        <v>701</v>
-      </c>
-      <c r="B209" s="2" t="s">
-        <v>703</v>
-      </c>
-      <c r="C209" s="2" t="s">
-        <v>709</v>
+        <v>692</v>
+      </c>
+      <c r="B209" s="4" t="s">
+        <v>696</v>
+      </c>
+      <c r="C209" s="4" t="s">
+        <v>706</v>
       </c>
     </row>
     <row r="210" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A210" s="2" t="s">
-        <v>711</v>
+        <v>699</v>
       </c>
       <c r="B210" s="2" t="s">
-        <v>711</v>
+        <v>698</v>
       </c>
       <c r="C210" s="2" t="s">
-        <v>712</v>
+        <v>707</v>
       </c>
     </row>
     <row r="211" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A211" s="2" t="s">
-        <v>713</v>
+        <v>700</v>
       </c>
       <c r="B211" s="2" t="s">
-        <v>714</v>
+        <v>702</v>
       </c>
       <c r="C211" s="2" t="s">
-        <v>715</v>
+        <v>708</v>
       </c>
     </row>
     <row r="212" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A212" s="2" t="s">
-        <v>716</v>
+        <v>701</v>
       </c>
       <c r="B212" s="2" t="s">
-        <v>717</v>
+        <v>703</v>
       </c>
       <c r="C212" s="2" t="s">
-        <v>718</v>
+        <v>709</v>
       </c>
     </row>
     <row r="213" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A213" s="2" t="s">
-        <v>719</v>
+        <v>711</v>
       </c>
       <c r="B213" s="2" t="s">
-        <v>720</v>
+        <v>711</v>
       </c>
       <c r="C213" s="2" t="s">
-        <v>721</v>
+        <v>712</v>
       </c>
     </row>
     <row r="214" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A214" s="2" t="s">
-        <v>732</v>
+        <v>713</v>
       </c>
       <c r="B214" s="2" t="s">
-        <v>733</v>
+        <v>714</v>
       </c>
       <c r="C214" s="2" t="s">
-        <v>736</v>
+        <v>715</v>
       </c>
     </row>
     <row r="215" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A215" s="2" t="s">
-        <v>734</v>
+        <v>716</v>
       </c>
       <c r="B215" s="2" t="s">
-        <v>735</v>
+        <v>717</v>
       </c>
       <c r="C215" s="2" t="s">
-        <v>737</v>
-      </c>
-    </row>
-    <row r="216" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+        <v>718</v>
+      </c>
+    </row>
+    <row r="216" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A216" s="2" t="s">
-        <v>728</v>
+        <v>719</v>
       </c>
       <c r="B216" s="2" t="s">
-        <v>729</v>
+        <v>720</v>
       </c>
       <c r="C216" s="2" t="s">
-        <v>738</v>
-      </c>
-    </row>
-    <row r="217" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+        <v>721</v>
+      </c>
+    </row>
+    <row r="217" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A217" s="2" t="s">
-        <v>730</v>
+        <v>732</v>
       </c>
       <c r="B217" s="2" t="s">
-        <v>731</v>
+        <v>733</v>
       </c>
       <c r="C217" s="2" t="s">
-        <v>739</v>
+        <v>736</v>
       </c>
     </row>
     <row r="218" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A218" s="2" t="s">
-        <v>743</v>
+        <v>734</v>
       </c>
       <c r="B218" s="2" t="s">
-        <v>744</v>
+        <v>735</v>
       </c>
       <c r="C218" s="2" t="s">
-        <v>744</v>
-      </c>
-    </row>
-    <row r="219" spans="1:3" x14ac:dyDescent="0.25">
+        <v>737</v>
+      </c>
+    </row>
+    <row r="219" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A219" s="2" t="s">
-        <v>745</v>
+        <v>728</v>
       </c>
       <c r="B219" s="2" t="s">
-        <v>746</v>
+        <v>729</v>
       </c>
       <c r="C219" s="2" t="s">
-        <v>747</v>
-      </c>
-    </row>
-    <row r="220" spans="1:3" x14ac:dyDescent="0.25">
+        <v>738</v>
+      </c>
+    </row>
+    <row r="220" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A220" s="2" t="s">
-        <v>751</v>
+        <v>730</v>
       </c>
       <c r="B220" s="2" t="s">
-        <v>752</v>
+        <v>731</v>
       </c>
       <c r="C220" s="2" t="s">
-        <v>753</v>
+        <v>739</v>
       </c>
     </row>
     <row r="221" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A221" s="2" t="s">
-        <v>754</v>
+        <v>743</v>
       </c>
       <c r="B221" s="2" t="s">
-        <v>755</v>
+        <v>744</v>
       </c>
       <c r="C221" s="2" t="s">
-        <v>756</v>
+        <v>744</v>
       </c>
     </row>
     <row r="222" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A222" s="2" t="s">
-        <v>757</v>
+        <v>745</v>
       </c>
       <c r="B222" s="2" t="s">
-        <v>758</v>
+        <v>746</v>
       </c>
       <c r="C222" s="2" t="s">
-        <v>759</v>
+        <v>747</v>
       </c>
     </row>
     <row r="223" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A223" s="2" t="s">
-        <v>760</v>
+        <v>751</v>
       </c>
       <c r="B223" s="2" t="s">
-        <v>761</v>
+        <v>752</v>
       </c>
       <c r="C223" s="2" t="s">
-        <v>762</v>
-      </c>
-    </row>
-    <row r="224" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+        <v>753</v>
+      </c>
+    </row>
+    <row r="224" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A224" s="2" t="s">
-        <v>763</v>
+        <v>754</v>
       </c>
       <c r="B224" s="2" t="s">
-        <v>764</v>
+        <v>755</v>
       </c>
       <c r="C224" s="2" t="s">
-        <v>765</v>
-      </c>
-    </row>
-    <row r="225" spans="1:3" ht="60" x14ac:dyDescent="0.25">
+        <v>756</v>
+      </c>
+    </row>
+    <row r="225" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A225" s="2" t="s">
-        <v>766</v>
+        <v>757</v>
       </c>
       <c r="B225" s="2" t="s">
-        <v>767</v>
+        <v>758</v>
       </c>
       <c r="C225" s="2" t="s">
-        <v>768</v>
+        <v>759</v>
       </c>
     </row>
     <row r="226" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A226" s="2" t="s">
+        <v>760</v>
+      </c>
+      <c r="B226" s="2" t="s">
+        <v>761</v>
+      </c>
+      <c r="C226" s="2" t="s">
+        <v>762</v>
+      </c>
+    </row>
+    <row r="227" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A227" s="2" t="s">
+        <v>763</v>
+      </c>
+      <c r="B227" s="2" t="s">
+        <v>764</v>
+      </c>
+      <c r="C227" s="2" t="s">
+        <v>765</v>
+      </c>
+    </row>
+    <row r="228" spans="1:3" ht="60" x14ac:dyDescent="0.25">
+      <c r="A228" s="2" t="s">
+        <v>766</v>
+      </c>
+      <c r="B228" s="2" t="s">
+        <v>767</v>
+      </c>
+      <c r="C228" s="2" t="s">
+        <v>768</v>
+      </c>
+    </row>
+    <row r="229" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A229" s="2" t="s">
         <v>769</v>
       </c>
-      <c r="B226" s="2" t="s">
+      <c r="B229" s="2" t="s">
         <v>770</v>
       </c>
-      <c r="C226" s="2" t="s">
+      <c r="C229" s="2" t="s">
         <v>770</v>
       </c>
     </row>
-    <row r="227" spans="1:3" ht="225" x14ac:dyDescent="0.25">
-      <c r="A227" s="2" t="s">
+    <row r="230" spans="1:3" ht="225" x14ac:dyDescent="0.25">
+      <c r="A230" s="2" t="s">
         <v>774</v>
       </c>
-      <c r="B227" s="2" t="s">
+      <c r="B230" s="2" t="s">
         <v>775</v>
+      </c>
+    </row>
+    <row r="231" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A231" s="2" t="s">
+        <v>788</v>
+      </c>
+      <c r="B231" s="2" t="s">
+        <v>789</v>
+      </c>
+      <c r="C231" s="2" t="s">
+        <v>790</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added the so necessary Flashlight and Water/Taser related translations on playmode.
</commit_message>
<xml_diff>
--- a/Translations/Translations.xlsx
+++ b/Translations/Translations.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programacion\MelonLoader\FS_LevelEditor\Translations\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Coding\FS\LE2cpp\Translations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{499E0310-3A6B-4531-90D8-D8321144CDE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F11A3049-1755-4AAA-B09A-3FBAC7632194}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{F5C22481-FF1A-482C-BF7E-EB5A7718AF49}"/>
+    <workbookView xWindow="22932" yWindow="972" windowWidth="23256" windowHeight="12696" xr2:uid="{F5C22481-FF1A-482C-BF7E-EB5A7718AF49}"/>
   </bookViews>
   <sheets>
     <sheet name="Translations" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1486" uniqueCount="791">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1492" uniqueCount="797">
   <si>
     <t>ID</t>
   </si>
@@ -2415,6 +2415,24 @@
   </si>
   <si>
     <t>Animación de Reaparición</t>
+  </si>
+  <si>
+    <t>FlashlightNotOperational</t>
+  </si>
+  <si>
+    <t>FlashlightOperational</t>
+  </si>
+  <si>
+    <t>TASER_WATER_UNUSABLE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flashlight is not available! </t>
+  </si>
+  <si>
+    <t>Flashlight is now available!</t>
+  </si>
+  <si>
+    <t>Cannot use Taser underwater!</t>
   </si>
 </sst>
 </file>
@@ -2528,7 +2546,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - Tema de 2022">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
     <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
@@ -2825,15 +2843,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6961A5F-F8EA-4989-8112-A0ACE51D011E}">
   <sheetPr codeName="Hoja1"/>
-  <dimension ref="A1:D231"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:D234"/>
+  <sheetFormatPr defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="37" style="2" customWidth="1"/>
-    <col min="2" max="4" width="45.7109375" style="2" customWidth="1"/>
-    <col min="5" max="16384" width="11.42578125" style="2"/>
+    <col min="2" max="4" width="45.6640625" style="2" customWidth="1"/>
+    <col min="5" max="16384" width="11.44140625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -2847,7 +2865,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>160</v>
       </c>
@@ -2861,7 +2879,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>123</v>
       </c>
@@ -2875,7 +2893,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>126</v>
       </c>
@@ -2889,7 +2907,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>129</v>
       </c>
@@ -2903,7 +2921,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>132</v>
       </c>
@@ -2917,7 +2935,7 @@
         <v>326</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>135</v>
       </c>
@@ -2931,7 +2949,7 @@
         <v>327</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>67</v>
       </c>
@@ -2945,7 +2963,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>5</v>
       </c>
@@ -2959,7 +2977,7 @@
         <v>329</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>7</v>
       </c>
@@ -2973,7 +2991,7 @@
         <v>330</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>9</v>
       </c>
@@ -2987,7 +3005,7 @@
         <v>331</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>11</v>
       </c>
@@ -3001,7 +3019,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>13</v>
       </c>
@@ -3015,7 +3033,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>15</v>
       </c>
@@ -3029,7 +3047,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>17</v>
       </c>
@@ -3043,7 +3061,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>19</v>
       </c>
@@ -3057,7 +3075,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
         <v>21</v>
       </c>
@@ -3071,7 +3089,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
         <v>23</v>
       </c>
@@ -3085,7 +3103,7 @@
         <v>338</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
         <v>25</v>
       </c>
@@ -3099,7 +3117,7 @@
         <v>339</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
         <v>27</v>
       </c>
@@ -3113,7 +3131,7 @@
         <v>340</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
         <v>29</v>
       </c>
@@ -3127,7 +3145,7 @@
         <v>341</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
         <v>31</v>
       </c>
@@ -3141,7 +3159,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
         <v>33</v>
       </c>
@@ -3155,7 +3173,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
         <v>35</v>
       </c>
@@ -3169,7 +3187,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
         <v>37</v>
       </c>
@@ -3183,7 +3201,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
         <v>39</v>
       </c>
@@ -3197,7 +3215,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
         <v>41</v>
       </c>
@@ -3211,7 +3229,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
         <v>43</v>
       </c>
@@ -3225,7 +3243,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
         <v>45</v>
       </c>
@@ -3239,7 +3257,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
         <v>47</v>
       </c>
@@ -3253,7 +3271,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
         <v>49</v>
       </c>
@@ -3267,7 +3285,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
         <v>51</v>
       </c>
@@ -3281,7 +3299,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
         <v>53</v>
       </c>
@@ -3295,7 +3313,7 @@
         <v>353</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
         <v>55</v>
       </c>
@@ -3309,7 +3327,7 @@
         <v>354</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
         <v>57</v>
       </c>
@@ -3323,7 +3341,7 @@
         <v>355</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
         <v>59</v>
       </c>
@@ -3337,7 +3355,7 @@
         <v>356</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A37" s="2" t="s">
         <v>61</v>
       </c>
@@ -3351,7 +3369,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A38" s="2" t="s">
         <v>63</v>
       </c>
@@ -3365,7 +3383,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="39" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="2" t="s">
         <v>65</v>
       </c>
@@ -3379,7 +3397,7 @@
         <v>359</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A40" s="2" t="s">
         <v>280</v>
       </c>
@@ -3393,7 +3411,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A41" s="2" t="s">
         <v>283</v>
       </c>
@@ -3407,7 +3425,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A42" s="2" t="s">
         <v>286</v>
       </c>
@@ -3421,7 +3439,7 @@
         <v>362</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A43" s="2" t="s">
         <v>303</v>
       </c>
@@ -3435,7 +3453,7 @@
         <v>363</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A44" s="2" t="s">
         <v>440</v>
       </c>
@@ -3449,7 +3467,7 @@
         <v>553</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A45" s="2" t="s">
         <v>442</v>
       </c>
@@ -3463,7 +3481,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A46" s="2" t="s">
         <v>452</v>
       </c>
@@ -3477,7 +3495,7 @@
         <v>454</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A47" s="2" t="s">
         <v>455</v>
       </c>
@@ -3491,7 +3509,7 @@
         <v>457</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A48" s="2" t="s">
         <v>464</v>
       </c>
@@ -3505,7 +3523,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A49" s="2" t="s">
         <v>467</v>
       </c>
@@ -3519,7 +3537,7 @@
         <v>555</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A50" s="2" t="s">
         <v>470</v>
       </c>
@@ -3533,7 +3551,7 @@
         <v>556</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A51" s="2" t="s">
         <v>509</v>
       </c>
@@ -3547,7 +3565,7 @@
         <v>511</v>
       </c>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A52" s="2" t="s">
         <v>515</v>
       </c>
@@ -3561,7 +3579,7 @@
         <v>517</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A53" s="2" t="s">
         <v>526</v>
       </c>
@@ -3575,7 +3593,7 @@
         <v>528</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A54" s="2" t="s">
         <v>529</v>
       </c>
@@ -3589,7 +3607,7 @@
         <v>531</v>
       </c>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A55" s="2" t="s">
         <v>546</v>
       </c>
@@ -3603,7 +3621,7 @@
         <v>548</v>
       </c>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A56" s="2" t="s">
         <v>549</v>
       </c>
@@ -3617,7 +3635,7 @@
         <v>551</v>
       </c>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A57" s="2" t="s">
         <v>543</v>
       </c>
@@ -3631,7 +3649,7 @@
         <v>545</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A58" s="2" t="s">
         <v>635</v>
       </c>
@@ -3642,7 +3660,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A59" s="2" t="s">
         <v>660</v>
       </c>
@@ -3653,7 +3671,7 @@
         <v>662</v>
       </c>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A60" s="2" t="s">
         <v>663</v>
       </c>
@@ -3664,7 +3682,7 @@
         <v>665</v>
       </c>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A61" s="2" t="s">
         <v>672</v>
       </c>
@@ -3675,7 +3693,7 @@
         <v>674</v>
       </c>
     </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A62" s="2" t="s">
         <v>722</v>
       </c>
@@ -3686,7 +3704,7 @@
         <v>724</v>
       </c>
     </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A63" s="2" t="s">
         <v>725</v>
       </c>
@@ -3697,7 +3715,7 @@
         <v>727</v>
       </c>
     </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A64" s="2" t="s">
         <v>748</v>
       </c>
@@ -3709,7 +3727,7 @@
       </c>
       <c r="D64" s="5"/>
     </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A65" s="2" t="s">
         <v>771</v>
       </c>
@@ -3720,7 +3738,7 @@
         <v>773</v>
       </c>
     </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A66" s="2" t="s">
         <v>779</v>
       </c>
@@ -3731,7 +3749,7 @@
         <v>781</v>
       </c>
     </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A67" s="2" t="s">
         <v>69</v>
       </c>
@@ -3745,7 +3763,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A68" s="2" t="s">
         <v>443</v>
       </c>
@@ -3759,7 +3777,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A69" s="2" t="s">
         <v>456</v>
       </c>
@@ -3773,7 +3791,7 @@
         <v>457</v>
       </c>
     </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A70" s="2" t="s">
         <v>105</v>
       </c>
@@ -3787,7 +3805,7 @@
         <v>365</v>
       </c>
     </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A71" s="2" t="s">
         <v>106</v>
       </c>
@@ -3801,7 +3819,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A72" s="2" t="s">
         <v>107</v>
       </c>
@@ -3815,7 +3833,7 @@
         <v>367</v>
       </c>
     </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A73" s="2" t="s">
         <v>108</v>
       </c>
@@ -3829,7 +3847,7 @@
         <v>365</v>
       </c>
     </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A74" s="2" t="s">
         <v>110</v>
       </c>
@@ -3843,7 +3861,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A75" s="2" t="s">
         <v>114</v>
       </c>
@@ -3857,7 +3875,7 @@
         <v>368</v>
       </c>
     </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A76" s="2" t="s">
         <v>117</v>
       </c>
@@ -3871,7 +3889,7 @@
         <v>369</v>
       </c>
     </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A77" s="2" t="s">
         <v>118</v>
       </c>
@@ -3885,7 +3903,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A78" s="2" t="s">
         <v>445</v>
       </c>
@@ -3899,7 +3917,7 @@
         <v>447</v>
       </c>
     </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A79" s="2" t="s">
         <v>512</v>
       </c>
@@ -3913,7 +3931,7 @@
         <v>514</v>
       </c>
     </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A80" s="2" t="s">
         <v>518</v>
       </c>
@@ -3927,7 +3945,7 @@
         <v>520</v>
       </c>
     </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A81" s="2" t="s">
         <v>521</v>
       </c>
@@ -3941,7 +3959,7 @@
         <v>523</v>
       </c>
     </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A82" s="2" t="s">
         <v>532</v>
       </c>
@@ -3955,7 +3973,7 @@
         <v>534</v>
       </c>
     </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A83" s="2" t="s">
         <v>537</v>
       </c>
@@ -3969,7 +3987,7 @@
         <v>536</v>
       </c>
     </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A84" s="2" t="s">
         <v>740</v>
       </c>
@@ -3980,7 +3998,7 @@
         <v>742</v>
       </c>
     </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A85" s="2" t="s">
         <v>776</v>
       </c>
@@ -3991,7 +4009,7 @@
         <v>778</v>
       </c>
     </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A86" s="2" t="s">
         <v>782</v>
       </c>
@@ -4002,7 +4020,7 @@
         <v>784</v>
       </c>
     </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A87" s="2" t="s">
         <v>785</v>
       </c>
@@ -4013,7 +4031,7 @@
         <v>787</v>
       </c>
     </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A88" s="2" t="s">
         <v>154</v>
       </c>
@@ -4027,7 +4045,7 @@
         <v>371</v>
       </c>
     </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A89" s="2" t="s">
         <v>164</v>
       </c>
@@ -4041,7 +4059,7 @@
         <v>372</v>
       </c>
     </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A90" s="2" t="s">
         <v>157</v>
       </c>
@@ -4055,7 +4073,7 @@
         <v>373</v>
       </c>
     </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A91" s="2" t="s">
         <v>167</v>
       </c>
@@ -4069,7 +4087,7 @@
         <v>374</v>
       </c>
     </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A92" s="2" t="s">
         <v>141</v>
       </c>
@@ -4083,7 +4101,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="93" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A93" s="2" t="s">
         <v>144</v>
       </c>
@@ -4097,7 +4115,7 @@
         <v>376</v>
       </c>
     </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A94" s="2" t="s">
         <v>153</v>
       </c>
@@ -4111,7 +4129,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A95" s="2" t="s">
         <v>147</v>
       </c>
@@ -4125,7 +4143,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A96" s="2" t="s">
         <v>150</v>
       </c>
@@ -4139,7 +4157,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A97" s="2" t="s">
         <v>172</v>
       </c>
@@ -4153,7 +4171,7 @@
         <v>379</v>
       </c>
     </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A98" s="2" t="s">
         <v>173</v>
       </c>
@@ -4167,7 +4185,7 @@
         <v>380</v>
       </c>
     </row>
-    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A99" s="2" t="s">
         <v>176</v>
       </c>
@@ -4181,7 +4199,7 @@
         <v>381</v>
       </c>
     </row>
-    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A100" s="2" t="s">
         <v>178</v>
       </c>
@@ -4195,7 +4213,7 @@
         <v>382</v>
       </c>
     </row>
-    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A101" s="2" t="s">
         <v>180</v>
       </c>
@@ -4209,7 +4227,7 @@
         <v>383</v>
       </c>
     </row>
-    <row r="102" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A102" s="2" t="s">
         <v>243</v>
       </c>
@@ -4223,7 +4241,7 @@
         <v>384</v>
       </c>
     </row>
-    <row r="103" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A103" s="2" t="s">
         <v>138</v>
       </c>
@@ -4237,7 +4255,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="104" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A104" s="2" t="s">
         <v>182</v>
       </c>
@@ -4251,7 +4269,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="105" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A105" s="2" t="s">
         <v>184</v>
       </c>
@@ -4265,7 +4283,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="106" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A106" s="2" t="s">
         <v>186</v>
       </c>
@@ -4279,7 +4297,7 @@
         <v>388</v>
       </c>
     </row>
-    <row r="107" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A107" s="2" t="s">
         <v>188</v>
       </c>
@@ -4293,7 +4311,7 @@
         <v>389</v>
       </c>
     </row>
-    <row r="108" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A108" s="2" t="s">
         <v>190</v>
       </c>
@@ -4307,7 +4325,7 @@
         <v>390</v>
       </c>
     </row>
-    <row r="109" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A109" s="2" t="s">
         <v>192</v>
       </c>
@@ -4321,7 +4339,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="110" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A110" s="2" t="s">
         <v>434</v>
       </c>
@@ -4335,7 +4353,7 @@
         <v>591</v>
       </c>
     </row>
-    <row r="111" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A111" s="2" t="s">
         <v>437</v>
       </c>
@@ -4349,7 +4367,7 @@
         <v>592</v>
       </c>
     </row>
-    <row r="112" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A112" s="2" t="s">
         <v>473</v>
       </c>
@@ -4363,7 +4381,7 @@
         <v>593</v>
       </c>
     </row>
-    <row r="113" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A113" s="2" t="s">
         <v>195</v>
       </c>
@@ -4377,7 +4395,7 @@
         <v>392</v>
       </c>
     </row>
-    <row r="114" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A114" s="2" t="s">
         <v>198</v>
       </c>
@@ -4391,7 +4409,7 @@
         <v>393</v>
       </c>
     </row>
-    <row r="115" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A115" s="2" t="s">
         <v>201</v>
       </c>
@@ -4405,7 +4423,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="116" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A116" s="2" t="s">
         <v>203</v>
       </c>
@@ -4419,7 +4437,7 @@
         <v>395</v>
       </c>
     </row>
-    <row r="117" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A117" s="2" t="s">
         <v>205</v>
       </c>
@@ -4433,7 +4451,7 @@
         <v>396</v>
       </c>
     </row>
-    <row r="118" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A118" s="2" t="s">
         <v>206</v>
       </c>
@@ -4447,7 +4465,7 @@
         <v>397</v>
       </c>
     </row>
-    <row r="119" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A119" s="2" t="s">
         <v>209</v>
       </c>
@@ -4461,7 +4479,7 @@
         <v>398</v>
       </c>
     </row>
-    <row r="120" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A120" s="2" t="s">
         <v>212</v>
       </c>
@@ -4475,7 +4493,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="121" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A121" s="2" t="s">
         <v>215</v>
       </c>
@@ -4489,7 +4507,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="122" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A122" s="2" t="s">
         <v>220</v>
       </c>
@@ -4503,7 +4521,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="123" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A123" s="2" t="s">
         <v>292</v>
       </c>
@@ -4517,7 +4535,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="124" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A124" s="2" t="s">
         <v>294</v>
       </c>
@@ -4531,7 +4549,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="125" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A125" s="2" t="s">
         <v>297</v>
       </c>
@@ -4545,7 +4563,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="126" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A126" s="2" t="s">
         <v>221</v>
       </c>
@@ -4559,7 +4577,7 @@
         <v>405</v>
       </c>
     </row>
-    <row r="127" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A127" s="2" t="s">
         <v>223</v>
       </c>
@@ -4573,7 +4591,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="128" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A128" s="2" t="s">
         <v>226</v>
       </c>
@@ -4587,7 +4605,7 @@
         <v>407</v>
       </c>
     </row>
-    <row r="129" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A129" s="2" t="s">
         <v>229</v>
       </c>
@@ -4601,7 +4619,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="130" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A130" s="2" t="s">
         <v>230</v>
       </c>
@@ -4615,7 +4633,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="131" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A131" s="2" t="s">
         <v>232</v>
       </c>
@@ -4629,7 +4647,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="132" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A132" s="2" t="s">
         <v>234</v>
       </c>
@@ -4643,7 +4661,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="133" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A133" s="2" t="s">
         <v>237</v>
       </c>
@@ -4657,7 +4675,7 @@
         <v>412</v>
       </c>
     </row>
-    <row r="134" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A134" s="2" t="s">
         <v>300</v>
       </c>
@@ -4671,7 +4689,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="135" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A135" s="2" t="s">
         <v>240</v>
       </c>
@@ -4685,7 +4703,7 @@
         <v>414</v>
       </c>
     </row>
-    <row r="136" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A136" s="2" t="s">
         <v>244</v>
       </c>
@@ -4699,7 +4717,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="137" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A137" s="2" t="s">
         <v>245</v>
       </c>
@@ -4713,7 +4731,7 @@
         <v>416</v>
       </c>
     </row>
-    <row r="138" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A138" s="2" t="s">
         <v>247</v>
       </c>
@@ -4727,7 +4745,7 @@
         <v>417</v>
       </c>
     </row>
-    <row r="139" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A139" s="2" t="s">
         <v>249</v>
       </c>
@@ -4741,7 +4759,7 @@
         <v>418</v>
       </c>
     </row>
-    <row r="140" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A140" s="2" t="s">
         <v>253</v>
       </c>
@@ -4755,7 +4773,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="141" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A141" s="2" t="s">
         <v>256</v>
       </c>
@@ -4769,7 +4787,7 @@
         <v>420</v>
       </c>
     </row>
-    <row r="142" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A142" s="2" t="s">
         <v>259</v>
       </c>
@@ -4783,7 +4801,7 @@
         <v>421</v>
       </c>
     </row>
-    <row r="143" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A143" s="2" t="s">
         <v>262</v>
       </c>
@@ -4797,7 +4815,7 @@
         <v>422</v>
       </c>
     </row>
-    <row r="144" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A144" s="2" t="s">
         <v>265</v>
       </c>
@@ -4811,7 +4829,7 @@
         <v>423</v>
       </c>
     </row>
-    <row r="145" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A145" s="2" t="s">
         <v>266</v>
       </c>
@@ -4825,7 +4843,7 @@
         <v>424</v>
       </c>
     </row>
-    <row r="146" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A146" s="2" t="s">
         <v>268</v>
       </c>
@@ -4839,7 +4857,7 @@
         <v>425</v>
       </c>
     </row>
-    <row r="147" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A147" s="2" t="s">
         <v>270</v>
       </c>
@@ -4853,7 +4871,7 @@
         <v>426</v>
       </c>
     </row>
-    <row r="148" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A148" s="2" t="s">
         <v>271</v>
       </c>
@@ -4867,7 +4885,7 @@
         <v>427</v>
       </c>
     </row>
-    <row r="149" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A149" s="2" t="s">
         <v>274</v>
       </c>
@@ -4878,7 +4896,7 @@
         <v>279</v>
       </c>
     </row>
-    <row r="150" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A150" s="2" t="s">
         <v>275</v>
       </c>
@@ -4889,7 +4907,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="151" spans="1:4" ht="75" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A151" s="2" t="s">
         <v>289</v>
       </c>
@@ -4900,7 +4918,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="152" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A152" s="2" t="s">
         <v>306</v>
       </c>
@@ -4914,7 +4932,7 @@
         <v>428</v>
       </c>
     </row>
-    <row r="153" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A153" s="2" t="s">
         <v>309</v>
       </c>
@@ -4928,7 +4946,7 @@
         <v>429</v>
       </c>
     </row>
-    <row r="154" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A154" s="2" t="s">
         <v>310</v>
       </c>
@@ -4942,7 +4960,7 @@
         <v>430</v>
       </c>
     </row>
-    <row r="155" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A155" s="2" t="s">
         <v>315</v>
       </c>
@@ -4956,7 +4974,7 @@
         <v>431</v>
       </c>
     </row>
-    <row r="156" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A156" s="2" t="s">
         <v>317</v>
       </c>
@@ -4970,7 +4988,7 @@
         <v>432</v>
       </c>
     </row>
-    <row r="157" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A157" s="2" t="s">
         <v>319</v>
       </c>
@@ -4984,7 +5002,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="158" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A158" s="2" t="s">
         <v>448</v>
       </c>
@@ -4998,7 +5016,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="159" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A159" s="2" t="s">
         <v>449</v>
       </c>
@@ -5012,7 +5030,7 @@
         <v>451</v>
       </c>
     </row>
-    <row r="160" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A160" s="2" t="s">
         <v>475</v>
       </c>
@@ -5026,7 +5044,7 @@
         <v>569</v>
       </c>
     </row>
-    <row r="161" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A161" s="2" t="s">
         <v>478</v>
       </c>
@@ -5040,7 +5058,7 @@
         <v>568</v>
       </c>
     </row>
-    <row r="162" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A162" s="2" t="s">
         <v>480</v>
       </c>
@@ -5054,7 +5072,7 @@
         <v>567</v>
       </c>
     </row>
-    <row r="163" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A163" s="2" t="s">
         <v>483</v>
       </c>
@@ -5068,7 +5086,7 @@
         <v>566</v>
       </c>
     </row>
-    <row r="164" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A164" s="2" t="s">
         <v>486</v>
       </c>
@@ -5082,7 +5100,7 @@
         <v>565</v>
       </c>
     </row>
-    <row r="165" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A165" s="2" t="s">
         <v>489</v>
       </c>
@@ -5096,7 +5114,7 @@
         <v>564</v>
       </c>
     </row>
-    <row r="166" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A166" s="2" t="s">
         <v>538</v>
       </c>
@@ -5110,7 +5128,7 @@
         <v>539</v>
       </c>
     </row>
-    <row r="167" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A167" s="2" t="s">
         <v>540</v>
       </c>
@@ -5124,7 +5142,7 @@
         <v>542</v>
       </c>
     </row>
-    <row r="168" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A168" s="2" t="s">
         <v>492</v>
       </c>
@@ -5138,7 +5156,7 @@
         <v>563</v>
       </c>
     </row>
-    <row r="169" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A169" s="2" t="s">
         <v>495</v>
       </c>
@@ -5152,7 +5170,7 @@
         <v>562</v>
       </c>
     </row>
-    <row r="170" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A170" s="2" t="s">
         <v>498</v>
       </c>
@@ -5166,7 +5184,7 @@
         <v>561</v>
       </c>
     </row>
-    <row r="171" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A171" s="2" t="s">
         <v>501</v>
       </c>
@@ -5180,7 +5198,7 @@
         <v>560</v>
       </c>
     </row>
-    <row r="172" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A172" s="2" t="s">
         <v>503</v>
       </c>
@@ -5194,7 +5212,7 @@
         <v>559</v>
       </c>
     </row>
-    <row r="173" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A173" s="2" t="s">
         <v>505</v>
       </c>
@@ -5208,7 +5226,7 @@
         <v>558</v>
       </c>
     </row>
-    <row r="174" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A174" s="2" t="s">
         <v>507</v>
       </c>
@@ -5222,7 +5240,7 @@
         <v>557</v>
       </c>
     </row>
-    <row r="175" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A175" s="2" t="s">
         <v>570</v>
       </c>
@@ -5233,7 +5251,7 @@
         <v>609</v>
       </c>
     </row>
-    <row r="176" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A176" s="2" t="s">
         <v>572</v>
       </c>
@@ -5244,7 +5262,7 @@
         <v>610</v>
       </c>
     </row>
-    <row r="177" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A177" s="2" t="s">
         <v>574</v>
       </c>
@@ -5255,7 +5273,7 @@
         <v>611</v>
       </c>
     </row>
-    <row r="178" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A178" s="2" t="s">
         <v>576</v>
       </c>
@@ -5266,7 +5284,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="179" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A179" s="2" t="s">
         <v>578</v>
       </c>
@@ -5277,7 +5295,7 @@
         <v>613</v>
       </c>
     </row>
-    <row r="180" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A180" s="2" t="s">
         <v>580</v>
       </c>
@@ -5288,7 +5306,7 @@
         <v>614</v>
       </c>
     </row>
-    <row r="181" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A181" s="2" t="s">
         <v>582</v>
       </c>
@@ -5299,7 +5317,7 @@
         <v>615</v>
       </c>
     </row>
-    <row r="182" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A182" s="2" t="s">
         <v>584</v>
       </c>
@@ -5310,7 +5328,7 @@
         <v>616</v>
       </c>
     </row>
-    <row r="183" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A183" s="2" t="s">
         <v>586</v>
       </c>
@@ -5321,7 +5339,7 @@
         <v>617</v>
       </c>
     </row>
-    <row r="184" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A184" s="2" t="s">
         <v>588</v>
       </c>
@@ -5332,7 +5350,7 @@
         <v>618</v>
       </c>
     </row>
-    <row r="185" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A185" s="2" t="s">
         <v>620</v>
       </c>
@@ -5343,7 +5361,7 @@
         <v>622</v>
       </c>
     </row>
-    <row r="186" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A186" s="2" t="s">
         <v>623</v>
       </c>
@@ -5354,7 +5372,7 @@
         <v>624</v>
       </c>
     </row>
-    <row r="187" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A187" s="2" t="s">
         <v>625</v>
       </c>
@@ -5365,7 +5383,7 @@
         <v>627</v>
       </c>
     </row>
-    <row r="188" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A188" s="2" t="s">
         <v>626</v>
       </c>
@@ -5376,7 +5394,7 @@
         <v>628</v>
       </c>
     </row>
-    <row r="189" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A189" s="2" t="s">
         <v>629</v>
       </c>
@@ -5387,7 +5405,7 @@
         <v>631</v>
       </c>
     </row>
-    <row r="190" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A190" s="2" t="s">
         <v>632</v>
       </c>
@@ -5398,7 +5416,7 @@
         <v>634</v>
       </c>
     </row>
-    <row r="191" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A191" s="2" t="s">
         <v>638</v>
       </c>
@@ -5409,7 +5427,7 @@
         <v>640</v>
       </c>
     </row>
-    <row r="192" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A192" s="2" t="s">
         <v>641</v>
       </c>
@@ -5420,7 +5438,7 @@
         <v>642</v>
       </c>
     </row>
-    <row r="193" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A193" s="2" t="s">
         <v>643</v>
       </c>
@@ -5431,7 +5449,7 @@
         <v>645</v>
       </c>
     </row>
-    <row r="194" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A194" s="2" t="s">
         <v>646</v>
       </c>
@@ -5442,7 +5460,7 @@
         <v>648</v>
       </c>
     </row>
-    <row r="195" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A195" s="2" t="s">
         <v>649</v>
       </c>
@@ -5453,7 +5471,7 @@
         <v>651</v>
       </c>
     </row>
-    <row r="196" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A196" s="2" t="s">
         <v>652</v>
       </c>
@@ -5464,7 +5482,7 @@
         <v>654</v>
       </c>
     </row>
-    <row r="197" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A197" s="2" t="s">
         <v>655</v>
       </c>
@@ -5475,7 +5493,7 @@
         <v>656</v>
       </c>
     </row>
-    <row r="198" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A198" s="2" t="s">
         <v>657</v>
       </c>
@@ -5486,7 +5504,7 @@
         <v>659</v>
       </c>
     </row>
-    <row r="199" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A199" s="2" t="s">
         <v>666</v>
       </c>
@@ -5497,7 +5515,7 @@
         <v>668</v>
       </c>
     </row>
-    <row r="200" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A200" s="2" t="s">
         <v>669</v>
       </c>
@@ -5508,7 +5526,7 @@
         <v>671</v>
       </c>
     </row>
-    <row r="201" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A201" s="2" t="s">
         <v>675</v>
       </c>
@@ -5519,7 +5537,7 @@
         <v>677</v>
       </c>
     </row>
-    <row r="202" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A202" s="2" t="s">
         <v>678</v>
       </c>
@@ -5530,7 +5548,7 @@
         <v>680</v>
       </c>
     </row>
-    <row r="203" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A203" s="2" t="s">
         <v>681</v>
       </c>
@@ -5541,7 +5559,7 @@
         <v>683</v>
       </c>
     </row>
-    <row r="204" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A204" s="2" t="s">
         <v>684</v>
       </c>
@@ -5552,7 +5570,7 @@
         <v>686</v>
       </c>
     </row>
-    <row r="205" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A205" s="2" t="s">
         <v>687</v>
       </c>
@@ -5563,7 +5581,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="206" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A206" s="2" t="s">
         <v>690</v>
       </c>
@@ -5574,7 +5592,7 @@
         <v>704</v>
       </c>
     </row>
-    <row r="207" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A207" s="2" t="s">
         <v>691</v>
       </c>
@@ -5585,7 +5603,7 @@
         <v>710</v>
       </c>
     </row>
-    <row r="208" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A208" s="2" t="s">
         <v>693</v>
       </c>
@@ -5596,7 +5614,7 @@
         <v>705</v>
       </c>
     </row>
-    <row r="209" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A209" s="2" t="s">
         <v>692</v>
       </c>
@@ -5607,7 +5625,7 @@
         <v>706</v>
       </c>
     </row>
-    <row r="210" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A210" s="2" t="s">
         <v>699</v>
       </c>
@@ -5618,7 +5636,7 @@
         <v>707</v>
       </c>
     </row>
-    <row r="211" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A211" s="2" t="s">
         <v>700</v>
       </c>
@@ -5629,7 +5647,7 @@
         <v>708</v>
       </c>
     </row>
-    <row r="212" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A212" s="2" t="s">
         <v>701</v>
       </c>
@@ -5640,7 +5658,7 @@
         <v>709</v>
       </c>
     </row>
-    <row r="213" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A213" s="2" t="s">
         <v>711</v>
       </c>
@@ -5651,7 +5669,7 @@
         <v>712</v>
       </c>
     </row>
-    <row r="214" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A214" s="2" t="s">
         <v>713</v>
       </c>
@@ -5662,7 +5680,7 @@
         <v>715</v>
       </c>
     </row>
-    <row r="215" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A215" s="2" t="s">
         <v>716</v>
       </c>
@@ -5673,7 +5691,7 @@
         <v>718</v>
       </c>
     </row>
-    <row r="216" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A216" s="2" t="s">
         <v>719</v>
       </c>
@@ -5684,7 +5702,7 @@
         <v>721</v>
       </c>
     </row>
-    <row r="217" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A217" s="2" t="s">
         <v>732</v>
       </c>
@@ -5695,7 +5713,7 @@
         <v>736</v>
       </c>
     </row>
-    <row r="218" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A218" s="2" t="s">
         <v>734</v>
       </c>
@@ -5706,7 +5724,7 @@
         <v>737</v>
       </c>
     </row>
-    <row r="219" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A219" s="2" t="s">
         <v>728</v>
       </c>
@@ -5717,7 +5735,7 @@
         <v>738</v>
       </c>
     </row>
-    <row r="220" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A220" s="2" t="s">
         <v>730</v>
       </c>
@@ -5728,7 +5746,7 @@
         <v>739</v>
       </c>
     </row>
-    <row r="221" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A221" s="2" t="s">
         <v>743</v>
       </c>
@@ -5739,7 +5757,7 @@
         <v>744</v>
       </c>
     </row>
-    <row r="222" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A222" s="2" t="s">
         <v>745</v>
       </c>
@@ -5750,7 +5768,7 @@
         <v>747</v>
       </c>
     </row>
-    <row r="223" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A223" s="2" t="s">
         <v>751</v>
       </c>
@@ -5761,7 +5779,7 @@
         <v>753</v>
       </c>
     </row>
-    <row r="224" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A224" s="2" t="s">
         <v>754</v>
       </c>
@@ -5772,7 +5790,7 @@
         <v>756</v>
       </c>
     </row>
-    <row r="225" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A225" s="2" t="s">
         <v>757</v>
       </c>
@@ -5783,7 +5801,7 @@
         <v>759</v>
       </c>
     </row>
-    <row r="226" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A226" s="2" t="s">
         <v>760</v>
       </c>
@@ -5794,7 +5812,7 @@
         <v>762</v>
       </c>
     </row>
-    <row r="227" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A227" s="2" t="s">
         <v>763</v>
       </c>
@@ -5805,7 +5823,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="228" spans="1:3" ht="60" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A228" s="2" t="s">
         <v>766</v>
       </c>
@@ -5816,7 +5834,7 @@
         <v>768</v>
       </c>
     </row>
-    <row r="229" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A229" s="2" t="s">
         <v>769</v>
       </c>
@@ -5827,7 +5845,7 @@
         <v>770</v>
       </c>
     </row>
-    <row r="230" spans="1:3" ht="225" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:3" ht="216" x14ac:dyDescent="0.3">
       <c r="A230" s="2" t="s">
         <v>774</v>
       </c>
@@ -5835,7 +5853,7 @@
         <v>775</v>
       </c>
     </row>
-    <row r="231" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A231" s="2" t="s">
         <v>788</v>
       </c>
@@ -5844,6 +5862,30 @@
       </c>
       <c r="C231" s="2" t="s">
         <v>790</v>
+      </c>
+    </row>
+    <row r="232" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A232" s="2" t="s">
+        <v>791</v>
+      </c>
+      <c r="B232" s="2" t="s">
+        <v>794</v>
+      </c>
+    </row>
+    <row r="233" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A233" s="2" t="s">
+        <v>792</v>
+      </c>
+      <c r="B233" s="2" t="s">
+        <v>795</v>
+      </c>
+    </row>
+    <row r="234" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A234" s="2" t="s">
+        <v>793</v>
+      </c>
+      <c r="B234" s="2" t="s">
+        <v>796</v>
       </c>
     </row>
   </sheetData>
@@ -5856,9 +5898,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE0107E6-A156-44A0-947B-0BE38822807A}">
   <dimension ref="A1:D171"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -5872,7 +5914,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>160</v>
       </c>
@@ -5886,7 +5928,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>123</v>
       </c>
@@ -5900,7 +5942,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>126</v>
       </c>
@@ -5914,7 +5956,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>129</v>
       </c>
@@ -5928,7 +5970,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>132</v>
       </c>
@@ -5942,7 +5984,7 @@
         <v>326</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>135</v>
       </c>
@@ -5956,7 +5998,7 @@
         <v>327</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>67</v>
       </c>
@@ -5970,7 +6012,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>5</v>
       </c>
@@ -5984,7 +6026,7 @@
         <v>329</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>7</v>
       </c>
@@ -5998,7 +6040,7 @@
         <v>330</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -6012,7 +6054,7 @@
         <v>331</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>11</v>
       </c>
@@ -6026,7 +6068,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>13</v>
       </c>
@@ -6040,7 +6082,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>15</v>
       </c>
@@ -6054,7 +6096,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>17</v>
       </c>
@@ -6068,7 +6110,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>19</v>
       </c>
@@ -6082,7 +6124,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>21</v>
       </c>
@@ -6096,7 +6138,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>23</v>
       </c>
@@ -6110,7 +6152,7 @@
         <v>338</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>25</v>
       </c>
@@ -6124,7 +6166,7 @@
         <v>339</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>27</v>
       </c>
@@ -6138,7 +6180,7 @@
         <v>340</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>29</v>
       </c>
@@ -6152,7 +6194,7 @@
         <v>341</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>31</v>
       </c>
@@ -6166,7 +6208,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>33</v>
       </c>
@@ -6180,7 +6222,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>35</v>
       </c>
@@ -6194,7 +6236,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>37</v>
       </c>
@@ -6208,7 +6250,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>39</v>
       </c>
@@ -6222,7 +6264,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>41</v>
       </c>
@@ -6236,7 +6278,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>43</v>
       </c>
@@ -6250,7 +6292,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>45</v>
       </c>
@@ -6264,7 +6306,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>47</v>
       </c>
@@ -6278,7 +6320,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>49</v>
       </c>
@@ -6292,7 +6334,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>51</v>
       </c>
@@ -6306,7 +6348,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>53</v>
       </c>
@@ -6320,7 +6362,7 @@
         <v>353</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>55</v>
       </c>
@@ -6334,7 +6376,7 @@
         <v>354</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>57</v>
       </c>
@@ -6348,7 +6390,7 @@
         <v>355</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>59</v>
       </c>
@@ -6362,7 +6404,7 @@
         <v>356</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>61</v>
       </c>
@@ -6376,7 +6418,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>63</v>
       </c>
@@ -6390,7 +6432,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>65</v>
       </c>
@@ -6404,7 +6446,7 @@
         <v>359</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>280</v>
       </c>
@@ -6418,7 +6460,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>283</v>
       </c>
@@ -6432,7 +6474,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>286</v>
       </c>
@@ -6446,7 +6488,7 @@
         <v>362</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>303</v>
       </c>
@@ -6460,7 +6502,7 @@
         <v>363</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>440</v>
       </c>
@@ -6474,7 +6516,7 @@
         <v>553</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>442</v>
       </c>
@@ -6488,7 +6530,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>452</v>
       </c>
@@ -6502,7 +6544,7 @@
         <v>454</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>455</v>
       </c>
@@ -6516,7 +6558,7 @@
         <v>457</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>464</v>
       </c>
@@ -6530,7 +6572,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>467</v>
       </c>
@@ -6544,7 +6586,7 @@
         <v>555</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>470</v>
       </c>
@@ -6558,7 +6600,7 @@
         <v>556</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>509</v>
       </c>
@@ -6569,7 +6611,7 @@
         <v>511</v>
       </c>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>515</v>
       </c>
@@ -6580,7 +6622,7 @@
         <v>517</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>526</v>
       </c>
@@ -6591,7 +6633,7 @@
         <v>528</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>529</v>
       </c>
@@ -6602,7 +6644,7 @@
         <v>531</v>
       </c>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>546</v>
       </c>
@@ -6613,7 +6655,7 @@
         <v>548</v>
       </c>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>549</v>
       </c>
@@ -6624,7 +6666,7 @@
         <v>551</v>
       </c>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>543</v>
       </c>
@@ -6635,7 +6677,7 @@
         <v>545</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>69</v>
       </c>
@@ -6649,7 +6691,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>443</v>
       </c>
@@ -6660,7 +6702,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>456</v>
       </c>
@@ -6671,7 +6713,7 @@
         <v>457</v>
       </c>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>105</v>
       </c>
@@ -6685,7 +6727,7 @@
         <v>365</v>
       </c>
     </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>106</v>
       </c>
@@ -6699,7 +6741,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>107</v>
       </c>
@@ -6713,7 +6755,7 @@
         <v>367</v>
       </c>
     </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>108</v>
       </c>
@@ -6727,7 +6769,7 @@
         <v>365</v>
       </c>
     </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>110</v>
       </c>
@@ -6741,7 +6783,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>114</v>
       </c>
@@ -6755,7 +6797,7 @@
         <v>368</v>
       </c>
     </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>117</v>
       </c>
@@ -6769,7 +6811,7 @@
         <v>369</v>
       </c>
     </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>118</v>
       </c>
@@ -6783,7 +6825,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>445</v>
       </c>
@@ -6797,7 +6839,7 @@
         <v>447</v>
       </c>
     </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>512</v>
       </c>
@@ -6808,7 +6850,7 @@
         <v>514</v>
       </c>
     </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>518</v>
       </c>
@@ -6819,7 +6861,7 @@
         <v>520</v>
       </c>
     </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>521</v>
       </c>
@@ -6830,7 +6872,7 @@
         <v>523</v>
       </c>
     </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>532</v>
       </c>
@@ -6841,7 +6883,7 @@
         <v>534</v>
       </c>
     </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>537</v>
       </c>
@@ -6852,7 +6894,7 @@
         <v>536</v>
       </c>
     </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>154</v>
       </c>
@@ -6866,7 +6908,7 @@
         <v>371</v>
       </c>
     </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>164</v>
       </c>
@@ -6880,7 +6922,7 @@
         <v>372</v>
       </c>
     </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>157</v>
       </c>
@@ -6894,7 +6936,7 @@
         <v>373</v>
       </c>
     </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>167</v>
       </c>
@@ -6908,7 +6950,7 @@
         <v>374</v>
       </c>
     </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>141</v>
       </c>
@@ -6922,7 +6964,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>144</v>
       </c>
@@ -6936,7 +6978,7 @@
         <v>376</v>
       </c>
     </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>153</v>
       </c>
@@ -6950,7 +6992,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>147</v>
       </c>
@@ -6964,7 +7006,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>150</v>
       </c>
@@ -6978,7 +7020,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
         <v>172</v>
       </c>
@@ -6992,7 +7034,7 @@
         <v>379</v>
       </c>
     </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
         <v>173</v>
       </c>
@@ -7006,7 +7048,7 @@
         <v>380</v>
       </c>
     </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
         <v>176</v>
       </c>
@@ -7020,7 +7062,7 @@
         <v>381</v>
       </c>
     </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
         <v>178</v>
       </c>
@@ -7034,7 +7076,7 @@
         <v>382</v>
       </c>
     </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
         <v>180</v>
       </c>
@@ -7048,7 +7090,7 @@
         <v>383</v>
       </c>
     </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
         <v>243</v>
       </c>
@@ -7062,7 +7104,7 @@
         <v>384</v>
       </c>
     </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
         <v>138</v>
       </c>
@@ -7076,7 +7118,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
         <v>182</v>
       </c>
@@ -7090,7 +7132,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
         <v>184</v>
       </c>
@@ -7104,7 +7146,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
         <v>186</v>
       </c>
@@ -7118,7 +7160,7 @@
         <v>388</v>
       </c>
     </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
         <v>188</v>
       </c>
@@ -7132,7 +7174,7 @@
         <v>389</v>
       </c>
     </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
         <v>190</v>
       </c>
@@ -7146,7 +7188,7 @@
         <v>390</v>
       </c>
     </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
         <v>192</v>
       </c>
@@ -7160,7 +7202,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
         <v>434</v>
       </c>
@@ -7177,7 +7219,7 @@
         <v>#NAME?</v>
       </c>
     </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
         <v>437</v>
       </c>
@@ -7194,7 +7236,7 @@
         <v>#NAME?</v>
       </c>
     </row>
-    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
         <v>473</v>
       </c>
@@ -7211,7 +7253,7 @@
         <v>#NAME?</v>
       </c>
     </row>
-    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
         <v>195</v>
       </c>
@@ -7225,7 +7267,7 @@
         <v>392</v>
       </c>
     </row>
-    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
         <v>198</v>
       </c>
@@ -7239,7 +7281,7 @@
         <v>393</v>
       </c>
     </row>
-    <row r="102" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
         <v>201</v>
       </c>
@@ -7253,7 +7295,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="103" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
         <v>203</v>
       </c>
@@ -7267,7 +7309,7 @@
         <v>395</v>
       </c>
     </row>
-    <row r="104" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
         <v>205</v>
       </c>
@@ -7281,7 +7323,7 @@
         <v>396</v>
       </c>
     </row>
-    <row r="105" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
         <v>206</v>
       </c>
@@ -7295,7 +7337,7 @@
         <v>397</v>
       </c>
     </row>
-    <row r="106" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
         <v>209</v>
       </c>
@@ -7309,7 +7351,7 @@
         <v>398</v>
       </c>
     </row>
-    <row r="107" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
         <v>212</v>
       </c>
@@ -7323,7 +7365,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="108" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
         <v>215</v>
       </c>
@@ -7337,7 +7379,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="109" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
         <v>220</v>
       </c>
@@ -7351,7 +7393,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="110" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
         <v>292</v>
       </c>
@@ -7365,7 +7407,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="111" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
         <v>294</v>
       </c>
@@ -7379,7 +7421,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="112" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
         <v>297</v>
       </c>
@@ -7393,7 +7435,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="113" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
         <v>221</v>
       </c>
@@ -7407,7 +7449,7 @@
         <v>405</v>
       </c>
     </row>
-    <row r="114" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
         <v>223</v>
       </c>
@@ -7421,7 +7463,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="115" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
         <v>226</v>
       </c>
@@ -7435,7 +7477,7 @@
         <v>407</v>
       </c>
     </row>
-    <row r="116" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
         <v>229</v>
       </c>
@@ -7449,7 +7491,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="117" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
         <v>230</v>
       </c>
@@ -7463,7 +7505,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="118" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
         <v>232</v>
       </c>
@@ -7477,7 +7519,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="119" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A119" t="s">
         <v>234</v>
       </c>
@@ -7491,7 +7533,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="120" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
         <v>237</v>
       </c>
@@ -7505,7 +7547,7 @@
         <v>412</v>
       </c>
     </row>
-    <row r="121" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A121" t="s">
         <v>300</v>
       </c>
@@ -7519,7 +7561,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="122" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A122" t="s">
         <v>240</v>
       </c>
@@ -7533,7 +7575,7 @@
         <v>414</v>
       </c>
     </row>
-    <row r="123" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A123" t="s">
         <v>244</v>
       </c>
@@ -7547,7 +7589,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="124" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A124" t="s">
         <v>245</v>
       </c>
@@ -7561,7 +7603,7 @@
         <v>416</v>
       </c>
     </row>
-    <row r="125" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A125" t="s">
         <v>247</v>
       </c>
@@ -7575,7 +7617,7 @@
         <v>417</v>
       </c>
     </row>
-    <row r="126" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A126" t="s">
         <v>249</v>
       </c>
@@ -7589,7 +7631,7 @@
         <v>418</v>
       </c>
     </row>
-    <row r="127" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A127" t="s">
         <v>253</v>
       </c>
@@ -7603,7 +7645,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="128" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A128" t="s">
         <v>256</v>
       </c>
@@ -7617,7 +7659,7 @@
         <v>420</v>
       </c>
     </row>
-    <row r="129" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A129" t="s">
         <v>259</v>
       </c>
@@ -7631,7 +7673,7 @@
         <v>421</v>
       </c>
     </row>
-    <row r="130" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A130" t="s">
         <v>262</v>
       </c>
@@ -7645,7 +7687,7 @@
         <v>422</v>
       </c>
     </row>
-    <row r="131" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A131" t="s">
         <v>265</v>
       </c>
@@ -7659,7 +7701,7 @@
         <v>423</v>
       </c>
     </row>
-    <row r="132" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A132" t="s">
         <v>266</v>
       </c>
@@ -7673,7 +7715,7 @@
         <v>424</v>
       </c>
     </row>
-    <row r="133" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A133" t="s">
         <v>268</v>
       </c>
@@ -7687,7 +7729,7 @@
         <v>425</v>
       </c>
     </row>
-    <row r="134" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A134" t="s">
         <v>270</v>
       </c>
@@ -7701,7 +7743,7 @@
         <v>426</v>
       </c>
     </row>
-    <row r="135" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A135" t="s">
         <v>271</v>
       </c>
@@ -7715,7 +7757,7 @@
         <v>427</v>
       </c>
     </row>
-    <row r="136" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A136" t="s">
         <v>274</v>
       </c>
@@ -7726,7 +7768,7 @@
         <v>279</v>
       </c>
     </row>
-    <row r="137" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A137" t="s">
         <v>275</v>
       </c>
@@ -7737,7 +7779,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="138" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A138" t="s">
         <v>289</v>
       </c>
@@ -7748,7 +7790,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="139" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A139" t="s">
         <v>306</v>
       </c>
@@ -7762,7 +7804,7 @@
         <v>428</v>
       </c>
     </row>
-    <row r="140" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A140" t="s">
         <v>309</v>
       </c>
@@ -7776,7 +7818,7 @@
         <v>429</v>
       </c>
     </row>
-    <row r="141" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A141" t="s">
         <v>310</v>
       </c>
@@ -7790,7 +7832,7 @@
         <v>430</v>
       </c>
     </row>
-    <row r="142" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A142" t="s">
         <v>315</v>
       </c>
@@ -7804,7 +7846,7 @@
         <v>431</v>
       </c>
     </row>
-    <row r="143" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A143" t="s">
         <v>317</v>
       </c>
@@ -7818,7 +7860,7 @@
         <v>432</v>
       </c>
     </row>
-    <row r="144" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A144" t="s">
         <v>319</v>
       </c>
@@ -7832,7 +7874,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="145" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A145" t="s">
         <v>448</v>
       </c>
@@ -7846,7 +7888,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="146" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A146" t="s">
         <v>449</v>
       </c>
@@ -7860,7 +7902,7 @@
         <v>451</v>
       </c>
     </row>
-    <row r="147" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A147" t="s">
         <v>475</v>
       </c>
@@ -7874,7 +7916,7 @@
         <v>569</v>
       </c>
     </row>
-    <row r="148" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A148" t="s">
         <v>478</v>
       </c>
@@ -7888,7 +7930,7 @@
         <v>568</v>
       </c>
     </row>
-    <row r="149" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A149" t="s">
         <v>480</v>
       </c>
@@ -7902,7 +7944,7 @@
         <v>567</v>
       </c>
     </row>
-    <row r="150" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A150" t="s">
         <v>483</v>
       </c>
@@ -7916,7 +7958,7 @@
         <v>566</v>
       </c>
     </row>
-    <row r="151" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A151" t="s">
         <v>486</v>
       </c>
@@ -7930,7 +7972,7 @@
         <v>565</v>
       </c>
     </row>
-    <row r="152" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A152" t="s">
         <v>489</v>
       </c>
@@ -7944,7 +7986,7 @@
         <v>564</v>
       </c>
     </row>
-    <row r="153" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A153" t="s">
         <v>538</v>
       </c>
@@ -7955,7 +7997,7 @@
         <v>539</v>
       </c>
     </row>
-    <row r="154" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A154" t="s">
         <v>540</v>
       </c>
@@ -7966,7 +8008,7 @@
         <v>542</v>
       </c>
     </row>
-    <row r="155" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A155" t="s">
         <v>492</v>
       </c>
@@ -7980,7 +8022,7 @@
         <v>563</v>
       </c>
     </row>
-    <row r="156" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A156" t="s">
         <v>495</v>
       </c>
@@ -7994,7 +8036,7 @@
         <v>562</v>
       </c>
     </row>
-    <row r="157" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A157" t="s">
         <v>498</v>
       </c>
@@ -8008,7 +8050,7 @@
         <v>561</v>
       </c>
     </row>
-    <row r="158" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A158" t="s">
         <v>501</v>
       </c>
@@ -8022,7 +8064,7 @@
         <v>560</v>
       </c>
     </row>
-    <row r="159" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A159" t="s">
         <v>503</v>
       </c>
@@ -8036,7 +8078,7 @@
         <v>559</v>
       </c>
     </row>
-    <row r="160" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A160" t="s">
         <v>505</v>
       </c>
@@ -8050,7 +8092,7 @@
         <v>558</v>
       </c>
     </row>
-    <row r="161" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A161" t="s">
         <v>507</v>
       </c>
@@ -8064,7 +8106,7 @@
         <v>557</v>
       </c>
     </row>
-    <row r="162" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A162" t="s">
         <v>570</v>
       </c>
@@ -8072,7 +8114,7 @@
         <v>571</v>
       </c>
     </row>
-    <row r="163" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A163" t="s">
         <v>572</v>
       </c>
@@ -8080,7 +8122,7 @@
         <v>573</v>
       </c>
     </row>
-    <row r="164" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A164" t="s">
         <v>574</v>
       </c>
@@ -8088,7 +8130,7 @@
         <v>575</v>
       </c>
     </row>
-    <row r="165" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A165" t="s">
         <v>576</v>
       </c>
@@ -8096,7 +8138,7 @@
         <v>577</v>
       </c>
     </row>
-    <row r="166" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A166" t="s">
         <v>578</v>
       </c>
@@ -8104,7 +8146,7 @@
         <v>579</v>
       </c>
     </row>
-    <row r="167" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A167" t="s">
         <v>580</v>
       </c>
@@ -8112,7 +8154,7 @@
         <v>581</v>
       </c>
     </row>
-    <row r="168" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A168" t="s">
         <v>582</v>
       </c>
@@ -8120,7 +8162,7 @@
         <v>583</v>
       </c>
     </row>
-    <row r="169" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A169" t="s">
         <v>584</v>
       </c>
@@ -8128,7 +8170,7 @@
         <v>585</v>
       </c>
     </row>
-    <row r="170" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A170" t="s">
         <v>586</v>
       </c>
@@ -8136,7 +8178,7 @@
         <v>587</v>
       </c>
     </row>
-    <row r="171" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A171" t="s">
         <v>588</v>
       </c>

</xml_diff>

<commit_message>
Putting the broken translations fixes inside of ChapterLocPatch is not necessary, the mod already hooks the Localization.Get method, so we can just use the OG keys in the translations file and it will replace them automatically.
</commit_message>
<xml_diff>
--- a/Translations/Translations.xlsx
+++ b/Translations/Translations.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Coding\FS\LE2cpp\Translations\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programacion\MelonLoader\FS_LevelEditor\Translations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F11A3049-1755-4AAA-B09A-3FBAC7632194}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01731B24-1764-4CA6-9FA2-28A0CB5C8F89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="972" windowWidth="23256" windowHeight="12696" xr2:uid="{F5C22481-FF1A-482C-BF7E-EB5A7718AF49}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{F5C22481-FF1A-482C-BF7E-EB5A7718AF49}"/>
   </bookViews>
   <sheets>
     <sheet name="Translations" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1492" uniqueCount="797">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1493" uniqueCount="798">
   <si>
     <t>ID</t>
   </si>
@@ -2417,15 +2417,6 @@
     <t>Animación de Reaparición</t>
   </si>
   <si>
-    <t>FlashlightNotOperational</t>
-  </si>
-  <si>
-    <t>FlashlightOperational</t>
-  </si>
-  <si>
-    <t>TASER_WATER_UNUSABLE</t>
-  </si>
-  <si>
     <t xml:space="preserve">Flashlight is not available! </t>
   </si>
   <si>
@@ -2433,6 +2424,18 @@
   </si>
   <si>
     <t>Cannot use Taser underwater!</t>
+  </si>
+  <si>
+    <t>Notification_FlashlightNotOperational</t>
+  </si>
+  <si>
+    <t>Notification_FlashlightOperational</t>
+  </si>
+  <si>
+    <t>Notification_TASER_WATER_UNUSABLE</t>
+  </si>
+  <si>
+    <t># Broken translations in the main game.</t>
   </si>
 </sst>
 </file>
@@ -2546,7 +2549,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - Tema de 2022">
   <a:themeElements>
     <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
@@ -2843,15 +2846,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6961A5F-F8EA-4989-8112-A0ACE51D011E}">
   <sheetPr codeName="Hoja1"/>
-  <dimension ref="A1:D234"/>
-  <sheetFormatPr defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:D236"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="37" style="2" customWidth="1"/>
-    <col min="2" max="4" width="45.6640625" style="2" customWidth="1"/>
-    <col min="5" max="16384" width="11.44140625" style="2"/>
+    <col min="2" max="4" width="45.7109375" style="2" customWidth="1"/>
+    <col min="5" max="16384" width="11.42578125" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -2865,7 +2868,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>160</v>
       </c>
@@ -2879,7 +2882,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>123</v>
       </c>
@@ -2893,7 +2896,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>126</v>
       </c>
@@ -2907,7 +2910,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>129</v>
       </c>
@@ -2921,7 +2924,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>132</v>
       </c>
@@ -2935,7 +2938,7 @@
         <v>326</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>135</v>
       </c>
@@ -2949,7 +2952,7 @@
         <v>327</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>67</v>
       </c>
@@ -2963,7 +2966,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>5</v>
       </c>
@@ -2977,7 +2980,7 @@
         <v>329</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>7</v>
       </c>
@@ -2991,7 +2994,7 @@
         <v>330</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>9</v>
       </c>
@@ -3005,7 +3008,7 @@
         <v>331</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>11</v>
       </c>
@@ -3019,7 +3022,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>13</v>
       </c>
@@ -3033,7 +3036,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>15</v>
       </c>
@@ -3047,7 +3050,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>17</v>
       </c>
@@ -3061,7 +3064,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>19</v>
       </c>
@@ -3075,7 +3078,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>21</v>
       </c>
@@ -3089,7 +3092,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>23</v>
       </c>
@@ -3103,7 +3106,7 @@
         <v>338</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>25</v>
       </c>
@@ -3117,7 +3120,7 @@
         <v>339</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>27</v>
       </c>
@@ -3131,7 +3134,7 @@
         <v>340</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>29</v>
       </c>
@@ -3145,7 +3148,7 @@
         <v>341</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>31</v>
       </c>
@@ -3159,7 +3162,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>33</v>
       </c>
@@ -3173,7 +3176,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>35</v>
       </c>
@@ -3187,7 +3190,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>37</v>
       </c>
@@ -3201,7 +3204,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>39</v>
       </c>
@@ -3215,7 +3218,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>41</v>
       </c>
@@ -3229,7 +3232,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>43</v>
       </c>
@@ -3243,7 +3246,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>45</v>
       </c>
@@ -3257,7 +3260,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>47</v>
       </c>
@@ -3271,7 +3274,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>49</v>
       </c>
@@ -3285,7 +3288,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>51</v>
       </c>
@@ -3299,7 +3302,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>53</v>
       </c>
@@ -3313,7 +3316,7 @@
         <v>353</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
         <v>55</v>
       </c>
@@ -3327,7 +3330,7 @@
         <v>354</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
         <v>57</v>
       </c>
@@ -3341,7 +3344,7 @@
         <v>355</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
         <v>59</v>
       </c>
@@ -3355,7 +3358,7 @@
         <v>356</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
         <v>61</v>
       </c>
@@ -3369,7 +3372,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
         <v>63</v>
       </c>
@@ -3383,7 +3386,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="39" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
         <v>65</v>
       </c>
@@ -3397,7 +3400,7 @@
         <v>359</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
         <v>280</v>
       </c>
@@ -3411,7 +3414,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
         <v>283</v>
       </c>
@@ -3425,7 +3428,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
         <v>286</v>
       </c>
@@ -3439,7 +3442,7 @@
         <v>362</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
         <v>303</v>
       </c>
@@ -3453,7 +3456,7 @@
         <v>363</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
         <v>440</v>
       </c>
@@ -3467,7 +3470,7 @@
         <v>553</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
         <v>442</v>
       </c>
@@ -3481,7 +3484,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
         <v>452</v>
       </c>
@@ -3495,7 +3498,7 @@
         <v>454</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
         <v>455</v>
       </c>
@@ -3509,7 +3512,7 @@
         <v>457</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
         <v>464</v>
       </c>
@@ -3523,7 +3526,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
         <v>467</v>
       </c>
@@ -3537,7 +3540,7 @@
         <v>555</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
         <v>470</v>
       </c>
@@ -3551,7 +3554,7 @@
         <v>556</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
         <v>509</v>
       </c>
@@ -3565,7 +3568,7 @@
         <v>511</v>
       </c>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
         <v>515</v>
       </c>
@@ -3579,7 +3582,7 @@
         <v>517</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" s="2" t="s">
         <v>526</v>
       </c>
@@ -3593,7 +3596,7 @@
         <v>528</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" s="2" t="s">
         <v>529</v>
       </c>
@@ -3607,7 +3610,7 @@
         <v>531</v>
       </c>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A55" s="2" t="s">
         <v>546</v>
       </c>
@@ -3621,7 +3624,7 @@
         <v>548</v>
       </c>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
         <v>549</v>
       </c>
@@ -3635,7 +3638,7 @@
         <v>551</v>
       </c>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57" s="2" t="s">
         <v>543</v>
       </c>
@@ -3649,7 +3652,7 @@
         <v>545</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" s="2" t="s">
         <v>635</v>
       </c>
@@ -3660,7 +3663,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" s="2" t="s">
         <v>660</v>
       </c>
@@ -3671,7 +3674,7 @@
         <v>662</v>
       </c>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
         <v>663</v>
       </c>
@@ -3682,7 +3685,7 @@
         <v>665</v>
       </c>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61" s="2" t="s">
         <v>672</v>
       </c>
@@ -3693,7 +3696,7 @@
         <v>674</v>
       </c>
     </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" s="2" t="s">
         <v>722</v>
       </c>
@@ -3704,7 +3707,7 @@
         <v>724</v>
       </c>
     </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63" s="2" t="s">
         <v>725</v>
       </c>
@@ -3715,7 +3718,7 @@
         <v>727</v>
       </c>
     </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" s="2" t="s">
         <v>748</v>
       </c>
@@ -3727,7 +3730,7 @@
       </c>
       <c r="D64" s="5"/>
     </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A65" s="2" t="s">
         <v>771</v>
       </c>
@@ -3738,7 +3741,7 @@
         <v>773</v>
       </c>
     </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66" s="2" t="s">
         <v>779</v>
       </c>
@@ -3749,7 +3752,7 @@
         <v>781</v>
       </c>
     </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A67" s="2" t="s">
         <v>69</v>
       </c>
@@ -3763,7 +3766,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A68" s="2" t="s">
         <v>443</v>
       </c>
@@ -3777,7 +3780,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A69" s="2" t="s">
         <v>456</v>
       </c>
@@ -3791,7 +3794,7 @@
         <v>457</v>
       </c>
     </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A70" s="2" t="s">
         <v>105</v>
       </c>
@@ -3805,7 +3808,7 @@
         <v>365</v>
       </c>
     </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A71" s="2" t="s">
         <v>106</v>
       </c>
@@ -3819,7 +3822,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A72" s="2" t="s">
         <v>107</v>
       </c>
@@ -3833,7 +3836,7 @@
         <v>367</v>
       </c>
     </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A73" s="2" t="s">
         <v>108</v>
       </c>
@@ -3847,7 +3850,7 @@
         <v>365</v>
       </c>
     </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A74" s="2" t="s">
         <v>110</v>
       </c>
@@ -3861,7 +3864,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A75" s="2" t="s">
         <v>114</v>
       </c>
@@ -3875,7 +3878,7 @@
         <v>368</v>
       </c>
     </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A76" s="2" t="s">
         <v>117</v>
       </c>
@@ -3889,7 +3892,7 @@
         <v>369</v>
       </c>
     </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A77" s="2" t="s">
         <v>118</v>
       </c>
@@ -3903,7 +3906,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A78" s="2" t="s">
         <v>445</v>
       </c>
@@ -3917,7 +3920,7 @@
         <v>447</v>
       </c>
     </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A79" s="2" t="s">
         <v>512</v>
       </c>
@@ -3931,7 +3934,7 @@
         <v>514</v>
       </c>
     </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
         <v>518</v>
       </c>
@@ -3945,7 +3948,7 @@
         <v>520</v>
       </c>
     </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A81" s="2" t="s">
         <v>521</v>
       </c>
@@ -3959,7 +3962,7 @@
         <v>523</v>
       </c>
     </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A82" s="2" t="s">
         <v>532</v>
       </c>
@@ -3973,7 +3976,7 @@
         <v>534</v>
       </c>
     </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A83" s="2" t="s">
         <v>537</v>
       </c>
@@ -3987,7 +3990,7 @@
         <v>536</v>
       </c>
     </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A84" s="2" t="s">
         <v>740</v>
       </c>
@@ -3998,7 +4001,7 @@
         <v>742</v>
       </c>
     </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A85" s="2" t="s">
         <v>776</v>
       </c>
@@ -4009,7 +4012,7 @@
         <v>778</v>
       </c>
     </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A86" s="2" t="s">
         <v>782</v>
       </c>
@@ -4020,7 +4023,7 @@
         <v>784</v>
       </c>
     </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A87" s="2" t="s">
         <v>785</v>
       </c>
@@ -4031,7 +4034,7 @@
         <v>787</v>
       </c>
     </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A88" s="2" t="s">
         <v>154</v>
       </c>
@@ -4045,7 +4048,7 @@
         <v>371</v>
       </c>
     </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A89" s="2" t="s">
         <v>164</v>
       </c>
@@ -4059,7 +4062,7 @@
         <v>372</v>
       </c>
     </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A90" s="2" t="s">
         <v>157</v>
       </c>
@@ -4073,7 +4076,7 @@
         <v>373</v>
       </c>
     </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A91" s="2" t="s">
         <v>167</v>
       </c>
@@ -4087,7 +4090,7 @@
         <v>374</v>
       </c>
     </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A92" s="2" t="s">
         <v>141</v>
       </c>
@@ -4101,7 +4104,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="93" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A93" s="2" t="s">
         <v>144</v>
       </c>
@@ -4115,7 +4118,7 @@
         <v>376</v>
       </c>
     </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A94" s="2" t="s">
         <v>153</v>
       </c>
@@ -4129,7 +4132,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A95" s="2" t="s">
         <v>147</v>
       </c>
@@ -4143,7 +4146,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A96" s="2" t="s">
         <v>150</v>
       </c>
@@ -4157,7 +4160,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A97" s="2" t="s">
         <v>172</v>
       </c>
@@ -4171,7 +4174,7 @@
         <v>379</v>
       </c>
     </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A98" s="2" t="s">
         <v>173</v>
       </c>
@@ -4185,7 +4188,7 @@
         <v>380</v>
       </c>
     </row>
-    <row r="99" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A99" s="2" t="s">
         <v>176</v>
       </c>
@@ -4199,7 +4202,7 @@
         <v>381</v>
       </c>
     </row>
-    <row r="100" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A100" s="2" t="s">
         <v>178</v>
       </c>
@@ -4213,7 +4216,7 @@
         <v>382</v>
       </c>
     </row>
-    <row r="101" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A101" s="2" t="s">
         <v>180</v>
       </c>
@@ -4227,7 +4230,7 @@
         <v>383</v>
       </c>
     </row>
-    <row r="102" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A102" s="2" t="s">
         <v>243</v>
       </c>
@@ -4241,7 +4244,7 @@
         <v>384</v>
       </c>
     </row>
-    <row r="103" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A103" s="2" t="s">
         <v>138</v>
       </c>
@@ -4255,7 +4258,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="104" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A104" s="2" t="s">
         <v>182</v>
       </c>
@@ -4269,7 +4272,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="105" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A105" s="2" t="s">
         <v>184</v>
       </c>
@@ -4283,7 +4286,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="106" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A106" s="2" t="s">
         <v>186</v>
       </c>
@@ -4297,7 +4300,7 @@
         <v>388</v>
       </c>
     </row>
-    <row r="107" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A107" s="2" t="s">
         <v>188</v>
       </c>
@@ -4311,7 +4314,7 @@
         <v>389</v>
       </c>
     </row>
-    <row r="108" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A108" s="2" t="s">
         <v>190</v>
       </c>
@@ -4325,7 +4328,7 @@
         <v>390</v>
       </c>
     </row>
-    <row r="109" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A109" s="2" t="s">
         <v>192</v>
       </c>
@@ -4339,7 +4342,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="110" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A110" s="2" t="s">
         <v>434</v>
       </c>
@@ -4353,7 +4356,7 @@
         <v>591</v>
       </c>
     </row>
-    <row r="111" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A111" s="2" t="s">
         <v>437</v>
       </c>
@@ -4367,7 +4370,7 @@
         <v>592</v>
       </c>
     </row>
-    <row r="112" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A112" s="2" t="s">
         <v>473</v>
       </c>
@@ -4381,7 +4384,7 @@
         <v>593</v>
       </c>
     </row>
-    <row r="113" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A113" s="2" t="s">
         <v>195</v>
       </c>
@@ -4395,7 +4398,7 @@
         <v>392</v>
       </c>
     </row>
-    <row r="114" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A114" s="2" t="s">
         <v>198</v>
       </c>
@@ -4409,7 +4412,7 @@
         <v>393</v>
       </c>
     </row>
-    <row r="115" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A115" s="2" t="s">
         <v>201</v>
       </c>
@@ -4423,7 +4426,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="116" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A116" s="2" t="s">
         <v>203</v>
       </c>
@@ -4437,7 +4440,7 @@
         <v>395</v>
       </c>
     </row>
-    <row r="117" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A117" s="2" t="s">
         <v>205</v>
       </c>
@@ -4451,7 +4454,7 @@
         <v>396</v>
       </c>
     </row>
-    <row r="118" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A118" s="2" t="s">
         <v>206</v>
       </c>
@@ -4465,7 +4468,7 @@
         <v>397</v>
       </c>
     </row>
-    <row r="119" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A119" s="2" t="s">
         <v>209</v>
       </c>
@@ -4479,7 +4482,7 @@
         <v>398</v>
       </c>
     </row>
-    <row r="120" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A120" s="2" t="s">
         <v>212</v>
       </c>
@@ -4493,7 +4496,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="121" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A121" s="2" t="s">
         <v>215</v>
       </c>
@@ -4507,7 +4510,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="122" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A122" s="2" t="s">
         <v>220</v>
       </c>
@@ -4521,7 +4524,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="123" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A123" s="2" t="s">
         <v>292</v>
       </c>
@@ -4535,7 +4538,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="124" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A124" s="2" t="s">
         <v>294</v>
       </c>
@@ -4549,7 +4552,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="125" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A125" s="2" t="s">
         <v>297</v>
       </c>
@@ -4563,7 +4566,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="126" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A126" s="2" t="s">
         <v>221</v>
       </c>
@@ -4577,7 +4580,7 @@
         <v>405</v>
       </c>
     </row>
-    <row r="127" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A127" s="2" t="s">
         <v>223</v>
       </c>
@@ -4591,7 +4594,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="128" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A128" s="2" t="s">
         <v>226</v>
       </c>
@@ -4605,7 +4608,7 @@
         <v>407</v>
       </c>
     </row>
-    <row r="129" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A129" s="2" t="s">
         <v>229</v>
       </c>
@@ -4619,7 +4622,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="130" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A130" s="2" t="s">
         <v>230</v>
       </c>
@@ -4633,7 +4636,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="131" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A131" s="2" t="s">
         <v>232</v>
       </c>
@@ -4647,7 +4650,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="132" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A132" s="2" t="s">
         <v>234</v>
       </c>
@@ -4661,7 +4664,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="133" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A133" s="2" t="s">
         <v>237</v>
       </c>
@@ -4675,7 +4678,7 @@
         <v>412</v>
       </c>
     </row>
-    <row r="134" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A134" s="2" t="s">
         <v>300</v>
       </c>
@@ -4689,7 +4692,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="135" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A135" s="2" t="s">
         <v>240</v>
       </c>
@@ -4703,7 +4706,7 @@
         <v>414</v>
       </c>
     </row>
-    <row r="136" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A136" s="2" t="s">
         <v>244</v>
       </c>
@@ -4717,7 +4720,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="137" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A137" s="2" t="s">
         <v>245</v>
       </c>
@@ -4731,7 +4734,7 @@
         <v>416</v>
       </c>
     </row>
-    <row r="138" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A138" s="2" t="s">
         <v>247</v>
       </c>
@@ -4745,7 +4748,7 @@
         <v>417</v>
       </c>
     </row>
-    <row r="139" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A139" s="2" t="s">
         <v>249</v>
       </c>
@@ -4759,7 +4762,7 @@
         <v>418</v>
       </c>
     </row>
-    <row r="140" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A140" s="2" t="s">
         <v>253</v>
       </c>
@@ -4773,7 +4776,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="141" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A141" s="2" t="s">
         <v>256</v>
       </c>
@@ -4787,7 +4790,7 @@
         <v>420</v>
       </c>
     </row>
-    <row r="142" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A142" s="2" t="s">
         <v>259</v>
       </c>
@@ -4801,7 +4804,7 @@
         <v>421</v>
       </c>
     </row>
-    <row r="143" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A143" s="2" t="s">
         <v>262</v>
       </c>
@@ -4815,7 +4818,7 @@
         <v>422</v>
       </c>
     </row>
-    <row r="144" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A144" s="2" t="s">
         <v>265</v>
       </c>
@@ -4829,7 +4832,7 @@
         <v>423</v>
       </c>
     </row>
-    <row r="145" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A145" s="2" t="s">
         <v>266</v>
       </c>
@@ -4843,7 +4846,7 @@
         <v>424</v>
       </c>
     </row>
-    <row r="146" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A146" s="2" t="s">
         <v>268</v>
       </c>
@@ -4857,7 +4860,7 @@
         <v>425</v>
       </c>
     </row>
-    <row r="147" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A147" s="2" t="s">
         <v>270</v>
       </c>
@@ -4871,7 +4874,7 @@
         <v>426</v>
       </c>
     </row>
-    <row r="148" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A148" s="2" t="s">
         <v>271</v>
       </c>
@@ -4885,7 +4888,7 @@
         <v>427</v>
       </c>
     </row>
-    <row r="149" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A149" s="2" t="s">
         <v>274</v>
       </c>
@@ -4896,7 +4899,7 @@
         <v>279</v>
       </c>
     </row>
-    <row r="150" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A150" s="2" t="s">
         <v>275</v>
       </c>
@@ -4907,7 +4910,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="151" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:4" ht="75" x14ac:dyDescent="0.25">
       <c r="A151" s="2" t="s">
         <v>289</v>
       </c>
@@ -4918,7 +4921,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="152" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A152" s="2" t="s">
         <v>306</v>
       </c>
@@ -4932,7 +4935,7 @@
         <v>428</v>
       </c>
     </row>
-    <row r="153" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A153" s="2" t="s">
         <v>309</v>
       </c>
@@ -4946,7 +4949,7 @@
         <v>429</v>
       </c>
     </row>
-    <row r="154" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A154" s="2" t="s">
         <v>310</v>
       </c>
@@ -4960,7 +4963,7 @@
         <v>430</v>
       </c>
     </row>
-    <row r="155" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A155" s="2" t="s">
         <v>315</v>
       </c>
@@ -4974,7 +4977,7 @@
         <v>431</v>
       </c>
     </row>
-    <row r="156" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A156" s="2" t="s">
         <v>317</v>
       </c>
@@ -4988,7 +4991,7 @@
         <v>432</v>
       </c>
     </row>
-    <row r="157" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A157" s="2" t="s">
         <v>319</v>
       </c>
@@ -5002,7 +5005,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="158" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A158" s="2" t="s">
         <v>448</v>
       </c>
@@ -5016,7 +5019,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="159" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A159" s="2" t="s">
         <v>449</v>
       </c>
@@ -5030,7 +5033,7 @@
         <v>451</v>
       </c>
     </row>
-    <row r="160" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A160" s="2" t="s">
         <v>475</v>
       </c>
@@ -5044,7 +5047,7 @@
         <v>569</v>
       </c>
     </row>
-    <row r="161" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A161" s="2" t="s">
         <v>478</v>
       </c>
@@ -5058,7 +5061,7 @@
         <v>568</v>
       </c>
     </row>
-    <row r="162" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A162" s="2" t="s">
         <v>480</v>
       </c>
@@ -5072,7 +5075,7 @@
         <v>567</v>
       </c>
     </row>
-    <row r="163" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A163" s="2" t="s">
         <v>483</v>
       </c>
@@ -5086,7 +5089,7 @@
         <v>566</v>
       </c>
     </row>
-    <row r="164" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A164" s="2" t="s">
         <v>486</v>
       </c>
@@ -5100,7 +5103,7 @@
         <v>565</v>
       </c>
     </row>
-    <row r="165" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A165" s="2" t="s">
         <v>489</v>
       </c>
@@ -5114,7 +5117,7 @@
         <v>564</v>
       </c>
     </row>
-    <row r="166" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A166" s="2" t="s">
         <v>538</v>
       </c>
@@ -5128,7 +5131,7 @@
         <v>539</v>
       </c>
     </row>
-    <row r="167" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A167" s="2" t="s">
         <v>540</v>
       </c>
@@ -5142,7 +5145,7 @@
         <v>542</v>
       </c>
     </row>
-    <row r="168" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A168" s="2" t="s">
         <v>492</v>
       </c>
@@ -5156,7 +5159,7 @@
         <v>563</v>
       </c>
     </row>
-    <row r="169" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A169" s="2" t="s">
         <v>495</v>
       </c>
@@ -5170,7 +5173,7 @@
         <v>562</v>
       </c>
     </row>
-    <row r="170" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A170" s="2" t="s">
         <v>498</v>
       </c>
@@ -5184,7 +5187,7 @@
         <v>561</v>
       </c>
     </row>
-    <row r="171" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A171" s="2" t="s">
         <v>501</v>
       </c>
@@ -5198,7 +5201,7 @@
         <v>560</v>
       </c>
     </row>
-    <row r="172" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A172" s="2" t="s">
         <v>503</v>
       </c>
@@ -5212,7 +5215,7 @@
         <v>559</v>
       </c>
     </row>
-    <row r="173" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A173" s="2" t="s">
         <v>505</v>
       </c>
@@ -5226,7 +5229,7 @@
         <v>558</v>
       </c>
     </row>
-    <row r="174" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A174" s="2" t="s">
         <v>507</v>
       </c>
@@ -5240,7 +5243,7 @@
         <v>557</v>
       </c>
     </row>
-    <row r="175" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A175" s="2" t="s">
         <v>570</v>
       </c>
@@ -5251,7 +5254,7 @@
         <v>609</v>
       </c>
     </row>
-    <row r="176" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A176" s="2" t="s">
         <v>572</v>
       </c>
@@ -5262,7 +5265,7 @@
         <v>610</v>
       </c>
     </row>
-    <row r="177" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A177" s="2" t="s">
         <v>574</v>
       </c>
@@ -5273,7 +5276,7 @@
         <v>611</v>
       </c>
     </row>
-    <row r="178" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A178" s="2" t="s">
         <v>576</v>
       </c>
@@ -5284,7 +5287,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="179" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A179" s="2" t="s">
         <v>578</v>
       </c>
@@ -5295,7 +5298,7 @@
         <v>613</v>
       </c>
     </row>
-    <row r="180" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A180" s="2" t="s">
         <v>580</v>
       </c>
@@ -5306,7 +5309,7 @@
         <v>614</v>
       </c>
     </row>
-    <row r="181" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A181" s="2" t="s">
         <v>582</v>
       </c>
@@ -5317,7 +5320,7 @@
         <v>615</v>
       </c>
     </row>
-    <row r="182" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A182" s="2" t="s">
         <v>584</v>
       </c>
@@ -5328,7 +5331,7 @@
         <v>616</v>
       </c>
     </row>
-    <row r="183" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A183" s="2" t="s">
         <v>586</v>
       </c>
@@ -5339,7 +5342,7 @@
         <v>617</v>
       </c>
     </row>
-    <row r="184" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A184" s="2" t="s">
         <v>588</v>
       </c>
@@ -5350,7 +5353,7 @@
         <v>618</v>
       </c>
     </row>
-    <row r="185" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A185" s="2" t="s">
         <v>620</v>
       </c>
@@ -5361,7 +5364,7 @@
         <v>622</v>
       </c>
     </row>
-    <row r="186" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A186" s="2" t="s">
         <v>623</v>
       </c>
@@ -5372,7 +5375,7 @@
         <v>624</v>
       </c>
     </row>
-    <row r="187" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A187" s="2" t="s">
         <v>625</v>
       </c>
@@ -5383,7 +5386,7 @@
         <v>627</v>
       </c>
     </row>
-    <row r="188" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A188" s="2" t="s">
         <v>626</v>
       </c>
@@ -5394,7 +5397,7 @@
         <v>628</v>
       </c>
     </row>
-    <row r="189" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A189" s="2" t="s">
         <v>629</v>
       </c>
@@ -5405,7 +5408,7 @@
         <v>631</v>
       </c>
     </row>
-    <row r="190" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A190" s="2" t="s">
         <v>632</v>
       </c>
@@ -5416,7 +5419,7 @@
         <v>634</v>
       </c>
     </row>
-    <row r="191" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A191" s="2" t="s">
         <v>638</v>
       </c>
@@ -5427,7 +5430,7 @@
         <v>640</v>
       </c>
     </row>
-    <row r="192" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A192" s="2" t="s">
         <v>641</v>
       </c>
@@ -5438,7 +5441,7 @@
         <v>642</v>
       </c>
     </row>
-    <row r="193" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A193" s="2" t="s">
         <v>643</v>
       </c>
@@ -5449,7 +5452,7 @@
         <v>645</v>
       </c>
     </row>
-    <row r="194" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="194" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A194" s="2" t="s">
         <v>646</v>
       </c>
@@ -5460,7 +5463,7 @@
         <v>648</v>
       </c>
     </row>
-    <row r="195" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A195" s="2" t="s">
         <v>649</v>
       </c>
@@ -5471,7 +5474,7 @@
         <v>651</v>
       </c>
     </row>
-    <row r="196" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A196" s="2" t="s">
         <v>652</v>
       </c>
@@ -5482,7 +5485,7 @@
         <v>654</v>
       </c>
     </row>
-    <row r="197" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A197" s="2" t="s">
         <v>655</v>
       </c>
@@ -5493,7 +5496,7 @@
         <v>656</v>
       </c>
     </row>
-    <row r="198" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="198" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A198" s="2" t="s">
         <v>657</v>
       </c>
@@ -5504,7 +5507,7 @@
         <v>659</v>
       </c>
     </row>
-    <row r="199" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="199" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A199" s="2" t="s">
         <v>666</v>
       </c>
@@ -5515,7 +5518,7 @@
         <v>668</v>
       </c>
     </row>
-    <row r="200" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="200" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A200" s="2" t="s">
         <v>669</v>
       </c>
@@ -5526,7 +5529,7 @@
         <v>671</v>
       </c>
     </row>
-    <row r="201" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="201" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A201" s="2" t="s">
         <v>675</v>
       </c>
@@ -5537,7 +5540,7 @@
         <v>677</v>
       </c>
     </row>
-    <row r="202" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A202" s="2" t="s">
         <v>678</v>
       </c>
@@ -5548,7 +5551,7 @@
         <v>680</v>
       </c>
     </row>
-    <row r="203" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="203" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A203" s="2" t="s">
         <v>681</v>
       </c>
@@ -5559,7 +5562,7 @@
         <v>683</v>
       </c>
     </row>
-    <row r="204" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="204" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A204" s="2" t="s">
         <v>684</v>
       </c>
@@ -5570,7 +5573,7 @@
         <v>686</v>
       </c>
     </row>
-    <row r="205" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="205" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A205" s="2" t="s">
         <v>687</v>
       </c>
@@ -5581,7 +5584,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="206" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="206" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A206" s="2" t="s">
         <v>690</v>
       </c>
@@ -5592,7 +5595,7 @@
         <v>704</v>
       </c>
     </row>
-    <row r="207" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="207" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A207" s="2" t="s">
         <v>691</v>
       </c>
@@ -5603,7 +5606,7 @@
         <v>710</v>
       </c>
     </row>
-    <row r="208" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="208" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A208" s="2" t="s">
         <v>693</v>
       </c>
@@ -5614,7 +5617,7 @@
         <v>705</v>
       </c>
     </row>
-    <row r="209" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="209" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A209" s="2" t="s">
         <v>692</v>
       </c>
@@ -5625,7 +5628,7 @@
         <v>706</v>
       </c>
     </row>
-    <row r="210" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="210" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A210" s="2" t="s">
         <v>699</v>
       </c>
@@ -5636,7 +5639,7 @@
         <v>707</v>
       </c>
     </row>
-    <row r="211" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="211" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A211" s="2" t="s">
         <v>700</v>
       </c>
@@ -5647,7 +5650,7 @@
         <v>708</v>
       </c>
     </row>
-    <row r="212" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="212" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A212" s="2" t="s">
         <v>701</v>
       </c>
@@ -5658,7 +5661,7 @@
         <v>709</v>
       </c>
     </row>
-    <row r="213" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="213" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A213" s="2" t="s">
         <v>711</v>
       </c>
@@ -5669,7 +5672,7 @@
         <v>712</v>
       </c>
     </row>
-    <row r="214" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="214" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A214" s="2" t="s">
         <v>713</v>
       </c>
@@ -5680,7 +5683,7 @@
         <v>715</v>
       </c>
     </row>
-    <row r="215" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="215" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A215" s="2" t="s">
         <v>716</v>
       </c>
@@ -5691,7 +5694,7 @@
         <v>718</v>
       </c>
     </row>
-    <row r="216" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="216" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A216" s="2" t="s">
         <v>719</v>
       </c>
@@ -5702,7 +5705,7 @@
         <v>721</v>
       </c>
     </row>
-    <row r="217" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="217" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A217" s="2" t="s">
         <v>732</v>
       </c>
@@ -5713,7 +5716,7 @@
         <v>736</v>
       </c>
     </row>
-    <row r="218" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="218" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A218" s="2" t="s">
         <v>734</v>
       </c>
@@ -5724,7 +5727,7 @@
         <v>737</v>
       </c>
     </row>
-    <row r="219" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="219" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A219" s="2" t="s">
         <v>728</v>
       </c>
@@ -5735,7 +5738,7 @@
         <v>738</v>
       </c>
     </row>
-    <row r="220" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="220" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A220" s="2" t="s">
         <v>730</v>
       </c>
@@ -5746,7 +5749,7 @@
         <v>739</v>
       </c>
     </row>
-    <row r="221" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="221" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A221" s="2" t="s">
         <v>743</v>
       </c>
@@ -5757,7 +5760,7 @@
         <v>744</v>
       </c>
     </row>
-    <row r="222" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="222" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A222" s="2" t="s">
         <v>745</v>
       </c>
@@ -5768,7 +5771,7 @@
         <v>747</v>
       </c>
     </row>
-    <row r="223" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="223" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A223" s="2" t="s">
         <v>751</v>
       </c>
@@ -5779,7 +5782,7 @@
         <v>753</v>
       </c>
     </row>
-    <row r="224" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="224" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A224" s="2" t="s">
         <v>754</v>
       </c>
@@ -5790,7 +5793,7 @@
         <v>756</v>
       </c>
     </row>
-    <row r="225" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="225" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A225" s="2" t="s">
         <v>757</v>
       </c>
@@ -5801,7 +5804,7 @@
         <v>759</v>
       </c>
     </row>
-    <row r="226" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="226" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A226" s="2" t="s">
         <v>760</v>
       </c>
@@ -5812,7 +5815,7 @@
         <v>762</v>
       </c>
     </row>
-    <row r="227" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="227" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A227" s="2" t="s">
         <v>763</v>
       </c>
@@ -5823,7 +5826,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="228" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="228" spans="1:3" ht="60" x14ac:dyDescent="0.25">
       <c r="A228" s="2" t="s">
         <v>766</v>
       </c>
@@ -5834,7 +5837,7 @@
         <v>768</v>
       </c>
     </row>
-    <row r="229" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="229" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A229" s="2" t="s">
         <v>769</v>
       </c>
@@ -5845,7 +5848,7 @@
         <v>770</v>
       </c>
     </row>
-    <row r="230" spans="1:3" ht="216" x14ac:dyDescent="0.3">
+    <row r="230" spans="1:3" ht="225" x14ac:dyDescent="0.25">
       <c r="A230" s="2" t="s">
         <v>774</v>
       </c>
@@ -5853,7 +5856,7 @@
         <v>775</v>
       </c>
     </row>
-    <row r="231" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="231" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A231" s="2" t="s">
         <v>788</v>
       </c>
@@ -5864,28 +5867,33 @@
         <v>790</v>
       </c>
     </row>
-    <row r="232" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A232" s="2" t="s">
+    <row r="233" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A233" s="2" t="s">
+        <v>797</v>
+      </c>
+    </row>
+    <row r="234" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A234" s="2" t="s">
+        <v>794</v>
+      </c>
+      <c r="B234" s="2" t="s">
         <v>791</v>
       </c>
-      <c r="B232" s="2" t="s">
-        <v>794</v>
-      </c>
-    </row>
-    <row r="233" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A233" s="2" t="s">
+    </row>
+    <row r="235" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A235" s="2" t="s">
+        <v>795</v>
+      </c>
+      <c r="B235" s="2" t="s">
         <v>792</v>
       </c>
-      <c r="B233" s="2" t="s">
-        <v>795</v>
-      </c>
-    </row>
-    <row r="234" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A234" s="2" t="s">
+    </row>
+    <row r="236" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A236" s="2" t="s">
+        <v>796</v>
+      </c>
+      <c r="B236" s="2" t="s">
         <v>793</v>
-      </c>
-      <c r="B234" s="2" t="s">
-        <v>796</v>
       </c>
     </row>
   </sheetData>
@@ -5898,9 +5906,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE0107E6-A156-44A0-947B-0BE38822807A}">
   <dimension ref="A1:D171"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -5914,7 +5922,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>160</v>
       </c>
@@ -5928,7 +5936,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>123</v>
       </c>
@@ -5942,7 +5950,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>126</v>
       </c>
@@ -5956,7 +5964,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>129</v>
       </c>
@@ -5970,7 +5978,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>132</v>
       </c>
@@ -5984,7 +5992,7 @@
         <v>326</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>135</v>
       </c>
@@ -5998,7 +6006,7 @@
         <v>327</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>67</v>
       </c>
@@ -6012,7 +6020,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>5</v>
       </c>
@@ -6026,7 +6034,7 @@
         <v>329</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>7</v>
       </c>
@@ -6040,7 +6048,7 @@
         <v>330</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -6054,7 +6062,7 @@
         <v>331</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>11</v>
       </c>
@@ -6068,7 +6076,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>13</v>
       </c>
@@ -6082,7 +6090,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>15</v>
       </c>
@@ -6096,7 +6104,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>17</v>
       </c>
@@ -6110,7 +6118,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>19</v>
       </c>
@@ -6124,7 +6132,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>21</v>
       </c>
@@ -6138,7 +6146,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>23</v>
       </c>
@@ -6152,7 +6160,7 @@
         <v>338</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>25</v>
       </c>
@@ -6166,7 +6174,7 @@
         <v>339</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>27</v>
       </c>
@@ -6180,7 +6188,7 @@
         <v>340</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>29</v>
       </c>
@@ -6194,7 +6202,7 @@
         <v>341</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>31</v>
       </c>
@@ -6208,7 +6216,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>33</v>
       </c>
@@ -6222,7 +6230,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>35</v>
       </c>
@@ -6236,7 +6244,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>37</v>
       </c>
@@ -6250,7 +6258,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>39</v>
       </c>
@@ -6264,7 +6272,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>41</v>
       </c>
@@ -6278,7 +6286,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>43</v>
       </c>
@@ -6292,7 +6300,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>45</v>
       </c>
@@ -6306,7 +6314,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>47</v>
       </c>
@@ -6320,7 +6328,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>49</v>
       </c>
@@ -6334,7 +6342,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>51</v>
       </c>
@@ -6348,7 +6356,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>53</v>
       </c>
@@ -6362,7 +6370,7 @@
         <v>353</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>55</v>
       </c>
@@ -6376,7 +6384,7 @@
         <v>354</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>57</v>
       </c>
@@ -6390,7 +6398,7 @@
         <v>355</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>59</v>
       </c>
@@ -6404,7 +6412,7 @@
         <v>356</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>61</v>
       </c>
@@ -6418,7 +6426,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>63</v>
       </c>
@@ -6432,7 +6440,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>65</v>
       </c>
@@ -6446,7 +6454,7 @@
         <v>359</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>280</v>
       </c>
@@ -6460,7 +6468,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>283</v>
       </c>
@@ -6474,7 +6482,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>286</v>
       </c>
@@ -6488,7 +6496,7 @@
         <v>362</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>303</v>
       </c>
@@ -6502,7 +6510,7 @@
         <v>363</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>440</v>
       </c>
@@ -6516,7 +6524,7 @@
         <v>553</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>442</v>
       </c>
@@ -6530,7 +6538,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>452</v>
       </c>
@@ -6544,7 +6552,7 @@
         <v>454</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>455</v>
       </c>
@@ -6558,7 +6566,7 @@
         <v>457</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>464</v>
       </c>
@@ -6572,7 +6580,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>467</v>
       </c>
@@ -6586,7 +6594,7 @@
         <v>555</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>470</v>
       </c>
@@ -6600,7 +6608,7 @@
         <v>556</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>509</v>
       </c>
@@ -6611,7 +6619,7 @@
         <v>511</v>
       </c>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>515</v>
       </c>
@@ -6622,7 +6630,7 @@
         <v>517</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>526</v>
       </c>
@@ -6633,7 +6641,7 @@
         <v>528</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>529</v>
       </c>
@@ -6644,7 +6652,7 @@
         <v>531</v>
       </c>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>546</v>
       </c>
@@ -6655,7 +6663,7 @@
         <v>548</v>
       </c>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>549</v>
       </c>
@@ -6666,7 +6674,7 @@
         <v>551</v>
       </c>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>543</v>
       </c>
@@ -6677,7 +6685,7 @@
         <v>545</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>69</v>
       </c>
@@ -6691,7 +6699,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>443</v>
       </c>
@@ -6702,7 +6710,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>456</v>
       </c>
@@ -6713,7 +6721,7 @@
         <v>457</v>
       </c>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>105</v>
       </c>
@@ -6727,7 +6735,7 @@
         <v>365</v>
       </c>
     </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>106</v>
       </c>
@@ -6741,7 +6749,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>107</v>
       </c>
@@ -6755,7 +6763,7 @@
         <v>367</v>
       </c>
     </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>108</v>
       </c>
@@ -6769,7 +6777,7 @@
         <v>365</v>
       </c>
     </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>110</v>
       </c>
@@ -6783,7 +6791,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>114</v>
       </c>
@@ -6797,7 +6805,7 @@
         <v>368</v>
       </c>
     </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>117</v>
       </c>
@@ -6811,7 +6819,7 @@
         <v>369</v>
       </c>
     </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>118</v>
       </c>
@@ -6825,7 +6833,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>445</v>
       </c>
@@ -6839,7 +6847,7 @@
         <v>447</v>
       </c>
     </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>512</v>
       </c>
@@ -6850,7 +6858,7 @@
         <v>514</v>
       </c>
     </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>518</v>
       </c>
@@ -6861,7 +6869,7 @@
         <v>520</v>
       </c>
     </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>521</v>
       </c>
@@ -6872,7 +6880,7 @@
         <v>523</v>
       </c>
     </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>532</v>
       </c>
@@ -6883,7 +6891,7 @@
         <v>534</v>
       </c>
     </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>537</v>
       </c>
@@ -6894,7 +6902,7 @@
         <v>536</v>
       </c>
     </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>154</v>
       </c>
@@ -6908,7 +6916,7 @@
         <v>371</v>
       </c>
     </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>164</v>
       </c>
@@ -6922,7 +6930,7 @@
         <v>372</v>
       </c>
     </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>157</v>
       </c>
@@ -6936,7 +6944,7 @@
         <v>373</v>
       </c>
     </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>167</v>
       </c>
@@ -6950,7 +6958,7 @@
         <v>374</v>
       </c>
     </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>141</v>
       </c>
@@ -6964,7 +6972,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>144</v>
       </c>
@@ -6978,7 +6986,7 @@
         <v>376</v>
       </c>
     </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>153</v>
       </c>
@@ -6992,7 +7000,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>147</v>
       </c>
@@ -7006,7 +7014,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>150</v>
       </c>
@@ -7020,7 +7028,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>172</v>
       </c>
@@ -7034,7 +7042,7 @@
         <v>379</v>
       </c>
     </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>173</v>
       </c>
@@ -7048,7 +7056,7 @@
         <v>380</v>
       </c>
     </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>176</v>
       </c>
@@ -7062,7 +7070,7 @@
         <v>381</v>
       </c>
     </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>178</v>
       </c>
@@ -7076,7 +7084,7 @@
         <v>382</v>
       </c>
     </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>180</v>
       </c>
@@ -7090,7 +7098,7 @@
         <v>383</v>
       </c>
     </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>243</v>
       </c>
@@ -7104,7 +7112,7 @@
         <v>384</v>
       </c>
     </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>138</v>
       </c>
@@ -7118,7 +7126,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>182</v>
       </c>
@@ -7132,7 +7140,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>184</v>
       </c>
@@ -7146,7 +7154,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>186</v>
       </c>
@@ -7160,7 +7168,7 @@
         <v>388</v>
       </c>
     </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>188</v>
       </c>
@@ -7174,7 +7182,7 @@
         <v>389</v>
       </c>
     </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>190</v>
       </c>
@@ -7188,7 +7196,7 @@
         <v>390</v>
       </c>
     </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>192</v>
       </c>
@@ -7202,7 +7210,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>434</v>
       </c>
@@ -7219,7 +7227,7 @@
         <v>#NAME?</v>
       </c>
     </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>437</v>
       </c>
@@ -7236,7 +7244,7 @@
         <v>#NAME?</v>
       </c>
     </row>
-    <row r="99" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>473</v>
       </c>
@@ -7253,7 +7261,7 @@
         <v>#NAME?</v>
       </c>
     </row>
-    <row r="100" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>195</v>
       </c>
@@ -7267,7 +7275,7 @@
         <v>392</v>
       </c>
     </row>
-    <row r="101" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>198</v>
       </c>
@@ -7281,7 +7289,7 @@
         <v>393</v>
       </c>
     </row>
-    <row r="102" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>201</v>
       </c>
@@ -7295,7 +7303,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="103" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>203</v>
       </c>
@@ -7309,7 +7317,7 @@
         <v>395</v>
       </c>
     </row>
-    <row r="104" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
         <v>205</v>
       </c>
@@ -7323,7 +7331,7 @@
         <v>396</v>
       </c>
     </row>
-    <row r="105" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
         <v>206</v>
       </c>
@@ -7337,7 +7345,7 @@
         <v>397</v>
       </c>
     </row>
-    <row r="106" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
         <v>209</v>
       </c>
@@ -7351,7 +7359,7 @@
         <v>398</v>
       </c>
     </row>
-    <row r="107" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
         <v>212</v>
       </c>
@@ -7365,7 +7373,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="108" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
         <v>215</v>
       </c>
@@ -7379,7 +7387,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="109" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
         <v>220</v>
       </c>
@@ -7393,7 +7401,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="110" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
         <v>292</v>
       </c>
@@ -7407,7 +7415,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="111" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
         <v>294</v>
       </c>
@@ -7421,7 +7429,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="112" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
         <v>297</v>
       </c>
@@ -7435,7 +7443,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="113" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
         <v>221</v>
       </c>
@@ -7449,7 +7457,7 @@
         <v>405</v>
       </c>
     </row>
-    <row r="114" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
         <v>223</v>
       </c>
@@ -7463,7 +7471,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="115" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
         <v>226</v>
       </c>
@@ -7477,7 +7485,7 @@
         <v>407</v>
       </c>
     </row>
-    <row r="116" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
         <v>229</v>
       </c>
@@ -7491,7 +7499,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="117" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
         <v>230</v>
       </c>
@@ -7505,7 +7513,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="118" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
         <v>232</v>
       </c>
@@ -7519,7 +7527,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="119" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
         <v>234</v>
       </c>
@@ -7533,7 +7541,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="120" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
         <v>237</v>
       </c>
@@ -7547,7 +7555,7 @@
         <v>412</v>
       </c>
     </row>
-    <row r="121" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
         <v>300</v>
       </c>
@@ -7561,7 +7569,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="122" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
         <v>240</v>
       </c>
@@ -7575,7 +7583,7 @@
         <v>414</v>
       </c>
     </row>
-    <row r="123" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
         <v>244</v>
       </c>
@@ -7589,7 +7597,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="124" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
         <v>245</v>
       </c>
@@ -7603,7 +7611,7 @@
         <v>416</v>
       </c>
     </row>
-    <row r="125" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
         <v>247</v>
       </c>
@@ -7617,7 +7625,7 @@
         <v>417</v>
       </c>
     </row>
-    <row r="126" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
         <v>249</v>
       </c>
@@ -7631,7 +7639,7 @@
         <v>418</v>
       </c>
     </row>
-    <row r="127" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
         <v>253</v>
       </c>
@@ -7645,7 +7653,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="128" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
         <v>256</v>
       </c>
@@ -7659,7 +7667,7 @@
         <v>420</v>
       </c>
     </row>
-    <row r="129" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
         <v>259</v>
       </c>
@@ -7673,7 +7681,7 @@
         <v>421</v>
       </c>
     </row>
-    <row r="130" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
         <v>262</v>
       </c>
@@ -7687,7 +7695,7 @@
         <v>422</v>
       </c>
     </row>
-    <row r="131" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
         <v>265</v>
       </c>
@@ -7701,7 +7709,7 @@
         <v>423</v>
       </c>
     </row>
-    <row r="132" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
         <v>266</v>
       </c>
@@ -7715,7 +7723,7 @@
         <v>424</v>
       </c>
     </row>
-    <row r="133" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
         <v>268</v>
       </c>
@@ -7729,7 +7737,7 @@
         <v>425</v>
       </c>
     </row>
-    <row r="134" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
         <v>270</v>
       </c>
@@ -7743,7 +7751,7 @@
         <v>426</v>
       </c>
     </row>
-    <row r="135" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
         <v>271</v>
       </c>
@@ -7757,7 +7765,7 @@
         <v>427</v>
       </c>
     </row>
-    <row r="136" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
         <v>274</v>
       </c>
@@ -7768,7 +7776,7 @@
         <v>279</v>
       </c>
     </row>
-    <row r="137" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
         <v>275</v>
       </c>
@@ -7779,7 +7787,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="138" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
         <v>289</v>
       </c>
@@ -7790,7 +7798,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="139" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
         <v>306</v>
       </c>
@@ -7804,7 +7812,7 @@
         <v>428</v>
       </c>
     </row>
-    <row r="140" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
         <v>309</v>
       </c>
@@ -7818,7 +7826,7 @@
         <v>429</v>
       </c>
     </row>
-    <row r="141" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
         <v>310</v>
       </c>
@@ -7832,7 +7840,7 @@
         <v>430</v>
       </c>
     </row>
-    <row r="142" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
         <v>315</v>
       </c>
@@ -7846,7 +7854,7 @@
         <v>431</v>
       </c>
     </row>
-    <row r="143" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
         <v>317</v>
       </c>
@@ -7860,7 +7868,7 @@
         <v>432</v>
       </c>
     </row>
-    <row r="144" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
         <v>319</v>
       </c>
@@ -7874,7 +7882,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="145" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
         <v>448</v>
       </c>
@@ -7888,7 +7896,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="146" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
         <v>449</v>
       </c>
@@ -7902,7 +7910,7 @@
         <v>451</v>
       </c>
     </row>
-    <row r="147" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
         <v>475</v>
       </c>
@@ -7916,7 +7924,7 @@
         <v>569</v>
       </c>
     </row>
-    <row r="148" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
         <v>478</v>
       </c>
@@ -7930,7 +7938,7 @@
         <v>568</v>
       </c>
     </row>
-    <row r="149" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
         <v>480</v>
       </c>
@@ -7944,7 +7952,7 @@
         <v>567</v>
       </c>
     </row>
-    <row r="150" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
         <v>483</v>
       </c>
@@ -7958,7 +7966,7 @@
         <v>566</v>
       </c>
     </row>
-    <row r="151" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
         <v>486</v>
       </c>
@@ -7972,7 +7980,7 @@
         <v>565</v>
       </c>
     </row>
-    <row r="152" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
         <v>489</v>
       </c>
@@ -7986,7 +7994,7 @@
         <v>564</v>
       </c>
     </row>
-    <row r="153" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
         <v>538</v>
       </c>
@@ -7997,7 +8005,7 @@
         <v>539</v>
       </c>
     </row>
-    <row r="154" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
         <v>540</v>
       </c>
@@ -8008,7 +8016,7 @@
         <v>542</v>
       </c>
     </row>
-    <row r="155" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
         <v>492</v>
       </c>
@@ -8022,7 +8030,7 @@
         <v>563</v>
       </c>
     </row>
-    <row r="156" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
         <v>495</v>
       </c>
@@ -8036,7 +8044,7 @@
         <v>562</v>
       </c>
     </row>
-    <row r="157" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
         <v>498</v>
       </c>
@@ -8050,7 +8058,7 @@
         <v>561</v>
       </c>
     </row>
-    <row r="158" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
         <v>501</v>
       </c>
@@ -8064,7 +8072,7 @@
         <v>560</v>
       </c>
     </row>
-    <row r="159" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
         <v>503</v>
       </c>
@@ -8078,7 +8086,7 @@
         <v>559</v>
       </c>
     </row>
-    <row r="160" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
         <v>505</v>
       </c>
@@ -8092,7 +8100,7 @@
         <v>558</v>
       </c>
     </row>
-    <row r="161" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
         <v>507</v>
       </c>
@@ -8106,7 +8114,7 @@
         <v>557</v>
       </c>
     </row>
-    <row r="162" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
         <v>570</v>
       </c>
@@ -8114,7 +8122,7 @@
         <v>571</v>
       </c>
     </row>
-    <row r="163" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
         <v>572</v>
       </c>
@@ -8122,7 +8130,7 @@
         <v>573</v>
       </c>
     </row>
-    <row r="164" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
         <v>574</v>
       </c>
@@ -8130,7 +8138,7 @@
         <v>575</v>
       </c>
     </row>
-    <row r="165" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
         <v>576</v>
       </c>
@@ -8138,7 +8146,7 @@
         <v>577</v>
       </c>
     </row>
-    <row r="166" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
         <v>578</v>
       </c>
@@ -8146,7 +8154,7 @@
         <v>579</v>
       </c>
     </row>
-    <row r="167" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
         <v>580</v>
       </c>
@@ -8154,7 +8162,7 @@
         <v>581</v>
       </c>
     </row>
-    <row r="168" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
         <v>582</v>
       </c>
@@ -8162,7 +8170,7 @@
         <v>583</v>
       </c>
     </row>
-    <row r="169" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
         <v>584</v>
       </c>
@@ -8170,7 +8178,7 @@
         <v>585</v>
       </c>
     </row>
-    <row r="170" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
         <v>586</v>
       </c>
@@ -8178,7 +8186,7 @@
         <v>587</v>
       </c>
     </row>
-    <row r="171" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A171" t="s">
         <v>588</v>
       </c>

</xml_diff>

<commit_message>
Added new "With Offset" checkbox for reloc triggers!
</commit_message>
<xml_diff>
--- a/Translations/Translations.xlsx
+++ b/Translations/Translations.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programacion\MelonLoader\FS_LevelEditor\Translations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01731B24-1764-4CA6-9FA2-28A0CB5C8F89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7EF9B84-F478-4BB0-AE50-7581EA2A73C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{F5C22481-FF1A-482C-BF7E-EB5A7718AF49}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1493" uniqueCount="798">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1496" uniqueCount="801">
   <si>
     <t>ID</t>
   </si>
@@ -2436,6 +2436,15 @@
   </si>
   <si>
     <t># Broken translations in the main game.</t>
+  </si>
+  <si>
+    <t>WithOffset</t>
+  </si>
+  <si>
+    <t>With Offset</t>
+  </si>
+  <si>
+    <t>Compensar Diferencia</t>
   </si>
 </sst>
 </file>
@@ -2846,7 +2855,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6961A5F-F8EA-4989-8112-A0ACE51D011E}">
   <sheetPr codeName="Hoja1"/>
-  <dimension ref="A1:D236"/>
+  <dimension ref="A1:D237"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="37" style="2" customWidth="1"/>
@@ -5867,32 +5876,43 @@
         <v>790</v>
       </c>
     </row>
-    <row r="233" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A233" s="2" t="s">
-        <v>797</v>
+    <row r="232" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A232" s="2" t="s">
+        <v>798</v>
+      </c>
+      <c r="B232" s="2" t="s">
+        <v>799</v>
+      </c>
+      <c r="C232" s="2" t="s">
+        <v>800</v>
       </c>
     </row>
     <row r="234" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A234" s="2" t="s">
-        <v>794</v>
-      </c>
-      <c r="B234" s="2" t="s">
-        <v>791</v>
+        <v>797</v>
       </c>
     </row>
     <row r="235" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A235" s="2" t="s">
-        <v>795</v>
+        <v>794</v>
       </c>
       <c r="B235" s="2" t="s">
-        <v>792</v>
+        <v>791</v>
       </c>
     </row>
     <row r="236" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A236" s="2" t="s">
+        <v>795</v>
+      </c>
+      <c r="B236" s="2" t="s">
+        <v>792</v>
+      </c>
+    </row>
+    <row r="237" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A237" s="2" t="s">
         <v>796</v>
       </c>
-      <c r="B236" s="2" t="s">
+      <c r="B237" s="2" t="s">
         <v>793</v>
       </c>
     </row>

</xml_diff>